<commit_message>
Grade Cidade Jardim: mosaicos Bisazza (PA49) em alta resolução na aba IMAGENS ESPECIFICAÇÕES
- Painel (New Sterlizia, Narciso e degradê) e pilar do Espaço Termas com as imagens enviadas pelo usuário

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PQR4X6TCfpk7hYXx3JGbK9
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -4108,7 +4108,7 @@
       <row>12</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="1428750" cy="1428750"/>
+    <ext cx="1438275" cy="1428750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -4183,7 +4183,7 @@
       <row>13</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="1476375" cy="1428750"/>
+    <ext cx="1495425" cy="1428750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -4204,7 +4204,7 @@
   <oneCellAnchor>
     <from>
       <col>5</col>
-      <colOff>1609725</colOff>
+      <colOff>1628775</colOff>
       <row>13</row>
       <rowOff>95250</rowOff>
     </from>

</xml_diff>

<commit_message>
Grade Cidade Jardim: chuveiro D70 e monocomando D33 em alta resolução
- Foto e desenho técnico do chuveiro Docol Eden (D70) e do monocomando Mix&Match (D33) do Vestiário Termas, enviados pelo usuário

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PQR4X6TCfpk7hYXx3JGbK9
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -4433,7 +4433,7 @@
       <row>14</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="1485900" cy="1428750"/>
+    <ext cx="1476375" cy="1428750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="22" name="Image 22" descr="Picture"/>
@@ -4454,11 +4454,11 @@
   <oneCellAnchor>
     <from>
       <col>15</col>
-      <colOff>1619250</colOff>
+      <colOff>1609725</colOff>
       <row>14</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="2381250" cy="1428750"/>
+    <ext cx="2419350" cy="1428750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="23" name="Image 23" descr="Picture"/>
@@ -4508,7 +4508,7 @@
       <row>15</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="1428750" cy="1428750"/>
+    <ext cx="1419225" cy="1428750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -4529,11 +4529,11 @@
   <oneCellAnchor>
     <from>
       <col>15</col>
-      <colOff>1562100</colOff>
+      <colOff>1552575</colOff>
       <row>15</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="1390650" cy="1428750"/>
+    <ext cx="1419225" cy="1428750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>

</xml_diff>

<commit_message>
Grade Cidade Jardim: cores no padrão EPO
- Faixas pretas em verde-escuro EPO (#243F2E), linha GERAL em #2A7050, cabeçalhos em #E2E2E2, coluna de ambientes em #F2F2F2, aviso em verde claro
- Cores tiradas da planilha de histogramas enviada como modelo EPO; legenda INFO. REVISADA mantida

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -360,13 +360,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
+        <fgColor rgb="FFE2E2E2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.09997863704336681"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -378,31 +378,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1"/>
+        <fgColor rgb="FF243F2E"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.249977111117893"/>
+        <fgColor rgb="FF2A7050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
+        <fgColor rgb="FFC5DFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003A7D22"/>
+        <fgColor rgb="FF243F2E"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>

<commit_message>
Grade Cidade Jardim: especificações conflitantes em vermelho claro
Vestiários do Bar Piscina mantêm as duas versões (lista R04 e pranchas
37/38) na bancada e na torneira; legenda INFO. CONFLITANTE nas abas de
pavimento. D27 (porta papel higiênico) sai de Portas para Outros
Complementares.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -32,7 +32,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;* #,##0.00_-;\-&quot;R$&quot;* #,##0.00_-;_-&quot;R$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="57">
+  <fonts count="59">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -376,8 +376,19 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color rgb="FF9C0006"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="FF9C0006"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -429,6 +440,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF243F2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1344,7 +1360,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="281">
+  <cellXfs count="284">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -2098,6 +2114,13 @@
     </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="57" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="58" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6028,8 +6051,12 @@
       <c r="G9" s="7" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="8" t="n"/>
-      <c r="J9" s="193" t="n"/>
-      <c r="K9" s="193" t="n"/>
+      <c r="J9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="K9" s="229" t="n"/>
       <c r="L9" s="10" t="n"/>
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="10" t="n"/>
@@ -6038,8 +6065,12 @@
       <c r="Q9" s="10" t="n"/>
       <c r="R9" s="10" t="n"/>
       <c r="S9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
+      <c r="T9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="U9" s="229" t="n"/>
       <c r="V9" s="10" t="n"/>
       <c r="W9" s="10" t="n"/>
       <c r="X9" s="10" t="n"/>
@@ -6049,8 +6080,12 @@
       <c r="AB9" s="10" t="n"/>
       <c r="AC9" s="10" t="n"/>
       <c r="AD9" s="10" t="n"/>
-      <c r="AE9" s="10" t="n"/>
-      <c r="AF9" s="10" t="n"/>
+      <c r="AE9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="AF9" s="229" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -6951,14 +6986,14 @@
       <c r="W28" s="35" t="n"/>
       <c r="X28" s="269" t="inlineStr">
         <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
-D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y28" s="31" t="n"/>
       <c r="Z28" s="269" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -7643,7 +7678,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="31">
     <mergeCell ref="L10:U10"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="T5:U5"/>
@@ -7651,12 +7686,14 @@
     <mergeCell ref="AE1:AF4"/>
     <mergeCell ref="T1:U4"/>
     <mergeCell ref="A1:A4"/>
+    <mergeCell ref="J9:K9"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="L1:S4"/>
     <mergeCell ref="V10:Z10"/>
     <mergeCell ref="V5:AD6"/>
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="B5:I6"/>
+    <mergeCell ref="T9:U9"/>
     <mergeCell ref="AE8:AF8"/>
     <mergeCell ref="B7:I8"/>
     <mergeCell ref="V1:AD4"/>
@@ -7664,6 +7701,7 @@
     <mergeCell ref="B12:K12"/>
     <mergeCell ref="L7:S8"/>
     <mergeCell ref="T8:U8"/>
+    <mergeCell ref="AE9:AF9"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="T6:U6"/>
     <mergeCell ref="J1:K4"/>
@@ -8064,8 +8102,12 @@
       <c r="G9" s="7" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="8" t="n"/>
-      <c r="J9" s="193" t="n"/>
-      <c r="K9" s="193" t="n"/>
+      <c r="J9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="K9" s="229" t="n"/>
       <c r="L9" s="10" t="n"/>
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="10" t="n"/>
@@ -8074,8 +8116,12 @@
       <c r="Q9" s="10" t="n"/>
       <c r="R9" s="10" t="n"/>
       <c r="S9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
+      <c r="T9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="U9" s="229" t="n"/>
       <c r="V9" s="10" t="n"/>
       <c r="W9" s="10" t="n"/>
       <c r="X9" s="10" t="n"/>
@@ -8085,8 +8131,12 @@
       <c r="AB9" s="10" t="n"/>
       <c r="AC9" s="10" t="n"/>
       <c r="AD9" s="10" t="n"/>
-      <c r="AE9" s="10" t="n"/>
-      <c r="AF9" s="10" t="n"/>
+      <c r="AE9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="AF9" s="229" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -8823,7 +8873,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="31">
     <mergeCell ref="L10:U10"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="T5:U5"/>
@@ -8831,12 +8881,14 @@
     <mergeCell ref="AE1:AF4"/>
     <mergeCell ref="T1:U4"/>
     <mergeCell ref="A1:A4"/>
+    <mergeCell ref="J9:K9"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="L1:S4"/>
     <mergeCell ref="V10:Z10"/>
     <mergeCell ref="V5:AD6"/>
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="B5:I6"/>
+    <mergeCell ref="T9:U9"/>
     <mergeCell ref="AE8:AF8"/>
     <mergeCell ref="B7:I8"/>
     <mergeCell ref="V1:AD4"/>
@@ -8844,6 +8896,7 @@
     <mergeCell ref="B12:K12"/>
     <mergeCell ref="L7:S8"/>
     <mergeCell ref="T8:U8"/>
+    <mergeCell ref="AE9:AF9"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="T6:U6"/>
     <mergeCell ref="J1:K4"/>
@@ -9254,8 +9307,12 @@
       <c r="G9" s="7" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="8" t="n"/>
-      <c r="J9" s="193" t="n"/>
-      <c r="K9" s="193" t="n"/>
+      <c r="J9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="K9" s="229" t="n"/>
       <c r="L9" s="10" t="n"/>
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="10" t="n"/>
@@ -9264,8 +9321,12 @@
       <c r="Q9" s="10" t="n"/>
       <c r="R9" s="10" t="n"/>
       <c r="S9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
+      <c r="T9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="U9" s="229" t="n"/>
       <c r="V9" s="10" t="n"/>
       <c r="W9" s="10" t="n"/>
       <c r="X9" s="10" t="n"/>
@@ -9275,8 +9336,12 @@
       <c r="AB9" s="10" t="n"/>
       <c r="AC9" s="10" t="n"/>
       <c r="AD9" s="10" t="n"/>
-      <c r="AE9" s="10" t="n"/>
-      <c r="AF9" s="10" t="n"/>
+      <c r="AE9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="AF9" s="229" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -9756,14 +9821,14 @@
       <c r="W17" s="32" t="n"/>
       <c r="X17" s="269" t="inlineStr">
         <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
-D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
+          <t>D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y17" s="31" t="n"/>
       <c r="Z17" s="278" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -9835,14 +9900,14 @@
       <c r="W18" s="32" t="n"/>
       <c r="X18" s="269" t="inlineStr">
         <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
-D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
+          <t>D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y18" s="31" t="n"/>
       <c r="Z18" s="278" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -10110,14 +10175,14 @@
       <c r="W23" s="35" t="n"/>
       <c r="X23" s="269" t="inlineStr">
         <is>
-          <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
-D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco</t>
+          <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y23" s="31" t="n"/>
       <c r="Z23" s="277" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -10190,14 +10255,14 @@
       <c r="W24" s="35" t="n"/>
       <c r="X24" s="269" t="inlineStr">
         <is>
-          <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
-D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco</t>
+          <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y24" s="35" t="n"/>
       <c r="Z24" s="277" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -10739,9 +10804,10 @@
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J35" s="277" t="inlineStr">
-        <is>
-          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
+      <c r="J35" s="283" t="inlineStr">
+        <is>
+          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
         </is>
       </c>
       <c r="K35" s="246" t="inlineStr">
@@ -10752,9 +10818,10 @@
       <c r="L35" s="35" t="n"/>
       <c r="M35" s="37" t="n"/>
       <c r="N35" s="38" t="n"/>
-      <c r="O35" s="245" t="inlineStr">
-        <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
+      <c r="O35" s="283" t="inlineStr">
+        <is>
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
       <c r="P35" s="277" t="inlineStr">
@@ -10788,14 +10855,14 @@
       <c r="W35" s="35" t="n"/>
       <c r="X35" s="269" t="inlineStr">
         <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
-D32 - Divisórias e portas pivotantes com estrutura em alumínio e fechamento em vidro, cor Dark Beige. Ref.: Duo. Puxador tipo cava com fechaduras tipo rolete espelho modelo redondo acabamento cromo-acetinado.</t>
+          <t>D32 - Divisórias e portas pivotantes com estrutura em alumínio e fechamento em vidro, cor Dark Beige. Ref.: Duo. Puxador tipo cava com fechaduras tipo rolete espelho modelo redondo acabamento cromo-acetinado.</t>
         </is>
       </c>
       <c r="Y35" s="35" t="n"/>
       <c r="Z35" s="278" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -10832,9 +10899,10 @@
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J36" s="277" t="inlineStr">
-        <is>
-          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
+      <c r="J36" s="283" t="inlineStr">
+        <is>
+          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
         </is>
       </c>
       <c r="K36" s="246" t="inlineStr">
@@ -10845,9 +10913,10 @@
       <c r="L36" s="35" t="n"/>
       <c r="M36" s="37" t="n"/>
       <c r="N36" s="38" t="n"/>
-      <c r="O36" s="245" t="inlineStr">
-        <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
+      <c r="O36" s="283" t="inlineStr">
+        <is>
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
       <c r="P36" s="277" t="inlineStr">
@@ -10881,14 +10950,14 @@
       <c r="W36" s="35" t="n"/>
       <c r="X36" s="269" t="inlineStr">
         <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
-D32 - Divisórias e portas pivotantes com estrutura em alumínio e fechamento em vidro, cor Dark Beige. Ref.: Duo. Puxador tipo cava com fechaduras tipo rolete espelho modelo redondo acabamento cromo-acetinado.</t>
+          <t>D32 - Divisórias e portas pivotantes com estrutura em alumínio e fechamento em vidro, cor Dark Beige. Ref.: Duo. Puxador tipo cava com fechaduras tipo rolete espelho modelo redondo acabamento cromo-acetinado.</t>
         </is>
       </c>
       <c r="Y36" s="35" t="n"/>
       <c r="Z36" s="278" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -11565,15 +11634,12 @@
         </is>
       </c>
       <c r="W48" s="35" t="n"/>
-      <c r="X48" s="269" t="inlineStr">
-        <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco</t>
-        </is>
-      </c>
+      <c r="X48" s="269" t="n"/>
       <c r="Y48" s="35" t="n"/>
       <c r="Z48" s="270" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -11663,15 +11729,12 @@
         </is>
       </c>
       <c r="W49" s="35" t="n"/>
-      <c r="X49" s="269" t="inlineStr">
-        <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco</t>
-        </is>
-      </c>
+      <c r="X49" s="269" t="n"/>
       <c r="Y49" s="35" t="n"/>
       <c r="Z49" s="270" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -12019,15 +12082,15 @@
       <c r="W55" s="35" t="n"/>
       <c r="X55" s="269" t="inlineStr">
         <is>
-          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
-D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
+          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
 D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y55" s="35" t="n"/>
       <c r="Z55" s="278" t="inlineStr">
         <is>
-          <t>D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
+          <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
+D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
@@ -12385,7 +12448,7 @@
     </row>
     <row r="64" ht="2.1" customHeight="1"/>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="31">
     <mergeCell ref="L10:U10"/>
     <mergeCell ref="B10:K10"/>
     <mergeCell ref="J5:K5"/>
@@ -12394,11 +12457,13 @@
     <mergeCell ref="AE1:AF4"/>
     <mergeCell ref="T1:U4"/>
     <mergeCell ref="A1:A4"/>
+    <mergeCell ref="J9:K9"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="L1:S4"/>
     <mergeCell ref="V10:Z10"/>
     <mergeCell ref="V5:AD6"/>
     <mergeCell ref="B5:I6"/>
+    <mergeCell ref="T9:U9"/>
     <mergeCell ref="AE8:AF8"/>
     <mergeCell ref="B7:I8"/>
     <mergeCell ref="V1:AD4"/>
@@ -12406,6 +12471,7 @@
     <mergeCell ref="B12:K12"/>
     <mergeCell ref="L7:S8"/>
     <mergeCell ref="T8:U8"/>
+    <mergeCell ref="AE9:AF9"/>
     <mergeCell ref="J1:K4"/>
     <mergeCell ref="T6:U6"/>
     <mergeCell ref="AE6:AF6"/>

</xml_diff>

<commit_message>
Grade Cidade Jardim: aba APTO TIPO
Tabela JARDIM-ACABAMENTOS R01 e detalhamento CDJ_DET_EX PR001-PR008,
CDJ-ARQ-DT PR406/407 e PR721-728 (halls de serviço dos andares);
divergências entre tabela e detalhamento em vermelho claro.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -10,8 +10,9 @@
     <sheet name="TÉRREO " sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2° PAVTO" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="PILOTIS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="IMAGENS ESPECIFICAÇÕES " sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="PENDÊNCIAS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="APTO TIPO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="IMAGENS ESPECIFICAÇÕES " sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PENDÊNCIAS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'TÉRREO '!$1:$11,'TÉRREO '!$A:$A</definedName>
@@ -20,8 +21,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">'2° PAVTO'!$A$1:$AF$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'PILOTIS'!$1:$11,'PILOTIS'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'PILOTIS'!$A$1:$AF$63</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'IMAGENS ESPECIFICAÇÕES '!$1:$11,'IMAGENS ESPECIFICAÇÕES '!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'IMAGENS ESPECIFICAÇÕES '!$A$1:$U$26</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'IMAGENS ESPECIFICAÇÕES '!$1:$11,'IMAGENS ESPECIFICAÇÕES '!$A:$A</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'IMAGENS ESPECIFICAÇÕES '!$A$1:$U$26</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +33,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;* #,##0.00_-;\-&quot;R$&quot;* #,##0.00_-;_-&quot;R$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="60">
+  <fonts count="61">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -393,6 +394,12 @@
       <color rgb="FF9C0006"/>
       <sz val="16"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color rgb="FF9C0006"/>
+      <sz val="48"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1367,7 +1374,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="288">
+  <cellXfs count="289">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -2138,6 +2145,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="60" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3919,6 +3929,548 @@
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>1368136</colOff>
+      <row>7</row>
+      <rowOff>454083</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Imagem 1"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="3414278" y="2501610"/>
+          <a:ext cx="935183" cy="924273"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>0</col>
+      <colOff>831275</colOff>
+      <row>0</row>
+      <rowOff>103909</rowOff>
+    </from>
+    <to>
+      <col>0</col>
+      <colOff>2753592</colOff>
+      <row>3</row>
+      <rowOff>335785</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Imagem 6"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill rotWithShape="1">
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:srcRect b="16485"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="831275" y="103909"/>
+          <a:ext cx="1922317" cy="1470126"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>9</col>
+      <colOff>2247902</colOff>
+      <row>0</row>
+      <rowOff>100446</rowOff>
+    </from>
+    <to>
+      <col>10</col>
+      <colOff>1780310</colOff>
+      <row>3</row>
+      <rowOff>332322</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Imagem 7"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill rotWithShape="1">
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:srcRect b="16485"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="25650827" y="100446"/>
+          <a:ext cx="1913658" cy="1470126"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>19</col>
+      <colOff>1513612</colOff>
+      <row>0</row>
+      <rowOff>128154</rowOff>
+    </from>
+    <to>
+      <col>20</col>
+      <colOff>1046020</colOff>
+      <row>4</row>
+      <rowOff>2843</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Imagem 8"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill rotWithShape="1">
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:srcRect b="16485"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="49910137" y="128154"/>
+          <a:ext cx="1913658" cy="1470126"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>30</col>
+      <colOff>1437412</colOff>
+      <row>0</row>
+      <rowOff>69272</rowOff>
+    </from>
+    <to>
+      <col>31</col>
+      <colOff>969820</colOff>
+      <row>3</row>
+      <rowOff>301148</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Imagem 9"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill rotWithShape="1">
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:srcRect b="16485"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="76218187" y="69272"/>
+          <a:ext cx="1913658" cy="1470126"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="944708"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Imagem 2"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="29779478" y="2501610"/>
+          <a:ext cx="935183" cy="944708"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="944708"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Imagem 3"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="53591978" y="2501610"/>
+          <a:ext cx="935183" cy="944708"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="927787"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Imagem 4"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="29779478" y="2501610"/>
+          <a:ext cx="935183" cy="927787"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="927787"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Imagem 5"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="53591978" y="2501610"/>
+          <a:ext cx="935183" cy="927787"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="921675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Imagem 10"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="29779478" y="2501610"/>
+          <a:ext cx="935183" cy="921675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="921675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Imagem 11"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="53591978" y="2501610"/>
+          <a:ext cx="935183" cy="921675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="944708"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Imagem 12"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="53591978" y="2501610"/>
+          <a:ext cx="935183" cy="944708"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="927787"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Imagem 13"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="53591978" y="2501610"/>
+          <a:ext cx="935183" cy="927787"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>432953</colOff>
+      <row>6</row>
+      <rowOff>34635</rowOff>
+    </from>
+    <ext cx="935183" cy="921675"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Imagem 14"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm flipH="1">
+          <a:off x="53591978" y="2501610"/>
+          <a:ext cx="935183" cy="921675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
       <colOff>394853</colOff>
       <row>4</row>
       <rowOff>72735</rowOff>
@@ -9787,9 +10339,6 @@
       <c r="Y31" s="31" t="n"/>
       <c r="Z31" s="35" t="n"/>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
     <row r="35">
       <c r="S35" s="3" t="inlineStr">
         <is>
@@ -13515,6 +14064,1649 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AF35"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
+  <cols>
+    <col width="50.140625" customWidth="1" style="14" min="1" max="1"/>
+    <col width="56.28515625" customWidth="1" style="3" min="2" max="2"/>
+    <col width="35.7109375" customWidth="1" style="3" min="3" max="10"/>
+    <col width="53.42578125" customWidth="1" style="3" min="11" max="11"/>
+    <col width="35.7109375" customWidth="1" style="3" min="12" max="25"/>
+    <col width="38.5703125" customWidth="1" style="3" min="26" max="26"/>
+    <col width="35.7109375" customWidth="1" style="3" min="27" max="32"/>
+    <col width="9.140625" customWidth="1" style="3" min="33" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34.5" customHeight="1">
+      <c r="A1" s="153" t="n"/>
+      <c r="B1" s="137" t="inlineStr">
+        <is>
+          <t>GRADE DE ESPECIFICAÇÕES – APARTAMENTO TIPO
+EDIFÍCIO JARDIM</t>
+        </is>
+      </c>
+      <c r="C1" s="209" t="n"/>
+      <c r="D1" s="209" t="n"/>
+      <c r="E1" s="209" t="n"/>
+      <c r="F1" s="209" t="n"/>
+      <c r="G1" s="209" t="n"/>
+      <c r="H1" s="209" t="n"/>
+      <c r="I1" s="208" t="n"/>
+      <c r="J1" s="113" t="n"/>
+      <c r="K1" s="208" t="n"/>
+      <c r="L1" s="137">
+        <f>B1</f>
+        <v/>
+      </c>
+      <c r="M1" s="209" t="n"/>
+      <c r="N1" s="209" t="n"/>
+      <c r="O1" s="209" t="n"/>
+      <c r="P1" s="209" t="n"/>
+      <c r="Q1" s="209" t="n"/>
+      <c r="R1" s="209" t="n"/>
+      <c r="S1" s="208" t="n"/>
+      <c r="T1" s="113" t="n"/>
+      <c r="U1" s="208" t="n"/>
+      <c r="V1" s="137">
+        <f>B1</f>
+        <v/>
+      </c>
+      <c r="W1" s="209" t="n"/>
+      <c r="X1" s="209" t="n"/>
+      <c r="Y1" s="209" t="n"/>
+      <c r="Z1" s="209" t="n"/>
+      <c r="AA1" s="209" t="n"/>
+      <c r="AB1" s="209" t="n"/>
+      <c r="AC1" s="209" t="n"/>
+      <c r="AD1" s="208" t="n"/>
+      <c r="AE1" s="113" t="n"/>
+      <c r="AF1" s="208" t="n"/>
+    </row>
+    <row r="2" ht="28.5" customHeight="1">
+      <c r="A2" s="238" t="n"/>
+      <c r="B2" s="210" t="n"/>
+      <c r="I2" s="211" t="n"/>
+      <c r="J2" s="210" t="n"/>
+      <c r="K2" s="211" t="n"/>
+      <c r="L2" s="210" t="n"/>
+      <c r="S2" s="211" t="n"/>
+      <c r="T2" s="210" t="n"/>
+      <c r="U2" s="211" t="n"/>
+      <c r="V2" s="210" t="n"/>
+      <c r="AD2" s="211" t="n"/>
+      <c r="AE2" s="210" t="n"/>
+      <c r="AF2" s="211" t="n"/>
+    </row>
+    <row r="3" ht="34.5" customHeight="1">
+      <c r="A3" s="238" t="n"/>
+      <c r="B3" s="210" t="n"/>
+      <c r="I3" s="211" t="n"/>
+      <c r="J3" s="210" t="n"/>
+      <c r="K3" s="211" t="n"/>
+      <c r="L3" s="210" t="n"/>
+      <c r="S3" s="211" t="n"/>
+      <c r="T3" s="210" t="n"/>
+      <c r="U3" s="211" t="n"/>
+      <c r="V3" s="210" t="n"/>
+      <c r="AD3" s="211" t="n"/>
+      <c r="AE3" s="210" t="n"/>
+      <c r="AF3" s="211" t="n"/>
+    </row>
+    <row r="4" ht="28.5" customHeight="1" thickBot="1">
+      <c r="A4" s="239" t="n"/>
+      <c r="B4" s="213" t="n"/>
+      <c r="C4" s="216" t="n"/>
+      <c r="D4" s="216" t="n"/>
+      <c r="E4" s="216" t="n"/>
+      <c r="F4" s="216" t="n"/>
+      <c r="G4" s="216" t="n"/>
+      <c r="H4" s="216" t="n"/>
+      <c r="I4" s="214" t="n"/>
+      <c r="J4" s="213" t="n"/>
+      <c r="K4" s="214" t="n"/>
+      <c r="L4" s="213" t="n"/>
+      <c r="M4" s="216" t="n"/>
+      <c r="N4" s="216" t="n"/>
+      <c r="O4" s="216" t="n"/>
+      <c r="P4" s="216" t="n"/>
+      <c r="Q4" s="216" t="n"/>
+      <c r="R4" s="216" t="n"/>
+      <c r="S4" s="214" t="n"/>
+      <c r="T4" s="213" t="n"/>
+      <c r="U4" s="214" t="n"/>
+      <c r="V4" s="213" t="n"/>
+      <c r="W4" s="216" t="n"/>
+      <c r="X4" s="216" t="n"/>
+      <c r="Y4" s="216" t="n"/>
+      <c r="Z4" s="216" t="n"/>
+      <c r="AA4" s="216" t="n"/>
+      <c r="AB4" s="216" t="n"/>
+      <c r="AC4" s="216" t="n"/>
+      <c r="AD4" s="214" t="n"/>
+      <c r="AE4" s="213" t="n"/>
+      <c r="AF4" s="214" t="n"/>
+    </row>
+    <row r="5" ht="39.95" customHeight="1">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="127" t="inlineStr">
+        <is>
+          <t>PADRÃO DE FORMATAÇÃO: ITEM, LINHA, MARCA, TAMANHO, COR E/OU ACABAMENTOS. CÓDIGO. COR DE REJUNTE.</t>
+        </is>
+      </c>
+      <c r="C5" s="209" t="n"/>
+      <c r="D5" s="209" t="n"/>
+      <c r="E5" s="209" t="n"/>
+      <c r="F5" s="209" t="n"/>
+      <c r="G5" s="209" t="n"/>
+      <c r="H5" s="209" t="n"/>
+      <c r="I5" s="208" t="n"/>
+      <c r="J5" s="119" t="inlineStr">
+        <is>
+          <t>XXXXXXX</t>
+        </is>
+      </c>
+      <c r="K5" s="240" t="n"/>
+      <c r="L5" s="127" t="inlineStr">
+        <is>
+          <t>*ATENÇÃO: PARA TODOS OS REJUNTES, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO
+COM PROJETOS EXECUTIVOS DE ACORDO COM ALTURA DO CONTRAPISO</t>
+        </is>
+      </c>
+      <c r="M5" s="209" t="n"/>
+      <c r="N5" s="209" t="n"/>
+      <c r="O5" s="209" t="n"/>
+      <c r="P5" s="209" t="n"/>
+      <c r="Q5" s="209" t="n"/>
+      <c r="R5" s="209" t="n"/>
+      <c r="S5" s="208" t="n"/>
+      <c r="T5" s="119" t="inlineStr">
+        <is>
+          <t>XXXXXX</t>
+        </is>
+      </c>
+      <c r="U5" s="240" t="n"/>
+      <c r="V5" s="127" t="inlineStr">
+        <is>
+          <t>*ATENÇÃO: PARA TODOS OS REJUNTES, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO
+COM PROJETOS EXECUTIVOS DE ACORDO COM ALTURA DO CONTRAPISO</t>
+        </is>
+      </c>
+      <c r="W5" s="209" t="n"/>
+      <c r="X5" s="209" t="n"/>
+      <c r="Y5" s="209" t="n"/>
+      <c r="Z5" s="209" t="n"/>
+      <c r="AA5" s="209" t="n"/>
+      <c r="AB5" s="209" t="n"/>
+      <c r="AC5" s="209" t="n"/>
+      <c r="AD5" s="208" t="n"/>
+      <c r="AE5" s="119" t="inlineStr">
+        <is>
+          <t>XXXXXX</t>
+        </is>
+      </c>
+      <c r="AF5" s="240" t="n"/>
+    </row>
+    <row r="6" ht="28.5" customFormat="1" customHeight="1" s="4" thickBot="1">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="B6" s="213" t="n"/>
+      <c r="C6" s="216" t="n"/>
+      <c r="D6" s="216" t="n"/>
+      <c r="E6" s="216" t="n"/>
+      <c r="F6" s="216" t="n"/>
+      <c r="G6" s="216" t="n"/>
+      <c r="H6" s="216" t="n"/>
+      <c r="I6" s="214" t="n"/>
+      <c r="J6" s="201" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL</t>
+        </is>
+      </c>
+      <c r="K6" s="221" t="n"/>
+      <c r="L6" s="213" t="n"/>
+      <c r="M6" s="216" t="n"/>
+      <c r="N6" s="216" t="n"/>
+      <c r="O6" s="216" t="n"/>
+      <c r="P6" s="216" t="n"/>
+      <c r="Q6" s="216" t="n"/>
+      <c r="R6" s="216" t="n"/>
+      <c r="S6" s="214" t="n"/>
+      <c r="T6" s="201" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL</t>
+        </is>
+      </c>
+      <c r="U6" s="221" t="n"/>
+      <c r="V6" s="213" t="n"/>
+      <c r="W6" s="216" t="n"/>
+      <c r="X6" s="216" t="n"/>
+      <c r="Y6" s="216" t="n"/>
+      <c r="Z6" s="216" t="n"/>
+      <c r="AA6" s="216" t="n"/>
+      <c r="AB6" s="216" t="n"/>
+      <c r="AC6" s="216" t="n"/>
+      <c r="AD6" s="214" t="n"/>
+      <c r="AE6" s="201" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL</t>
+        </is>
+      </c>
+      <c r="AF6" s="221" t="n"/>
+    </row>
+    <row r="7" ht="39.95" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>REV. R00</t>
+        </is>
+      </c>
+      <c r="B7" s="131" t="inlineStr">
+        <is>
+          <t>*ATENÇÃO: PARA TODOS OS REJUNTES E TEXTURAS, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO ARQUITETURA DE ACORDO COM ALTURA DO CONTRAPISO. A DEFINIÇÃO DA ALTURA DE RODABANCAS E TESTEIRAS DEVEM SER DEFINIDAS CASO A CASO CONFORME IMAGENS E/OU ELEMENTOS DO PROJETO, COMO PEITORIL E PAGINAÇÃO DA PAREDE. QUANDO O REVESTIMENTO DA PAREDE NÃO FOR CERÂMICO, CONSIDERAR UMA ALTURA MAIOR DE RODABANCA. AS ESPECIFICAÇÕES PODERAM SER ALTERADAS CONFORME DISPONIBILIDADE DE MERCADO, VALIDAR JUNTO A ARQUITETURA CASO NO MOMENTO DA COMPRA O ITEM TENHA SAÍDO DE LINHA.</t>
+        </is>
+      </c>
+      <c r="C7" s="209" t="n"/>
+      <c r="D7" s="209" t="n"/>
+      <c r="E7" s="209" t="n"/>
+      <c r="F7" s="209" t="n"/>
+      <c r="G7" s="209" t="n"/>
+      <c r="H7" s="209" t="n"/>
+      <c r="I7" s="208" t="n"/>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFO. ANTERIOR </t>
+        </is>
+      </c>
+      <c r="K7" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFO. REVISADA </t>
+        </is>
+      </c>
+      <c r="L7" s="131" t="inlineStr">
+        <is>
+          <t>*ATENÇÃO: PARA TODOS OS REJUNTES E TEXTURAS, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO ARQUITETURA DE ACORDO COM ALTURA DO CONTRAPISO. A DEFINIÇÃO DA ALTURA DE RODABANCAS E TESTEIRAS DEVEM SER DEFINIDAS CASO A CASO CONFORME IMAGENS E/OU ELEMENTOS DO PROJETO, COMO PEITORIL E PAGINAÇÃO DA PAREDE. QUANDO O REVESTIMENTO DA PAREDE NÃO FOR CERÂMICO, CONSIDERAR UMA ALTURA MAIOR DE RODABANCA. AS ESPECIFICAÇÕES PODERAM SER ALTERADAS CONFORME DISPONIBILIDADE DE MERCADO, VALIDAR JUNTO A ARQUITETURA CASO NO MOMENTO DA COMPRA O ITEM TENHA SAÍDO DE LINHA.</t>
+        </is>
+      </c>
+      <c r="M7" s="209" t="n"/>
+      <c r="N7" s="209" t="n"/>
+      <c r="O7" s="209" t="n"/>
+      <c r="P7" s="209" t="n"/>
+      <c r="Q7" s="209" t="n"/>
+      <c r="R7" s="209" t="n"/>
+      <c r="S7" s="208" t="n"/>
+      <c r="T7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFO. ANTERIOR </t>
+        </is>
+      </c>
+      <c r="U7" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFO. REVISADA </t>
+        </is>
+      </c>
+      <c r="V7" s="146" t="inlineStr">
+        <is>
+          <t>*ATENÇÃO: PARA TODOS OS REJUNTES E TEXTURAS, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO ARQUITETURA DE ACORDO COM ALTURA DO CONTRAPISO. A DEFINIÇÃO DA ALTURA DE RODABANCAS E TESTEIRAS DEVEM SER DEFINIDAS CASO A CASO CONFORME IMAGENS E/OU ELEMENTOS DO PROJETO, COMO PEITORIL E PAGINAÇÃO DA PAREDE. QUANDO O REVESTIMENTO DA PAREDE NÃO FOR CERÂMICO, CONSIDERAR UMA ALTURA MAIOR DE RODABANCA. AS ESPECIFICAÇÕES PODERAM SER ALTERADAS CONFORME DISPONIBILIDADE DE MERCADO, VALIDAR JUNTO A ARQUITETURA CASO NO MOMENTO DA COMPRA O ITEM TENHA SAÍDO DE LINHA.</t>
+        </is>
+      </c>
+      <c r="W7" s="209" t="n"/>
+      <c r="X7" s="209" t="n"/>
+      <c r="Y7" s="209" t="n"/>
+      <c r="Z7" s="209" t="n"/>
+      <c r="AA7" s="209" t="n"/>
+      <c r="AB7" s="209" t="n"/>
+      <c r="AC7" s="209" t="n"/>
+      <c r="AD7" s="208" t="n"/>
+      <c r="AE7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFO. ANTERIOR </t>
+        </is>
+      </c>
+      <c r="AF7" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INFO. REVISADA </t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60.75" customFormat="1" customHeight="1" s="4" thickBot="1">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>REVISÃO</t>
+        </is>
+      </c>
+      <c r="B8" s="213" t="n"/>
+      <c r="C8" s="216" t="n"/>
+      <c r="D8" s="216" t="n"/>
+      <c r="E8" s="216" t="n"/>
+      <c r="F8" s="216" t="n"/>
+      <c r="G8" s="216" t="n"/>
+      <c r="H8" s="216" t="n"/>
+      <c r="I8" s="214" t="n"/>
+      <c r="J8" s="121" t="inlineStr">
+        <is>
+          <t>LEGENDA</t>
+        </is>
+      </c>
+      <c r="K8" s="221" t="n"/>
+      <c r="L8" s="213" t="n"/>
+      <c r="M8" s="216" t="n"/>
+      <c r="N8" s="216" t="n"/>
+      <c r="O8" s="216" t="n"/>
+      <c r="P8" s="216" t="n"/>
+      <c r="Q8" s="216" t="n"/>
+      <c r="R8" s="216" t="n"/>
+      <c r="S8" s="214" t="n"/>
+      <c r="T8" s="121" t="inlineStr">
+        <is>
+          <t>LEGENDA</t>
+        </is>
+      </c>
+      <c r="U8" s="221" t="n"/>
+      <c r="V8" s="213" t="n"/>
+      <c r="W8" s="216" t="n"/>
+      <c r="X8" s="216" t="n"/>
+      <c r="Y8" s="216" t="n"/>
+      <c r="Z8" s="216" t="n"/>
+      <c r="AA8" s="216" t="n"/>
+      <c r="AB8" s="216" t="n"/>
+      <c r="AC8" s="216" t="n"/>
+      <c r="AD8" s="214" t="n"/>
+      <c r="AE8" s="121" t="inlineStr">
+        <is>
+          <t>LEGENDA</t>
+        </is>
+      </c>
+      <c r="AF8" s="221" t="n"/>
+    </row>
+    <row r="9" ht="14.1" customFormat="1" customHeight="1" s="6">
+      <c r="A9" s="5" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="K9" s="229" t="n"/>
+      <c r="L9" s="10" t="n"/>
+      <c r="M9" s="10" t="n"/>
+      <c r="N9" s="10" t="n"/>
+      <c r="O9" s="11" t="n"/>
+      <c r="P9" s="11" t="n"/>
+      <c r="Q9" s="10" t="n"/>
+      <c r="R9" s="10" t="n"/>
+      <c r="S9" s="10" t="n"/>
+      <c r="T9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="U9" s="229" t="n"/>
+      <c r="V9" s="10" t="n"/>
+      <c r="W9" s="10" t="n"/>
+      <c r="X9" s="10" t="n"/>
+      <c r="Y9" s="10" t="n"/>
+      <c r="Z9" s="11" t="n"/>
+      <c r="AA9" s="11" t="n"/>
+      <c r="AB9" s="10" t="n"/>
+      <c r="AC9" s="10" t="n"/>
+      <c r="AD9" s="10" t="n"/>
+      <c r="AE9" s="281" t="inlineStr">
+        <is>
+          <t>INFO. CONFLITANTE (manter as duas)</t>
+        </is>
+      </c>
+      <c r="AF9" s="229" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="152" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="C10" s="216" t="n"/>
+      <c r="D10" s="216" t="n"/>
+      <c r="E10" s="216" t="n"/>
+      <c r="F10" s="216" t="n"/>
+      <c r="G10" s="216" t="n"/>
+      <c r="H10" s="216" t="n"/>
+      <c r="I10" s="216" t="n"/>
+      <c r="J10" s="216" t="n"/>
+      <c r="K10" s="214" t="n"/>
+      <c r="L10" s="152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOUÇAS E METAIS </t>
+        </is>
+      </c>
+      <c r="M10" s="216" t="n"/>
+      <c r="N10" s="216" t="n"/>
+      <c r="O10" s="216" t="n"/>
+      <c r="P10" s="216" t="n"/>
+      <c r="Q10" s="216" t="n"/>
+      <c r="R10" s="216" t="n"/>
+      <c r="S10" s="216" t="n"/>
+      <c r="T10" s="216" t="n"/>
+      <c r="U10" s="214" t="n"/>
+      <c r="V10" s="152" t="inlineStr">
+        <is>
+          <t>COMPLEMENTARES</t>
+        </is>
+      </c>
+      <c r="W10" s="216" t="n"/>
+      <c r="X10" s="216" t="n"/>
+      <c r="Y10" s="216" t="n"/>
+      <c r="Z10" s="214" t="n"/>
+    </row>
+    <row r="11" ht="93.75" customFormat="1" customHeight="1" s="12" thickBot="1">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>CÔMODO/AMBIENTE</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>PISO/REJUNTE</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>SOLEIRA</t>
+        </is>
+      </c>
+      <c r="D11" s="46" t="inlineStr">
+        <is>
+          <t>FILETE</t>
+        </is>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>PEITORIL</t>
+        </is>
+      </c>
+      <c r="F11" s="46" t="inlineStr">
+        <is>
+          <t>RODAPÉ</t>
+        </is>
+      </c>
+      <c r="G11" s="46" t="inlineStr">
+        <is>
+          <t>SÓCULO</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>PAREDE/REJUNTE</t>
+        </is>
+      </c>
+      <c r="I11" s="46" t="inlineStr">
+        <is>
+          <t>TETO</t>
+        </is>
+      </c>
+      <c r="J11" s="46" t="inlineStr">
+        <is>
+          <t>BANCADA</t>
+        </is>
+      </c>
+      <c r="K11" s="46" t="inlineStr">
+        <is>
+          <t>OUTROS REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="L11" s="46" t="inlineStr">
+        <is>
+          <t>LOUÇAS, CUBAS E TANQUES</t>
+        </is>
+      </c>
+      <c r="M11" s="46" t="inlineStr">
+        <is>
+          <t>VÁLVULAS DE CUBAS E TANQUES</t>
+        </is>
+      </c>
+      <c r="N11" s="46" t="inlineStr">
+        <is>
+          <t>SIFÕES</t>
+        </is>
+      </c>
+      <c r="O11" s="46" t="inlineStr">
+        <is>
+          <t>TORNEIRAS</t>
+        </is>
+      </c>
+      <c r="P11" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> BACIAS SANITÁRIAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="46" t="inlineStr">
+        <is>
+          <t>DUCHAS HIGIÊNICAS</t>
+        </is>
+      </c>
+      <c r="R11" s="46" t="inlineStr">
+        <is>
+          <t>ACABAMENTOS DE REGISTROS GERAL</t>
+        </is>
+      </c>
+      <c r="S11" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACIONAMENTO DE CHUVEIRO </t>
+        </is>
+      </c>
+      <c r="T11" s="46" t="inlineStr">
+        <is>
+          <t>RALOS</t>
+        </is>
+      </c>
+      <c r="U11" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUTROS
+ LOUÇAS E METAIS </t>
+        </is>
+      </c>
+      <c r="V11" s="46" t="inlineStr">
+        <is>
+          <t>ACABAMENTOS ELÉTRICOS</t>
+        </is>
+      </c>
+      <c r="W11" s="46" t="inlineStr">
+        <is>
+          <t>MAÇANETAS</t>
+        </is>
+      </c>
+      <c r="X11" s="46" t="inlineStr">
+        <is>
+          <t>PORTAS</t>
+        </is>
+      </c>
+      <c r="Y11" s="46" t="inlineStr">
+        <is>
+          <t>JANELAS</t>
+        </is>
+      </c>
+      <c r="Z11" s="46" t="inlineStr">
+        <is>
+          <t>OUTROS
+COMPLEMENTARES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customFormat="1" customHeight="1" s="13" thickBot="1">
+      <c r="A12" s="51" t="n"/>
+      <c r="B12" s="124" t="inlineStr">
+        <is>
+          <t>GERAL — APARTAMENTO TIPO: TABELA JARDIM-ACABAMENTOS R01 E DETALHAMENTO CDJ_DET_EX PR001-PR008, CDJ-ARQ-DT PR406/407 E PR721-728</t>
+        </is>
+      </c>
+      <c r="C12" s="241" t="n"/>
+      <c r="D12" s="241" t="n"/>
+      <c r="E12" s="241" t="n"/>
+      <c r="F12" s="241" t="n"/>
+      <c r="G12" s="241" t="n"/>
+      <c r="H12" s="241" t="n"/>
+      <c r="I12" s="241" t="n"/>
+      <c r="J12" s="241" t="n"/>
+      <c r="K12" s="242" t="n"/>
+      <c r="L12" s="123" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="M12" s="241" t="n"/>
+      <c r="N12" s="241" t="n"/>
+      <c r="O12" s="241" t="n"/>
+      <c r="P12" s="241" t="n"/>
+      <c r="Q12" s="241" t="n"/>
+      <c r="R12" s="241" t="n"/>
+      <c r="S12" s="241" t="n"/>
+      <c r="T12" s="241" t="n"/>
+      <c r="U12" s="242" t="n"/>
+      <c r="V12" s="123" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="W12" s="241" t="n"/>
+      <c r="X12" s="241" t="n"/>
+      <c r="Y12" s="241" t="n"/>
+      <c r="Z12" s="242" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="45" t="inlineStr">
+        <is>
+          <t>SALA / VARANDA DA SALA</t>
+        </is>
+      </c>
+      <c r="B13" s="269" t="inlineStr">
+        <is>
+          <t>Piso em mármore travertino romano bruto, 85x130cm, paginação conforme detalhamento. Rejunte Infinity Hard, cor Areia ou Palha (validar com o Setor de Produto). (DET PR001/PR002; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="32" t="n"/>
+      <c r="F13" s="288" t="inlineStr">
+        <is>
+          <t>Rodapé em mármore travertino romano bruto, semi-embutido, h=15cm. (DET PR001/PR002)
+CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="n"/>
+      <c r="H13" s="271" t="inlineStr">
+        <is>
+          <t>Pintura acrílica cor branco neve, acabamento acetinado. (DET PR001; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I13" s="271" t="n"/>
+      <c r="J13" s="32" t="n"/>
+      <c r="K13" s="32" t="n"/>
+      <c r="L13" s="32" t="n"/>
+      <c r="M13" s="32" t="n"/>
+      <c r="N13" s="32" t="n"/>
+      <c r="O13" s="32" t="n"/>
+      <c r="P13" s="32" t="n"/>
+      <c r="Q13" s="32" t="n"/>
+      <c r="R13" s="32" t="n"/>
+      <c r="S13" s="32" t="n"/>
+      <c r="T13" s="32" t="inlineStr">
+        <is>
+          <t>Varanda: ralo linear oculto; caimento do piso para o ralo i=1%. (DET PR001)</t>
+        </is>
+      </c>
+      <c r="U13" s="32" t="n"/>
+      <c r="V13" s="32" t="n"/>
+      <c r="W13" s="32" t="n"/>
+      <c r="X13" s="31" t="n"/>
+      <c r="Y13" s="31" t="n"/>
+      <c r="Z13" s="32" t="inlineStr">
+        <is>
+          <t>Varanda: mureta h=90cm. (DET PR001)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="45" t="inlineStr">
+        <is>
+          <t>LAVABO</t>
+        </is>
+      </c>
+      <c r="B14" s="269" t="inlineStr">
+        <is>
+          <t>Piso em mármore travertino romano bruto. Rejunte Infinity Hard, cor Areia ou Palha (validar com o Setor de Produto). (DET PR004; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>Soleira indicada em planta, material não especificado. (DET PR004)</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="32" t="n"/>
+      <c r="F14" s="288" t="inlineStr">
+        <is>
+          <t>Rodapé semi-embutido em mármore travertino romano bruto, h=15cm. (DET PR004)
+CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+        </is>
+      </c>
+      <c r="G14" s="32" t="n"/>
+      <c r="H14" s="271" t="inlineStr">
+        <is>
+          <t>Pintura acrílica cor branco neve, acabamento acetinado. (DET PR004; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I14" s="271" t="inlineStr">
+        <is>
+          <t>Forro em gesso acartonado, pintura acrílica acetinada cor branco neve, tabica metálica. PD 298cm. (DET PR004)</t>
+        </is>
+      </c>
+      <c r="J14" s="32" t="inlineStr">
+        <is>
+          <t>Bancada esculpida em mármore travertino romano resinado (cuba esculpida). (DET PR004; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="K14" s="32" t="n"/>
+      <c r="L14" s="32" t="n"/>
+      <c r="M14" s="32" t="n"/>
+      <c r="N14" s="32" t="n"/>
+      <c r="O14" s="32" t="inlineStr">
+        <is>
+          <t>Torneira de mesa bica baixa para lavatório, cromado, linha Unic, cód. 1197.C90. Ref.: Deca. (DET PR004; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="P14" s="32" t="inlineStr">
+        <is>
+          <t>Bacia convencional suspensa branca, linha LK, cód. P.232.17. Ref.: Deca. Caixa de descarga embutida para alvenaria. (DET PR004; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="Q14" s="32" t="n"/>
+      <c r="R14" s="32" t="inlineStr">
+        <is>
+          <t>Acabamento para registro de gaveta 1 1/4" e 1 1/2", cromado, Unic, cód. 4900.C90.GD. Ref.: Deca
+Acabamento para caixa de descarga embutida, cromado, H Quadra Duo, cód. 4900.C.HQD.DUO. Ref.: Deca. (DET PR004)</t>
+        </is>
+      </c>
+      <c r="S14" s="32" t="n"/>
+      <c r="T14" s="32" t="inlineStr">
+        <is>
+          <t>Ralo oculto 15x15cm, tampa revestida com o mesmo mármore. (DET PR004)</t>
+        </is>
+      </c>
+      <c r="U14" s="32" t="n"/>
+      <c r="V14" s="32" t="n"/>
+      <c r="W14" s="32" t="inlineStr">
+        <is>
+          <t>Maçaneta Pado Sara, cromo acetinado, interna. (DET PR004)</t>
+        </is>
+      </c>
+      <c r="X14" s="31" t="inlineStr">
+        <is>
+          <t>Porta piso-forro, cor branca, alizar 10cm. (DET PR004)</t>
+        </is>
+      </c>
+      <c r="Y14" s="31" t="n"/>
+      <c r="Z14" s="32" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="45" t="inlineStr">
+        <is>
+          <t>BANHO SUÍTE MASTER</t>
+        </is>
+      </c>
+      <c r="B15" s="269" t="inlineStr">
+        <is>
+          <t>Piso em mármore travertino romano bruto resinado, paginado conforme detalhamento. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="n"/>
+      <c r="D15" s="32" t="n"/>
+      <c r="E15" s="32" t="n"/>
+      <c r="F15" s="32" t="n"/>
+      <c r="G15" s="32" t="n"/>
+      <c r="H15" s="271" t="inlineStr">
+        <is>
+          <t>Parede em mármore travertino romano bruto paginado. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I15" s="271" t="n"/>
+      <c r="J15" s="32" t="inlineStr">
+        <is>
+          <t>Bancada em mármore travertino romano resinado. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="K15" s="32" t="n"/>
+      <c r="L15" s="32" t="inlineStr">
+        <is>
+          <t>Cuba de apoio retangular Jader Almeida, branca. Ref.: Deca ou similar. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="M15" s="32" t="n"/>
+      <c r="N15" s="32" t="n"/>
+      <c r="O15" s="32" t="inlineStr">
+        <is>
+          <t>Misturador monocomando de mesa bica alta para lavatório, cromado, linha Level. Ref.: Deca ou similar. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="P15" s="32" t="inlineStr">
+        <is>
+          <t>Bacia convencional Carrara branca com caixa acoplada. Ref.: Deca ou similar
+Bidê 3 furos Carrara branco. Ref.: Deca ou similar. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="Q15" s="32" t="n"/>
+      <c r="R15" s="32" t="n"/>
+      <c r="S15" s="32" t="inlineStr">
+        <is>
+          <t>Acabamento de monocomando de chuveiro, cromado, linha Level. Ref.: Deca ou similar. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="T15" s="32" t="n"/>
+      <c r="U15" s="32" t="inlineStr">
+        <is>
+          <t>Misturador para bidê, cromado, linha Level. Ref.: Deca ou similar. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="V15" s="32" t="n"/>
+      <c r="W15" s="32" t="n"/>
+      <c r="X15" s="31" t="n"/>
+      <c r="Y15" s="31" t="n"/>
+      <c r="Z15" s="32" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="45" t="inlineStr">
+        <is>
+          <t>BANHO SUÍTES</t>
+        </is>
+      </c>
+      <c r="B16" s="269" t="inlineStr">
+        <is>
+          <t>Piso em mármore travertino romano bruto resinado, paginado. Rejunte Infinity Hard, cor Areia ou Palha (validar com o Setor de Produto). Desnível do box 1cm. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="32" t="n"/>
+      <c r="F16" s="32" t="n"/>
+      <c r="G16" s="32" t="n"/>
+      <c r="H16" s="271" t="inlineStr">
+        <is>
+          <t>Parede em mármore travertino romano bruto: piso ao teto na área do box e barrado semi-embutido até 110cm nas demais paredes; acima, pintura acrílica cor branco neve, acetinado. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I16" s="271" t="inlineStr">
+        <is>
+          <t>Forro em gesso acartonado, pintura acrílica acetinada cor branco neve, tabica metálica e sanca. PD 298cm. (DET PR008)</t>
+        </is>
+      </c>
+      <c r="J16" s="32" t="inlineStr">
+        <is>
+          <t>Bancada esculpida em mármore travertino romano resinado. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="K16" s="32" t="n"/>
+      <c r="L16" s="32" t="inlineStr">
+        <is>
+          <t>Cuba retangular de apoio 60cm com deck, branca, linha Slim, cód. L.13060.M.17. Ref.: Deca. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="M16" s="32" t="n"/>
+      <c r="N16" s="32" t="n"/>
+      <c r="O16" s="32" t="inlineStr">
+        <is>
+          <t>Misturador monocomando de mesa bica baixa para lavatório, cromado, linha Level, cód. 2875.C26. Ref.: Deca. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="P16" s="32" t="inlineStr">
+        <is>
+          <t>Bacia convencional Carrara branca com caixa acoplada, cód. KP.606.17. Ref.: Deca. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="Q16" s="32" t="inlineStr">
+        <is>
+          <t>Ducha higiênica com registro e derivação, cromada, linha Level. Ref.: Deca. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="R16" s="32" t="inlineStr">
+        <is>
+          <t>Acabamento para registro de gaveta 1 1/4" e 1 1/2", cromado, Level, cód. 4900.C26.GD. Ref.: Deca. (DET PR008)</t>
+        </is>
+      </c>
+      <c r="S16" s="32" t="inlineStr">
+        <is>
+          <t>Acabamento monocomando para chuveiro, cromado, linha Level, cód. 4993.C26.CHU. Ref.: Deca. (DET PR008; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="T16" s="32" t="inlineStr">
+        <is>
+          <t>Ralo oculto 15x15cm e ralo linear oculto 90x5cm, tampas revestidas com a mesma pedra. (DET PR008)</t>
+        </is>
+      </c>
+      <c r="U16" s="32" t="n"/>
+      <c r="V16" s="32" t="n"/>
+      <c r="W16" s="32" t="n"/>
+      <c r="X16" s="31" t="n"/>
+      <c r="Y16" s="31" t="n"/>
+      <c r="Z16" s="32" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="45" t="inlineStr">
+        <is>
+          <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
+        </is>
+      </c>
+      <c r="B17" s="269" t="inlineStr">
+        <is>
+          <t>Piso em cumaru, assoalho piso pronto. Ref.: Indusparquet. (DET PR001/PR002; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="n"/>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>Transição madeira x pedra: perfil metálico (DET 05) ou filete de mármore (DET 07). (DET PR001)</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="n"/>
+      <c r="F17" s="288" t="inlineStr">
+        <is>
+          <t>Rodapé maciço com o mesmo acabamento do piso, h=10cm. Ref.: Indusparquet. (Tab. R01; quadro do DET PR001)
+CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
+        </is>
+      </c>
+      <c r="G17" s="32" t="n"/>
+      <c r="H17" s="271" t="inlineStr">
+        <is>
+          <t>Pintura acrílica cor branco neve. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I17" s="271" t="n"/>
+      <c r="J17" s="32" t="n"/>
+      <c r="K17" s="32" t="n"/>
+      <c r="L17" s="32" t="n"/>
+      <c r="M17" s="32" t="n"/>
+      <c r="N17" s="32" t="n"/>
+      <c r="O17" s="32" t="n"/>
+      <c r="P17" s="32" t="n"/>
+      <c r="Q17" s="32" t="n"/>
+      <c r="R17" s="32" t="n"/>
+      <c r="S17" s="32" t="n"/>
+      <c r="T17" s="32" t="n"/>
+      <c r="U17" s="32" t="n"/>
+      <c r="V17" s="32" t="n"/>
+      <c r="W17" s="32" t="n"/>
+      <c r="X17" s="31" t="n"/>
+      <c r="Y17" s="31" t="n"/>
+      <c r="Z17" s="32" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="45" t="inlineStr">
+        <is>
+          <t>COPA NOTURNA</t>
+        </is>
+      </c>
+      <c r="B18" s="269" t="inlineStr">
+        <is>
+          <t>Piso em cumaru, assoalho piso pronto. Ref.: Indusparquet. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="32" t="n"/>
+      <c r="E18" s="32" t="n"/>
+      <c r="F18" s="32" t="inlineStr">
+        <is>
+          <t>Rodapé maciço com o mesmo acabamento do piso, h=10cm. Ref.: Indusparquet. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="n"/>
+      <c r="H18" s="271" t="n"/>
+      <c r="I18" s="271" t="n"/>
+      <c r="J18" s="288" t="inlineStr">
+        <is>
+          <t>Bancada esculpida em mármore travertino romano resinado. (DET PR003)
+CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
+        </is>
+      </c>
+      <c r="K18" s="32" t="n"/>
+      <c r="L18" s="32" t="inlineStr">
+        <is>
+          <t>Cuba redonda CR-30, escovada, cód. 01018116 / 90010181016. Ref.: Mekal. (DET PR003; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="M18" s="32" t="n"/>
+      <c r="N18" s="32" t="n"/>
+      <c r="O18" s="32" t="inlineStr">
+        <is>
+          <t>Torneira de mesa bica alta para lavatório, cromada, linha Link, cód. 1198.C.LNK. Ref.: Deca. (DET PR003; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="P18" s="32" t="n"/>
+      <c r="Q18" s="32" t="n"/>
+      <c r="R18" s="32" t="n"/>
+      <c r="S18" s="32" t="n"/>
+      <c r="T18" s="32" t="n"/>
+      <c r="U18" s="32" t="n"/>
+      <c r="V18" s="32" t="n"/>
+      <c r="W18" s="32" t="n"/>
+      <c r="X18" s="31" t="n"/>
+      <c r="Y18" s="31" t="n"/>
+      <c r="Z18" s="32" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="45" t="inlineStr">
+        <is>
+          <t>COZINHA / DESPENSAS</t>
+        </is>
+      </c>
+      <c r="B19" s="269" t="inlineStr">
+        <is>
+          <t>Piso em granito branco siena escovado, 85x130cm. Rejunte Infinity Hard, cor Branco Pérola ou Palha (validar com o Setor de Produto). (DET PR001, PR406/407; Tab. R01: paginação a definir)</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>Soleira em granito branco siena. (PR406)</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>Rodapé semi-embutido em granito branco siena escovado, h=15cm (DET 22). (DET PR001, PR406/407; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="271" t="inlineStr">
+        <is>
+          <t>Rodabanca em granito branco siena escovado, h=60cm
+Pintura acrílica; cor a definir (Tab. R01). (PR406/407)</t>
+        </is>
+      </c>
+      <c r="I19" s="271" t="n"/>
+      <c r="J19" s="32" t="inlineStr">
+        <is>
+          <t>Bancada e ilha em granito branco siena escovado; parte seca h=90cm, área molhada com desnível 1cm h=92cm; suporte em metalon chumbado na parede; emendas seguem a paginação do piso. (PR406/407; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="K19" s="32" t="n"/>
+      <c r="L19" s="32" t="inlineStr">
+        <is>
+          <t>Cuba de embutir 600x400x230mm em aço inox, linha Retta. Ref.: Mekal ou similar. (Tab. R01; PR406 sem modelo)</t>
+        </is>
+      </c>
+      <c r="M19" s="32" t="n"/>
+      <c r="N19" s="32" t="n"/>
+      <c r="O19" s="32" t="inlineStr">
+        <is>
+          <t>Monocomando de mesa para cozinha, cromado, linha Level. Ref.: Deca ou similar. (Tab. R01; PR406 sem modelo)</t>
+        </is>
+      </c>
+      <c r="P19" s="32" t="n"/>
+      <c r="Q19" s="32" t="n"/>
+      <c r="R19" s="32" t="n"/>
+      <c r="S19" s="32" t="n"/>
+      <c r="T19" s="32" t="n"/>
+      <c r="U19" s="32" t="n"/>
+      <c r="V19" s="32" t="n"/>
+      <c r="W19" s="32" t="n"/>
+      <c r="X19" s="31" t="inlineStr">
+        <is>
+          <t>Porta em marcenaria. (PR406/407)</t>
+        </is>
+      </c>
+      <c r="Y19" s="31" t="n"/>
+      <c r="Z19" s="32" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>ÁREA DE SERVIÇO / CIRCULAÇÃO SERVIÇO</t>
+        </is>
+      </c>
+      <c r="B20" s="269" t="inlineStr">
+        <is>
+          <t>Piso em granito branco siena escovado, 85x130cm, ver paginação. Rejunte Infinity Hard, cor Branco Pérola ou Palha. (DET PR001, PR005; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>Soleira indicada em planta, material não especificado. (DET PR005)</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="32" t="inlineStr">
+        <is>
+          <t>Rodapé semi-embutido em granito branco siena escovado, h=15cm. (DET PR005)</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="271" t="inlineStr">
+        <is>
+          <t>Parede em Formica Branco Real L515, 308x125cm. (DET PR005/PR006; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I20" s="271" t="inlineStr">
+        <is>
+          <t>Forro de gesso com tabica metálica (DET 11) e cortineiro 25x16cm (DET 24). (DET PR006)</t>
+        </is>
+      </c>
+      <c r="J20" s="32" t="inlineStr">
+        <is>
+          <t>Bancada em granito branco siena escovado, molhada com 1cm de rebaixo, rodabanca h=60cm com topo polido; bancada seca com laterais polidas. (DET PR005/PR006; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="K20" s="32" t="n"/>
+      <c r="L20" s="32" t="inlineStr">
+        <is>
+          <t>Tanque para lavanderia CT-60, escovado, cód. 01019616 / 90010196016, 2 unidades, instalados sob a pedra da bancada. Ref.: Mekal. (DET PR005; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="M20" s="32" t="n"/>
+      <c r="N20" s="32" t="n"/>
+      <c r="O20" s="32" t="inlineStr">
+        <is>
+          <t>Torneira de parede com arejador para cozinha, cromada, linha Link, cód. 1159.C.LNK, 2 unidades. Ref.: Deca. (DET PR005; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="P20" s="32" t="n"/>
+      <c r="Q20" s="32" t="n"/>
+      <c r="R20" s="32" t="inlineStr">
+        <is>
+          <t>Acabamento para registro de gaveta 1 1/4" e 1 1/2", cromado, Link, cód. 4900.C.GD.LNK. Ref.: Deca. (DET PR005)</t>
+        </is>
+      </c>
+      <c r="S20" s="32" t="n"/>
+      <c r="T20" s="32" t="inlineStr">
+        <is>
+          <t>Ralo oculto 15x15cm, tampa revestida com a mesma pedra (o DET diz "mármore"; o piso é granito). (DET PR005)</t>
+        </is>
+      </c>
+      <c r="U20" s="32" t="n"/>
+      <c r="V20" s="32" t="n"/>
+      <c r="W20" s="32" t="inlineStr">
+        <is>
+          <t>Maçaneta Pado Sara, cromo acetinado, interna. Porta de segurança: fechadura digital FDE-600W. (DET PR005/PR006)</t>
+        </is>
+      </c>
+      <c r="X20" s="31" t="inlineStr">
+        <is>
+          <t>Porta piso-forro, cor branca, alizar 10cm
+Porta piso-forro especial de segurança, cor branca, alizar 10cm. (DET PR006)</t>
+        </is>
+      </c>
+      <c r="Y20" s="31" t="n"/>
+      <c r="Z20" s="32" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="45" t="inlineStr">
+        <is>
+          <t>BANHO SERVIÇO</t>
+        </is>
+      </c>
+      <c r="B21" s="269" t="inlineStr">
+        <is>
+          <t>Piso em granito branco siena escovado. (DET PR007; Tab. R01: paginação a definir)</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>Filete em granito na transição para o vinílico (DET 04). (DET PR007)</t>
+        </is>
+      </c>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="271" t="inlineStr">
+        <is>
+          <t>Revestimento Forma Branco AC retificado 32,5x59cm. Ref.: Eliane. (DET PR007; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I21" s="271" t="inlineStr">
+        <is>
+          <t>Forro em gesso acartonado, pintura acrílica acetinada cor branco neve, tabica metálica, sanca 25x16cm. PD 298cm. (DET PR007)</t>
+        </is>
+      </c>
+      <c r="J21" s="32" t="inlineStr">
+        <is>
+          <t>Bancada em granito branco siena escovado. (DET PR007; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="K21" s="32" t="n"/>
+      <c r="L21" s="32" t="inlineStr">
+        <is>
+          <t>Cuba redonda de embutir 31cm branca, linha L, cód. L.41.17. Ref.: Deca. (DET PR007; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="M21" s="32" t="n"/>
+      <c r="N21" s="32" t="n"/>
+      <c r="O21" s="32" t="inlineStr">
+        <is>
+          <t>Torneira de mesa bica baixa para lavatório, cromada, linha Link, cód. 1197.C.LNK. Ref.: Deca. (DET PR007; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="P21" s="32" t="inlineStr">
+        <is>
+          <t>Bacia com caixa acoplada branca, linha Axis, cód. KP.470.17. Ref.: Deca. (DET PR007; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="Q21" s="32" t="inlineStr">
+        <is>
+          <t>Ducha higiênica com registro e derivação, cromada, linha Link, cód. 1984.C.ACT.LNK.BR. Ref.: Deca. (DET PR007)</t>
+        </is>
+      </c>
+      <c r="R21" s="32" t="inlineStr">
+        <is>
+          <t>Acabamento para registro de gaveta e pressão até 1", cromado, Link, cód. 4900.C.PQ.LNK. Ref.: Deca. (DET PR007; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="S21" s="32" t="n"/>
+      <c r="T21" s="32" t="inlineStr">
+        <is>
+          <t>Ralo linear oculto e ralo quadrado oculto. (DET PR007)</t>
+        </is>
+      </c>
+      <c r="U21" s="32" t="n"/>
+      <c r="V21" s="32" t="n"/>
+      <c r="W21" s="32" t="n"/>
+      <c r="X21" s="31" t="n"/>
+      <c r="Y21" s="31" t="n"/>
+      <c r="Z21" s="32" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="45" t="inlineStr">
+        <is>
+          <t>QUARTO / ESTAR FUNCIONÁRIOS</t>
+        </is>
+      </c>
+      <c r="B22" s="269" t="inlineStr">
+        <is>
+          <t>Piso vinílico Austin, linha Urban, 18x121cm. Ref.: Durafloor. (DET PR001; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>Filete em granito na transição vinílico x granito (DET 04). (DET PR001)</t>
+        </is>
+      </c>
+      <c r="E22" s="32" t="n"/>
+      <c r="F22" s="32" t="inlineStr">
+        <is>
+          <t>Rodapé Easy Y.01 120. Ref.: Durafloor. (DET PR001; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="n"/>
+      <c r="H22" s="271" t="inlineStr">
+        <is>
+          <t>Pintura acrílica cor branco neve. (Tab. R01)</t>
+        </is>
+      </c>
+      <c r="I22" s="271" t="n"/>
+      <c r="J22" s="32" t="n"/>
+      <c r="K22" s="32" t="n"/>
+      <c r="L22" s="32" t="n"/>
+      <c r="M22" s="32" t="n"/>
+      <c r="N22" s="32" t="n"/>
+      <c r="O22" s="32" t="n"/>
+      <c r="P22" s="32" t="n"/>
+      <c r="Q22" s="32" t="n"/>
+      <c r="R22" s="32" t="n"/>
+      <c r="S22" s="32" t="n"/>
+      <c r="T22" s="32" t="n"/>
+      <c r="U22" s="32" t="n"/>
+      <c r="V22" s="32" t="n"/>
+      <c r="W22" s="32" t="n"/>
+      <c r="X22" s="31" t="n"/>
+      <c r="Y22" s="31" t="n"/>
+      <c r="Z22" s="32" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>VARANDA TÉCNICA</t>
+        </is>
+      </c>
+      <c r="B23" s="269" t="inlineStr">
+        <is>
+          <t>Piso em concreto. (DET PR001)</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="n"/>
+      <c r="D23" s="32" t="n"/>
+      <c r="E23" s="32" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="32" t="n"/>
+      <c r="H23" s="271" t="n"/>
+      <c r="I23" s="271" t="n"/>
+      <c r="J23" s="32" t="n"/>
+      <c r="K23" s="32" t="n"/>
+      <c r="L23" s="32" t="n"/>
+      <c r="M23" s="32" t="n"/>
+      <c r="N23" s="32" t="n"/>
+      <c r="O23" s="32" t="n"/>
+      <c r="P23" s="32" t="n"/>
+      <c r="Q23" s="32" t="n"/>
+      <c r="R23" s="32" t="n"/>
+      <c r="S23" s="32" t="n"/>
+      <c r="T23" s="32" t="n"/>
+      <c r="U23" s="32" t="n"/>
+      <c r="V23" s="32" t="n"/>
+      <c r="W23" s="32" t="n"/>
+      <c r="X23" s="31" t="n"/>
+      <c r="Y23" s="31" t="n"/>
+      <c r="Z23" s="32" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>HALL ELEVADOR SOCIAL (ANDAR)</t>
+        </is>
+      </c>
+      <c r="B24" s="269" t="inlineStr">
+        <is>
+          <t>Piso em mármore travertino romano bruto. (DET PR003)</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="32" t="n"/>
+      <c r="E24" s="32" t="n"/>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>Rodapé em mármore travertino romano bruto, semi-embutido, h=15cm. (DET PR003)</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="n"/>
+      <c r="H24" s="271" t="inlineStr">
+        <is>
+          <t>Parede pintada com tinta acrílica cor branco neve, acabamento acetinado
+Aduela do elevador (2cm) em mármore travertino romano bruto. (DET PR003)</t>
+        </is>
+      </c>
+      <c r="I24" s="271" t="n"/>
+      <c r="J24" s="32" t="n"/>
+      <c r="K24" s="32" t="n"/>
+      <c r="L24" s="32" t="n"/>
+      <c r="M24" s="32" t="n"/>
+      <c r="N24" s="32" t="n"/>
+      <c r="O24" s="32" t="n"/>
+      <c r="P24" s="32" t="n"/>
+      <c r="Q24" s="32" t="n"/>
+      <c r="R24" s="32" t="n"/>
+      <c r="S24" s="32" t="n"/>
+      <c r="T24" s="32" t="n"/>
+      <c r="U24" s="32" t="n"/>
+      <c r="V24" s="32" t="n"/>
+      <c r="W24" s="32" t="n"/>
+      <c r="X24" s="31" t="n"/>
+      <c r="Y24" s="31" t="n"/>
+      <c r="Z24" s="32" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>HALL ELEVADOR SERVIÇO (ANDAR)</t>
+        </is>
+      </c>
+      <c r="B25" s="269" t="inlineStr">
+        <is>
+          <t>Piso em granito branco siena escovado. (DET PR003)</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>Rodapé em granito branco siena escovado, semi-embutido, h=15cm. (DET PR003)</t>
+        </is>
+      </c>
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="271" t="inlineStr">
+        <is>
+          <t>Parede pintada com tinta acrílica cor branco neve, acabamento acetinado
+Aduela do elevador (2cm) em granito branco siena escovado. (DET PR003)</t>
+        </is>
+      </c>
+      <c r="I25" s="271" t="n"/>
+      <c r="J25" s="32" t="n"/>
+      <c r="K25" s="32" t="n"/>
+      <c r="L25" s="32" t="n"/>
+      <c r="M25" s="32" t="n"/>
+      <c r="N25" s="32" t="n"/>
+      <c r="O25" s="32" t="n"/>
+      <c r="P25" s="32" t="n"/>
+      <c r="Q25" s="32" t="n"/>
+      <c r="R25" s="32" t="n"/>
+      <c r="S25" s="32" t="n"/>
+      <c r="T25" s="32" t="n"/>
+      <c r="U25" s="32" t="n"/>
+      <c r="V25" s="32" t="n"/>
+      <c r="W25" s="32" t="n"/>
+      <c r="X25" s="31" t="n"/>
+      <c r="Y25" s="31" t="n"/>
+      <c r="Z25" s="32" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="45" t="inlineStr">
+        <is>
+          <t>HALL SERVIÇO / ANTECÂMARA – GARDEN, TIPO E COBERTURA</t>
+        </is>
+      </c>
+      <c r="B26" s="269" t="inlineStr">
+        <is>
+          <t>Piso em granito ("revestimento conforme ambiente"). (PR721-728)</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="32" t="n"/>
+      <c r="F26" s="32" t="inlineStr">
+        <is>
+          <t>Rodapé em granito semi-embutido, seguir alinhamento do piso (DET 22). (PR722/724/726/728)</t>
+        </is>
+      </c>
+      <c r="G26" s="32" t="n"/>
+      <c r="H26" s="271" t="inlineStr">
+        <is>
+          <t>Parede pintada. (PR722/724/726/728)</t>
+        </is>
+      </c>
+      <c r="I26" s="271" t="inlineStr">
+        <is>
+          <t>Forro em gesso com sanca: PD 259cm (Garden e Tipo), 267,5cm (Cobertura 1º nível), 272,5cm (Cobertura 2º nível); junta de dilatação em perfil metálico "Z" (DET 09); trechos em laje de concreto aparente. (PR721-728)</t>
+        </is>
+      </c>
+      <c r="J26" s="32" t="n"/>
+      <c r="K26" s="32" t="n"/>
+      <c r="L26" s="32" t="n"/>
+      <c r="M26" s="32" t="n"/>
+      <c r="N26" s="32" t="n"/>
+      <c r="O26" s="32" t="n"/>
+      <c r="P26" s="32" t="n"/>
+      <c r="Q26" s="32" t="n"/>
+      <c r="R26" s="32" t="n"/>
+      <c r="S26" s="32" t="n"/>
+      <c r="T26" s="32" t="n"/>
+      <c r="U26" s="32" t="n"/>
+      <c r="V26" s="32" t="n"/>
+      <c r="W26" s="32" t="n"/>
+      <c r="X26" s="31" t="inlineStr">
+        <is>
+          <t>PCF1, PCF2, PE-A, P13, P23, PA05, PCF3, P15A, P15C (vão 90x240cm); material não especificado nas pranchas de circulação. (PR721-728)</t>
+        </is>
+      </c>
+      <c r="Y26" s="31" t="n"/>
+      <c r="Z26" s="32" t="inlineStr">
+        <is>
+          <t>Sirene de alarme e botoeira; hidrante nos halls conforme projeto PCI. (PR722-728)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="45" t="n"/>
+      <c r="B27" s="269" t="n"/>
+      <c r="C27" s="32" t="n"/>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="32" t="n"/>
+      <c r="F27" s="32" t="n"/>
+      <c r="G27" s="32" t="n"/>
+      <c r="H27" s="271" t="n"/>
+      <c r="I27" s="271" t="n"/>
+      <c r="J27" s="32" t="n"/>
+      <c r="K27" s="32" t="n"/>
+      <c r="L27" s="32" t="n"/>
+      <c r="M27" s="32" t="n"/>
+      <c r="N27" s="32" t="n"/>
+      <c r="O27" s="32" t="n"/>
+      <c r="P27" s="32" t="n"/>
+      <c r="Q27" s="32" t="n"/>
+      <c r="R27" s="32" t="n"/>
+      <c r="S27" s="32" t="n"/>
+      <c r="T27" s="32" t="n"/>
+      <c r="U27" s="32" t="n"/>
+      <c r="V27" s="32" t="n"/>
+      <c r="W27" s="32" t="n"/>
+      <c r="X27" s="31" t="n"/>
+      <c r="Y27" s="31" t="n"/>
+      <c r="Z27" s="32" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="45" t="n"/>
+      <c r="B28" s="269" t="n"/>
+      <c r="C28" s="32" t="n"/>
+      <c r="D28" s="32" t="n"/>
+      <c r="E28" s="32" t="n"/>
+      <c r="F28" s="32" t="n"/>
+      <c r="G28" s="32" t="n"/>
+      <c r="H28" s="271" t="n"/>
+      <c r="I28" s="271" t="n"/>
+      <c r="J28" s="32" t="n"/>
+      <c r="K28" s="32" t="n"/>
+      <c r="L28" s="32" t="n"/>
+      <c r="M28" s="32" t="n"/>
+      <c r="N28" s="32" t="n"/>
+      <c r="O28" s="32" t="n"/>
+      <c r="P28" s="32" t="n"/>
+      <c r="Q28" s="32" t="n"/>
+      <c r="R28" s="32" t="n"/>
+      <c r="S28" s="32" t="n"/>
+      <c r="T28" s="32" t="n"/>
+      <c r="U28" s="32" t="n"/>
+      <c r="V28" s="32" t="n"/>
+      <c r="W28" s="32" t="n"/>
+      <c r="X28" s="31" t="n"/>
+      <c r="Y28" s="31" t="n"/>
+      <c r="Z28" s="32" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="45" t="n"/>
+      <c r="B29" s="269" t="n"/>
+      <c r="C29" s="32" t="n"/>
+      <c r="D29" s="32" t="n"/>
+      <c r="E29" s="32" t="n"/>
+      <c r="F29" s="32" t="n"/>
+      <c r="G29" s="32" t="n"/>
+      <c r="H29" s="271" t="n"/>
+      <c r="I29" s="271" t="n"/>
+      <c r="J29" s="32" t="n"/>
+      <c r="K29" s="32" t="n"/>
+      <c r="L29" s="32" t="n"/>
+      <c r="M29" s="32" t="n"/>
+      <c r="N29" s="32" t="n"/>
+      <c r="O29" s="32" t="n"/>
+      <c r="P29" s="32" t="n"/>
+      <c r="Q29" s="32" t="n"/>
+      <c r="R29" s="32" t="n"/>
+      <c r="S29" s="32" t="n"/>
+      <c r="T29" s="32" t="n"/>
+      <c r="U29" s="32" t="n"/>
+      <c r="V29" s="32" t="n"/>
+      <c r="W29" s="32" t="n"/>
+      <c r="X29" s="31" t="n"/>
+      <c r="Y29" s="31" t="n"/>
+      <c r="Z29" s="32" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="45" t="n"/>
+      <c r="B30" s="269" t="n"/>
+      <c r="C30" s="32" t="n"/>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="32" t="n"/>
+      <c r="F30" s="32" t="n"/>
+      <c r="G30" s="32" t="n"/>
+      <c r="H30" s="271" t="n"/>
+      <c r="I30" s="271" t="n"/>
+      <c r="J30" s="32" t="n"/>
+      <c r="K30" s="32" t="n"/>
+      <c r="L30" s="32" t="n"/>
+      <c r="M30" s="32" t="n"/>
+      <c r="N30" s="32" t="n"/>
+      <c r="O30" s="32" t="n"/>
+      <c r="P30" s="32" t="n"/>
+      <c r="Q30" s="32" t="n"/>
+      <c r="R30" s="32" t="n"/>
+      <c r="S30" s="32" t="n"/>
+      <c r="T30" s="32" t="n"/>
+      <c r="U30" s="32" t="n"/>
+      <c r="V30" s="32" t="n"/>
+      <c r="W30" s="32" t="n"/>
+      <c r="X30" s="31" t="n"/>
+      <c r="Y30" s="31" t="n"/>
+      <c r="Z30" s="32" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="45" t="n"/>
+      <c r="B31" s="269" t="n"/>
+      <c r="C31" s="32" t="n"/>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="32" t="n"/>
+      <c r="F31" s="32" t="n"/>
+      <c r="G31" s="32" t="n"/>
+      <c r="H31" s="271" t="n"/>
+      <c r="I31" s="271" t="n"/>
+      <c r="J31" s="32" t="n"/>
+      <c r="K31" s="32" t="n"/>
+      <c r="L31" s="32" t="n"/>
+      <c r="M31" s="32" t="n"/>
+      <c r="N31" s="32" t="n"/>
+      <c r="O31" s="32" t="n"/>
+      <c r="P31" s="32" t="n"/>
+      <c r="Q31" s="32" t="n"/>
+      <c r="R31" s="32" t="n"/>
+      <c r="S31" s="32" t="n"/>
+      <c r="T31" s="32" t="n"/>
+      <c r="U31" s="32" t="n"/>
+      <c r="V31" s="32" t="n"/>
+      <c r="W31" s="32" t="n"/>
+      <c r="X31" s="31" t="n"/>
+      <c r="Y31" s="31" t="n"/>
+      <c r="Z31" s="32" t="n"/>
+    </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35">
+      <c r="S35" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="31">
+    <mergeCell ref="L10:U10"/>
+    <mergeCell ref="B10:K10"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="T5:U5"/>
+    <mergeCell ref="B1:I4"/>
+    <mergeCell ref="AE1:AF4"/>
+    <mergeCell ref="T1:U4"/>
+    <mergeCell ref="A1:A4"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="L1:S4"/>
+    <mergeCell ref="V10:Z10"/>
+    <mergeCell ref="V5:AD6"/>
+    <mergeCell ref="B5:I6"/>
+    <mergeCell ref="T9:U9"/>
+    <mergeCell ref="AE8:AF8"/>
+    <mergeCell ref="B7:I8"/>
+    <mergeCell ref="V1:AD4"/>
+    <mergeCell ref="L12:U12"/>
+    <mergeCell ref="B12:K12"/>
+    <mergeCell ref="L7:S8"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="AE9:AF9"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="J1:K4"/>
+    <mergeCell ref="AE5:AF5"/>
+    <mergeCell ref="L5:S6"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="V12:Z12"/>
+    <mergeCell ref="V7:AD8"/>
+  </mergeCells>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0.3149606299212598" footer="0.3149606299212598"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" pageOrder="overThenDown"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor theme="0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AA33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
   <cols>
@@ -14446,13 +16638,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E532"/>
+  <dimension ref="A1:E543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -26615,6 +28807,121 @@
         </is>
       </c>
     </row>
+    <row r="534">
+      <c r="A534" s="279" t="inlineStr">
+        <is>
+          <t>6. APARTAMENTO TIPO (pasta DTL - DETALHAMENTO / APARTAMENTOS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>SALA / VARANDA DA SALA</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>RODAPÉ: CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>LAVABO</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>RODAPÉ: CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>RODAPÉ: CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>COPA NOTURNA</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>BANCADA: CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>BANHO SUÍTE MASTER</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Prancha CDJ-ARQ-DT-PR408-ISSM_TIPO-R05 não tem texto legível pelo conector; linha preenchida só com a tabela R01. Anexar o PDF para conferir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>ÁREA DE SERVIÇO</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Ralo com "tampa revestida com o mesmo mármore", mas o piso é granito branco siena. Confirmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>SOLEIRAS</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Indicadas em planta no lavabo e na área de serviço sem material; só a cozinha define (granito branco siena).</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>COZINHA</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>PR406/407 não trazem modelo de cuba e monocomando; valem os da tabela R01 (Mekal Retta e Deca Level).</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>REJUNTES</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>DET indica "validar com o Setor de Produto"; PR001/PR002 "não liberado para execução, paginação poderá sofrer alterações".</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Grade Cidade Jardim: banho suíte master pela prancha PR408
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -14823,60 +14823,99 @@
       </c>
       <c r="B15" s="269" t="inlineStr">
         <is>
-          <t>Piso em mármore travertino romano bruto resinado, paginado conforme detalhamento. (Tab. R01)</t>
+          <t>11 - Piso em contrapiso regularizado, revestido em mármore travertino romano resinado. Rejunte creme ou marfim (ver padrão da chapa). Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (PR408; Tab. R01: "bruto resinado")</t>
         </is>
       </c>
       <c r="C15" s="32" t="n"/>
       <c r="D15" s="32" t="n"/>
-      <c r="E15" s="32" t="n"/>
-      <c r="F15" s="32" t="n"/>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>Peitoril a definir conforme projeto de esquadrias. (PR408)</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>23 - Rodapé em mármore travertino romano bruto semi-embutido, h=15cm; paginação segue alinhamento do piso. (PR408)</t>
+        </is>
+      </c>
       <c r="G15" s="32" t="n"/>
-      <c r="H15" s="271" t="inlineStr">
-        <is>
-          <t>Parede em mármore travertino romano bruto paginado. (Tab. R01)</t>
-        </is>
-      </c>
-      <c r="I15" s="271" t="n"/>
+      <c r="H15" s="285" t="inlineStr">
+        <is>
+          <t>14 - Parede revestida em mármore travertino romano resinado. Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (PR408)
+1 - Parede em alvenaria emassada e regularizada, pintada com tinta acrílica cor branco neve, acabamento acetinado. Ref.: Suvinil. (PR408)
+CONFLITO – Tabela R01: parede em mármore travertino romano BRUTO paginado</t>
+        </is>
+      </c>
+      <c r="I15" s="271" t="inlineStr">
+        <is>
+          <t>1 - Forro em gesso acartonado liso, tinta acrílica cor branco neve, acabamento fosco, junta de dilatação metálica branca. Ref.: Suvinil. Sanca (DET 20). (PR408)</t>
+        </is>
+      </c>
       <c r="J15" s="32" t="inlineStr">
         <is>
-          <t>Bancada em mármore travertino romano resinado. (Tab. R01)</t>
+          <t>35 - Bancada em mármore travertino romano resinado. Rejunte creme ou marfim (ver padrão da chapa). Dimensões conforme detalhamento. (PR408; Tab. R01)</t>
         </is>
       </c>
       <c r="K15" s="32" t="n"/>
       <c r="L15" s="32" t="inlineStr">
         <is>
-          <t>Cuba de apoio retangular Jader Almeida, branca. Ref.: Deca ou similar. (Tab. R01)</t>
+          <t>33 - Cuba de apoio retangular Jader Almeida 670x495x120mm, branca, cód. L.310.17. Ref.: Deca. (PR408; Tab. R01)</t>
         </is>
       </c>
       <c r="M15" s="32" t="n"/>
       <c r="N15" s="32" t="n"/>
       <c r="O15" s="32" t="inlineStr">
         <is>
-          <t>Misturador monocomando de mesa bica alta para lavatório, cromado, linha Level. Ref.: Deca ou similar. (Tab. R01)</t>
+          <t>36 - Misturador monocomando de mesa bica alta para lavatório, Level cromado, cód. 2885.C26. Ref.: Deca. (PR408; Tab. R01)</t>
         </is>
       </c>
       <c r="P15" s="32" t="inlineStr">
         <is>
-          <t>Bacia convencional Carrara branca com caixa acoplada. Ref.: Deca ou similar
-Bidê 3 furos Carrara branco. Ref.: Deca ou similar. (Tab. R01)</t>
-        </is>
-      </c>
-      <c r="Q15" s="32" t="n"/>
-      <c r="R15" s="32" t="n"/>
+          <t>34 - Bacia convencional Carrara branca com caixa acoplada e acionamento duo, cód. P.606.17. Ref.: Deca. (PR408; Tab. R01)
+46 - Bidê 3 furos Carrara branco, cód. B.60.17. Ref.: Deca. (PR408; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="Q15" s="32" t="inlineStr">
+        <is>
+          <t>37 - Ducha higiênica Level cromada, cód. 1984.C26.ACT.CR. (PR408)</t>
+        </is>
+      </c>
+      <c r="R15" s="32" t="inlineStr">
+        <is>
+          <t>49 - Acabamento para registro Level cromado, cód. 4900.C26.PQ. Ref.: Deca. (PR408)</t>
+        </is>
+      </c>
       <c r="S15" s="32" t="inlineStr">
         <is>
-          <t>Acabamento de monocomando de chuveiro, cromado, linha Level. Ref.: Deca ou similar. (Tab. R01)</t>
-        </is>
-      </c>
-      <c r="T15" s="32" t="n"/>
+          <t>44 - Acabamento de monocomando de chuveiro para alta e baixa pressão, Level cromado, cód. 4993.C26.CHU. (PR408; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="T15" s="32" t="inlineStr">
+        <is>
+          <t>47 - Ralo linear oculto Royal 70cm
+48 - Ralo oculto 15x15cm Square. (PR408)</t>
+        </is>
+      </c>
       <c r="U15" s="32" t="inlineStr">
         <is>
-          <t>Misturador para bidê, cromado, linha Level. Ref.: Deca ou similar. (Tab. R01)</t>
-        </is>
-      </c>
-      <c r="V15" s="32" t="n"/>
-      <c r="W15" s="32" t="n"/>
-      <c r="X15" s="31" t="n"/>
+          <t>45 - Misturador para bidê Level cromado, cód. 1895.C26. (PR408; Tab. R01)</t>
+        </is>
+      </c>
+      <c r="V15" s="32" t="inlineStr">
+        <is>
+          <t>39 - Tomadas e interruptores Arteor quadrado branco. Ref.: Legrand. (PR408)</t>
+        </is>
+      </c>
+      <c r="W15" s="32" t="inlineStr">
+        <is>
+          <t>Maçaneta Sara cromo acetinado. Ref.: Pado. (PR408)</t>
+        </is>
+      </c>
+      <c r="X15" s="31" t="inlineStr">
+        <is>
+          <t>38 - Porta em marcenaria piso-forro, cor branca, alizar 10cm. (PR408)</t>
+        </is>
+      </c>
       <c r="Y15" s="31" t="n"/>
       <c r="Z15" s="32" t="n"/>
     </row>
@@ -16644,7 +16683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E543"/>
+  <dimension ref="A1:E544"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -28841,82 +28880,94 @@
     <row r="537">
       <c r="B537" t="inlineStr">
         <is>
-          <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
+          <t>BANHO SUÍTE MASTER</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>RODAPÉ: CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
+          <t>PAREDE/REJUNTE: CONFLITO – Tabela R01: parede em mármore travertino romano BRUTO paginado</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="B538" t="inlineStr">
         <is>
-          <t>COPA NOTURNA</t>
+          <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>BANCADA: CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
+          <t>RODAPÉ: CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="B539" t="inlineStr">
         <is>
-          <t>BANHO SUÍTE MASTER</t>
+          <t>COPA NOTURNA</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>Prancha CDJ-ARQ-DT-PR408-ISSM_TIPO-R05 não tem texto legível pelo conector; linha preenchida só com a tabela R01. Anexar o PDF para conferir.</t>
+          <t>BANCADA: CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="B540" t="inlineStr">
         <is>
-          <t>ÁREA DE SERVIÇO</t>
+          <t>BANHO SUÍTE MASTER</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>Ralo com "tampa revestida com o mesmo mármore", mas o piso é granito branco siena. Confirmar.</t>
+          <t>Prancha CDJ-ARQ-DT-PR408-ISSM_TIPO-R05 lida pelo PDF anexado (só imagem vetorial, sem texto); códigos da legenda da prancha.</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="B541" t="inlineStr">
         <is>
-          <t>SOLEIRAS</t>
+          <t>ÁREA DE SERVIÇO</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>Indicadas em planta no lavabo e na área de serviço sem material; só a cozinha define (granito branco siena).</t>
+          <t>Ralo com "tampa revestida com o mesmo mármore", mas o piso é granito branco siena. Confirmar.</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="B542" t="inlineStr">
         <is>
-          <t>COZINHA</t>
+          <t>SOLEIRAS</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
         <is>
-          <t>PR406/407 não trazem modelo de cuba e monocomando; valem os da tabela R01 (Mekal Retta e Deca Level).</t>
+          <t>Indicadas em planta no lavabo e na área de serviço sem material; só a cozinha define (granito branco siena).</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="B543" t="inlineStr">
         <is>
+          <t>COZINHA</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>PR406/407 não trazem modelo de cuba e monocomando; valem os da tabela R01 (Mekal Retta e Deca Level).</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="B544" t="inlineStr">
+        <is>
           <t>REJUNTES</t>
         </is>
       </c>
-      <c r="D543" t="inlineStr">
+      <c r="D544" t="inlineStr">
         <is>
           <t>DET indica "validar com o Setor de Produto"; PR001/PR002 "não liberado para execução, paginação poderá sofrer alterações".</t>
         </is>

</xml_diff>

<commit_message>
Grade Cidade Jardim: área de impressão dinâmica em todas as abas
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -15,14 +15,18 @@
     <sheet name="PENDÊNCIAS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">OFFSET('CONTROLE DE REVISÕES '!$A$1,0,0,MAX(1,MAX(INDEX(('CONTROLE DE REVISÕES '!$A$1:$I$3000&amp;""&lt;&gt;"")*ROW('CONTROLE DE REVISÕES '!$A$1:$I$3000),0))),9)</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'TÉRREO '!$1:$11,'TÉRREO '!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'TÉRREO '!$A$1:$AF$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">OFFSET('TÉRREO '!$A$1,0,0,MAX(11,MAX(INDEX(('TÉRREO '!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('TÉRREO '!$A$1:$AF$3000),0))),32)</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'2° PAVTO'!$1:$11,'2° PAVTO'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'2° PAVTO'!$A$1:$AF$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">OFFSET('2° PAVTO'!$A$1,0,0,MAX(11,MAX(INDEX(('2° PAVTO'!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('2° PAVTO'!$A$1:$AF$3000),0))),32)</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'PILOTIS'!$1:$11,'PILOTIS'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'PILOTIS'!$A$1:$AF$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">OFFSET('PILOTIS'!$A$1,0,0,MAX(11,MAX(INDEX(('PILOTIS'!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('PILOTIS'!$A$1:$AF$3000),0))),32)</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'APTO TIPO'!$1:$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">OFFSET('APTO TIPO'!$A$1,0,0,MAX(11,MAX(INDEX(('APTO TIPO'!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('APTO TIPO'!$A$1:$AF$3000),0))),32)</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'IMAGENS ESPECIFICAÇÕES '!$1:$11,'IMAGENS ESPECIFICAÇÕES '!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'IMAGENS ESPECIFICAÇÕES '!$A$1:$U$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">OFFSET('IMAGENS ESPECIFICAÇÕES '!$A$1,0,0,MAX(26,MAX(INDEX(('IMAGENS ESPECIFICAÇÕES '!$A$1:$U$3000&amp;""&lt;&gt;"")*ROW('IMAGENS ESPECIFICAÇÕES '!$A$1:$U$3000),0))),21)</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">OFFSET('PENDÊNCIAS'!$A$1,0,0,MAX(1,MAX(INDEX(('PENDÊNCIAS'!$A$1:$E$3000&amp;""&lt;&gt;"")*ROW('PENDÊNCIAS'!$A$1:$E$3000),0))),5)</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -6196,6 +6200,7 @@
       <c r="H33" s="230" t="n"/>
       <c r="I33" s="217" t="n"/>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="E35" s="21" t="n"/>
     </row>
@@ -6252,7 +6257,7 @@
     <mergeCell ref="C11:I11"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="8" scale="71" fitToHeight="0"/>
+  <pageSetup orientation="portrait" paperSize="8" scale="71" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -6262,7 +6267,7 @@
   <sheetPr>
     <tabColor theme="0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
@@ -8893,7 +8898,7 @@
     <mergeCell ref="V7:AD8"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" pageOrder="overThenDown"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" fitToWidth="1" pageOrder="overThenDown"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;L&amp;"Aptos Narrow,Negrito"&amp;18  Página &amp;P de &amp;N</oddFooter>
@@ -8915,7 +8920,7 @@
   <sheetPr>
     <tabColor theme="0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
@@ -10395,7 +10400,7 @@
     <mergeCell ref="V7:AD8"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" pageOrder="overThenDown"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" fitToWidth="1" pageOrder="overThenDown"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;L&amp;"Aptos Narrow,Negrito"&amp;18  Página &amp;P de &amp;N</oddFooter>
@@ -10417,7 +10422,7 @@
   <sheetPr codeName="Planilha2">
     <tabColor theme="0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
@@ -14054,7 +14059,7 @@
     <mergeCell ref="V7:AD8"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" pageOrder="overThenDown"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" fitToWidth="1" pageOrder="overThenDown"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;L&amp;"Aptos Narrow,Negrito"&amp;18  Página &amp;P de &amp;N</oddFooter>
@@ -14076,7 +14081,7 @@
   <sheetPr>
     <tabColor theme="0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
@@ -15748,7 +15753,7 @@
     <mergeCell ref="V7:AD8"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" pageOrder="overThenDown"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" fitToWidth="1" pageOrder="overThenDown"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -15758,7 +15763,7 @@
   <sheetPr>
     <tabColor theme="0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AA33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
@@ -16623,6 +16628,10 @@
     </row>
     <row r="27" ht="125.25" customHeight="1"/>
     <row r="28" ht="2.1" customHeight="1"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
     <row r="33">
       <c r="P33" s="3" t="inlineStr">
         <is>
@@ -16675,7 +16684,7 @@
     <mergeCell ref="G22:H22"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" pageOrder="overThenDown"/>
+  <pageSetup orientation="landscape" paperSize="8" scale="38" fitToHeight="0" fitToWidth="1" pageOrder="overThenDown"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;L&amp;"Aptos Narrow,Negrito"&amp;18  Página &amp;P de &amp;N</oddFooter>
@@ -16721,6 +16730,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="265" t="inlineStr">
         <is>
@@ -17180,6 +17190,8 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="265" t="inlineStr">
         <is>
@@ -17410,6 +17422,8 @@
       <c r="D42" s="268" t="inlineStr"/>
       <c r="E42" s="268" t="inlineStr"/>
     </row>
+    <row r="43"/>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="265" t="inlineStr">
         <is>
@@ -17929,6 +17943,8 @@
       <c r="D75" s="268" t="inlineStr"/>
       <c r="E75" s="268" t="inlineStr"/>
     </row>
+    <row r="76"/>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="265" t="inlineStr">
         <is>
@@ -18106,6 +18122,7 @@
       </c>
       <c r="E86" s="268" t="inlineStr"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="279" t="inlineStr">
         <is>
@@ -23740,6 +23757,7 @@
         </is>
       </c>
     </row>
+    <row r="314"/>
     <row r="315">
       <c r="A315" s="279" t="inlineStr">
         <is>
@@ -23867,6 +23885,7 @@
         </is>
       </c>
     </row>
+    <row r="326"/>
     <row r="327">
       <c r="A327" s="279" t="inlineStr">
         <is>
@@ -28776,6 +28795,8 @@
         </is>
       </c>
     </row>
+    <row r="524"/>
+    <row r="525"/>
     <row r="526">
       <c r="B526" t="inlineStr">
         <is>
@@ -28860,6 +28881,7 @@
         </is>
       </c>
     </row>
+    <row r="533"/>
     <row r="534">
       <c r="A534" s="279" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Grade Cidade Jardim: imagens por link nas células, sem a aba de imagens
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -11,8 +11,7 @@
     <sheet name="2° PAVTO" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="PILOTIS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="APTO TIPO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="IMAGENS ESPECIFICAÇÕES " sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="PENDÊNCIAS" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="PENDÊNCIAS" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">OFFSET('CONTROLE DE REVISÕES '!$A$1,0,0,MAX(1,MAX(INDEX(('CONTROLE DE REVISÕES '!$A$1:$I$3000&amp;""&lt;&gt;"")*ROW('CONTROLE DE REVISÕES '!$A$1:$I$3000),0))),9)</definedName>
@@ -24,9 +23,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="3">OFFSET('PILOTIS'!$A$1,0,0,MAX(11,MAX(INDEX(('PILOTIS'!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('PILOTIS'!$A$1:$AF$3000),0))),32)</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'APTO TIPO'!$1:$11,'APTO TIPO'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">OFFSET('APTO TIPO'!$A$1,0,0,MAX(11,MAX(INDEX(('APTO TIPO'!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('APTO TIPO'!$A$1:$AF$3000),0))),32)</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'IMAGENS ESPECIFICAÇÕES '!$1:$11,'IMAGENS ESPECIFICAÇÕES '!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">OFFSET('IMAGENS ESPECIFICAÇÕES '!$A$1,0,0,MAX(26,MAX(INDEX(('IMAGENS ESPECIFICAÇÕES '!$A$1:$U$3000&amp;""&lt;&gt;"")*ROW('IMAGENS ESPECIFICAÇÕES '!$A$1:$U$3000),0))),21)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">OFFSET('PENDÊNCIAS'!$A$1,0,0,MAX(1,MAX(INDEX(('PENDÊNCIAS'!$A$1:$E$3000&amp;""&lt;&gt;"")*ROW('PENDÊNCIAS'!$A$1:$E$3000),0))),5)</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">OFFSET('PENDÊNCIAS'!$A$1,0,0,MAX(1,MAX(INDEX(('PENDÊNCIAS'!$A$1:$E$3000&amp;""&lt;&gt;"")*ROW('PENDÊNCIAS'!$A$1:$E$3000),0))),5)</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -4607,805 +4604,6 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>1</col>
-      <colOff>394853</colOff>
-      <row>4</row>
-      <rowOff>72735</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>1330036</colOff>
-      <row>5</row>
-      <rowOff>492183</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Imagem 1"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm flipH="1">
-          <a:off x="3366653" y="1749135"/>
-          <a:ext cx="935183" cy="914748"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>831275</colOff>
-      <row>0</row>
-      <rowOff>103909</rowOff>
-    </from>
-    <to>
-      <col>0</col>
-      <colOff>2753592</colOff>
-      <row>3</row>
-      <rowOff>335785</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Imagem 6"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip cstate="print" r:embed="rId24"/>
-        <a:srcRect b="16485"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="831275" y="103909"/>
-          <a:ext cx="1922317" cy="1470126"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>6</col>
-      <colOff>2247902</colOff>
-      <row>0</row>
-      <rowOff>100446</rowOff>
-    </from>
-    <to>
-      <col>7</col>
-      <colOff>1548246</colOff>
-      <row>3</row>
-      <rowOff>332322</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Imagem 7"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip cstate="print" r:embed="rId25"/>
-        <a:srcRect b="16485"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="25650827" y="100446"/>
-          <a:ext cx="1913658" cy="1470126"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>19</col>
-      <colOff>1513612</colOff>
-      <row>0</row>
-      <rowOff>128154</rowOff>
-    </from>
-    <to>
-      <col>20</col>
-      <colOff>1046019</colOff>
-      <row>3</row>
-      <rowOff>360030</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Imagem 8"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill rotWithShape="1">
-        <a:blip cstate="print" r:embed="rId26"/>
-        <a:srcRect b="16485"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="49910137" y="128154"/>
-          <a:ext cx="1913658" cy="1470126"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>370607</colOff>
-      <row>4</row>
-      <rowOff>117762</rowOff>
-    </from>
-    <ext cx="935183" cy="927787"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Imagem 4"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm flipH="1">
-          <a:off x="33212807" y="1794162"/>
-          <a:ext cx="935183" cy="927787"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>76200</colOff>
-      <row>12</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="981075" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>76200</colOff>
-      <row>12</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1562100" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>1695450</colOff>
-      <row>12</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1428750" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>3181350</colOff>
-      <row>12</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1438275" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>76200</colOff>
-      <row>12</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1428750" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>1562100</colOff>
-      <row>12</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1152525" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>76200</colOff>
-      <row>13</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1495425" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>1628775</colOff>
-      <row>13</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1428750" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="981075" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1628775" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="981075" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1809750" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>11</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="942975" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1219200" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>1352550</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1190625" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>2600325</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1428750" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>76200</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1476375" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>1609725</colOff>
-      <row>14</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="2419350" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>76200</colOff>
-      <row>15</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1428750" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>76200</colOff>
-      <row>15</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1419225" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="25" name="Image 25" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>1552575</colOff>
-      <row>15</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="1419225" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="26" name="Image 26" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
@@ -6043,7 +5241,7 @@
       <c r="B19" s="217" t="n"/>
       <c r="C19" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMAGENS ESPECIFICAÇÕES </t>
+          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
         </is>
       </c>
       <c r="D19" s="230" t="n"/>
@@ -6062,7 +5260,7 @@
       <c r="B20" s="217" t="n"/>
       <c r="C20" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMAGENS ESPECIFICAÇÕES </t>
+          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
         </is>
       </c>
       <c r="D20" s="230" t="n"/>
@@ -6081,7 +5279,7 @@
       <c r="B21" s="217" t="n"/>
       <c r="C21" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMAGENS ESPECIFICAÇÕES </t>
+          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
         </is>
       </c>
       <c r="D21" s="230" t="n"/>
@@ -6100,7 +5298,7 @@
       <c r="B22" s="221" t="n"/>
       <c r="C22" s="111" t="inlineStr">
         <is>
-          <t>IMAGENS ESPECIFICAÇÕES</t>
+          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
         </is>
       </c>
       <c r="D22" s="231" t="n"/>
@@ -6246,7 +5444,7 @@
       </c>
       <c r="E28" s="237" t="inlineStr">
         <is>
-          <t>Imagens das fichas TERMAS e VESTIÁRIOS - TERMAS da tabela v00 (págs. 7 e 8).</t>
+          <t>Imagens das fichas TERMAS e VESTIÁRIOS - TERMAS da tabela de acabamentos v00. Em 01/10/2026 a aba de imagens foi substituída pelo link "► VER IMAGEM (clique)" nas próprias células da grade.</t>
         </is>
       </c>
       <c r="F28" s="230" t="n"/>
@@ -12844,7 +12042,7 @@
       <c r="Y40" s="307" t="n"/>
       <c r="Z40" s="300" t="n"/>
     </row>
-    <row r="41" ht="224" customHeight="1">
+    <row r="41" ht="254" customHeight="1">
       <c r="A41" s="298" t="inlineStr">
         <is>
           <t>ESPAÇO TERMAS</t>
@@ -12852,7 +12050,8 @@
       </c>
       <c r="B41" s="320" t="inlineStr">
         <is>
-          <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
+          <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="C41" s="300" t="n"/>
@@ -12868,7 +12067,8 @@
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA48 - Parede rebocada e regularizada revestida em mármore branco selecionado, lote a ser aprovado, acabamento frisado com ranhuras de 4x4mm espassada a cada 12mm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-PA49 - Pilar em concreto rebocados e regularizados revestidos em mosaico de pastilhas, módulos de 32x259cm com pastilhas de 20x20mm, NARCISO Shading BlendDesenho e paginação conforme detalhamento. Argamassa e rejunte recomendados: Filgel plus 1101 bianco alabastro. Ref.:Bisazza. Amostra a ser aprovada pela GPA&amp;A</t>
+PA49 - Pilar em concreto rebocados e regularizados revestidos em mosaico de pastilhas, módulos de 32x259cm com pastilhas de 20x20mm, NARCISO Shading BlendDesenho e paginação conforme detalhamento. Argamassa e rejunte recomendados: Filgel plus 1101 bianco alabastro. Ref.:Bisazza. Amostra a ser aprovada pela GPA&amp;A
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="I41" s="316" t="inlineStr">
@@ -12898,7 +12098,8 @@
       </c>
       <c r="U41" s="317" t="inlineStr">
         <is>
-          <t>D54 - Chuveiro de embutir no teto Raindream, Roca, acabamento cromado, cód.: A5B3250C0C. Ref.: Roca. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
+          <t>D54 - Chuveiro de embutir no teto Raindream, Roca, acabamento cromado, cód.: A5B3250C0C. Ref.: Roca. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="V41" s="299" t="inlineStr">
@@ -13711,7 +12912,7 @@
       <c r="Y54" s="307" t="n"/>
       <c r="Z54" s="300" t="n"/>
     </row>
-    <row r="55" ht="194" customHeight="1">
+    <row r="55" ht="224" customHeight="1">
       <c r="A55" s="298" t="inlineStr">
         <is>
           <t>VESTIÁRIO FEM./MASC. - TERMAS</t>
@@ -13719,7 +12920,8 @@
       </c>
       <c r="B55" s="320" t="inlineStr">
         <is>
-          <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
+          <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="C55" s="300" t="n"/>
@@ -13735,7 +12937,8 @@
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA47 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 930, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A
-PA48 - Parede rebocada e regularizada revestida em mármore branco selecionado, lote a ser aprovado, acabamento frisado com ranhuras de 4x4mm espassada a cada 12mm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
+PA48 - Parede rebocada e regularizada revestida em mármore branco selecionado, lote a ser aprovado, acabamento frisado com ranhuras de 4x4mm espassada a cada 12mm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="I55" s="316" t="inlineStr">
@@ -13745,36 +12948,42 @@
       </c>
       <c r="J55" s="320" t="inlineStr">
         <is>
-          <t>D73 - Bancada em pedra natural, mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D73 - Bancada em pedra natural, mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="K55" s="317" t="inlineStr">
         <is>
-          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
+          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="L55" s="320" t="inlineStr">
         <is>
-          <t>D72 - Cuba de semiencaixe, linha Slim, cor branco, cód.: L.61040.M.17. Ref.: Deca</t>
+          <t>D72 - Cuba de semiencaixe, linha Slim, cor branco, cód.: L.61040.M.17. Ref.: Deca
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="M55" s="308" t="n"/>
       <c r="N55" s="308" t="n"/>
       <c r="O55" s="320" t="inlineStr">
         <is>
-          <t>D69 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca</t>
+          <t>D69 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="P55" s="316" t="inlineStr">
         <is>
-          <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="Q55" s="300" t="n"/>
       <c r="R55" s="307" t="n"/>
       <c r="S55" s="320" t="inlineStr">
         <is>
-          <t>D33 - Monocomando para chuveiro, linha Mix&amp;Match, acabamento cromado, cód.:90009312006. Ref.: Docol</t>
+          <t>D33 - Monocomando para chuveiro, linha Mix&amp;Match, acabamento cromado, cód.:90009312006. Ref.: Docol
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="T55" s="299" t="inlineStr">
@@ -13785,7 +12994,8 @@
       </c>
       <c r="U55" s="317" t="inlineStr">
         <is>
-          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
+          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.
+► VER IMAGEM (clique)</t>
         </is>
       </c>
       <c r="V55" s="299" t="inlineStr">
@@ -14249,6 +13459,20 @@
     <mergeCell ref="V12:Z12"/>
     <mergeCell ref="V7:AD8"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" tooltip="Abrir imagem: P10 - Piso elevado em mármore branco selecionado" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" tooltip="Abrir imagem: PA49 - Mosaico Bisazza (painel e pilar)" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" tooltip="Abrir imagem: D54 - Chuveiro de embutir no teto Raindream, Roca" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" tooltip="Abrir imagem: P10 - Piso elevado em mármore branco selecionado" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" tooltip="Abrir imagem: PA47 - Pintura com tinta mineral, cor 930, Terracor" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" tooltip="Abrir imagem: D73 - Bancada em mármore branco selecionado" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" tooltip="Abrir imagem: D38 - Espelho liso incolor 4mm" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" tooltip="Abrir imagem: D72 - Cuba de semi-encaixe slim, Deca" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" tooltip="Abrir imagem: D69 - Torneira com sensor Decalux, Deca" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" tooltip="Abrir imagem: D22 - Bacia Carrara / Panache e assento" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S55" tooltip="Abrir imagem: D33 - Monocomando para chuveiro Mix&amp;Match, Docol" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U55" tooltip="Abrir imagem: D70 - Chuveiro 200 de parede Docol Eden" r:id="rId12"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="8" scale="38" pageOrder="overThenDown"/>
@@ -14264,7 +13488,7 @@
     <brk id="11" min="0" max="16383" man="1"/>
     <brk id="21" min="0" max="16383" man="1"/>
   </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
 </worksheet>
 </file>
 
@@ -15986,945 +15210,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor theme="0"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:AA33"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
-  <cols>
-    <col width="44.7109375" customWidth="1" style="14" min="1" max="1"/>
-    <col width="70.5703125" customWidth="1" style="3" min="2" max="6"/>
-    <col width="39.42578125" customWidth="1" style="3" min="7" max="8"/>
-    <col width="35.7109375" customWidth="1" style="3" min="9" max="14"/>
-    <col width="40.28515625" customWidth="1" style="3" min="15" max="15"/>
-    <col width="42" customWidth="1" style="3" min="16" max="16"/>
-    <col width="35.7109375" customWidth="1" style="3" min="17" max="17"/>
-    <col width="42.5703125" customWidth="1" style="3" min="18" max="18"/>
-    <col width="35.7109375" customWidth="1" style="3" min="19" max="27"/>
-    <col width="9.140625" customWidth="1" style="3" min="28" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="34.5" customHeight="1">
-      <c r="A1" s="153" t="n"/>
-      <c r="B1" s="137" t="inlineStr">
-        <is>
-          <t>GRADE DE ESPECIFICAÇÕES PARA ÁREA COMUM
-EDIFÍCIO JARDIM</t>
-        </is>
-      </c>
-      <c r="C1" s="209" t="n"/>
-      <c r="D1" s="209" t="n"/>
-      <c r="E1" s="209" t="n"/>
-      <c r="F1" s="208" t="n"/>
-      <c r="G1" s="113" t="n"/>
-      <c r="H1" s="208" t="n"/>
-      <c r="I1" s="248">
-        <f>B1</f>
-        <v/>
-      </c>
-      <c r="J1" s="209" t="n"/>
-      <c r="K1" s="209" t="n"/>
-      <c r="L1" s="209" t="n"/>
-      <c r="M1" s="209" t="n"/>
-      <c r="N1" s="209" t="n"/>
-      <c r="O1" s="209" t="n"/>
-      <c r="P1" s="209" t="n"/>
-      <c r="Q1" s="209" t="n"/>
-      <c r="R1" s="209" t="n"/>
-      <c r="S1" s="249" t="n"/>
-      <c r="T1" s="113" t="n"/>
-      <c r="U1" s="208" t="n"/>
-      <c r="V1" s="55" t="n"/>
-      <c r="W1" s="55" t="n"/>
-      <c r="X1" s="55" t="n"/>
-      <c r="Y1" s="55" t="n"/>
-      <c r="Z1" s="194" t="n"/>
-    </row>
-    <row r="2" ht="28.5" customHeight="1">
-      <c r="A2" s="238" t="n"/>
-      <c r="B2" s="210" t="n"/>
-      <c r="F2" s="211" t="n"/>
-      <c r="G2" s="210" t="n"/>
-      <c r="H2" s="211" t="n"/>
-      <c r="I2" s="210" t="n"/>
-      <c r="S2" s="250" t="n"/>
-      <c r="T2" s="210" t="n"/>
-      <c r="U2" s="211" t="n"/>
-      <c r="V2" s="55" t="n"/>
-      <c r="W2" s="55" t="n"/>
-      <c r="X2" s="55" t="n"/>
-      <c r="Y2" s="55" t="n"/>
-    </row>
-    <row r="3" ht="34.5" customHeight="1">
-      <c r="A3" s="238" t="n"/>
-      <c r="B3" s="210" t="n"/>
-      <c r="F3" s="211" t="n"/>
-      <c r="G3" s="210" t="n"/>
-      <c r="H3" s="211" t="n"/>
-      <c r="I3" s="210" t="n"/>
-      <c r="S3" s="250" t="n"/>
-      <c r="T3" s="210" t="n"/>
-      <c r="U3" s="211" t="n"/>
-      <c r="V3" s="55" t="n"/>
-      <c r="W3" s="55" t="n"/>
-      <c r="X3" s="55" t="n"/>
-      <c r="Y3" s="55" t="n"/>
-    </row>
-    <row r="4" ht="28.5" customHeight="1" thickBot="1">
-      <c r="A4" s="239" t="n"/>
-      <c r="B4" s="213" t="n"/>
-      <c r="C4" s="216" t="n"/>
-      <c r="D4" s="216" t="n"/>
-      <c r="E4" s="216" t="n"/>
-      <c r="F4" s="214" t="n"/>
-      <c r="G4" s="213" t="n"/>
-      <c r="H4" s="214" t="n"/>
-      <c r="I4" s="251" t="n"/>
-      <c r="J4" s="223" t="n"/>
-      <c r="K4" s="223" t="n"/>
-      <c r="L4" s="223" t="n"/>
-      <c r="M4" s="223" t="n"/>
-      <c r="N4" s="223" t="n"/>
-      <c r="O4" s="223" t="n"/>
-      <c r="P4" s="223" t="n"/>
-      <c r="Q4" s="223" t="n"/>
-      <c r="R4" s="223" t="n"/>
-      <c r="S4" s="252" t="n"/>
-      <c r="T4" s="213" t="n"/>
-      <c r="U4" s="214" t="n"/>
-      <c r="V4" s="55" t="n"/>
-      <c r="W4" s="55" t="n"/>
-      <c r="X4" s="55" t="n"/>
-      <c r="Y4" s="55" t="n"/>
-    </row>
-    <row r="5" ht="39.95" customHeight="1">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="127" t="inlineStr">
-        <is>
-          <t>PADRÃO DE FORMATAÇÃO: ITEM, LINHA, MARCA, TAMANHO, COR E/OU ACABAMENTOS. CÓDIGO. COR DE REJUNTE.</t>
-        </is>
-      </c>
-      <c r="C5" s="209" t="n"/>
-      <c r="D5" s="209" t="n"/>
-      <c r="E5" s="209" t="n"/>
-      <c r="F5" s="208" t="n"/>
-      <c r="G5" s="27" t="inlineStr">
-        <is>
-          <t>XXXXXXX</t>
-        </is>
-      </c>
-      <c r="H5" s="229" t="n"/>
-      <c r="I5" s="253" t="inlineStr">
-        <is>
-          <t>*ATENÇÃO: PARA TODOS OS REJUNTES, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO
-COM PROJETOS EXECUTIVOS DE ACORDO COM ALTURA DO CONTRAPISO</t>
-        </is>
-      </c>
-      <c r="S5" s="250" t="n"/>
-      <c r="T5" s="119" t="inlineStr">
-        <is>
-          <t>XXXXXX</t>
-        </is>
-      </c>
-      <c r="U5" s="240" t="n"/>
-      <c r="V5" s="56" t="n"/>
-      <c r="W5" s="56" t="n"/>
-      <c r="X5" s="56" t="n"/>
-      <c r="Y5" s="56" t="n"/>
-      <c r="Z5" s="198" t="n"/>
-    </row>
-    <row r="6" ht="43.5" customFormat="1" customHeight="1" s="4" thickBot="1">
-      <c r="A6" s="52" t="inlineStr">
-        <is>
-          <t>DATA</t>
-        </is>
-      </c>
-      <c r="B6" s="213" t="n"/>
-      <c r="C6" s="216" t="n"/>
-      <c r="D6" s="216" t="n"/>
-      <c r="E6" s="216" t="n"/>
-      <c r="F6" s="214" t="n"/>
-      <c r="G6" s="52" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL</t>
-        </is>
-      </c>
-      <c r="H6" s="226" t="n"/>
-      <c r="I6" s="210" t="n"/>
-      <c r="S6" s="250" t="n"/>
-      <c r="T6" s="201" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL</t>
-        </is>
-      </c>
-      <c r="U6" s="221" t="n"/>
-      <c r="V6" s="56" t="n"/>
-      <c r="W6" s="56" t="n"/>
-      <c r="X6" s="56" t="n"/>
-      <c r="Y6" s="56" t="n"/>
-      <c r="Z6" s="203" t="n"/>
-    </row>
-    <row r="7" ht="69.75" customHeight="1">
-      <c r="A7" s="27" t="inlineStr">
-        <is>
-          <t>REV. R00</t>
-        </is>
-      </c>
-      <c r="B7" s="186" t="inlineStr">
-        <is>
-          <t>*ATENÇÃO: PARA TODOS OS REJUNTES E TEXTURAS, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO ARQUITETURA DE ACORDO COM ALTURA DO CONTRAPISO. A DEFINIÇÃO DA ALTURA DE RODABANCAS E TESTEIRAS DEVEM SER DEFINIDAS CASO A CASO CONFORME IMAGENS E/OU ELEMENTOS DO PROJETO, COMO PEITORIL E PAGINAÇÃO DA PAREDE. QUANDO O REVESTIMENTO DA PAREDE NÃO FOR CERÂMICO, CONSIDERAR UMA ALTURA MAIOR DE RODABANCA. AS ESPECIFICAÇÕES PODERAM SER ALTERADAS CONFORME DISPONIBILIDADE DE MERCADO, VALIDAR JUNTO A ARQUITETURA CASO NO MOMENTO DA COMPRA O ITEM TENHA SAÍDO DE LINHA.</t>
-        </is>
-      </c>
-      <c r="C7" s="209" t="n"/>
-      <c r="D7" s="209" t="n"/>
-      <c r="E7" s="209" t="n"/>
-      <c r="F7" s="208" t="n"/>
-      <c r="G7" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INFO. ANTERIOR </t>
-        </is>
-      </c>
-      <c r="H7" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INFO. REVISADA </t>
-        </is>
-      </c>
-      <c r="I7" s="254" t="inlineStr">
-        <is>
-          <t>*ATENÇÃO: PARA TODOS OS REJUNTES E TEXTURAS, FAZER TESTES E APROVAR COM ARQUITETURA. PARA TODOS OS RALOS, APROVAR MODELO ARQUITETURA DE ACORDO COM ALTURA DO CONTRAPISO. A DEFINIÇÃO DA ALTURA DE RODABANCAS E TESTEIRAS DEVEM SER DEFINIDAS CASO A CASO CONFORME IMAGENS E/OU ELEMENTOS DO PROJETO, COMO PEITORIL E PAGINAÇÃO DA PAREDE. QUANDO O REVESTIMENTO DA PAREDE NÃO FOR CERÂMICO, CONSIDERAR UMA ALTURA MAIOR DE RODABANCA. AS ESPECIFICAÇÕES PODERAM SER ALTERADAS CONFORME DISPONIBILIDADE DE MERCADO, VALIDAR JUNTO A ARQUITETURA CASO NO MOMENTO DA COMPRA O ITEM TENHA SAÍDO DE LINHA.</t>
-        </is>
-      </c>
-      <c r="J7" s="209" t="n"/>
-      <c r="K7" s="209" t="n"/>
-      <c r="L7" s="209" t="n"/>
-      <c r="M7" s="209" t="n"/>
-      <c r="N7" s="209" t="n"/>
-      <c r="O7" s="209" t="n"/>
-      <c r="P7" s="209" t="n"/>
-      <c r="Q7" s="209" t="n"/>
-      <c r="R7" s="209" t="n"/>
-      <c r="S7" s="249" t="n"/>
-      <c r="T7" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INFO. ANTERIOR </t>
-        </is>
-      </c>
-      <c r="U7" s="53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INFO. REVISADA </t>
-        </is>
-      </c>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
-      <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="57" t="n"/>
-      <c r="AA7" s="58" t="n"/>
-    </row>
-    <row r="8" ht="69.75" customFormat="1" customHeight="1" s="4" thickBot="1">
-      <c r="A8" s="52" t="inlineStr">
-        <is>
-          <t>REVISÃO</t>
-        </is>
-      </c>
-      <c r="B8" s="213" t="n"/>
-      <c r="C8" s="216" t="n"/>
-      <c r="D8" s="216" t="n"/>
-      <c r="E8" s="216" t="n"/>
-      <c r="F8" s="214" t="n"/>
-      <c r="G8" s="255" t="inlineStr">
-        <is>
-          <t>LEGENDA</t>
-        </is>
-      </c>
-      <c r="H8" s="226" t="n"/>
-      <c r="I8" s="251" t="n"/>
-      <c r="J8" s="223" t="n"/>
-      <c r="K8" s="223" t="n"/>
-      <c r="L8" s="223" t="n"/>
-      <c r="M8" s="223" t="n"/>
-      <c r="N8" s="223" t="n"/>
-      <c r="O8" s="223" t="n"/>
-      <c r="P8" s="223" t="n"/>
-      <c r="Q8" s="223" t="n"/>
-      <c r="R8" s="223" t="n"/>
-      <c r="S8" s="252" t="n"/>
-      <c r="T8" s="121" t="inlineStr">
-        <is>
-          <t>LEGENDA</t>
-        </is>
-      </c>
-      <c r="U8" s="221" t="n"/>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="5" t="n"/>
-      <c r="X8" s="5" t="n"/>
-      <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="193" t="n"/>
-    </row>
-    <row r="9" ht="14.1" customFormat="1" customHeight="1" s="6">
-      <c r="A9" s="5" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="193" t="n"/>
-      <c r="H9" s="193" t="n"/>
-      <c r="I9" s="10" t="n"/>
-      <c r="J9" s="10" t="n"/>
-      <c r="K9" s="10" t="n"/>
-      <c r="L9" s="11" t="n"/>
-      <c r="M9" s="11" t="n"/>
-      <c r="N9" s="10" t="n"/>
-      <c r="O9" s="10" t="n"/>
-      <c r="P9" s="10" t="n"/>
-      <c r="Q9" s="10" t="n"/>
-      <c r="R9" s="10" t="n"/>
-      <c r="S9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
-      <c r="V9" s="11" t="n"/>
-      <c r="W9" s="10" t="n"/>
-      <c r="X9" s="10" t="n"/>
-      <c r="Y9" s="10" t="n"/>
-      <c r="Z9" s="10" t="n"/>
-      <c r="AA9" s="10" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="152" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="C10" s="216" t="n"/>
-      <c r="D10" s="216" t="n"/>
-      <c r="E10" s="216" t="n"/>
-      <c r="F10" s="216" t="n"/>
-      <c r="G10" s="216" t="n"/>
-      <c r="H10" s="214" t="n"/>
-      <c r="I10" s="152" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOUÇAS E METAIS </t>
-        </is>
-      </c>
-      <c r="J10" s="216" t="n"/>
-      <c r="K10" s="216" t="n"/>
-      <c r="L10" s="216" t="n"/>
-      <c r="M10" s="216" t="n"/>
-      <c r="N10" s="216" t="n"/>
-      <c r="O10" s="216" t="n"/>
-      <c r="P10" s="216" t="n"/>
-      <c r="Q10" s="216" t="n"/>
-      <c r="R10" s="214" t="n"/>
-      <c r="S10" s="152" t="inlineStr">
-        <is>
-          <t>COMPLEMENTARES</t>
-        </is>
-      </c>
-      <c r="T10" s="216" t="n"/>
-      <c r="U10" s="214" t="n"/>
-    </row>
-    <row r="11" ht="171.75" customFormat="1" customHeight="1" s="12" thickBot="1">
-      <c r="A11" s="46" t="n"/>
-      <c r="B11" s="46" t="inlineStr">
-        <is>
-          <t>PISO</t>
-        </is>
-      </c>
-      <c r="C11" s="46" t="inlineStr">
-        <is>
-          <t>FILETE</t>
-        </is>
-      </c>
-      <c r="D11" s="46" t="inlineStr">
-        <is>
-          <t>PEITORIL</t>
-        </is>
-      </c>
-      <c r="E11" s="46" t="inlineStr">
-        <is>
-          <t>RODAPÉ</t>
-        </is>
-      </c>
-      <c r="F11" s="46" t="inlineStr">
-        <is>
-          <t>PAREDE</t>
-        </is>
-      </c>
-      <c r="G11" s="256" t="inlineStr">
-        <is>
-          <t>BANCADA</t>
-        </is>
-      </c>
-      <c r="H11" s="221" t="n"/>
-      <c r="I11" s="46" t="inlineStr">
-        <is>
-          <t>LOUÇAS, CUBAS E TANQUES</t>
-        </is>
-      </c>
-      <c r="J11" s="46" t="inlineStr">
-        <is>
-          <t>VÁLVULAS DE CUBAS E TANQUES</t>
-        </is>
-      </c>
-      <c r="K11" s="46" t="inlineStr">
-        <is>
-          <t>SIFÕES</t>
-        </is>
-      </c>
-      <c r="L11" s="46" t="inlineStr">
-        <is>
-          <t>TORNEIRAS</t>
-        </is>
-      </c>
-      <c r="M11" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> BACIAS SANITÁRIAS</t>
-        </is>
-      </c>
-      <c r="N11" s="46" t="inlineStr">
-        <is>
-          <t>DUCHAS HIGIÊNICAS</t>
-        </is>
-      </c>
-      <c r="O11" s="46" t="inlineStr">
-        <is>
-          <t>ACABAMENTOS DE REGISTROS GERAL</t>
-        </is>
-      </c>
-      <c r="P11" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ACIONAMENTO DE CHUVEIRO </t>
-        </is>
-      </c>
-      <c r="Q11" s="46" t="inlineStr">
-        <is>
-          <t>RALOS</t>
-        </is>
-      </c>
-      <c r="R11" s="46" t="inlineStr">
-        <is>
-          <t>ACABAMENTOS ELÉTRICOS</t>
-        </is>
-      </c>
-      <c r="S11" s="46" t="inlineStr">
-        <is>
-          <t>MAÇANETAS</t>
-        </is>
-      </c>
-      <c r="T11" s="46" t="inlineStr">
-        <is>
-          <t>PORTAS</t>
-        </is>
-      </c>
-      <c r="U11" s="54" t="inlineStr">
-        <is>
-          <t>PORTAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customFormat="1" customHeight="1" s="13" thickBot="1">
-      <c r="A12" s="51" t="n"/>
-      <c r="B12" s="124" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="C12" s="241" t="n"/>
-      <c r="D12" s="241" t="n"/>
-      <c r="E12" s="241" t="n"/>
-      <c r="F12" s="241" t="n"/>
-      <c r="G12" s="241" t="n"/>
-      <c r="H12" s="242" t="n"/>
-      <c r="I12" s="123" t="inlineStr">
-        <is>
-          <t>GERAL</t>
-        </is>
-      </c>
-      <c r="J12" s="241" t="n"/>
-      <c r="K12" s="241" t="n"/>
-      <c r="L12" s="241" t="n"/>
-      <c r="M12" s="241" t="n"/>
-      <c r="N12" s="241" t="n"/>
-      <c r="O12" s="241" t="n"/>
-      <c r="P12" s="241" t="n"/>
-      <c r="Q12" s="241" t="n"/>
-      <c r="R12" s="241" t="n"/>
-      <c r="S12" s="241" t="n"/>
-      <c r="T12" s="241" t="n"/>
-      <c r="U12" s="242" t="n"/>
-    </row>
-    <row r="13" ht="203.25" customHeight="1">
-      <c r="A13" s="156" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IMAGENS CONFORME ESPECIFICAÇÕES </t>
-        </is>
-      </c>
-      <c r="B13" s="257" t="inlineStr">
-        <is>
-          <t>ESPAÇO TERMAS
-P10 - Piso elevado em mármore branco selecionado</t>
-        </is>
-      </c>
-      <c r="C13" s="49" t="n"/>
-      <c r="D13" s="49" t="n"/>
-      <c r="E13" s="49" t="n"/>
-      <c r="F13" s="258" t="inlineStr">
-        <is>
-          <t>ESPAÇO TERMAS
-PA49 - Mosaico Bisazza (painel): New Sterlizia / Narciso</t>
-        </is>
-      </c>
-      <c r="G13" s="259" t="n"/>
-      <c r="H13" s="240" t="n"/>
-      <c r="I13" s="49" t="n"/>
-      <c r="J13" s="49" t="n"/>
-      <c r="K13" s="49" t="n"/>
-      <c r="L13" s="49" t="n"/>
-      <c r="M13" s="49" t="n"/>
-      <c r="N13" s="49" t="n"/>
-      <c r="O13" s="49" t="n"/>
-      <c r="P13" s="258" t="inlineStr">
-        <is>
-          <t>ESPAÇO TERMAS
-D54 - Chuveiro de embutir no teto Raindream, Roca</t>
-        </is>
-      </c>
-      <c r="Q13" s="49" t="n"/>
-      <c r="R13" s="49" t="n"/>
-      <c r="S13" s="49" t="n"/>
-      <c r="T13" s="49" t="n"/>
-      <c r="U13" s="48" t="n"/>
-    </row>
-    <row r="14" ht="203.25" customHeight="1">
-      <c r="A14" s="260" t="n"/>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="32" t="n"/>
-      <c r="D14" s="32" t="n"/>
-      <c r="E14" s="32" t="n"/>
-      <c r="F14" s="261" t="inlineStr">
-        <is>
-          <t>ESPAÇO TERMAS
-PA49 - Mosaico Bisazza (pilar): Narciso</t>
-        </is>
-      </c>
-      <c r="G14" s="32" t="n"/>
-      <c r="H14" s="217" t="n"/>
-      <c r="I14" s="32" t="n"/>
-      <c r="J14" s="32" t="n"/>
-      <c r="K14" s="32" t="n"/>
-      <c r="L14" s="32" t="n"/>
-      <c r="M14" s="32" t="n"/>
-      <c r="N14" s="32" t="n"/>
-      <c r="O14" s="32" t="n"/>
-      <c r="P14" s="32" t="n"/>
-      <c r="Q14" s="32" t="n"/>
-      <c r="R14" s="32" t="n"/>
-      <c r="S14" s="32" t="n"/>
-      <c r="T14" s="32" t="n"/>
-      <c r="U14" s="31" t="n"/>
-    </row>
-    <row r="15" ht="203.25" customHeight="1">
-      <c r="A15" s="260" t="n"/>
-      <c r="B15" s="262" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-P10 - Piso elevado em mármore branco selecionado</t>
-        </is>
-      </c>
-      <c r="C15" s="32" t="n"/>
-      <c r="D15" s="32" t="n"/>
-      <c r="E15" s="32" t="n"/>
-      <c r="F15" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-D38 - Espelho liso incolor 4mm</t>
-        </is>
-      </c>
-      <c r="G15" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-D73 - Bancada em mármore branco selecionado</t>
-        </is>
-      </c>
-      <c r="H15" s="217" t="n"/>
-      <c r="I15" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-D72 - Cuba de semi-encaixe slim, Deca</t>
-        </is>
-      </c>
-      <c r="J15" s="32" t="n"/>
-      <c r="K15" s="32" t="n"/>
-      <c r="L15" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-D69 - Torneira com sensor Decalux, Deca</t>
-        </is>
-      </c>
-      <c r="M15" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-D22 - Bacia Carrara (Deca) / Panache (Kohler) e assento</t>
-        </is>
-      </c>
-      <c r="N15" s="32" t="n"/>
-      <c r="O15" s="32" t="n"/>
-      <c r="P15" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-D33 - Monocomando para chuveiro Mix&amp;Match, Docol</t>
-        </is>
-      </c>
-      <c r="Q15" s="32" t="n"/>
-      <c r="R15" s="32" t="n"/>
-      <c r="S15" s="32" t="n"/>
-      <c r="T15" s="32" t="n"/>
-      <c r="U15" s="31" t="n"/>
-    </row>
-    <row r="16" ht="203.25" customHeight="1">
-      <c r="A16" s="260" t="n"/>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="32" t="n"/>
-      <c r="D16" s="32" t="n"/>
-      <c r="E16" s="32" t="n"/>
-      <c r="F16" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-PA47 - Pintura com tinta mineral, cor 930, Terracor</t>
-        </is>
-      </c>
-      <c r="G16" s="32" t="n"/>
-      <c r="H16" s="217" t="n"/>
-      <c r="I16" s="32" t="n"/>
-      <c r="J16" s="32" t="n"/>
-      <c r="K16" s="32" t="n"/>
-      <c r="L16" s="32" t="n"/>
-      <c r="M16" s="32" t="n"/>
-      <c r="N16" s="32" t="n"/>
-      <c r="O16" s="32" t="n"/>
-      <c r="P16" s="261" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEM./MASC. - TERMAS
-D70 - Chuveiro 200 de parede Docol Eden</t>
-        </is>
-      </c>
-      <c r="Q16" s="32" t="n"/>
-      <c r="R16" s="32" t="n"/>
-      <c r="S16" s="32" t="n"/>
-      <c r="T16" s="32" t="n"/>
-      <c r="U16" s="31" t="n"/>
-    </row>
-    <row r="17" ht="203.25" customHeight="1">
-      <c r="A17" s="260" t="n"/>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="32" t="n"/>
-      <c r="D17" s="32" t="n"/>
-      <c r="E17" s="32" t="n"/>
-      <c r="F17" s="33" t="n"/>
-      <c r="G17" s="32" t="n"/>
-      <c r="H17" s="217" t="n"/>
-      <c r="I17" s="32" t="n"/>
-      <c r="J17" s="32" t="n"/>
-      <c r="K17" s="32" t="n"/>
-      <c r="L17" s="32" t="n"/>
-      <c r="M17" s="32" t="n"/>
-      <c r="N17" s="32" t="n"/>
-      <c r="O17" s="32" t="n"/>
-      <c r="P17" s="32" t="n"/>
-      <c r="Q17" s="32" t="n"/>
-      <c r="R17" s="32" t="n"/>
-      <c r="S17" s="32" t="n"/>
-      <c r="T17" s="32" t="n"/>
-      <c r="U17" s="31" t="n"/>
-    </row>
-    <row r="18" ht="203.25" customHeight="1">
-      <c r="A18" s="260" t="n"/>
-      <c r="B18" s="31" t="n"/>
-      <c r="C18" s="32" t="n"/>
-      <c r="D18" s="32" t="n"/>
-      <c r="E18" s="32" t="n"/>
-      <c r="F18" s="33" t="n"/>
-      <c r="G18" s="32" t="n"/>
-      <c r="H18" s="217" t="n"/>
-      <c r="I18" s="32" t="n"/>
-      <c r="J18" s="32" t="n"/>
-      <c r="K18" s="32" t="n"/>
-      <c r="L18" s="32" t="n"/>
-      <c r="M18" s="32" t="n"/>
-      <c r="N18" s="32" t="n"/>
-      <c r="O18" s="32" t="n"/>
-      <c r="P18" s="32" t="n"/>
-      <c r="Q18" s="32" t="n"/>
-      <c r="R18" s="32" t="n"/>
-      <c r="S18" s="32" t="n"/>
-      <c r="T18" s="32" t="n"/>
-      <c r="U18" s="31" t="n"/>
-    </row>
-    <row r="19" ht="203.25" customHeight="1" thickBot="1">
-      <c r="A19" s="260" t="n"/>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="32" t="n"/>
-      <c r="D19" s="32" t="n"/>
-      <c r="E19" s="32" t="n"/>
-      <c r="F19" s="33" t="n"/>
-      <c r="G19" s="32" t="n"/>
-      <c r="H19" s="217" t="n"/>
-      <c r="I19" s="32" t="n"/>
-      <c r="J19" s="32" t="n"/>
-      <c r="K19" s="32" t="n"/>
-      <c r="L19" s="32" t="n"/>
-      <c r="M19" s="32" t="n"/>
-      <c r="N19" s="32" t="n"/>
-      <c r="O19" s="32" t="n"/>
-      <c r="P19" s="32" t="n"/>
-      <c r="Q19" s="32" t="n"/>
-      <c r="R19" s="32" t="n"/>
-      <c r="S19" s="32" t="n"/>
-      <c r="T19" s="32" t="n"/>
-      <c r="U19" s="31" t="n"/>
-    </row>
-    <row r="20" ht="203.25" customHeight="1">
-      <c r="A20" s="156" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IMAGENS CONFORME ESPECIFICAÇÕES </t>
-        </is>
-      </c>
-      <c r="B20" s="31" t="n"/>
-      <c r="C20" s="32" t="n"/>
-      <c r="D20" s="32" t="n"/>
-      <c r="F20" s="33" t="n"/>
-      <c r="G20" s="32" t="n"/>
-      <c r="H20" s="217" t="n"/>
-      <c r="I20" s="32" t="n"/>
-      <c r="J20" s="32" t="n"/>
-      <c r="K20" s="32" t="n"/>
-      <c r="L20" s="32" t="n"/>
-      <c r="M20" s="32" t="n"/>
-      <c r="N20" s="32" t="n"/>
-      <c r="O20" s="32" t="n"/>
-      <c r="P20" s="32" t="n"/>
-      <c r="Q20" s="32" t="n"/>
-      <c r="R20" s="32" t="n"/>
-      <c r="S20" s="32" t="n"/>
-      <c r="T20" s="32" t="n"/>
-      <c r="U20" s="31" t="n"/>
-    </row>
-    <row r="21" ht="203.25" customHeight="1">
-      <c r="A21" s="260" t="n"/>
-      <c r="B21" s="31" t="n"/>
-      <c r="C21" s="32" t="n"/>
-      <c r="D21" s="32" t="n"/>
-      <c r="E21" s="32" t="n"/>
-      <c r="F21" s="33" t="n"/>
-      <c r="G21" s="32" t="n"/>
-      <c r="H21" s="217" t="n"/>
-      <c r="I21" s="32" t="n"/>
-      <c r="J21" s="32" t="n"/>
-      <c r="K21" s="32" t="n"/>
-      <c r="L21" s="32" t="n"/>
-      <c r="M21" s="32" t="n"/>
-      <c r="N21" s="32" t="n"/>
-      <c r="O21" s="32" t="n"/>
-      <c r="P21" s="32" t="n"/>
-      <c r="Q21" s="32" t="n"/>
-      <c r="R21" s="32" t="n"/>
-      <c r="S21" s="32" t="n"/>
-      <c r="T21" s="32" t="n"/>
-      <c r="U21" s="31" t="n"/>
-    </row>
-    <row r="22" ht="203.25" customHeight="1">
-      <c r="A22" s="260" t="n"/>
-      <c r="B22" s="34" t="n"/>
-      <c r="C22" s="32" t="n"/>
-      <c r="D22" s="32" t="n"/>
-      <c r="E22" s="34" t="n"/>
-      <c r="F22" s="34" t="n"/>
-      <c r="G22" s="32" t="n"/>
-      <c r="H22" s="217" t="n"/>
-      <c r="I22" s="32" t="n"/>
-      <c r="J22" s="32" t="n"/>
-      <c r="K22" s="32" t="n"/>
-      <c r="L22" s="32" t="n"/>
-      <c r="M22" s="32" t="n"/>
-      <c r="N22" s="32" t="n"/>
-      <c r="O22" s="32" t="n"/>
-      <c r="P22" s="32" t="n"/>
-      <c r="Q22" s="32" t="n"/>
-      <c r="R22" s="32" t="n"/>
-      <c r="S22" s="31" t="n"/>
-      <c r="T22" s="34" t="n"/>
-      <c r="U22" s="31" t="n"/>
-    </row>
-    <row r="23" ht="203.25" customHeight="1">
-      <c r="A23" s="260" t="n"/>
-      <c r="B23" s="34" t="n"/>
-      <c r="C23" s="34" t="n"/>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="34" t="n"/>
-      <c r="F23" s="34" t="n"/>
-      <c r="G23" s="32" t="n"/>
-      <c r="H23" s="217" t="n"/>
-      <c r="I23" s="32" t="n"/>
-      <c r="J23" s="32" t="n"/>
-      <c r="K23" s="32" t="n"/>
-      <c r="L23" s="32" t="n"/>
-      <c r="M23" s="32" t="n"/>
-      <c r="N23" s="32" t="n"/>
-      <c r="O23" s="32" t="n"/>
-      <c r="P23" s="32" t="n"/>
-      <c r="Q23" s="32" t="n"/>
-      <c r="R23" s="32" t="n"/>
-      <c r="S23" s="31" t="n"/>
-      <c r="T23" s="35" t="n"/>
-      <c r="U23" s="31" t="n"/>
-    </row>
-    <row r="24" ht="203.25" customHeight="1">
-      <c r="A24" s="260" t="n"/>
-      <c r="B24" s="35" t="n"/>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="32" t="n"/>
-      <c r="E24" s="35" t="n"/>
-      <c r="F24" s="35" t="n"/>
-      <c r="G24" s="32" t="n"/>
-      <c r="H24" s="217" t="n"/>
-      <c r="I24" s="32" t="n"/>
-      <c r="J24" s="37" t="n"/>
-      <c r="K24" s="37" t="n"/>
-      <c r="L24" s="31" t="n"/>
-      <c r="M24" s="31" t="n"/>
-      <c r="N24" s="32" t="n"/>
-      <c r="O24" s="35" t="n"/>
-      <c r="P24" s="32" t="n"/>
-      <c r="Q24" s="35" t="n"/>
-      <c r="R24" s="32" t="n"/>
-      <c r="S24" s="31" t="n"/>
-      <c r="T24" s="35" t="n"/>
-      <c r="U24" s="35" t="n"/>
-    </row>
-    <row r="25" ht="203.25" customHeight="1">
-      <c r="A25" s="260" t="n"/>
-      <c r="B25" s="35" t="n"/>
-      <c r="C25" s="35" t="n"/>
-      <c r="D25" s="37" t="n"/>
-      <c r="E25" s="35" t="n"/>
-      <c r="F25" s="35" t="n"/>
-      <c r="G25" s="32" t="n"/>
-      <c r="H25" s="217" t="n"/>
-      <c r="I25" s="32" t="n"/>
-      <c r="J25" s="32" t="n"/>
-      <c r="K25" s="32" t="n"/>
-      <c r="L25" s="32" t="n"/>
-      <c r="M25" s="32" t="n"/>
-      <c r="N25" s="32" t="n"/>
-      <c r="O25" s="32" t="n"/>
-      <c r="P25" s="32" t="n"/>
-      <c r="Q25" s="35" t="n"/>
-      <c r="R25" s="32" t="n"/>
-      <c r="S25" s="31" t="n"/>
-      <c r="T25" s="35" t="n"/>
-      <c r="U25" s="31" t="n"/>
-    </row>
-    <row r="26" ht="203.25" customHeight="1">
-      <c r="A26" s="260" t="n"/>
-      <c r="B26" s="35" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="37" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="35" t="n"/>
-      <c r="G26" s="32" t="n"/>
-      <c r="H26" s="217" t="n"/>
-      <c r="I26" s="35" t="n"/>
-      <c r="J26" s="35" t="n"/>
-      <c r="K26" s="35" t="n"/>
-      <c r="L26" s="35" t="n"/>
-      <c r="M26" s="32" t="n"/>
-      <c r="N26" s="32" t="n"/>
-      <c r="O26" s="35" t="n"/>
-      <c r="P26" s="32" t="n"/>
-      <c r="Q26" s="32" t="n"/>
-      <c r="R26" s="32" t="n"/>
-      <c r="S26" s="31" t="n"/>
-      <c r="T26" s="32" t="n"/>
-      <c r="U26" s="32" t="n"/>
-    </row>
-    <row r="27" ht="125.25" customHeight="1"/>
-    <row r="28" ht="2.1" customHeight="1"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33">
-      <c r="P33" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="T5:U5"/>
-    <mergeCell ref="T1:U4"/>
-    <mergeCell ref="A1:A4"/>
-    <mergeCell ref="B1:F4"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="A20:A26"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="I5:S6"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I10:R10"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="Z1:AA4"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="B5:F6"/>
-    <mergeCell ref="G1:H4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I1:S4"/>
-    <mergeCell ref="Z8:AA8"/>
-    <mergeCell ref="B7:F8"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="Z5:AA5"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="I12:U12"/>
-    <mergeCell ref="I7:S8"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="G22:H22"/>
-  </mergeCells>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0" right="0" top="0" bottom="0" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="8" scale="38" pageOrder="overThenDown"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;L&amp;"Aptos Narrow,Negrito"&amp;18  Página &amp;P de &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <colBreaks count="1" manualBreakCount="1">
-    <brk id="8" min="0" max="25" man="1"/>
-  </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>

<commit_message>
Grade Cidade Jardim: imagens na própria aba, com link interno VER IMAGEM / VOLTAR
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -34,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;* #,##0.00_-;\-&quot;R$&quot;* #,##0.00_-;_-&quot;R$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="68">
+  <fonts count="70">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -442,8 +442,20 @@
       <color rgb="FF9C0006"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00243F2E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="20"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -500,6 +512,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00243F2E"/>
       </patternFill>
     </fill>
   </fills>
@@ -1415,7 +1437,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="322">
+  <cellXfs count="324">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -2285,6 +2307,12 @@
     </xf>
     <xf numFmtId="0" fontId="67" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -3543,7 +3571,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
+        <a:blip cstate="print" r:embed="rId22"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3584,7 +3612,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip cstate="print" r:embed="rId11"/>
+        <a:blip cstate="print" r:embed="rId23"/>
         <a:srcRect b="16485"/>
         <a:stretch>
           <a:fillRect/>
@@ -3627,7 +3655,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip cstate="print" r:embed="rId12"/>
+        <a:blip cstate="print" r:embed="rId24"/>
         <a:srcRect b="16485"/>
         <a:stretch>
           <a:fillRect/>
@@ -3670,7 +3698,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip cstate="print" r:embed="rId13"/>
+        <a:blip cstate="print" r:embed="rId25"/>
         <a:srcRect b="16485"/>
         <a:stretch>
           <a:fillRect/>
@@ -3713,7 +3741,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip cstate="print" r:embed="rId14"/>
+        <a:blip cstate="print" r:embed="rId26"/>
         <a:srcRect b="16485"/>
         <a:stretch>
           <a:fillRect/>
@@ -4052,6 +4080,342 @@
         <a:prstGeom prst="rect">
           <avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>33</col>
+      <colOff>676275</colOff>
+      <row>40</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3486150" cy="2743200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>34</col>
+      <colOff>962025</colOff>
+      <row>40</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="2914650" cy="2743200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>35</col>
+      <colOff>676275</colOff>
+      <row>40</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3486150" cy="2743200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>33</col>
+      <colOff>923925</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3000375" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>34</col>
+      <colOff>923925</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3000375" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>35</col>
+      <colOff>923925</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3000375" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>36</col>
+      <colOff>923925</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3000375" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>37</col>
+      <colOff>923925</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3000375" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>38</col>
+      <colOff>923925</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="3000375" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>39</col>
+      <colOff>38100</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="4762500" cy="2000250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>40</col>
+      <colOff>38100</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="4762500" cy="2028825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>41</col>
+      <colOff>371475</colOff>
+      <row>54</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="4105275" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -5241,7 +5605,7 @@
       <c r="B19" s="217" t="n"/>
       <c r="C19" s="61" t="inlineStr">
         <is>
-          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
+          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
         </is>
       </c>
       <c r="D19" s="230" t="n"/>
@@ -5260,7 +5624,7 @@
       <c r="B20" s="217" t="n"/>
       <c r="C20" s="61" t="inlineStr">
         <is>
-          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
+          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
         </is>
       </c>
       <c r="D20" s="230" t="n"/>
@@ -5279,7 +5643,7 @@
       <c r="B21" s="217" t="n"/>
       <c r="C21" s="61" t="inlineStr">
         <is>
-          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
+          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
         </is>
       </c>
       <c r="D21" s="230" t="n"/>
@@ -5298,7 +5662,7 @@
       <c r="B22" s="221" t="n"/>
       <c r="C22" s="111" t="inlineStr">
         <is>
-          <t>IMAGENS: LINK "VER IMAGEM" NAS CÉLULAS DA GRADE</t>
+          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
         </is>
       </c>
       <c r="D22" s="231" t="n"/>
@@ -5444,7 +5808,7 @@
       </c>
       <c r="E28" s="237" t="inlineStr">
         <is>
-          <t>Imagens das fichas TERMAS e VESTIÁRIOS - TERMAS da tabela de acabamentos v00. Em 01/10/2026 a aba de imagens foi substituída pelo link "► VER IMAGEM (clique)" nas próprias células da grade.</t>
+          <t>Imagens das fichas TERMAS e VESTIÁRIOS - TERMAS da tabela de acabamentos v00. Em 02/10/2026 passaram para a própria aba PILOTIS, à direita da grade (a partir da coluna AH); o link "► VER IMAGEM (clique)" na célula leva à foto e "◄ VOLTAR" retorna.</t>
         </is>
       </c>
       <c r="F28" s="230" t="n"/>
@@ -9799,7 +10163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AF64"/>
+  <dimension ref="A1:AQ64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9834,6 +10198,18 @@
     <col width="31" customWidth="1" min="30" max="30"/>
     <col width="31" customWidth="1" min="31" max="31"/>
     <col width="31" customWidth="1" min="32" max="32"/>
+    <col width="72" customWidth="1" min="34" max="34"/>
+    <col width="72" customWidth="1" min="35" max="35"/>
+    <col width="72" customWidth="1" min="36" max="36"/>
+    <col width="72" customWidth="1" min="37" max="37"/>
+    <col width="72" customWidth="1" min="38" max="38"/>
+    <col width="72" customWidth="1" min="39" max="39"/>
+    <col width="72" customWidth="1" min="40" max="40"/>
+    <col width="72" customWidth="1" min="41" max="41"/>
+    <col width="72" customWidth="1" min="42" max="42"/>
+    <col width="72" customWidth="1" min="43" max="43"/>
+    <col width="72" customWidth="1" min="44" max="44"/>
+    <col width="72" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1" ht="34.5" customHeight="1">
@@ -10398,6 +10774,11 @@
 COMPLEMENTARES</t>
         </is>
       </c>
+      <c r="AH11" s="322" t="inlineStr">
+        <is>
+          <t>IMAGENS DAS ESPECIFICAÇÕES (fora da área de impressão)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customFormat="1" customHeight="1" s="13" thickBot="1">
       <c r="A12" s="51" t="n"/>
@@ -12115,6 +12496,24 @@
       </c>
       <c r="Y41" s="307" t="n"/>
       <c r="Z41" s="300" t="n"/>
+      <c r="AH41" s="323" t="inlineStr">
+        <is>
+          <t>P10 - Piso elevado em mármore branco selecionado
+◄ VOLTAR para B41</t>
+        </is>
+      </c>
+      <c r="AI41" s="323" t="inlineStr">
+        <is>
+          <t>PA49 - Mosaico Bisazza (painel e pilar)
+◄ VOLTAR para H41</t>
+        </is>
+      </c>
+      <c r="AJ41" s="323" t="inlineStr">
+        <is>
+          <t>D54 - Chuveiro de embutir no teto Raindream, Roca
+◄ VOLTAR para U41</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="89" customHeight="1">
       <c r="A42" s="298" t="inlineStr">
@@ -13018,6 +13417,60 @@
 D28 - Papeleira em aço Inox para papel interfolhado, modelo Basic, cód.:74.103. Ref.: Draco</t>
         </is>
       </c>
+      <c r="AH55" s="323" t="inlineStr">
+        <is>
+          <t>P10 - Piso elevado em mármore branco selecionado
+◄ VOLTAR para B55</t>
+        </is>
+      </c>
+      <c r="AI55" s="323" t="inlineStr">
+        <is>
+          <t>PA47 - Pintura com tinta mineral, cor 930, Terracor
+◄ VOLTAR para H55</t>
+        </is>
+      </c>
+      <c r="AJ55" s="323" t="inlineStr">
+        <is>
+          <t>D73 - Bancada em mármore branco selecionado
+◄ VOLTAR para J55</t>
+        </is>
+      </c>
+      <c r="AK55" s="323" t="inlineStr">
+        <is>
+          <t>D38 - Espelho liso incolor 4mm
+◄ VOLTAR para K55</t>
+        </is>
+      </c>
+      <c r="AL55" s="323" t="inlineStr">
+        <is>
+          <t>D72 - Cuba de semi-encaixe slim, Deca
+◄ VOLTAR para L55</t>
+        </is>
+      </c>
+      <c r="AM55" s="323" t="inlineStr">
+        <is>
+          <t>D69 - Torneira com sensor Decalux, Deca
+◄ VOLTAR para O55</t>
+        </is>
+      </c>
+      <c r="AN55" s="323" t="inlineStr">
+        <is>
+          <t>D22 - Bacia Carrara / Panache e assento
+◄ VOLTAR para P55</t>
+        </is>
+      </c>
+      <c r="AO55" s="323" t="inlineStr">
+        <is>
+          <t>D33 - Monocomando para chuveiro Mix&amp;Match, Docol
+◄ VOLTAR para S55</t>
+        </is>
+      </c>
+      <c r="AP55" s="323" t="inlineStr">
+        <is>
+          <t>D70 - Chuveiro 200 de parede Docol Eden
+◄ VOLTAR para U55</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="60" customHeight="1">
       <c r="A56" s="298" t="inlineStr">
@@ -13426,8 +13879,9 @@
       <c r="Z64" s="300" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="32">
     <mergeCell ref="L10:U10"/>
+    <mergeCell ref="AH11:AQ11"/>
     <mergeCell ref="B10:K10"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="T5:U5"/>
@@ -13460,18 +13914,30 @@
     <mergeCell ref="V7:AD8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" tooltip="Abrir imagem: P10 - Piso elevado em mármore branco selecionado" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" tooltip="Abrir imagem: PA49 - Mosaico Bisazza (painel e pilar)" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" tooltip="Abrir imagem: D54 - Chuveiro de embutir no teto Raindream, Roca" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" tooltip="Abrir imagem: P10 - Piso elevado em mármore branco selecionado" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" tooltip="Abrir imagem: PA47 - Pintura com tinta mineral, cor 930, Terracor" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" tooltip="Abrir imagem: D73 - Bancada em mármore branco selecionado" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" tooltip="Abrir imagem: D38 - Espelho liso incolor 4mm" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" tooltip="Abrir imagem: D72 - Cuba de semi-encaixe slim, Deca" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" tooltip="Abrir imagem: D69 - Torneira com sensor Decalux, Deca" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" tooltip="Abrir imagem: D22 - Bacia Carrara / Panache e assento" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S55" tooltip="Abrir imagem: D33 - Monocomando para chuveiro Mix&amp;Match, Docol" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U55" tooltip="Abrir imagem: D70 - Chuveiro 200 de parede Docol Eden" r:id="rId12"/>
+    <hyperlink ref="B41" location="'PILOTIS'!AH41" tooltip="Ver imagem: P10 - Piso elevado em mármore branco selecionado"/>
+    <hyperlink ref="H41" location="'PILOTIS'!AI41" tooltip="Ver imagem: PA49 - Mosaico Bisazza (painel e pilar)"/>
+    <hyperlink ref="U41" location="'PILOTIS'!AJ41" tooltip="Ver imagem: D54 - Chuveiro de embutir no teto Raindream, Roca"/>
+    <hyperlink ref="AH41" location="'PILOTIS'!B41" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AI41" location="'PILOTIS'!H41" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AJ41" location="'PILOTIS'!U41" tooltip="Voltar para a grade"/>
+    <hyperlink ref="B55" location="'PILOTIS'!AH55" tooltip="Ver imagem: P10 - Piso elevado em mármore branco selecionado"/>
+    <hyperlink ref="H55" location="'PILOTIS'!AI55" tooltip="Ver imagem: PA47 - Pintura com tinta mineral, cor 930, Terracor"/>
+    <hyperlink ref="J55" location="'PILOTIS'!AJ55" tooltip="Ver imagem: D73 - Bancada em mármore branco selecionado"/>
+    <hyperlink ref="K55" location="'PILOTIS'!AK55" tooltip="Ver imagem: D38 - Espelho liso incolor 4mm"/>
+    <hyperlink ref="L55" location="'PILOTIS'!AL55" tooltip="Ver imagem: D72 - Cuba de semi-encaixe slim, Deca"/>
+    <hyperlink ref="O55" location="'PILOTIS'!AM55" tooltip="Ver imagem: D69 - Torneira com sensor Decalux, Deca"/>
+    <hyperlink ref="P55" location="'PILOTIS'!AN55" tooltip="Ver imagem: D22 - Bacia Carrara / Panache e assento"/>
+    <hyperlink ref="S55" location="'PILOTIS'!AO55" tooltip="Ver imagem: D33 - Monocomando para chuveiro Mix&amp;Match, Docol"/>
+    <hyperlink ref="U55" location="'PILOTIS'!AP55" tooltip="Ver imagem: D70 - Chuveiro 200 de parede Docol Eden"/>
+    <hyperlink ref="AH55" location="'PILOTIS'!B55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AI55" location="'PILOTIS'!H55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AJ55" location="'PILOTIS'!J55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AK55" location="'PILOTIS'!K55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AL55" location="'PILOTIS'!L55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AM55" location="'PILOTIS'!O55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AN55" location="'PILOTIS'!P55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AO55" location="'PILOTIS'!S55" tooltip="Voltar para a grade"/>
+    <hyperlink ref="AP55" location="'PILOTIS'!U55" tooltip="Voltar para a grade"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
@@ -13488,7 +13954,7 @@
     <brk id="11" min="0" max="16383" man="1"/>
     <brk id="21" min="0" max="16383" man="1"/>
   </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Grade Cidade Jardim: R00 sem marcação de info revisada, aba CONFLITOS, sem linhas de grade
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -11,7 +11,8 @@
     <sheet name="2° PAVTO" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="PILOTIS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="APTO TIPO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="PENDÊNCIAS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CONFLITOS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PENDÊNCIAS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">OFFSET('CONTROLE DE REVISÕES '!$A$1,0,0,MAX(1,MAX(INDEX(('CONTROLE DE REVISÕES '!$A$1:$I$3000&amp;""&lt;&gt;"")*ROW('CONTROLE DE REVISÕES '!$A$1:$I$3000),0))),9)</definedName>
@@ -23,7 +24,9 @@
     <definedName name="_xlnm.Print_Area" localSheetId="3">OFFSET('PILOTIS'!$A$1,0,0,MAX(11,MAX(INDEX(('PILOTIS'!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('PILOTIS'!$A$1:$AF$3000),0))),32)</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'APTO TIPO'!$1:$11,'APTO TIPO'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">OFFSET('APTO TIPO'!$A$1,0,0,MAX(11,MAX(INDEX(('APTO TIPO'!$A$1:$AF$3000&amp;""&lt;&gt;"")*ROW('APTO TIPO'!$A$1:$AF$3000),0))),32)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">OFFSET('PENDÊNCIAS'!$A$1,0,0,MAX(1,MAX(INDEX(('PENDÊNCIAS'!$A$1:$E$3000&amp;""&lt;&gt;"")*ROW('PENDÊNCIAS'!$A$1:$E$3000),0))),5)</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'CONFLITOS'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">OFFSET('CONFLITOS'!$A$1,0,0,MAX(4,MAX(INDEX(('CONFLITOS'!$A$1:$H$3000&amp;""&lt;&gt;"")*ROW('CONFLITOS'!$A$1:$H$3000),0))),8)</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">OFFSET('PENDÊNCIAS'!$A$1,0,0,MAX(1,MAX(INDEX(('PENDÊNCIAS'!$A$1:$E$3000&amp;""&lt;&gt;"")*ROW('PENDÊNCIAS'!$A$1:$E$3000),0))),5)</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,7 +37,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;* #,##0.00_-;\-&quot;R$&quot;* #,##0.00_-;_-&quot;R$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="70">
+  <fonts count="75">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -454,8 +457,36 @@
       <color rgb="00FFFFFF"/>
       <sz val="20"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="009C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -524,8 +555,18 @@
         <fgColor rgb="00243F2E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="73">
+  <borders count="74">
     <border>
       <left/>
       <right/>
@@ -1424,6 +1465,20 @@
         <color rgb="00808080"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="008C8C8C"/>
+      </left>
+      <right style="thin">
+        <color rgb="008C8C8C"/>
+      </right>
+      <top style="thin">
+        <color rgb="008C8C8C"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="008C8C8C"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
@@ -1437,7 +1492,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="324">
+  <cellXfs count="335">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -2313,6 +2368,39 @@
     </xf>
     <xf numFmtId="0" fontId="68" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="65" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="13" borderId="73" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="73" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="73" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="73" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="14" borderId="73" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -6708,7 +6796,7 @@
           <t>ANTECÂMARA(ECLUSA PEDESTRE)</t>
         </is>
       </c>
-      <c r="B16" s="299" t="inlineStr">
+      <c r="B16" s="307" t="inlineStr">
         <is>
           <t>P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados na pedra devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -6716,18 +6804,18 @@
       <c r="C16" s="300" t="n"/>
       <c r="D16" s="300" t="n"/>
       <c r="E16" s="300" t="n"/>
-      <c r="F16" s="301" t="inlineStr">
+      <c r="F16" s="308" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G16" s="300" t="n"/>
-      <c r="H16" s="301" t="inlineStr">
+      <c r="H16" s="308" t="inlineStr">
         <is>
           <t>PA56 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica,  revestimento em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I16" s="301" t="inlineStr">
+      <c r="I16" s="308" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -6744,13 +6832,13 @@
       <c r="S16" s="300" t="n"/>
       <c r="T16" s="300" t="n"/>
       <c r="U16" s="300" t="n"/>
-      <c r="V16" s="301" t="inlineStr">
+      <c r="V16" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W16" s="300" t="n"/>
-      <c r="X16" s="299" t="inlineStr">
+      <c r="X16" s="307" t="inlineStr">
         <is>
           <t>D41 - Porta estruturada em alumínio com fechamento interno e externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A
 D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
@@ -6774,7 +6862,7 @@
       <c r="C17" s="300" t="n"/>
       <c r="D17" s="300" t="n"/>
       <c r="E17" s="300" t="n"/>
-      <c r="F17" s="301" t="inlineStr">
+      <c r="F17" s="308" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.
 ARQ-RD20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
@@ -6787,7 +6875,7 @@
 CONFLITO – Arquitetura: ARQ-PA02 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor a definir, acabamento acetinado.</t>
         </is>
       </c>
-      <c r="I17" s="301" t="inlineStr">
+      <c r="I17" s="308" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil
 ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
@@ -6805,7 +6893,7 @@
       <c r="S17" s="300" t="n"/>
       <c r="T17" s="300" t="n"/>
       <c r="U17" s="300" t="n"/>
-      <c r="V17" s="301" t="inlineStr">
+      <c r="V17" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
@@ -6821,7 +6909,7 @@
           <t>LAVABO GUARITA</t>
         </is>
       </c>
-      <c r="B18" s="299" t="inlineStr">
+      <c r="B18" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -6829,18 +6917,18 @@
       <c r="C18" s="300" t="n"/>
       <c r="D18" s="300" t="n"/>
       <c r="E18" s="300" t="n"/>
-      <c r="F18" s="301" t="inlineStr">
+      <c r="F18" s="308" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G18" s="300" t="n"/>
-      <c r="H18" s="301" t="inlineStr">
+      <c r="H18" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA02 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor a definir, acabamento acetinado.</t>
         </is>
       </c>
-      <c r="I18" s="301" t="inlineStr">
+      <c r="I18" s="308" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -6869,7 +6957,7 @@
           <t>CIRCULAÇÃO GUARITA</t>
         </is>
       </c>
-      <c r="B19" s="299" t="inlineStr">
+      <c r="B19" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -6877,18 +6965,18 @@
       <c r="C19" s="300" t="n"/>
       <c r="D19" s="300" t="n"/>
       <c r="E19" s="300" t="n"/>
-      <c r="F19" s="301" t="inlineStr">
+      <c r="F19" s="308" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G19" s="300" t="n"/>
-      <c r="H19" s="301" t="inlineStr">
+      <c r="H19" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I19" s="301" t="inlineStr">
+      <c r="I19" s="308" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -6917,7 +7005,7 @@
           <t>LOBBY ENTRADA</t>
         </is>
       </c>
-      <c r="B20" s="299" t="inlineStr">
+      <c r="B20" s="307" t="inlineStr">
         <is>
           <t>P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados na pedra devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -6925,13 +7013,13 @@
       <c r="C20" s="300" t="n"/>
       <c r="D20" s="300" t="n"/>
       <c r="E20" s="300" t="n"/>
-      <c r="F20" s="301" t="inlineStr">
+      <c r="F20" s="308" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G20" s="300" t="n"/>
-      <c r="H20" s="301" t="inlineStr">
+      <c r="H20" s="308" t="inlineStr">
         <is>
           <t>PA1 - Parede em alvenaria com reboco convencional 2,5cm, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.
 PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
@@ -6939,7 +7027,7 @@
 PA56 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica,  revestimento em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I20" s="301" t="inlineStr">
+      <c r="I20" s="308" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil
 T12 - Forro em chapa metálica dourada colada sobre MDF cru 6mm aparafusado em estrutura auxiliar do guarda corpo em metalon</t>
@@ -6957,20 +7045,20 @@
       <c r="S20" s="300" t="n"/>
       <c r="T20" s="300" t="n"/>
       <c r="U20" s="300" t="n"/>
-      <c r="V20" s="301" t="inlineStr">
+      <c r="V20" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W20" s="300" t="n"/>
-      <c r="X20" s="299" t="inlineStr">
+      <c r="X20" s="307" t="inlineStr">
         <is>
           <t>D41 - Porta estruturada em alumínio com fechamento interno e externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A
 D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y20" s="302" t="n"/>
-      <c r="Z20" s="301" t="inlineStr">
+      <c r="Z20" s="308" t="inlineStr">
         <is>
           <t>D63 - Guarda corpo em chapa metálica dourada colada sobre fechamento em MDF cru 6mm aparafusado em estrutura auxiliar de metalon. Dimensões e detalhes conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -6982,7 +7070,7 @@
           <t>HALL ELEVADORES</t>
         </is>
       </c>
-      <c r="B21" s="299" t="inlineStr">
+      <c r="B21" s="307" t="inlineStr">
         <is>
           <t>P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados na pedra devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -6990,20 +7078,20 @@
       <c r="C21" s="300" t="n"/>
       <c r="D21" s="300" t="n"/>
       <c r="E21" s="300" t="n"/>
-      <c r="F21" s="301" t="inlineStr">
+      <c r="F21" s="308" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G21" s="300" t="n"/>
-      <c r="H21" s="301" t="inlineStr">
+      <c r="H21" s="308" t="inlineStr">
         <is>
           <t>PA1 - Parede em alvenaria com reboco convencional 2,5cm, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.
 PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA54 - Parede em alvenaria regularizada, revestida em pedra natural, Basaltina, acabamento frisado. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I21" s="301" t="inlineStr">
+      <c r="I21" s="308" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7020,7 +7108,7 @@
       <c r="S21" s="300" t="n"/>
       <c r="T21" s="300" t="n"/>
       <c r="U21" s="300" t="n"/>
-      <c r="V21" s="301" t="inlineStr">
+      <c r="V21" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
@@ -7028,7 +7116,7 @@
       <c r="W21" s="300" t="n"/>
       <c r="X21" s="302" t="n"/>
       <c r="Y21" s="302" t="n"/>
-      <c r="Z21" s="301" t="inlineStr">
+      <c r="Z21" s="308" t="inlineStr">
         <is>
           <t>D64 - Quadro para elevador em chapa metálica 8mm com acabamento em pintura eletrostática, cor branca. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -7040,7 +7128,7 @@
           <t>CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTICÂRA</t>
         </is>
       </c>
-      <c r="B22" s="299" t="inlineStr">
+      <c r="B22" s="307" t="inlineStr">
         <is>
           <t>ARQ-P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -7048,18 +7136,18 @@
       <c r="C22" s="300" t="n"/>
       <c r="D22" s="300" t="n"/>
       <c r="E22" s="300" t="n"/>
-      <c r="F22" s="301" t="inlineStr">
+      <c r="F22" s="308" t="inlineStr">
         <is>
           <t>ARQ-RD20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G22" s="300" t="n"/>
-      <c r="H22" s="301" t="inlineStr">
+      <c r="H22" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I22" s="301" t="inlineStr">
+      <c r="I22" s="308" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7088,7 +7176,7 @@
           <t xml:space="preserve">HALL GARGEM </t>
         </is>
       </c>
-      <c r="B23" s="299" t="inlineStr">
+      <c r="B23" s="307" t="inlineStr">
         <is>
           <t>P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados na pedra devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -7096,19 +7184,19 @@
       <c r="C23" s="300" t="n"/>
       <c r="D23" s="300" t="n"/>
       <c r="E23" s="300" t="n"/>
-      <c r="F23" s="305" t="inlineStr">
+      <c r="F23" s="324" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G23" s="300" t="n"/>
-      <c r="H23" s="301" t="inlineStr">
+      <c r="H23" s="308" t="inlineStr">
         <is>
           <t>PA1 - Parede em alvenaria com reboco convencional 2,5cm, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.
 PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I23" s="301" t="inlineStr">
+      <c r="I23" s="308" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7125,20 +7213,20 @@
       <c r="S23" s="300" t="n"/>
       <c r="T23" s="300" t="n"/>
       <c r="U23" s="300" t="n"/>
-      <c r="V23" s="301" t="inlineStr">
+      <c r="V23" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W23" s="300" t="n"/>
-      <c r="X23" s="299" t="inlineStr">
+      <c r="X23" s="307" t="inlineStr">
         <is>
           <t>D44 - Porta pivotante em MDF com acabamento em pintura acrílica fosca. Tom a definir. Dimensões conforme Mapa de Esquadrias. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 D45 - Porta pivotante em MDF com acabamento em pintura acrílica fosca. Tom a definir. Dimensões conforme Mapa de Esquadrias. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y23" s="302" t="n"/>
-      <c r="Z23" s="301" t="inlineStr">
+      <c r="Z23" s="308" t="inlineStr">
         <is>
           <t>D64 - Quadro para elevador em chapa metálica 8mm com acabamento em pintura eletrostática, cor branca. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -7150,7 +7238,7 @@
           <t xml:space="preserve">GARAGEM </t>
         </is>
       </c>
-      <c r="B24" s="299" t="inlineStr">
+      <c r="B24" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -7160,12 +7248,12 @@
       <c r="E24" s="300" t="n"/>
       <c r="F24" s="300" t="n"/>
       <c r="G24" s="300" t="n"/>
-      <c r="H24" s="301" t="inlineStr">
+      <c r="H24" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I24" s="301" t="inlineStr">
+      <c r="I24" s="308" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -7194,7 +7282,7 @@
           <t>CASA DE BOMBAS</t>
         </is>
       </c>
-      <c r="B25" s="299" t="inlineStr">
+      <c r="B25" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -7204,12 +7292,12 @@
       <c r="E25" s="300" t="n"/>
       <c r="F25" s="306" t="n"/>
       <c r="G25" s="300" t="n"/>
-      <c r="H25" s="299" t="inlineStr">
+      <c r="H25" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I25" s="299" t="inlineStr">
+      <c r="I25" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -7270,7 +7358,7 @@
           <t xml:space="preserve">CIRCULAÇÃO </t>
         </is>
       </c>
-      <c r="B27" s="299" t="inlineStr">
+      <c r="B27" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7278,18 +7366,18 @@
       <c r="C27" s="300" t="n"/>
       <c r="D27" s="308" t="n"/>
       <c r="E27" s="300" t="n"/>
-      <c r="F27" s="299" t="inlineStr">
+      <c r="F27" s="307" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G27" s="300" t="n"/>
-      <c r="H27" s="299" t="inlineStr">
+      <c r="H27" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I27" s="299" t="inlineStr">
+      <c r="I27" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7318,7 +7406,7 @@
           <t>I.S P.C.D</t>
         </is>
       </c>
-      <c r="B28" s="299" t="inlineStr">
+      <c r="B28" s="307" t="inlineStr">
         <is>
           <t>P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados na pedra devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -7326,29 +7414,29 @@
       <c r="C28" s="300" t="n"/>
       <c r="D28" s="307" t="n"/>
       <c r="E28" s="308" t="n"/>
-      <c r="F28" s="299" t="inlineStr">
+      <c r="F28" s="307" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G28" s="300" t="n"/>
-      <c r="H28" s="299" t="inlineStr">
+      <c r="H28" s="307" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I28" s="301" t="inlineStr">
+      <c r="I28" s="308" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J28" s="301" t="inlineStr">
+      <c r="J28" s="308" t="inlineStr">
         <is>
           <t>D65 - Bancada em pedra natural Basaltina com cuba esculpida e bandeja removível. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="K28" s="301" t="inlineStr">
+      <c r="K28" s="308" t="inlineStr">
         <is>
           <t>D37 - Armário em MDF Kahimir ref. Arauco com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF 12mm com acabamento da lateral das portas cantoneiras em aço inox polido e lateral do armário em chapa de aço inox polido. Dimensões e desenho conforme detalhamento. Obs.: MDF possui certificação FSC.</t>
         </is>
@@ -7356,12 +7444,12 @@
       <c r="L28" s="300" t="n"/>
       <c r="M28" s="300" t="n"/>
       <c r="N28" s="300" t="n"/>
-      <c r="O28" s="301" t="inlineStr">
+      <c r="O28" s="308" t="inlineStr">
         <is>
           <t>D66 - Monocomando de mesa para lavatório, linha Mix&amp;Match, bica baixa, acabamento grafite escovado, cód.: 01739870. Ref.: Docol. Obs.: Se necessário instalar cardal para aquecimento de água. ATENÇÃO: vazão máxima de 6 l/min, instalar redutor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="P28" s="301" t="inlineStr">
+      <c r="P28" s="308" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7369,25 +7457,25 @@
       <c r="Q28" s="300" t="n"/>
       <c r="R28" s="300" t="n"/>
       <c r="S28" s="300" t="n"/>
-      <c r="T28" s="299" t="inlineStr">
+      <c r="T28" s="307" t="inlineStr">
         <is>
           <t>D34 - Ralo 15x15cm com tampa lisa em aço inox, linha Square. Ref.: Elleve</t>
         </is>
       </c>
       <c r="U28" s="300" t="n"/>
-      <c r="V28" s="299" t="inlineStr">
+      <c r="V28" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W28" s="307" t="n"/>
-      <c r="X28" s="299" t="inlineStr">
+      <c r="X28" s="307" t="inlineStr">
         <is>
           <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y28" s="302" t="n"/>
-      <c r="Z28" s="299" t="inlineStr">
+      <c r="Z28" s="307" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -7401,7 +7489,7 @@
           <t>VESTÍBULO</t>
         </is>
       </c>
-      <c r="B29" s="299" t="inlineStr">
+      <c r="B29" s="307" t="inlineStr">
         <is>
           <t>P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados na pedra devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -7409,19 +7497,19 @@
       <c r="C29" s="300" t="n"/>
       <c r="D29" s="300" t="n"/>
       <c r="E29" s="308" t="n"/>
-      <c r="F29" s="301" t="inlineStr">
+      <c r="F29" s="308" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G29" s="307" t="n"/>
-      <c r="H29" s="299" t="inlineStr">
+      <c r="H29" s="307" t="inlineStr">
         <is>
           <t>PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA55 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica,  revestimento em vidro 4mm temperado, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I29" s="299" t="inlineStr">
+      <c r="I29" s="307" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7438,13 +7526,13 @@
       <c r="S29" s="300" t="n"/>
       <c r="T29" s="300" t="n"/>
       <c r="U29" s="300" t="n"/>
-      <c r="V29" s="299" t="inlineStr">
+      <c r="V29" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W29" s="300" t="n"/>
-      <c r="X29" s="301" t="inlineStr">
+      <c r="X29" s="308" t="inlineStr">
         <is>
           <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
 D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
@@ -7459,7 +7547,7 @@
           <t>CONCIERGE</t>
         </is>
       </c>
-      <c r="B30" s="299" t="inlineStr">
+      <c r="B30" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7467,18 +7555,18 @@
       <c r="C30" s="300" t="n"/>
       <c r="D30" s="300" t="n"/>
       <c r="E30" s="308" t="n"/>
-      <c r="F30" s="301" t="inlineStr">
+      <c r="F30" s="308" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G30" s="307" t="n"/>
-      <c r="H30" s="299" t="inlineStr">
+      <c r="H30" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I30" s="299" t="inlineStr">
+      <c r="I30" s="307" t="inlineStr">
         <is>
           <t>ARQ-T19 - código não existe no quadro de tetos (01 a 06); conferir na planta</t>
         </is>
@@ -7507,7 +7595,7 @@
           <t>DELIVERY</t>
         </is>
       </c>
-      <c r="B31" s="299" t="inlineStr">
+      <c r="B31" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7515,18 +7603,18 @@
       <c r="C31" s="300" t="n"/>
       <c r="D31" s="308" t="n"/>
       <c r="E31" s="308" t="n"/>
-      <c r="F31" s="299" t="inlineStr">
+      <c r="F31" s="307" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G31" s="300" t="n"/>
-      <c r="H31" s="299" t="inlineStr">
+      <c r="H31" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I31" s="299" t="inlineStr">
+      <c r="I31" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7555,7 +7643,7 @@
           <t xml:space="preserve">CIRCULAÇÃO SERVIÇO </t>
         </is>
       </c>
-      <c r="B32" s="299" t="inlineStr">
+      <c r="B32" s="307" t="inlineStr">
         <is>
           <t>ARQ-P07 - Piso assentado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -7563,18 +7651,18 @@
       <c r="C32" s="300" t="n"/>
       <c r="D32" s="308" t="n"/>
       <c r="E32" s="308" t="n"/>
-      <c r="F32" s="299" t="inlineStr">
+      <c r="F32" s="307" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G32" s="300" t="n"/>
-      <c r="H32" s="299" t="inlineStr">
+      <c r="H32" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I32" s="299" t="inlineStr">
+      <c r="I32" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7603,7 +7691,7 @@
           <t>CAR WASH</t>
         </is>
       </c>
-      <c r="B33" s="299" t="inlineStr">
+      <c r="B33" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -7613,12 +7701,12 @@
       <c r="E33" s="300" t="n"/>
       <c r="F33" s="307" t="n"/>
       <c r="G33" s="300" t="n"/>
-      <c r="H33" s="299" t="inlineStr">
+      <c r="H33" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA13 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Acabamento de meia parede com porcelanato padrão cimentício 120x120cm, espessura 1cm, com acabamento fosco (antiderrapante). Ref.: CITTA SGR HARD; cód. 61588; Portinari. Paginação e altura conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I33" s="299" t="inlineStr">
+      <c r="I33" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -7647,7 +7735,7 @@
           <t xml:space="preserve">BICICLETÁRIO </t>
         </is>
       </c>
-      <c r="B34" s="299" t="inlineStr">
+      <c r="B34" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -7657,12 +7745,12 @@
       <c r="E34" s="308" t="n"/>
       <c r="F34" s="307" t="n"/>
       <c r="G34" s="300" t="n"/>
-      <c r="H34" s="299" t="inlineStr">
+      <c r="H34" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA13 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Acabamento de meia parede com porcelanato padrão cimentício 120x120cm, espessura 1cm, com acabamento fosco (antiderrapante). Ref.: CITTA SGR HARD; cód. 61588; Portinari. Paginação e altura conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I34" s="299" t="inlineStr">
+      <c r="I34" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -7691,7 +7779,7 @@
           <t xml:space="preserve">ZELADORIA </t>
         </is>
       </c>
-      <c r="B35" s="299" t="inlineStr">
+      <c r="B35" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7699,18 +7787,18 @@
       <c r="C35" s="300" t="n"/>
       <c r="D35" s="307" t="n"/>
       <c r="E35" s="308" t="n"/>
-      <c r="F35" s="299" t="inlineStr">
+      <c r="F35" s="307" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G35" s="300" t="n"/>
-      <c r="H35" s="299" t="inlineStr">
+      <c r="H35" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I35" s="299" t="inlineStr">
+      <c r="I35" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7739,7 +7827,7 @@
           <t>ARS 1</t>
         </is>
       </c>
-      <c r="B36" s="299" t="inlineStr">
+      <c r="B36" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7749,12 +7837,12 @@
       <c r="E36" s="308" t="n"/>
       <c r="F36" s="307" t="n"/>
       <c r="G36" s="300" t="n"/>
-      <c r="H36" s="299" t="inlineStr">
+      <c r="H36" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA11 - Parede revestida em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I36" s="299" t="inlineStr">
+      <c r="I36" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7783,7 +7871,7 @@
           <t>ARS 2</t>
         </is>
       </c>
-      <c r="B37" s="299" t="inlineStr">
+      <c r="B37" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7793,12 +7881,12 @@
       <c r="E37" s="308" t="n"/>
       <c r="F37" s="307" t="n"/>
       <c r="G37" s="300" t="n"/>
-      <c r="H37" s="299" t="inlineStr">
+      <c r="H37" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA11 - Parede revestida em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I37" s="299" t="inlineStr">
+      <c r="I37" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7827,7 +7915,7 @@
           <t>ARS 3</t>
         </is>
       </c>
-      <c r="B38" s="299" t="inlineStr">
+      <c r="B38" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7837,12 +7925,12 @@
       <c r="E38" s="308" t="n"/>
       <c r="F38" s="307" t="n"/>
       <c r="G38" s="300" t="n"/>
-      <c r="H38" s="299" t="inlineStr">
+      <c r="H38" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA11 - Parede revestida em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I38" s="299" t="inlineStr">
+      <c r="I38" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7871,7 +7959,7 @@
           <t>SALA MOTORISTA</t>
         </is>
       </c>
-      <c r="B39" s="299" t="inlineStr">
+      <c r="B39" s="307" t="inlineStr">
         <is>
           <t>ARQ-P06 - Piso em porcelanato padrão cimentício 120x120cm, espessura 1cm, com acabamento fosco (antiderrapante). Ref.: CITTA SGR HARD; cód. 61588; Portinari. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7879,18 +7967,18 @@
       <c r="C39" s="300" t="n"/>
       <c r="D39" s="307" t="n"/>
       <c r="E39" s="308" t="n"/>
-      <c r="F39" s="299" t="inlineStr">
+      <c r="F39" s="307" t="inlineStr">
         <is>
           <t>ARQ-RD20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G39" s="300" t="n"/>
-      <c r="H39" s="299" t="inlineStr">
+      <c r="H39" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA02 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor a definir, acabamento acetinado.</t>
         </is>
       </c>
-      <c r="I39" s="299" t="inlineStr">
+      <c r="I39" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -7919,7 +8007,7 @@
           <t>DML</t>
         </is>
       </c>
-      <c r="B40" s="299" t="inlineStr">
+      <c r="B40" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -7929,12 +8017,12 @@
       <c r="E40" s="308" t="n"/>
       <c r="F40" s="307" t="n"/>
       <c r="G40" s="300" t="n"/>
-      <c r="H40" s="299" t="inlineStr">
+      <c r="H40" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA12 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca branca. Ref.: branco neve; Suvinil. Acabamento de meia parede em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I40" s="299" t="inlineStr">
+      <c r="I40" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -7963,7 +8051,7 @@
           <t>VEST. P.C.D</t>
         </is>
       </c>
-      <c r="B41" s="299" t="inlineStr">
+      <c r="B41" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -7973,12 +8061,12 @@
       <c r="E41" s="308" t="n"/>
       <c r="F41" s="307" t="n"/>
       <c r="G41" s="300" t="n"/>
-      <c r="H41" s="299" t="inlineStr">
+      <c r="H41" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA11 - Parede revestida em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I41" s="299" t="inlineStr">
+      <c r="I41" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -8007,7 +8095,7 @@
           <t>VEST. FEMININO</t>
         </is>
       </c>
-      <c r="B42" s="299" t="inlineStr">
+      <c r="B42" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -8017,12 +8105,12 @@
       <c r="E42" s="308" t="n"/>
       <c r="F42" s="307" t="n"/>
       <c r="G42" s="300" t="n"/>
-      <c r="H42" s="299" t="inlineStr">
+      <c r="H42" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA11 - Parede revestida em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I42" s="299" t="inlineStr">
+      <c r="I42" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -8051,7 +8139,7 @@
           <t>VEST. MASC.</t>
         </is>
       </c>
-      <c r="B43" s="299" t="inlineStr">
+      <c r="B43" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -8061,12 +8149,12 @@
       <c r="E43" s="308" t="n"/>
       <c r="F43" s="307" t="n"/>
       <c r="G43" s="300" t="n"/>
-      <c r="H43" s="299" t="inlineStr">
+      <c r="H43" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA11 - Parede revestida em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I43" s="299" t="inlineStr">
+      <c r="I43" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -8095,7 +8183,7 @@
           <t>ESTAR/COPA FUNCIONÁRIOS</t>
         </is>
       </c>
-      <c r="B44" s="299" t="inlineStr">
+      <c r="B44" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -8105,12 +8193,12 @@
       <c r="E44" s="308" t="n"/>
       <c r="F44" s="307" t="n"/>
       <c r="G44" s="300" t="n"/>
-      <c r="H44" s="299" t="inlineStr">
+      <c r="H44" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I44" s="299" t="inlineStr">
+      <c r="I44" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -8139,7 +8227,7 @@
           <t xml:space="preserve">CIRCULAÇÃO </t>
         </is>
       </c>
-      <c r="B45" s="299" t="inlineStr">
+      <c r="B45" s="307" t="inlineStr">
         <is>
           <t>ARQ-P05 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -8147,18 +8235,18 @@
       <c r="C45" s="300" t="n"/>
       <c r="D45" s="307" t="n"/>
       <c r="E45" s="308" t="n"/>
-      <c r="F45" s="299" t="inlineStr">
+      <c r="F45" s="307" t="inlineStr">
         <is>
           <t>ARQ-RD19 - Rodapé em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação e altura conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="G45" s="300" t="n"/>
-      <c r="H45" s="299" t="inlineStr">
+      <c r="H45" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I45" s="299" t="inlineStr">
+      <c r="I45" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -8187,7 +8275,7 @@
           <t>GERADOR</t>
         </is>
       </c>
-      <c r="B46" s="299" t="inlineStr">
+      <c r="B46" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -8197,12 +8285,12 @@
       <c r="E46" s="308" t="n"/>
       <c r="F46" s="300" t="n"/>
       <c r="G46" s="300" t="n"/>
-      <c r="H46" s="299" t="inlineStr">
+      <c r="H46" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I46" s="299" t="inlineStr">
+      <c r="I46" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -8231,7 +8319,7 @@
           <t>VAGAS BOX</t>
         </is>
       </c>
-      <c r="B47" s="299" t="inlineStr">
+      <c r="B47" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -8241,12 +8329,12 @@
       <c r="E47" s="308" t="n"/>
       <c r="F47" s="300" t="n"/>
       <c r="G47" s="300" t="n"/>
-      <c r="H47" s="299" t="inlineStr">
+      <c r="H47" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I47" s="299" t="inlineStr">
+      <c r="I47" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -8275,7 +8363,7 @@
           <t>QUADROS ELÉTRICOS</t>
         </is>
       </c>
-      <c r="B48" s="299" t="inlineStr">
+      <c r="B48" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -8285,12 +8373,12 @@
       <c r="E48" s="308" t="n"/>
       <c r="F48" s="300" t="n"/>
       <c r="G48" s="300" t="n"/>
-      <c r="H48" s="299" t="inlineStr">
+      <c r="H48" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I48" s="299" t="inlineStr">
+      <c r="I48" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -8319,7 +8407,7 @@
           <t>ACESSO E SAÍDA DE VEÍCULOS</t>
         </is>
       </c>
-      <c r="B49" s="299" t="inlineStr">
+      <c r="B49" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -8329,12 +8417,12 @@
       <c r="E49" s="308" t="n"/>
       <c r="F49" s="300" t="n"/>
       <c r="G49" s="300" t="n"/>
-      <c r="H49" s="299" t="inlineStr">
+      <c r="H49" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I49" s="299" t="n"/>
+      <c r="I49" s="307" t="n"/>
       <c r="J49" s="307" t="n"/>
       <c r="K49" s="300" t="n"/>
       <c r="L49" s="307" t="n"/>
@@ -8359,7 +8447,7 @@
           <t>ESTACIONAMENTO VISITANTES</t>
         </is>
       </c>
-      <c r="B50" s="299" t="inlineStr">
+      <c r="B50" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -8369,12 +8457,12 @@
       <c r="E50" s="308" t="n"/>
       <c r="F50" s="300" t="n"/>
       <c r="G50" s="300" t="n"/>
-      <c r="H50" s="299" t="inlineStr">
+      <c r="H50" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I50" s="299" t="inlineStr">
+      <c r="I50" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -8403,7 +8491,7 @@
           <t>RAMPA VEÍCULOS</t>
         </is>
       </c>
-      <c r="B51" s="299" t="inlineStr">
+      <c r="B51" s="307" t="inlineStr">
         <is>
           <t>ARQ-P03 - Piso em concreto mecanizado com acabamento antiderrapante</t>
         </is>
@@ -8413,12 +8501,12 @@
       <c r="E51" s="308" t="n"/>
       <c r="F51" s="300" t="n"/>
       <c r="G51" s="300" t="n"/>
-      <c r="H51" s="299" t="inlineStr">
+      <c r="H51" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I51" s="299" t="inlineStr">
+      <c r="I51" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -8447,7 +8535,7 @@
           <t>DEPÓSITO (A=8,85 m²)</t>
         </is>
       </c>
-      <c r="B52" s="299" t="inlineStr">
+      <c r="B52" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -8457,12 +8545,12 @@
       <c r="E52" s="308" t="n"/>
       <c r="F52" s="300" t="n"/>
       <c r="G52" s="300" t="n"/>
-      <c r="H52" s="299" t="inlineStr">
+      <c r="H52" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I52" s="299" t="inlineStr">
+      <c r="I52" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -8491,7 +8579,7 @@
           <t>SERVIÇO JUNTO AO PORTÃO (A=6,87 m²)</t>
         </is>
       </c>
-      <c r="B53" s="299" t="inlineStr">
+      <c r="B53" s="307" t="inlineStr">
         <is>
           <t>ARQ-P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -8499,18 +8587,18 @@
       <c r="C53" s="300" t="n"/>
       <c r="D53" s="307" t="n"/>
       <c r="E53" s="308" t="n"/>
-      <c r="F53" s="301" t="inlineStr">
+      <c r="F53" s="308" t="inlineStr">
         <is>
           <t>ARQ-RD20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G53" s="300" t="n"/>
-      <c r="H53" s="299" t="inlineStr">
+      <c r="H53" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA02 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor a definir, acabamento acetinado.</t>
         </is>
       </c>
-      <c r="I53" s="299" t="inlineStr">
+      <c r="I53" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -8539,7 +8627,7 @@
           <t>CIRCULAÇÃO JUNTO À ESCADA (A=4,06 m²)</t>
         </is>
       </c>
-      <c r="B54" s="299" t="inlineStr">
+      <c r="B54" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -8547,14 +8635,14 @@
       <c r="C54" s="300" t="n"/>
       <c r="D54" s="307" t="n"/>
       <c r="E54" s="308" t="n"/>
-      <c r="F54" s="301" t="n"/>
+      <c r="F54" s="308" t="n"/>
       <c r="G54" s="300" t="n"/>
-      <c r="H54" s="299" t="inlineStr">
+      <c r="H54" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I54" s="299" t="inlineStr">
+      <c r="I54" s="307" t="inlineStr">
         <is>
           <t>ARQ-T02 - Laje em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9286,7 +9374,7 @@
           <t>CASA DE BOMBAS PISCINA 1</t>
         </is>
       </c>
-      <c r="B13" s="309" t="inlineStr">
+      <c r="B13" s="325" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9296,12 +9384,12 @@
       <c r="E13" s="296" t="n"/>
       <c r="F13" s="296" t="n"/>
       <c r="G13" s="296" t="n"/>
-      <c r="H13" s="310" t="inlineStr">
+      <c r="H13" s="326" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I13" s="310" t="inlineStr">
+      <c r="I13" s="326" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9330,7 +9418,7 @@
           <t>SHAFT ELÉTRICA</t>
         </is>
       </c>
-      <c r="B14" s="299" t="inlineStr">
+      <c r="B14" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9340,12 +9428,12 @@
       <c r="E14" s="300" t="n"/>
       <c r="F14" s="300" t="n"/>
       <c r="G14" s="300" t="n"/>
-      <c r="H14" s="301" t="inlineStr">
+      <c r="H14" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I14" s="301" t="inlineStr">
+      <c r="I14" s="308" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9438,7 +9526,7 @@
           <t>CIRCULAÇÃO/ANTECÂMARA</t>
         </is>
       </c>
-      <c r="B17" s="299" t="inlineStr">
+      <c r="B17" s="307" t="inlineStr">
         <is>
           <t>ARQ-P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -9446,18 +9534,18 @@
       <c r="C17" s="300" t="n"/>
       <c r="D17" s="300" t="n"/>
       <c r="E17" s="300" t="n"/>
-      <c r="F17" s="301" t="inlineStr">
+      <c r="F17" s="308" t="inlineStr">
         <is>
           <t>ARQ-RD20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G17" s="300" t="n"/>
-      <c r="H17" s="301" t="inlineStr">
+      <c r="H17" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I17" s="301" t="inlineStr">
+      <c r="I17" s="308" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil
 ARQ-T02 - Laje em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
@@ -9487,7 +9575,7 @@
           <t>PRESSURIZAÇÃO/ANTECÂMARA</t>
         </is>
       </c>
-      <c r="B18" s="299" t="inlineStr">
+      <c r="B18" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9497,12 +9585,12 @@
       <c r="E18" s="300" t="n"/>
       <c r="F18" s="300" t="n"/>
       <c r="G18" s="300" t="n"/>
-      <c r="H18" s="301" t="inlineStr">
+      <c r="H18" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I18" s="301" t="inlineStr">
+      <c r="I18" s="308" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9531,7 +9619,7 @@
           <t>ÁREA TÉCNICA 1</t>
         </is>
       </c>
-      <c r="B19" s="299" t="inlineStr">
+      <c r="B19" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9541,12 +9629,12 @@
       <c r="E19" s="300" t="n"/>
       <c r="F19" s="300" t="n"/>
       <c r="G19" s="300" t="n"/>
-      <c r="H19" s="301" t="inlineStr">
+      <c r="H19" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I19" s="301" t="inlineStr">
+      <c r="I19" s="308" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9575,7 +9663,7 @@
           <t>ÁREA TÉCNICA 2</t>
         </is>
       </c>
-      <c r="B20" s="299" t="inlineStr">
+      <c r="B20" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9585,12 +9673,12 @@
       <c r="E20" s="300" t="n"/>
       <c r="F20" s="312" t="n"/>
       <c r="G20" s="300" t="n"/>
-      <c r="H20" s="301" t="inlineStr">
+      <c r="H20" s="308" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I20" s="301" t="inlineStr">
+      <c r="I20" s="308" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9619,7 +9707,7 @@
           <t>GARAGEM</t>
         </is>
       </c>
-      <c r="B21" s="299" t="inlineStr">
+      <c r="B21" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -9629,12 +9717,12 @@
       <c r="E21" s="300" t="n"/>
       <c r="F21" s="306" t="n"/>
       <c r="G21" s="300" t="n"/>
-      <c r="H21" s="299" t="inlineStr">
+      <c r="H21" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I21" s="299" t="inlineStr">
+      <c r="I21" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9663,7 +9751,7 @@
           <t>VAGAS BOX</t>
         </is>
       </c>
-      <c r="B22" s="299" t="inlineStr">
+      <c r="B22" s="307" t="inlineStr">
         <is>
           <t>ARQ-P01 - Piso em concreto mecanizado com acabamento polido. Vagas demarcadas em pintura epóxi fosca de tom cinza médio com requadro em faixa de pintura epóxi fosca de tom cinza chumbo.</t>
         </is>
@@ -9673,12 +9761,12 @@
       <c r="E22" s="300" t="n"/>
       <c r="F22" s="306" t="n"/>
       <c r="G22" s="300" t="n"/>
-      <c r="H22" s="299" t="inlineStr">
+      <c r="H22" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I22" s="299" t="inlineStr">
+      <c r="I22" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9707,7 +9795,7 @@
           <t>TELECOM</t>
         </is>
       </c>
-      <c r="B23" s="299" t="inlineStr">
+      <c r="B23" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9717,12 +9805,12 @@
       <c r="E23" s="300" t="n"/>
       <c r="F23" s="307" t="n"/>
       <c r="G23" s="300" t="n"/>
-      <c r="H23" s="299" t="inlineStr">
+      <c r="H23" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I23" s="299" t="inlineStr">
+      <c r="I23" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9751,7 +9839,7 @@
           <t>SALA DE SEGURANÇA</t>
         </is>
       </c>
-      <c r="B24" s="299" t="inlineStr">
+      <c r="B24" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9761,12 +9849,12 @@
       <c r="E24" s="308" t="n"/>
       <c r="F24" s="307" t="n"/>
       <c r="G24" s="300" t="n"/>
-      <c r="H24" s="299" t="inlineStr">
+      <c r="H24" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I24" s="301" t="inlineStr">
+      <c r="I24" s="308" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9795,7 +9883,7 @@
           <t>CASA DE BOMBAS PISCINA 2 (FUNDO)</t>
         </is>
       </c>
-      <c r="B25" s="299" t="inlineStr">
+      <c r="B25" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9805,12 +9893,12 @@
       <c r="E25" s="308" t="n"/>
       <c r="F25" s="300" t="n"/>
       <c r="G25" s="307" t="n"/>
-      <c r="H25" s="299" t="inlineStr">
+      <c r="H25" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I25" s="299" t="inlineStr">
+      <c r="I25" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9839,7 +9927,7 @@
           <t>DML</t>
         </is>
       </c>
-      <c r="B26" s="299" t="inlineStr">
+      <c r="B26" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9849,12 +9937,12 @@
       <c r="E26" s="308" t="n"/>
       <c r="F26" s="300" t="n"/>
       <c r="G26" s="307" t="n"/>
-      <c r="H26" s="299" t="inlineStr">
+      <c r="H26" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA12 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca branca. Ref.: branco neve; Suvinil. Acabamento de meia parede em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane.</t>
         </is>
       </c>
-      <c r="I26" s="299" t="inlineStr">
+      <c r="I26" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9883,7 +9971,7 @@
           <t>RESERVATÓRIO INFERIOR</t>
         </is>
       </c>
-      <c r="B27" s="299" t="inlineStr">
+      <c r="B27" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9893,12 +9981,12 @@
       <c r="E27" s="308" t="n"/>
       <c r="F27" s="307" t="n"/>
       <c r="G27" s="300" t="n"/>
-      <c r="H27" s="299" t="inlineStr">
+      <c r="H27" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I27" s="299" t="inlineStr">
+      <c r="I27" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9927,7 +10015,7 @@
           <t>HALL TÉCNICO/CIRCULAÇÃO</t>
         </is>
       </c>
-      <c r="B28" s="299" t="inlineStr">
+      <c r="B28" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -9937,12 +10025,12 @@
       <c r="E28" s="308" t="n"/>
       <c r="F28" s="307" t="n"/>
       <c r="G28" s="300" t="n"/>
-      <c r="H28" s="299" t="inlineStr">
+      <c r="H28" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I28" s="299" t="inlineStr">
+      <c r="I28" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -9971,7 +10059,7 @@
           <t>RAMPA VEÍCULOS</t>
         </is>
       </c>
-      <c r="B29" s="299" t="inlineStr">
+      <c r="B29" s="307" t="inlineStr">
         <is>
           <t>ARQ-P04 - Piso em concreto mecanizado com acabamento em ladrilho hidráulico antiderrapante cinza, tom concreto. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -9981,12 +10069,12 @@
       <c r="E29" s="308" t="n"/>
       <c r="F29" s="307" t="n"/>
       <c r="G29" s="300" t="n"/>
-      <c r="H29" s="299" t="inlineStr">
+      <c r="H29" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA07 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza claro. Pintura de meia parede em epóxi monolítico de tom cinza médio, com arremate em faixa com tinta epóxi fosca de cor cinza chumbo. Altura conforme projeto arquitetônico. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I29" s="299" t="inlineStr">
+      <c r="I29" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -10015,7 +10103,7 @@
           <t>CIRCULAÇÃO ÁREA TÉCNICA (A=14,54 m²)</t>
         </is>
       </c>
-      <c r="B30" s="299" t="inlineStr">
+      <c r="B30" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -10025,12 +10113,12 @@
       <c r="E30" s="308" t="n"/>
       <c r="F30" s="307" t="n"/>
       <c r="G30" s="300" t="n"/>
-      <c r="H30" s="299" t="inlineStr">
+      <c r="H30" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I30" s="299" t="inlineStr">
+      <c r="I30" s="307" t="inlineStr">
         <is>
           <t>ARQ-T03 - Laje nervurada em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -10059,7 +10147,7 @@
           <t>CIRCULAÇÃO JUNTO À ESCADA (A=3,07 m²)</t>
         </is>
       </c>
-      <c r="B31" s="299" t="inlineStr">
+      <c r="B31" s="307" t="inlineStr">
         <is>
           <t>ARQ-P02 - Piso em concreto mecanizado com acabamento polido.</t>
         </is>
@@ -10069,12 +10157,12 @@
       <c r="E31" s="308" t="n"/>
       <c r="F31" s="307" t="n"/>
       <c r="G31" s="300" t="n"/>
-      <c r="H31" s="299" t="inlineStr">
+      <c r="H31" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I31" s="299" t="inlineStr">
+      <c r="I31" s="307" t="inlineStr">
         <is>
           <t>ARQ-T02 - Laje em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -10826,7 +10914,7 @@
           <t>LOBBY PILOTIS</t>
         </is>
       </c>
-      <c r="B13" s="313" t="inlineStr">
+      <c r="B13" s="327" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -10841,14 +10929,14 @@
         </is>
       </c>
       <c r="G13" s="296" t="n"/>
-      <c r="H13" s="315" t="inlineStr">
+      <c r="H13" s="314" t="inlineStr">
         <is>
           <t>PA44 - Parede em alvenaria emassada regularizada, revestida em massa acrílica texturizada cimento queimado, cor 107. Ref.: Terracor CQ. Amostra a ser aprovada pela GPA&amp;A.
 PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA58 - Pilar em concreto, com enchimento, revestido em pedra natural Basaltina conforme detalhamento.Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I13" s="315" t="inlineStr">
+      <c r="I13" s="314" t="inlineStr">
         <is>
           <t>FO2 - Forro em gesso acartonado perfurado de absorção acústica, modelo cleneo quadrado, furação 12/25, sistema de instalação tipo FGE - estruturado, Ref.: Knauf Ceiling Solutions ou similar. Bordas ou "tabeiras" em gesso liso, com acabamento em tinta acrílica fosca, cor branco neve. Preenchimento superior com 1 manta de lã de pet com 35Kg/m³ de densidade de 50mm de espessura, Ref.: Trisoft ou similar.
 T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
@@ -10870,13 +10958,13 @@
       <c r="S13" s="296" t="n"/>
       <c r="T13" s="296" t="n"/>
       <c r="U13" s="296" t="n"/>
-      <c r="V13" s="310" t="inlineStr">
+      <c r="V13" s="326" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W13" s="296" t="n"/>
-      <c r="X13" s="309" t="inlineStr">
+      <c r="X13" s="325" t="inlineStr">
         <is>
           <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
 D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
@@ -10893,7 +10981,7 @@
           <t>SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="B14" s="316" t="inlineStr">
+      <c r="B14" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -10915,7 +11003,7 @@
 PA31 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 107, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I14" s="318" t="inlineStr">
+      <c r="I14" s="317" t="inlineStr">
         <is>
           <t>FO1 - Forro de absorção acústica composto por 1 manta de lã de pet com 35Kg/m³ de densidade e 50mm de espessura, fixado perfis próprios metálicos, Ref.: Trisoft ou similar
 FO2 - Forro em gesso acartonado perfurado de absorção acústica, modelo cleneo quadrado, furação 12/25, sistema de instalação tipo FGE - estruturado, Ref.: Knauf Ceiling Solutions ou similar. Bordas ou "tabeiras" em gesso liso, com acabamento em tinta acrílica fosca, cor branco neve. Preenchimento superior com 1 manta de lã de pet com 35Kg/m³ de densidade de 50mm de espessura, Ref.: Trisoft ou similar.
@@ -10938,13 +11026,13 @@
       <c r="S14" s="300" t="n"/>
       <c r="T14" s="300" t="n"/>
       <c r="U14" s="300" t="n"/>
-      <c r="V14" s="301" t="inlineStr">
+      <c r="V14" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W14" s="300" t="n"/>
-      <c r="X14" s="299" t="inlineStr">
+      <c r="X14" s="307" t="inlineStr">
         <is>
           <t>D21 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxadores conforme detalhamento. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR
 D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
@@ -11023,7 +11111,7 @@
           <t>I.S FEMININO</t>
         </is>
       </c>
-      <c r="B17" s="316" t="inlineStr">
+      <c r="B17" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -11043,7 +11131,7 @@
           <t>PA39 - Parede em alvenaria rebocada regularizada revestida em pedra mármore Barrocci Honed, acabamento levigado, espessura 2cm. Ref.: Brasigran. Paginação e dimensões conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I17" s="318" t="inlineStr">
+      <c r="I17" s="317" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -11066,7 +11154,7 @@
           <t>D23 - Monocomando de mesa para lavatório, linha Mix&amp;Match, bica baixa, acabamento cromado, cód.: 90017398006. Ref.: Docol. Obs.: Se necessário instalar cardal para aquecimento de água. ATENÇÃO: vazão máxima de 6 l/min, instalar redutor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="P17" s="318" t="inlineStr">
+      <c r="P17" s="317" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -11076,19 +11164,19 @@
       <c r="S17" s="300" t="n"/>
       <c r="T17" s="300" t="n"/>
       <c r="U17" s="300" t="n"/>
-      <c r="V17" s="301" t="inlineStr">
+      <c r="V17" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W17" s="300" t="n"/>
-      <c r="X17" s="299" t="inlineStr">
+      <c r="X17" s="307" t="inlineStr">
         <is>
           <t>D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y17" s="302" t="n"/>
-      <c r="Z17" s="318" t="inlineStr">
+      <c r="Z17" s="317" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -11102,7 +11190,7 @@
           <t>I.S MASCULINO</t>
         </is>
       </c>
-      <c r="B18" s="316" t="inlineStr">
+      <c r="B18" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -11122,7 +11210,7 @@
           <t>PA39 - Parede em alvenaria rebocada regularizada revestida em pedra mármore Barrocci Honed, acabamento levigado, espessura 2cm. Ref.: Brasigran. Paginação e dimensões conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I18" s="318" t="inlineStr">
+      <c r="I18" s="317" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -11145,7 +11233,7 @@
           <t>D23 - Monocomando de mesa para lavatório, linha Mix&amp;Match, bica baixa, acabamento cromado, cód.: 90017398006. Ref.: Docol. Obs.: Se necessário instalar cardal para aquecimento de água. ATENÇÃO: vazão máxima de 6 l/min, instalar redutor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="P18" s="318" t="inlineStr">
+      <c r="P18" s="317" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -11155,19 +11243,19 @@
       <c r="S18" s="300" t="n"/>
       <c r="T18" s="300" t="n"/>
       <c r="U18" s="300" t="n"/>
-      <c r="V18" s="301" t="inlineStr">
+      <c r="V18" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W18" s="300" t="n"/>
-      <c r="X18" s="299" t="inlineStr">
+      <c r="X18" s="307" t="inlineStr">
         <is>
           <t>D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y18" s="302" t="n"/>
-      <c r="Z18" s="318" t="inlineStr">
+      <c r="Z18" s="317" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -11213,7 +11301,7 @@
           <t>COZINHA SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="B20" s="316" t="inlineStr">
+      <c r="B20" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -11234,7 +11322,7 @@
 PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
-      <c r="I20" s="318" t="inlineStr">
+      <c r="I20" s="317" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -11263,20 +11351,20 @@
       <c r="S20" s="300" t="n"/>
       <c r="T20" s="300" t="n"/>
       <c r="U20" s="300" t="n"/>
-      <c r="V20" s="301" t="inlineStr">
+      <c r="V20" s="308" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W20" s="300" t="n"/>
-      <c r="X20" s="299" t="inlineStr">
+      <c r="X20" s="307" t="inlineStr">
         <is>
           <t>D21 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxadores conforme detalhamento. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR
 D74 - Porta pivotante estruturada, fechamento em MDF cru, acabamento face interna e externa em micropintura cor S168-Sayerlack. Puxador tipo cava, prever tranca. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y20" s="302" t="n"/>
-      <c r="Z20" s="301" t="inlineStr">
+      <c r="Z20" s="308" t="inlineStr">
         <is>
           <t>D82 - Prateleira em granito cinza Santa Rosa, acabamento escovado, embutido na alvenaria. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -11344,7 +11432,7 @@
           <t>CIRCULAÇÃO/ANTECÂMARA ELEVADOR SERVIÇO</t>
         </is>
       </c>
-      <c r="B22" s="299" t="inlineStr">
+      <c r="B22" s="307" t="inlineStr">
         <is>
           <t>ARQ-P07 - Piso assentado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -11352,18 +11440,18 @@
       <c r="C22" s="306" t="n"/>
       <c r="D22" s="300" t="n"/>
       <c r="E22" s="300" t="n"/>
-      <c r="F22" s="299" t="inlineStr">
+      <c r="F22" s="307" t="inlineStr">
         <is>
           <t>ARQ-RD21 - Rodapé em granito cinza santa rosa, acabamento serrado, h=15cm, espessura 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
       <c r="G22" s="300" t="n"/>
-      <c r="H22" s="299" t="inlineStr">
+      <c r="H22" s="307" t="inlineStr">
         <is>
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I22" s="299" t="inlineStr">
+      <c r="I22" s="307" t="inlineStr">
         <is>
           <t>ARQ-T01 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -11406,14 +11494,14 @@
         </is>
       </c>
       <c r="G23" s="300" t="n"/>
-      <c r="H23" s="316" t="inlineStr">
+      <c r="H23" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural caravalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
 PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
-      <c r="I23" s="316" t="inlineStr">
+      <c r="I23" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -11436,7 +11524,7 @@
           <t>D23 - Monocomando de mesa para lavatório, linha Mix&amp;Match, bica baixa, acabamento cromado, cód.: 90017398006. Ref.: Docol. Obs.: Se necessário instalar cardal para aquecimento de água. ATENÇÃO: vazão máxima de 6 l/min, instalar redutor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="P23" s="318" t="inlineStr">
+      <c r="P23" s="317" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -11446,19 +11534,19 @@
       <c r="S23" s="300" t="n"/>
       <c r="T23" s="300" t="n"/>
       <c r="U23" s="300" t="n"/>
-      <c r="V23" s="299" t="inlineStr">
+      <c r="V23" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W23" s="307" t="n"/>
-      <c r="X23" s="299" t="inlineStr">
+      <c r="X23" s="307" t="inlineStr">
         <is>
           <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y23" s="302" t="n"/>
-      <c r="Z23" s="316" t="inlineStr">
+      <c r="Z23" s="320" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -11486,14 +11574,14 @@
         </is>
       </c>
       <c r="G24" s="300" t="n"/>
-      <c r="H24" s="316" t="inlineStr">
+      <c r="H24" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural caravalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
 PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
-      <c r="I24" s="316" t="inlineStr">
+      <c r="I24" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -11516,7 +11604,7 @@
           <t>D23 - Monocomando de mesa para lavatório, linha Mix&amp;Match, bica baixa, acabamento cromado, cód.: 90017398006. Ref.: Docol. Obs.: Se necessário instalar cardal para aquecimento de água. ATENÇÃO: vazão máxima de 6 l/min, instalar redutor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="P24" s="316" t="inlineStr">
+      <c r="P24" s="320" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -11526,19 +11614,19 @@
       <c r="S24" s="300" t="n"/>
       <c r="T24" s="307" t="n"/>
       <c r="U24" s="300" t="n"/>
-      <c r="V24" s="299" t="inlineStr">
+      <c r="V24" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W24" s="307" t="n"/>
-      <c r="X24" s="299" t="inlineStr">
+      <c r="X24" s="307" t="inlineStr">
         <is>
           <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y24" s="307" t="n"/>
-      <c r="Z24" s="316" t="inlineStr">
+      <c r="Z24" s="320" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -11584,7 +11672,7 @@
           <t>ESPAÇO KIDS</t>
         </is>
       </c>
-      <c r="B26" s="316" t="inlineStr">
+      <c r="B26" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P24 - Piso em contrapiso regularizado revestido em piso vinílico em manta, 2x20m, linha Polysafe Verona PUR, acabamento Rock Salt - cód: LRV-43. Paginação conforme detalhamento.</t>
@@ -11608,7 +11696,7 @@
 PA38 - Parede em alvenaria emassada regularizada, revestida em painel de marcenaria MDF Nude-linha VEL-Berneck. Amostra a ser aprovada pela GPA&amp;A. Obs.: MDF possui certificação FSC.</t>
         </is>
       </c>
-      <c r="I26" s="318" t="inlineStr">
+      <c r="I26" s="317" t="inlineStr">
         <is>
           <t>FO1 - Forro de absorção acústica composto por 1 manta de lã de pet com 35Kg/m³ de densidade e 50mm de espessura, fixado perfis próprios metálicos, Ref.: Trisoft ou similar
 FO2 - Forro em gesso acartonado perfurado de absorção acústica, modelo cleneo quadrado, furação 12/25, sistema de instalação tipo FGE - estruturado, Ref.: Knauf Ceiling Solutions ou similar. Bordas ou "tabeiras" em gesso liso, com acabamento em tinta acrílica fosca, cor branco neve. Preenchimento superior com 1 manta de lã de pet com 35Kg/m³ de densidade de 50mm de espessura, Ref.: Trisoft ou similar.
@@ -11627,20 +11715,20 @@
       <c r="S26" s="300" t="n"/>
       <c r="T26" s="307" t="n"/>
       <c r="U26" s="300" t="n"/>
-      <c r="V26" s="299" t="inlineStr">
+      <c r="V26" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W26" s="307" t="n"/>
-      <c r="X26" s="299" t="inlineStr">
+      <c r="X26" s="307" t="inlineStr">
         <is>
           <t>D11 - Porta pivotante estruturada, fechamento em  MDF cru, acabamento micro pintura face do kids cor S081-Sayerlack e acabamento face do gourmet em folha madeira natural caravalho tonalizado. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y26" s="302" t="n"/>
-      <c r="Z26" s="299" t="inlineStr">
+      <c r="Z26" s="307" t="inlineStr">
         <is>
           <t>D18 - Módulos compostos por três peças hexagonais com estruturado em peças de madeira maciça,   fechamento em reguas de madeira 25mmx70mm. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
 D56 - Pendente sob medida em peças de madeira maciça 60x50mm fixados no teto através de cabos de aço e estrutura auxiliar no entreforro, com acabamento no forro em canopla, cor branca. Retroiluminação em fitas de led na parte superior com dimensionamentos conforme projeto luminotécnico. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
@@ -11653,7 +11741,7 @@
           <t>ESPAÇO GOURMET</t>
         </is>
       </c>
-      <c r="B27" s="316" t="inlineStr">
+      <c r="B27" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -11668,14 +11756,14 @@
         </is>
       </c>
       <c r="G27" s="307" t="n"/>
-      <c r="H27" s="316" t="inlineStr">
+      <c r="H27" s="320" t="inlineStr">
         <is>
           <t>PA44 - Parede em alvenaria emassada regularizada, revestida em massa acrílica texturizada cimento queimado, cor 107. Ref.: Terracor CQ. Amostra a ser aprovada pela GPA&amp;A.
 PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural caravalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
 PA33 - Pilar em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina, acabamento frisado. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="I27" s="316" t="inlineStr">
+      <c r="I27" s="320" t="inlineStr">
         <is>
           <t>FO1 - Forro de absorção acústica composto por 1 manta de lã de pet com 35Kg/m³ de densidade e 50mm de espessura, fixado perfis próprios metálicos, Ref.: Trisoft ou similar
 FO2 - Forro em gesso acartonado perfurado de absorção acústica, modelo cleneo quadrado, furação 12/25, sistema de instalação tipo FGE - estruturado, Ref.: Knauf Ceiling Solutions ou similar. Bordas ou "tabeiras" em gesso liso, com acabamento em tinta acrílica fosca, cor branco neve. Preenchimento superior com 1 manta de lã de pet com 35Kg/m³ de densidade de 50mm de espessura, Ref.: Trisoft ou similar.</t>
@@ -11709,20 +11797,20 @@
       <c r="S27" s="300" t="n"/>
       <c r="T27" s="300" t="n"/>
       <c r="U27" s="300" t="n"/>
-      <c r="V27" s="299" t="inlineStr">
+      <c r="V27" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W27" s="300" t="n"/>
-      <c r="X27" s="301" t="inlineStr">
+      <c r="X27" s="308" t="inlineStr">
         <is>
           <t>D11 - Porta pivotante estruturada, fechamento em  MDF cru, acabamento micro pintura face do kids cor S081-Sayerlack e acabamento face do gourmet em folha madeira natural caravalho tonalizado. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y27" s="300" t="n"/>
-      <c r="Z27" s="299" t="inlineStr">
+      <c r="Z27" s="307" t="inlineStr">
         <is>
           <t>D13 - Estante suspensa em tubo retangular 25x25mm em aço inox com pintura ouro velho. Fixada no teto através de estrutura auxiliar. Apresentar amostra pintura e solda para aprovação GPA&amp;A.
 D14 - Fechamento cego em mdf cru com acabamento em folha madeira natural caravalho tonalizado. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
@@ -11770,7 +11858,7 @@
           <t>PISCINA DECOBERTA</t>
         </is>
       </c>
-      <c r="B29" s="316" t="inlineStr">
+      <c r="B29" s="320" t="inlineStr">
         <is>
           <t>P18 - Piso revestido em pastilhas de mármore branco selecionado, lote a ser aprovado, acabamento levigado, 3x3cm.  Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Amostra a ser aprovada pela GPA&amp;A
 P28 - Piso assentado em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -11781,7 +11869,7 @@
       <c r="E29" s="308" t="n"/>
       <c r="F29" s="307" t="n"/>
       <c r="G29" s="300" t="n"/>
-      <c r="H29" s="316" t="inlineStr">
+      <c r="H29" s="320" t="inlineStr">
         <is>
           <t>PA59 - Parede revestida em pastilha Jatobá, acabamento cinza cimento brilhante, 5x5cm. Cód.: CJC1614.. Ref.: Ceramicasa. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -11801,25 +11889,25 @@
       <c r="Q29" s="300" t="n"/>
       <c r="R29" s="300" t="n"/>
       <c r="S29" s="300" t="n"/>
-      <c r="T29" s="301" t="inlineStr">
+      <c r="T29" s="308" t="inlineStr">
         <is>
           <t>D78 - Ralo linear oculto para encaixe de granito. Dimensões conforme detalhamento. Ref.: Elleve</t>
         </is>
       </c>
-      <c r="U29" s="301" t="inlineStr">
+      <c r="U29" s="308" t="inlineStr">
         <is>
           <t>D79 - Chuveiro de piso para área externa em aço inox 316. cód.: DK5123B. Ref.: Doka</t>
         </is>
       </c>
       <c r="V29" s="302" t="n"/>
       <c r="W29" s="307" t="n"/>
-      <c r="X29" s="299" t="inlineStr">
+      <c r="X29" s="307" t="inlineStr">
         <is>
           <t>D77 - Porta pivotante para guarda corpo em vidro temperado laminado liso incolor com tubo para pivô em aço inox polido 1 1/4'' fixado no piso com barra lisa soltada com rosca na extremidade para fixação do vidro com botão de acabamento.</t>
         </is>
       </c>
       <c r="Y29" s="302" t="n"/>
-      <c r="Z29" s="299" t="inlineStr">
+      <c r="Z29" s="307" t="inlineStr">
         <is>
           <t>D76 - Guarda corpo em vidro temperado laminado liso incolor embutido no piso com ancoragem mínima de 70mm através de perfil fixador em aço inox e espaçamento entre vidros de 30mm.</t>
         </is>
@@ -11899,7 +11987,7 @@
           <t>BAR PISCINA</t>
         </is>
       </c>
-      <c r="B32" s="299" t="inlineStr">
+      <c r="B32" s="307" t="inlineStr">
         <is>
           <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -11907,38 +11995,38 @@
       <c r="C32" s="300" t="n"/>
       <c r="D32" s="308" t="n"/>
       <c r="E32" s="308" t="n"/>
-      <c r="F32" s="299" t="inlineStr">
+      <c r="F32" s="307" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G32" s="300" t="n"/>
-      <c r="H32" s="299" t="inlineStr">
+      <c r="H32" s="307" t="inlineStr">
         <is>
           <t>PA42 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento serrado, com arte em baixo relevo, corte a laser, profundidade 4mm Espessura da pedra: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA51 - Pilar em concreto aparente</t>
         </is>
       </c>
-      <c r="I32" s="299" t="inlineStr">
+      <c r="I32" s="307" t="inlineStr">
         <is>
           <t>T4 - Forro em madeira pinho autoclavado tonalizado, espessura de 3cm, réguas de 10cm.  ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR
 T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J32" s="301" t="inlineStr">
+      <c r="J32" s="308" t="inlineStr">
         <is>
           <t>D46 - Bancada/Mesa em pedra sinterizada, Lava satin fusion collection. Espessura: 5mm. Ref: Neo Lhít. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="K32" s="300" t="n"/>
-      <c r="L32" s="301" t="inlineStr">
+      <c r="L32" s="308" t="inlineStr">
         <is>
           <t>D10 - Cuba Design Collection Quadrum 70 em Aço Inox com Acabamento Scotch Brite. Cód Ref.: REF 94007103. Ref.: Tramontina</t>
         </is>
       </c>
       <c r="M32" s="300" t="n"/>
       <c r="N32" s="300" t="n"/>
-      <c r="O32" s="301" t="inlineStr">
+      <c r="O32" s="308" t="inlineStr">
         <is>
           <t>D9 - Misturador Monocomando Monde Filter Plus em Aço Inox com Saída Adicional para Água Filtrada + Filtro 3M. Cód Ref.:  REF 94520025. Ref.: Tramontina. ATENÇÃO: vazão máxima de 9 l/min, instalar redutor de vazão se necessário</t>
         </is>
@@ -11947,14 +12035,14 @@
       <c r="Q32" s="300" t="n"/>
       <c r="R32" s="300" t="n"/>
       <c r="S32" s="300" t="n"/>
-      <c r="T32" s="301" t="inlineStr">
+      <c r="T32" s="308" t="inlineStr">
         <is>
           <t>D34 - Ralo 15x15cm com tampa lisa em aço inox, linha Square. Ref.: Elleve
 D35 - Ralo linear com tampa lisa em aço inox. Dimensões conforme detalhamento. Ref.: Elleve</t>
         </is>
       </c>
       <c r="U32" s="300" t="n"/>
-      <c r="V32" s="299" t="inlineStr">
+      <c r="V32" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
@@ -11962,7 +12050,7 @@
       <c r="W32" s="307" t="n"/>
       <c r="X32" s="302" t="n"/>
       <c r="Y32" s="302" t="n"/>
-      <c r="Z32" s="299" t="inlineStr">
+      <c r="Z32" s="307" t="inlineStr">
         <is>
           <t>D47 - Marcenaria sob bancada em MDF Kashimir ref. Arauco - portas e frente gavetas em reguas de madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador em cava na marcenaria. Apresentar amostra para aprovação GPA&amp;A Obs.: MDF possui certificação FSC. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR
 D48 - Estante suspensa em tubo retangular 25x25mm em aço inox com pintura ouro velho. Fixada no teto através de estrutura auxiliar. Apresentar amostra pintura e solda para aprovação GPA&amp;A.
@@ -12009,7 +12097,7 @@
           <t>CIRCULAÇÃO VESTIÁRIOS</t>
         </is>
       </c>
-      <c r="B34" s="299" t="inlineStr">
+      <c r="B34" s="307" t="inlineStr">
         <is>
           <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -12019,12 +12107,12 @@
       <c r="E34" s="308" t="n"/>
       <c r="F34" s="307" t="n"/>
       <c r="G34" s="300" t="n"/>
-      <c r="H34" s="299" t="inlineStr">
+      <c r="H34" s="307" t="inlineStr">
         <is>
           <t>PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
-      <c r="I34" s="299" t="inlineStr">
+      <c r="I34" s="307" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -12041,7 +12129,7 @@
       <c r="S34" s="307" t="n"/>
       <c r="T34" s="307" t="n"/>
       <c r="U34" s="300" t="n"/>
-      <c r="V34" s="299" t="inlineStr">
+      <c r="V34" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
@@ -12057,7 +12145,7 @@
           <t>VESTIÁRIO FEMININO</t>
         </is>
       </c>
-      <c r="B35" s="316" t="inlineStr">
+      <c r="B35" s="320" t="inlineStr">
         <is>
           <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -12065,20 +12153,20 @@
       <c r="C35" s="300" t="n"/>
       <c r="D35" s="307" t="n"/>
       <c r="E35" s="308" t="n"/>
-      <c r="F35" s="299" t="inlineStr">
+      <c r="F35" s="307" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G35" s="300" t="n"/>
-      <c r="H35" s="316" t="inlineStr">
+      <c r="H35" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.
 PA60 - Parede revestida em chapa de aço inox 304, acabamento polido. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I35" s="316" t="inlineStr">
+      <c r="I35" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -12103,7 +12191,7 @@
 CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
-      <c r="P35" s="316" t="inlineStr">
+      <c r="P35" s="320" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -12126,19 +12214,19 @@
           <t>D31 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="V35" s="299" t="inlineStr">
+      <c r="V35" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W35" s="307" t="n"/>
-      <c r="X35" s="299" t="inlineStr">
+      <c r="X35" s="307" t="inlineStr">
         <is>
           <t>D32 - Divisórias e portas pivotantes com estrutura em alumínio e fechamento em vidro, cor Dark Beige. Ref.: Duo. Puxador tipo cava com fechaduras tipo rolete espelho modelo redondo acabamento cromo-acetinado.</t>
         </is>
       </c>
       <c r="Y35" s="307" t="n"/>
-      <c r="Z35" s="318" t="inlineStr">
+      <c r="Z35" s="317" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -12152,7 +12240,7 @@
           <t xml:space="preserve">VESTIÁRIO MASCULINO </t>
         </is>
       </c>
-      <c r="B36" s="316" t="inlineStr">
+      <c r="B36" s="320" t="inlineStr">
         <is>
           <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
@@ -12160,20 +12248,20 @@
       <c r="C36" s="300" t="n"/>
       <c r="D36" s="307" t="n"/>
       <c r="E36" s="308" t="n"/>
-      <c r="F36" s="299" t="inlineStr">
+      <c r="F36" s="307" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G36" s="300" t="n"/>
-      <c r="H36" s="316" t="inlineStr">
+      <c r="H36" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.
 PA60 - Parede revestida em chapa de aço inox 304, acabamento polido. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I36" s="316" t="inlineStr">
+      <c r="I36" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -12198,7 +12286,7 @@
 CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
-      <c r="P36" s="316" t="inlineStr">
+      <c r="P36" s="320" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -12221,19 +12309,19 @@
           <t>D31 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="V36" s="299" t="inlineStr">
+      <c r="V36" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W36" s="307" t="n"/>
-      <c r="X36" s="299" t="inlineStr">
+      <c r="X36" s="307" t="inlineStr">
         <is>
           <t>D32 - Divisórias e portas pivotantes com estrutura em alumínio e fechamento em vidro, cor Dark Beige. Ref.: Duo. Puxador tipo cava com fechaduras tipo rolete espelho modelo redondo acabamento cromo-acetinado.</t>
         </is>
       </c>
       <c r="Y36" s="307" t="n"/>
-      <c r="Z36" s="318" t="inlineStr">
+      <c r="Z36" s="317" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -12247,7 +12335,7 @@
           <t>ACADEMIA</t>
         </is>
       </c>
-      <c r="B37" s="316" t="inlineStr">
+      <c r="B37" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P22 - Piso em contrapiso regularizado, revestido em piso emborrachado isolante e antiderrapante, acabamernto preto, placas 100x100cm. Espessura: 8mm. Paginação conforme detalhamento. Ref.: Rubberkap ou similar. Amostra a ser aprovada pela GPA&amp;A.</t>
@@ -12262,7 +12350,7 @@
         </is>
       </c>
       <c r="G37" s="300" t="n"/>
-      <c r="H37" s="316" t="inlineStr">
+      <c r="H37" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA27 - Parede em alvenaria rebocada e regularizada revestida em espelho liso fumê 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
@@ -12271,7 +12359,7 @@
 PA30 - Pilar em concreto com acabamento em textura mineral Arch + Concrete ENG, Ref.: Novacolor. Fornecedor: Icolori (31)99952-2442. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I37" s="316" t="inlineStr">
+      <c r="I37" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil
 FO2 - Forro em gesso acartonado perfurado de absorção acústica, modelo cleneo quadrado, furação 12/25, sistema de instalação tipo FGE - estruturado, Ref.: Knauf Ceiling Solutions ou similar. Bordas ou "tabeiras" em gesso liso, com acabamento em tinta acrílica fosca, cor branco neve. Preenchimento superior com 1 manta de lã de pet com 35Kg/m³ de densidade de 50mm de espessura, Ref.: Trisoft ou similar.</t>
@@ -12289,19 +12377,19 @@
       <c r="S37" s="307" t="n"/>
       <c r="T37" s="307" t="n"/>
       <c r="U37" s="300" t="n"/>
-      <c r="V37" s="299" t="inlineStr">
+      <c r="V37" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W37" s="307" t="n"/>
-      <c r="X37" s="299" t="inlineStr">
+      <c r="X37" s="307" t="inlineStr">
         <is>
           <t>D57 - Porta de correr com duas folhas em vidro temperado liso incolor, com kit de instalação de sensor, modelo ES200. Ref.: Dorma</t>
         </is>
       </c>
       <c r="Y37" s="307" t="n"/>
-      <c r="Z37" s="301" t="inlineStr">
+      <c r="Z37" s="308" t="inlineStr">
         <is>
           <t>D3 - Estante em MDF Nero Rust Ref.: Berneck, desenho conforme detalhamento, Amostra a ser aprovada pela GPA&amp;A. Obs.: MDF possui certificação FSC.
 D4 - Armário em marcenaria, estruturado, com espaço para central de sonorização e automação, quadro de distribuição embutido - verificar dimensões com projetos específico, desenho conforme detalhamento. Porta.  de giro com sistema fecho-toque, acabamento em MDF Nero Rust. Ref.: Berneck. Obs.: MDF possui certificação FSC.
@@ -12349,7 +12437,7 @@
           <t>PISCINA RAIA</t>
         </is>
       </c>
-      <c r="B39" s="316" t="inlineStr">
+      <c r="B39" s="320" t="inlineStr">
         <is>
           <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -12359,7 +12447,7 @@
       <c r="E39" s="308" t="n"/>
       <c r="F39" s="300" t="n"/>
       <c r="G39" s="300" t="n"/>
-      <c r="H39" s="316" t="inlineStr">
+      <c r="H39" s="320" t="inlineStr">
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -12399,7 +12487,7 @@
       <c r="E40" s="308" t="n"/>
       <c r="F40" s="300" t="n"/>
       <c r="G40" s="300" t="n"/>
-      <c r="H40" s="316" t="inlineStr">
+      <c r="H40" s="320" t="inlineStr">
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -12438,7 +12526,7 @@
       <c r="C41" s="300" t="n"/>
       <c r="D41" s="307" t="n"/>
       <c r="E41" s="308" t="n"/>
-      <c r="F41" s="301" t="inlineStr">
+      <c r="F41" s="308" t="inlineStr">
         <is>
           <t>PA23 - Rodapé em mármore branco selecionado embutido na alvenaria, lote a ser aprovado, acabamento levigado. Arremate de topo com perfil "U" em aço inox 10x10mm. Paginação e dimensões seguem paginação do piso e detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada na GPA&amp;A</t>
         </is>
@@ -12452,7 +12540,7 @@
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
-      <c r="I41" s="316" t="inlineStr">
+      <c r="I41" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil
 T7 - Forro com resistência à umidade, especificação a ser definida. Projeto técnico a ser desenvolvido pelo fornecedor e validado pela GPAA&amp;A.</t>
@@ -12466,13 +12554,13 @@
       <c r="O41" s="307" t="n"/>
       <c r="P41" s="302" t="n"/>
       <c r="Q41" s="300" t="n"/>
-      <c r="R41" s="299" t="inlineStr">
+      <c r="R41" s="307" t="inlineStr">
         <is>
           <t>D58 - Acabamento para registro DocolBase, linha Mix&amp;Match, acabamento cromado. Ref.: Docol</t>
         </is>
       </c>
       <c r="S41" s="307" t="n"/>
-      <c r="T41" s="299" t="inlineStr">
+      <c r="T41" s="307" t="inlineStr">
         <is>
           <t>D35 - Ralo linear com tampa lisa em aço inox. Dimensões conforme detalhamento. Ref.: Elleve</t>
         </is>
@@ -12483,13 +12571,13 @@
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
-      <c r="V41" s="299" t="inlineStr">
+      <c r="V41" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W41" s="307" t="n"/>
-      <c r="X41" s="299" t="inlineStr">
+      <c r="X41" s="307" t="inlineStr">
         <is>
           <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -12549,18 +12637,18 @@
       <c r="O42" s="307" t="n"/>
       <c r="P42" s="302" t="n"/>
       <c r="Q42" s="300" t="n"/>
-      <c r="R42" s="299" t="inlineStr">
+      <c r="R42" s="307" t="inlineStr">
         <is>
           <t>D58 - Acabamento para registro DocolBase, linha Mix&amp;Match, acabamento cromado. Ref.: Docol</t>
         </is>
       </c>
       <c r="S42" s="307" t="n"/>
-      <c r="T42" s="299" t="inlineStr">
+      <c r="T42" s="307" t="inlineStr">
         <is>
           <t>D35 - Ralo linear com tampa lisa em aço inox. Dimensões conforme detalhamento. Ref.: Elleve</t>
         </is>
       </c>
-      <c r="U42" s="301" t="inlineStr">
+      <c r="U42" s="308" t="inlineStr">
         <is>
           <t>D54 - Chuveiro de embutir no teto Raindream, Roca, acabamento cromado, cód.: A5B3250C0C. Ref.: Roca. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
@@ -12667,14 +12755,14 @@
         </is>
       </c>
       <c r="G45" s="300" t="n"/>
-      <c r="H45" s="316" t="inlineStr">
+      <c r="H45" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA47 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 930, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I45" s="316" t="inlineStr">
+      <c r="I45" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -12687,7 +12775,7 @@
         </is>
       </c>
       <c r="K45" s="300" t="n"/>
-      <c r="L45" s="316" t="inlineStr">
+      <c r="L45" s="320" t="inlineStr">
         <is>
           <t>D55 - Cuba de apoio, modelo Ametista 26, cor branco, cód.:121003002. Ref.: Sabbia
 D62 - Cuba esculpida em mármore branco selecionado, lote a ser aprovado. Interior da cuba e bandeja removível em mármore liso. Fechamento lateral em mármore frisado e fechamento frontal em placa de mármore frisado fixado com imã em estrutura auxiliar de metalon. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
@@ -12695,7 +12783,7 @@
       </c>
       <c r="M45" s="308" t="n"/>
       <c r="N45" s="308" t="n"/>
-      <c r="O45" s="316" t="inlineStr">
+      <c r="O45" s="320" t="inlineStr">
         <is>
           <t>D51 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
 D53 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
@@ -12707,13 +12795,13 @@
       <c r="S45" s="307" t="n"/>
       <c r="T45" s="307" t="n"/>
       <c r="U45" s="300" t="n"/>
-      <c r="V45" s="299" t="inlineStr">
+      <c r="V45" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W45" s="307" t="n"/>
-      <c r="X45" s="316" t="inlineStr">
+      <c r="X45" s="320" t="inlineStr">
         <is>
           <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -12741,14 +12829,14 @@
         </is>
       </c>
       <c r="G46" s="300" t="n"/>
-      <c r="H46" s="316" t="inlineStr">
+      <c r="H46" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA47 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 930, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I46" s="316" t="inlineStr">
+      <c r="I46" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -12761,7 +12849,7 @@
         </is>
       </c>
       <c r="K46" s="300" t="n"/>
-      <c r="L46" s="299" t="inlineStr">
+      <c r="L46" s="307" t="inlineStr">
         <is>
           <t>D55 - Cuba de apoio, modelo Ametista 26, cor branco, cód.:121003002. Ref.: Sabbia
 D62 - Cuba esculpida em mármore branco selecionado, lote a ser aprovado. Interior da cuba e bandeja removível em mármore liso. Fechamento lateral em mármore frisado e fechamento frontal em placa de mármore frisado fixado com imã em estrutura auxiliar de metalon. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
@@ -12769,7 +12857,7 @@
       </c>
       <c r="M46" s="308" t="n"/>
       <c r="N46" s="308" t="n"/>
-      <c r="O46" s="316" t="inlineStr">
+      <c r="O46" s="320" t="inlineStr">
         <is>
           <t>D51 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
 D53 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
@@ -12781,13 +12869,13 @@
       <c r="S46" s="307" t="n"/>
       <c r="T46" s="307" t="n"/>
       <c r="U46" s="300" t="n"/>
-      <c r="V46" s="299" t="inlineStr">
+      <c r="V46" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W46" s="307" t="n"/>
-      <c r="X46" s="299" t="inlineStr">
+      <c r="X46" s="307" t="inlineStr">
         <is>
           <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
@@ -12801,7 +12889,7 @@
           <t>HALL VESTIÁRIOS</t>
         </is>
       </c>
-      <c r="B47" s="299" t="inlineStr">
+      <c r="B47" s="307" t="inlineStr">
         <is>
           <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -12809,19 +12897,19 @@
       <c r="C47" s="300" t="n"/>
       <c r="D47" s="307" t="n"/>
       <c r="E47" s="308" t="n"/>
-      <c r="F47" s="301" t="inlineStr">
+      <c r="F47" s="308" t="inlineStr">
         <is>
           <t>PA23 - Rodapé em mármore branco selecionado embutido na alvenaria, lote a ser aprovado, acabamento levigado. Arremate de topo com perfil "U" em aço inox 10x10mm. Paginação e dimensões seguem paginação do piso e detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada na GPA&amp;A</t>
         </is>
       </c>
       <c r="G47" s="300" t="n"/>
-      <c r="H47" s="299" t="inlineStr">
+      <c r="H47" s="307" t="inlineStr">
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA48 - Parede rebocada e regularizada revestida em mármore branco selecionado, lote a ser aprovado, acabamento frisado com ranhuras de 4x4mm espassada a cada 12mm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I47" s="299" t="inlineStr">
+      <c r="I47" s="307" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -12840,7 +12928,7 @@
       <c r="U47" s="300" t="n"/>
       <c r="V47" s="302" t="n"/>
       <c r="W47" s="307" t="n"/>
-      <c r="X47" s="299" t="inlineStr">
+      <c r="X47" s="307" t="inlineStr">
         <is>
           <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
 D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
@@ -12855,7 +12943,7 @@
           <t>VEST. P.C.D</t>
         </is>
       </c>
-      <c r="B48" s="299" t="inlineStr">
+      <c r="B48" s="307" t="inlineStr">
         <is>
           <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -12863,80 +12951,80 @@
       <c r="C48" s="300" t="n"/>
       <c r="D48" s="307" t="n"/>
       <c r="E48" s="308" t="n"/>
-      <c r="F48" s="301" t="inlineStr">
+      <c r="F48" s="308" t="inlineStr">
         <is>
           <t>PA23 - Rodapé em mármore branco selecionado embutido na alvenaria, lote a ser aprovado, acabamento levigado. Arremate de topo com perfil "U" em aço inox 10x10mm. Paginação e dimensões seguem paginação do piso e detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada na GPA&amp;A</t>
         </is>
       </c>
       <c r="G48" s="300" t="n"/>
-      <c r="H48" s="299" t="inlineStr">
+      <c r="H48" s="307" t="inlineStr">
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA47 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 930, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I48" s="299" t="inlineStr">
+      <c r="I48" s="307" t="inlineStr">
         <is>
           <t>T8 - Forro em gesso acartonado liso hidrofugante, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J48" s="299" t="inlineStr">
+      <c r="J48" s="307" t="inlineStr">
         <is>
           <t>D73 - Bancada em pedra natural, mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="K48" s="301" t="inlineStr">
+      <c r="K48" s="308" t="inlineStr">
         <is>
           <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
-      <c r="L48" s="299" t="inlineStr">
+      <c r="L48" s="307" t="inlineStr">
         <is>
           <t>D72 - Cuba de semiencaixe, linha Slim, cor branco, cód.: L.61040.M.17. Ref.: Deca</t>
         </is>
       </c>
       <c r="M48" s="308" t="n"/>
       <c r="N48" s="308" t="n"/>
-      <c r="O48" s="299" t="inlineStr">
+      <c r="O48" s="307" t="inlineStr">
         <is>
           <t>D69 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca</t>
         </is>
       </c>
-      <c r="P48" s="299" t="inlineStr">
+      <c r="P48" s="307" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="Q48" s="301" t="inlineStr">
+      <c r="Q48" s="308" t="inlineStr">
         <is>
           <t>D84 - Ducha higiênica com registro e derivação de parede linha Mix&amp;Match, acabamento cromado. Cód.: 90009316006. Ref.: Docol</t>
         </is>
       </c>
       <c r="R48" s="307" t="n"/>
-      <c r="S48" s="299" t="inlineStr">
+      <c r="S48" s="307" t="inlineStr">
         <is>
           <t>D33 - Monocomando para chuveiro, linha Mix&amp;Match, acabamento cromado, cód.:90009312006. Ref.: Docol</t>
         </is>
       </c>
-      <c r="T48" s="299" t="inlineStr">
+      <c r="T48" s="307" t="inlineStr">
         <is>
           <t>D35 - Ralo linear com tampa lisa em aço inox. Dimensões conforme detalhamento. Ref.: Elleve</t>
         </is>
       </c>
-      <c r="U48" s="301" t="inlineStr">
+      <c r="U48" s="308" t="inlineStr">
         <is>
           <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="V48" s="299" t="inlineStr">
+      <c r="V48" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W48" s="307" t="n"/>
-      <c r="X48" s="299" t="n"/>
+      <c r="X48" s="307" t="n"/>
       <c r="Y48" s="307" t="n"/>
-      <c r="Z48" s="301" t="inlineStr">
+      <c r="Z48" s="308" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -12950,7 +13038,7 @@
           <t>VEST. P.C.D</t>
         </is>
       </c>
-      <c r="B49" s="299" t="inlineStr">
+      <c r="B49" s="307" t="inlineStr">
         <is>
           <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -12958,80 +13046,80 @@
       <c r="C49" s="300" t="n"/>
       <c r="D49" s="307" t="n"/>
       <c r="E49" s="308" t="n"/>
-      <c r="F49" s="301" t="inlineStr">
+      <c r="F49" s="308" t="inlineStr">
         <is>
           <t>PA23 - Rodapé em mármore branco selecionado embutido na alvenaria, lote a ser aprovado, acabamento levigado. Arremate de topo com perfil "U" em aço inox 10x10mm. Paginação e dimensões seguem paginação do piso e detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada na GPA&amp;A</t>
         </is>
       </c>
       <c r="G49" s="300" t="n"/>
-      <c r="H49" s="299" t="inlineStr">
+      <c r="H49" s="307" t="inlineStr">
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA47 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 930, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I49" s="299" t="inlineStr">
+      <c r="I49" s="307" t="inlineStr">
         <is>
           <t>T8 - Forro em gesso acartonado liso hidrofugante, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J49" s="299" t="inlineStr">
+      <c r="J49" s="307" t="inlineStr">
         <is>
           <t>D73 - Bancada em pedra natural, mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="K49" s="301" t="inlineStr">
+      <c r="K49" s="308" t="inlineStr">
         <is>
           <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
-      <c r="L49" s="299" t="inlineStr">
+      <c r="L49" s="307" t="inlineStr">
         <is>
           <t>D72 - Cuba de semiencaixe, linha Slim, cor branco, cód.: L.61040.M.17. Ref.: Deca</t>
         </is>
       </c>
       <c r="M49" s="308" t="n"/>
       <c r="N49" s="308" t="n"/>
-      <c r="O49" s="299" t="inlineStr">
+      <c r="O49" s="307" t="inlineStr">
         <is>
           <t>D69 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca</t>
         </is>
       </c>
-      <c r="P49" s="299" t="inlineStr">
+      <c r="P49" s="307" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
-      <c r="Q49" s="301" t="inlineStr">
+      <c r="Q49" s="308" t="inlineStr">
         <is>
           <t>D84 - Ducha higiênica com registro e derivação de parede linha Mix&amp;Match, acabamento cromado. Cód.: 90009316006. Ref.: Docol</t>
         </is>
       </c>
       <c r="R49" s="307" t="n"/>
-      <c r="S49" s="299" t="inlineStr">
+      <c r="S49" s="307" t="inlineStr">
         <is>
           <t>D33 - Monocomando para chuveiro, linha Mix&amp;Match, acabamento cromado, cód.:90009312006. Ref.: Docol</t>
         </is>
       </c>
-      <c r="T49" s="299" t="inlineStr">
+      <c r="T49" s="307" t="inlineStr">
         <is>
           <t>D35 - Ralo linear com tampa lisa em aço inox. Dimensões conforme detalhamento. Ref.: Elleve</t>
         </is>
       </c>
-      <c r="U49" s="301" t="inlineStr">
+      <c r="U49" s="308" t="inlineStr">
         <is>
           <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="V49" s="299" t="inlineStr">
+      <c r="V49" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W49" s="307" t="n"/>
-      <c r="X49" s="299" t="n"/>
+      <c r="X49" s="307" t="n"/>
       <c r="Y49" s="307" t="n"/>
-      <c r="Z49" s="301" t="inlineStr">
+      <c r="Z49" s="308" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -13045,7 +13133,7 @@
           <t>DML</t>
         </is>
       </c>
-      <c r="B50" s="316" t="inlineStr">
+      <c r="B50" s="320" t="inlineStr">
         <is>
           <t>P10 - Piso elevado em mármore branco selecionado, lote a ser aprovado, acabamento levigado. Espessura: 3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
@@ -13053,7 +13141,7 @@
       <c r="C50" s="300" t="n"/>
       <c r="D50" s="307" t="n"/>
       <c r="E50" s="308" t="n"/>
-      <c r="F50" s="318" t="inlineStr">
+      <c r="F50" s="317" t="inlineStr">
         <is>
           <t>PA23 - Rodapé em mármore branco selecionado embutido na alvenaria, lote a ser aprovado, acabamento levigado. Arremate de topo com perfil "U" em aço inox 10x10mm. Paginação e dimensões seguem paginação do piso e detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada na GPA&amp;A</t>
         </is>
@@ -13064,7 +13152,7 @@
           <t>PA47 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 930, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I50" s="316" t="inlineStr">
+      <c r="I50" s="320" t="inlineStr">
         <is>
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -13150,7 +13238,7 @@
 ARQ-PA03 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza, tom a definir.</t>
         </is>
       </c>
-      <c r="I52" s="299" t="inlineStr">
+      <c r="I52" s="307" t="inlineStr">
         <is>
           <t>ARQ-T05 - Cobertura em telha sanduíche com estrutura espacial pintadas na cor cinza tom a definir.</t>
         </is>
@@ -13326,13 +13414,13 @@
       <c r="C55" s="300" t="n"/>
       <c r="D55" s="307" t="n"/>
       <c r="E55" s="308" t="n"/>
-      <c r="F55" s="318" t="inlineStr">
+      <c r="F55" s="317" t="inlineStr">
         <is>
           <t>PA23 - Rodapé em mármore branco selecionado embutido na alvenaria, lote a ser aprovado, acabamento levigado. Arremate de topo com perfil "U" em aço inox 10x10mm. Paginação e dimensões seguem paginação do piso e detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada na GPA&amp;A</t>
         </is>
       </c>
       <c r="G55" s="300" t="n"/>
-      <c r="H55" s="316" t="inlineStr">
+      <c r="H55" s="320" t="inlineStr">
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA47 - Parede em alvenaria emassada regularizada pintada com tinta mineral, cor 930, acabamento CQ. Ref.: Terracor. Amostra a ser aprovada pela GPA&amp;A
@@ -13340,7 +13428,7 @@
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
-      <c r="I55" s="316" t="inlineStr">
+      <c r="I55" s="320" t="inlineStr">
         <is>
           <t>T8 - Forro em gesso acartonado liso hidrofugante, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
@@ -13371,7 +13459,7 @@
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
-      <c r="P55" s="316" t="inlineStr">
+      <c r="P55" s="320" t="inlineStr">
         <is>
           <t>D22 - Bacia Sanitária com caixa acoplada, linha Carrara, acabamento branco, cód.: P.606.17. Ref.: Deca OU Bacia Sanitária com caixa acoplada, linha Panache, acabamento branco, cód.: K-18395BR-0.Amostra a ser aprovada pela GPA&amp;A.
 ► VER IMAGEM (clique)</t>
@@ -13385,7 +13473,7 @@
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
-      <c r="T55" s="299" t="inlineStr">
+      <c r="T55" s="307" t="inlineStr">
         <is>
           <t>D34 - Ralo 15x15cm com tampa lisa em aço inox, linha Square. Ref.: Elleve
 D35 - Ralo linear com tampa lisa em aço inox. Dimensões conforme detalhamento. Ref.: Elleve</t>
@@ -13397,20 +13485,20 @@
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
-      <c r="V55" s="299" t="inlineStr">
+      <c r="V55" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
       </c>
       <c r="W55" s="307" t="n"/>
-      <c r="X55" s="299" t="inlineStr">
+      <c r="X55" s="307" t="inlineStr">
         <is>
           <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
 D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y55" s="307" t="n"/>
-      <c r="Z55" s="318" t="inlineStr">
+      <c r="Z55" s="317" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
 D26 - Saboneteira de pressão em aço inox, instalação na parede, modelo Prime Press Espuma, cód.:70.032. Ref.: Draco
@@ -13574,7 +13662,7 @@
           <t>CIRCULAÇÃO</t>
         </is>
       </c>
-      <c r="B58" s="316" t="inlineStr">
+      <c r="B58" s="320" t="inlineStr">
         <is>
           <t>PI02 - Contrapiso flutuante: Contrapiso armado sobre painel de lã de vidro, (sistema optma piso, membrana flexível, 15mm de espessura, Ref.: ISOVER. Para evitar fissuras o contrapiso deverá ser armado com tela tipo "pop" soldada
 P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -13583,27 +13671,27 @@
       <c r="C58" s="300" t="n"/>
       <c r="D58" s="307" t="n"/>
       <c r="E58" s="308" t="n"/>
-      <c r="F58" s="318" t="inlineStr">
+      <c r="F58" s="317" t="inlineStr">
         <is>
           <t>PA20 - Rodapé de embutir em alvenaria em cantoneira metálica 50x15mm em alumínio anodizado pintado no tom da parede.</t>
         </is>
       </c>
       <c r="G58" s="300" t="n"/>
-      <c r="H58" s="316" t="inlineStr">
+      <c r="H58" s="320" t="inlineStr">
         <is>
           <t>PA44 - Parede em alvenaria emassada regularizada, revestida em massa acrílica texturizada cimento queimado, cor 107. Ref.: Terracor CQ. Amostra a ser aprovada pela GPA&amp;A.
 PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA58 - Pilar em concreto, com enchimento, revestido em pedra natural Basaltina conforme detalhamento.Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="I58" s="316" t="inlineStr">
+      <c r="I58" s="320" t="inlineStr">
         <is>
           <t>FO2 - Forro em gesso acartonado perfurado de absorção acústica, modelo cleneo quadrado, furação 12/25, sistema de instalação tipo FGE - estruturado, Ref.: Knauf Ceiling Solutions ou similar. Bordas ou "tabeiras" em gesso liso, com acabamento em tinta acrílica fosca, cor branco neve. Preenchimento superior com 1 manta de lã de pet com 35Kg/m³ de densidade de 50mm de espessura, Ref.: Trisoft ou similar.
 T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
       <c r="J58" s="320" t="n"/>
-      <c r="K58" s="318" t="inlineStr">
+      <c r="K58" s="317" t="inlineStr">
         <is>
           <t>D75 - Fechamento decorativo piso teto com quadro fixado no piso e no teto através de espaçadores e fechamento com desenho conforme base para corte de molde em CNC - peças em madeira maciça engenheirada, tonalizada,acabamento escovado, calandradas conforme molde. Ref.: Demuner. ATENÇÃO:a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
@@ -13618,7 +13706,7 @@
       <c r="S58" s="307" t="n"/>
       <c r="T58" s="307" t="n"/>
       <c r="U58" s="300" t="n"/>
-      <c r="V58" s="299" t="inlineStr">
+      <c r="V58" s="307" t="inlineStr">
         <is>
           <t>D12 - Acabamento de tomadas e interruptores, linha Arteor, cor a definir conforme superfície a ser instalado. Ref.: Legrand</t>
         </is>
@@ -13634,7 +13722,7 @@
           <t>ESTAR PISCINA / CIRCULAÇÃO</t>
         </is>
       </c>
-      <c r="B59" s="316" t="inlineStr">
+      <c r="B59" s="320" t="inlineStr">
         <is>
           <t>P28 - Piso assentado em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.
 P8 - Piso elevado em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofulgante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
@@ -13667,7 +13755,7 @@
       <c r="W59" s="307" t="n"/>
       <c r="X59" s="307" t="n"/>
       <c r="Y59" s="307" t="n"/>
-      <c r="Z59" s="301" t="inlineStr">
+      <c r="Z59" s="308" t="inlineStr">
         <is>
           <t>D76 - Guarda corpo em vidro temperado laminado liso incolor embutido no piso com ancoragem mínima de 70mm através de perfil fixador em aço inox e espaçamento entre vidros de 30mm.</t>
         </is>
@@ -13726,7 +13814,7 @@
       <c r="E61" s="308" t="n"/>
       <c r="F61" s="317" t="n"/>
       <c r="G61" s="300" t="n"/>
-      <c r="H61" s="316" t="inlineStr">
+      <c r="H61" s="320" t="inlineStr">
         <is>
           <t>ARQ-PA06 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica fosca cinza tom a definir. Meia parede pintada com tinta acrílica fosca na cor verde, tom a definir. Verificar altura conforme detalhamento.</t>
         </is>
@@ -13798,7 +13886,7 @@
           <t>APOIO QUADRAS</t>
         </is>
       </c>
-      <c r="B63" s="316" t="inlineStr">
+      <c r="B63" s="320" t="inlineStr">
         <is>
           <t>P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.
 P27 - Piso em deck de madeira, modelo Tauari Teak encaixe macho e femea, acabamento com cavilha, reguas 20mmx100mmx2000m-acima. Ref.: Indusparquet.  ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
@@ -13810,7 +13898,7 @@
       <c r="F63" s="317" t="n"/>
       <c r="G63" s="300" t="n"/>
       <c r="H63" s="320" t="n"/>
-      <c r="I63" s="316" t="inlineStr">
+      <c r="I63" s="320" t="inlineStr">
         <is>
           <t>FO2 - Forro em gesso acartonado perfurado de absorção acústica, modelo cleneo quadrado, furação 12/25, sistema de instalação tipo FGE - estruturado, Ref.: Knauf Ceiling Solutions ou similar. Bordas ou "tabeiras" em gesso liso, com acabamento em tinta acrílica fosca, cor branco neve. Preenchimento superior com 1 manta de lã de pet com 35Kg/m³ de densidade de 50mm de espessura, Ref.: Trisoft ou similar.
 T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
@@ -13840,7 +13928,7 @@
           <t>CIRCULAÇÃO JUNTO À ESCADA (A=2,91 m²)</t>
         </is>
       </c>
-      <c r="B64" s="316" t="inlineStr">
+      <c r="B64" s="320" t="inlineStr">
         <is>
           <t>ARQ-P03 - Piso em concreto mecanizado com acabamento antiderrapante</t>
         </is>
@@ -13850,12 +13938,12 @@
       <c r="E64" s="308" t="n"/>
       <c r="F64" s="317" t="n"/>
       <c r="G64" s="300" t="n"/>
-      <c r="H64" s="316" t="inlineStr">
+      <c r="H64" s="320" t="inlineStr">
         <is>
           <t>ARQ-PA09 - Parede em alvenaria, emassada e regularizada, revestida em textura acrílica rolada fosca branca. Ref.: Branco Neve; Suvinil.</t>
         </is>
       </c>
-      <c r="I64" s="316" t="inlineStr">
+      <c r="I64" s="320" t="inlineStr">
         <is>
           <t>ARQ-T02 - Laje em concreto aparente com tratamento a ser indicado pelo projeto estrutural.</t>
         </is>
@@ -14611,7 +14699,7 @@
           <t>SALA / VARANDA DA SALA</t>
         </is>
       </c>
-      <c r="B13" s="299" t="inlineStr">
+      <c r="B13" s="307" t="inlineStr">
         <is>
           <t>Piso em mármore travertino romano bruto, 85x130cm, paginação conforme detalhamento. Rejunte Infinity Hard, cor Areia ou Palha (validar com o Setor de Produto). (DET PR001/PR002; Tab. R01)</t>
         </is>
@@ -14626,12 +14714,12 @@
         </is>
       </c>
       <c r="G13" s="300" t="n"/>
-      <c r="H13" s="301" t="inlineStr">
+      <c r="H13" s="308" t="inlineStr">
         <is>
           <t>Pintura acrílica cor branco neve, acabamento acetinado. (DET PR001; Tab. R01)</t>
         </is>
       </c>
-      <c r="I13" s="301" t="n"/>
+      <c r="I13" s="308" t="n"/>
       <c r="J13" s="300" t="n"/>
       <c r="K13" s="300" t="n"/>
       <c r="L13" s="300" t="n"/>
@@ -14664,7 +14752,7 @@
           <t>LAVABO</t>
         </is>
       </c>
-      <c r="B14" s="299" t="inlineStr">
+      <c r="B14" s="307" t="inlineStr">
         <is>
           <t>Piso em mármore travertino romano bruto. Rejunte Infinity Hard, cor Areia ou Palha (validar com o Setor de Produto). (DET PR004; Tab. R01)</t>
         </is>
@@ -14683,12 +14771,12 @@
         </is>
       </c>
       <c r="G14" s="300" t="n"/>
-      <c r="H14" s="301" t="inlineStr">
+      <c r="H14" s="308" t="inlineStr">
         <is>
           <t>Pintura acrílica cor branco neve, acabamento acetinado. (DET PR004; Tab. R01)</t>
         </is>
       </c>
-      <c r="I14" s="301" t="inlineStr">
+      <c r="I14" s="308" t="inlineStr">
         <is>
           <t>Forro em gesso acartonado, pintura acrílica acetinada cor branco neve, tabica metálica. PD 298cm. (DET PR004)</t>
         </is>
@@ -14746,7 +14834,7 @@
           <t>BANHO SUÍTE MASTER</t>
         </is>
       </c>
-      <c r="B15" s="299" t="inlineStr">
+      <c r="B15" s="307" t="inlineStr">
         <is>
           <t>11 - Piso em contrapiso regularizado, revestido em mármore travertino romano resinado. Rejunte creme ou marfim (ver padrão da chapa). Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (PR408; Tab. R01: "bruto resinado")</t>
         </is>
@@ -14771,7 +14859,7 @@
 CONFLITO – Tabela R01: parede em mármore travertino romano BRUTO paginado</t>
         </is>
       </c>
-      <c r="I15" s="301" t="inlineStr">
+      <c r="I15" s="308" t="inlineStr">
         <is>
           <t>1 - Forro em gesso acartonado liso, tinta acrílica cor branco neve, acabamento fosco, junta de dilatação metálica branca. Ref.: Suvinil. Sanca (DET 20). (PR408)</t>
         </is>
@@ -14850,7 +14938,7 @@
           <t>BANHO SUÍTES</t>
         </is>
       </c>
-      <c r="B16" s="299" t="inlineStr">
+      <c r="B16" s="307" t="inlineStr">
         <is>
           <t>Piso em mármore travertino romano bruto resinado, paginado. Rejunte Infinity Hard, cor Areia ou Palha (validar com o Setor de Produto). Desnível do box 1cm. (DET PR008; Tab. R01)</t>
         </is>
@@ -14860,12 +14948,12 @@
       <c r="E16" s="300" t="n"/>
       <c r="F16" s="300" t="n"/>
       <c r="G16" s="300" t="n"/>
-      <c r="H16" s="301" t="inlineStr">
+      <c r="H16" s="308" t="inlineStr">
         <is>
           <t>Parede em mármore travertino romano bruto: piso ao teto na área do box e barrado semi-embutido até 110cm nas demais paredes; acima, pintura acrílica cor branco neve, acetinado. (DET PR008; Tab. R01)</t>
         </is>
       </c>
-      <c r="I16" s="301" t="inlineStr">
+      <c r="I16" s="308" t="inlineStr">
         <is>
           <t>Forro em gesso acartonado, pintura acrílica acetinada cor branco neve, tabica metálica e sanca. PD 298cm. (DET PR008)</t>
         </is>
@@ -14926,7 +15014,7 @@
           <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
         </is>
       </c>
-      <c r="B17" s="299" t="inlineStr">
+      <c r="B17" s="307" t="inlineStr">
         <is>
           <t>Piso em cumaru, assoalho piso pronto. Ref.: Indusparquet. (DET PR001/PR002; Tab. R01)</t>
         </is>
@@ -14945,12 +15033,12 @@
         </is>
       </c>
       <c r="G17" s="300" t="n"/>
-      <c r="H17" s="301" t="inlineStr">
+      <c r="H17" s="308" t="inlineStr">
         <is>
           <t>Pintura acrílica cor branco neve. (Tab. R01)</t>
         </is>
       </c>
-      <c r="I17" s="301" t="n"/>
+      <c r="I17" s="308" t="n"/>
       <c r="J17" s="300" t="n"/>
       <c r="K17" s="300" t="n"/>
       <c r="L17" s="300" t="n"/>
@@ -14975,7 +15063,7 @@
           <t>COPA NOTURNA</t>
         </is>
       </c>
-      <c r="B18" s="299" t="inlineStr">
+      <c r="B18" s="307" t="inlineStr">
         <is>
           <t>Piso em cumaru, assoalho piso pronto. Ref.: Indusparquet. (Tab. R01)</t>
         </is>
@@ -14989,8 +15077,8 @@
         </is>
       </c>
       <c r="G18" s="300" t="n"/>
-      <c r="H18" s="301" t="n"/>
-      <c r="I18" s="301" t="n"/>
+      <c r="H18" s="308" t="n"/>
+      <c r="I18" s="308" t="n"/>
       <c r="J18" s="304" t="inlineStr">
         <is>
           <t>Bancada esculpida em mármore travertino romano resinado. (DET PR003)
@@ -15028,7 +15116,7 @@
           <t>COZINHA / DESPENSAS</t>
         </is>
       </c>
-      <c r="B19" s="299" t="inlineStr">
+      <c r="B19" s="307" t="inlineStr">
         <is>
           <t>Piso em granito branco siena escovado, 85x130cm. Rejunte Infinity Hard, cor Branco Pérola ou Palha (validar com o Setor de Produto). (DET PR001, PR406/407; Tab. R01: paginação a definir)</t>
         </is>
@@ -15046,13 +15134,13 @@
         </is>
       </c>
       <c r="G19" s="300" t="n"/>
-      <c r="H19" s="301" t="inlineStr">
+      <c r="H19" s="308" t="inlineStr">
         <is>
           <t>Rodabanca em granito branco siena escovado, h=60cm
 Pintura acrílica; cor a definir (Tab. R01). (PR406/407)</t>
         </is>
       </c>
-      <c r="I19" s="301" t="n"/>
+      <c r="I19" s="308" t="n"/>
       <c r="J19" s="300" t="inlineStr">
         <is>
           <t>Bancada e ilha em granito branco siena escovado; parte seca h=90cm, área molhada com desnível 1cm h=92cm; suporte em metalon chumbado na parede; emendas seguem a paginação do piso. (PR406/407; Tab. R01)</t>
@@ -15093,7 +15181,7 @@
           <t>ÁREA DE SERVIÇO / CIRCULAÇÃO SERVIÇO</t>
         </is>
       </c>
-      <c r="B20" s="299" t="inlineStr">
+      <c r="B20" s="307" t="inlineStr">
         <is>
           <t>Piso em granito branco siena escovado, 85x130cm, ver paginação. Rejunte Infinity Hard, cor Branco Pérola ou Palha. (DET PR001, PR005; Tab. R01)</t>
         </is>
@@ -15111,12 +15199,12 @@
         </is>
       </c>
       <c r="G20" s="300" t="n"/>
-      <c r="H20" s="301" t="inlineStr">
+      <c r="H20" s="308" t="inlineStr">
         <is>
           <t>Parede em Formica Branco Real L515, 308x125cm. (DET PR005/PR006; Tab. R01)</t>
         </is>
       </c>
-      <c r="I20" s="301" t="inlineStr">
+      <c r="I20" s="308" t="inlineStr">
         <is>
           <t>Forro de gesso com tabica metálica (DET 11) e cortineiro 25x16cm (DET 24). (DET PR006)</t>
         </is>
@@ -15174,7 +15262,7 @@
           <t>BANHO SERVIÇO</t>
         </is>
       </c>
-      <c r="B21" s="299" t="inlineStr">
+      <c r="B21" s="307" t="inlineStr">
         <is>
           <t>Piso em granito branco siena escovado. (DET PR007; Tab. R01: paginação a definir)</t>
         </is>
@@ -15188,12 +15276,12 @@
       <c r="E21" s="300" t="n"/>
       <c r="F21" s="300" t="n"/>
       <c r="G21" s="300" t="n"/>
-      <c r="H21" s="301" t="inlineStr">
+      <c r="H21" s="308" t="inlineStr">
         <is>
           <t>Revestimento Forma Branco AC retificado 32,5x59cm. Ref.: Eliane. (DET PR007; Tab. R01)</t>
         </is>
       </c>
-      <c r="I21" s="301" t="inlineStr">
+      <c r="I21" s="308" t="inlineStr">
         <is>
           <t>Forro em gesso acartonado, pintura acrílica acetinada cor branco neve, tabica metálica, sanca 25x16cm. PD 298cm. (DET PR007)</t>
         </is>
@@ -15250,7 +15338,7 @@
           <t>QUARTO / ESTAR FUNCIONÁRIOS</t>
         </is>
       </c>
-      <c r="B22" s="299" t="inlineStr">
+      <c r="B22" s="307" t="inlineStr">
         <is>
           <t>Piso vinílico Austin, linha Urban, 18x121cm. Ref.: Durafloor. (DET PR001; Tab. R01)</t>
         </is>
@@ -15268,12 +15356,12 @@
         </is>
       </c>
       <c r="G22" s="300" t="n"/>
-      <c r="H22" s="301" t="inlineStr">
+      <c r="H22" s="308" t="inlineStr">
         <is>
           <t>Pintura acrílica cor branco neve. (Tab. R01)</t>
         </is>
       </c>
-      <c r="I22" s="301" t="n"/>
+      <c r="I22" s="308" t="n"/>
       <c r="J22" s="300" t="n"/>
       <c r="K22" s="300" t="n"/>
       <c r="L22" s="300" t="n"/>
@@ -15298,7 +15386,7 @@
           <t>VARANDA TÉCNICA</t>
         </is>
       </c>
-      <c r="B23" s="299" t="inlineStr">
+      <c r="B23" s="307" t="inlineStr">
         <is>
           <t>Piso em concreto. (DET PR001)</t>
         </is>
@@ -15308,8 +15396,8 @@
       <c r="E23" s="300" t="n"/>
       <c r="F23" s="300" t="n"/>
       <c r="G23" s="300" t="n"/>
-      <c r="H23" s="301" t="n"/>
-      <c r="I23" s="301" t="n"/>
+      <c r="H23" s="308" t="n"/>
+      <c r="I23" s="308" t="n"/>
       <c r="J23" s="300" t="n"/>
       <c r="K23" s="300" t="n"/>
       <c r="L23" s="300" t="n"/>
@@ -15334,7 +15422,7 @@
           <t>HALL ELEVADOR SOCIAL (ANDAR)</t>
         </is>
       </c>
-      <c r="B24" s="299" t="inlineStr">
+      <c r="B24" s="307" t="inlineStr">
         <is>
           <t>Piso em mármore travertino romano bruto. (DET PR003)</t>
         </is>
@@ -15348,13 +15436,13 @@
         </is>
       </c>
       <c r="G24" s="300" t="n"/>
-      <c r="H24" s="301" t="inlineStr">
+      <c r="H24" s="308" t="inlineStr">
         <is>
           <t>Parede pintada com tinta acrílica cor branco neve, acabamento acetinado
 Aduela do elevador (2cm) em mármore travertino romano bruto. (DET PR003)</t>
         </is>
       </c>
-      <c r="I24" s="301" t="n"/>
+      <c r="I24" s="308" t="n"/>
       <c r="J24" s="300" t="n"/>
       <c r="K24" s="300" t="n"/>
       <c r="L24" s="300" t="n"/>
@@ -15379,7 +15467,7 @@
           <t>HALL ELEVADOR SERVIÇO (ANDAR)</t>
         </is>
       </c>
-      <c r="B25" s="299" t="inlineStr">
+      <c r="B25" s="307" t="inlineStr">
         <is>
           <t>Piso em granito branco siena escovado. (DET PR003)</t>
         </is>
@@ -15393,13 +15481,13 @@
         </is>
       </c>
       <c r="G25" s="300" t="n"/>
-      <c r="H25" s="301" t="inlineStr">
+      <c r="H25" s="308" t="inlineStr">
         <is>
           <t>Parede pintada com tinta acrílica cor branco neve, acabamento acetinado
 Aduela do elevador (2cm) em granito branco siena escovado. (DET PR003)</t>
         </is>
       </c>
-      <c r="I25" s="301" t="n"/>
+      <c r="I25" s="308" t="n"/>
       <c r="J25" s="300" t="n"/>
       <c r="K25" s="300" t="n"/>
       <c r="L25" s="300" t="n"/>
@@ -15424,7 +15512,7 @@
           <t>HALL SERVIÇO / ANTECÂMARA – GARDEN, TIPO E COBERTURA</t>
         </is>
       </c>
-      <c r="B26" s="299" t="inlineStr">
+      <c r="B26" s="307" t="inlineStr">
         <is>
           <t>Piso em granito ("revestimento conforme ambiente"). (PR721-728)</t>
         </is>
@@ -15438,12 +15526,12 @@
         </is>
       </c>
       <c r="G26" s="300" t="n"/>
-      <c r="H26" s="301" t="inlineStr">
+      <c r="H26" s="308" t="inlineStr">
         <is>
           <t>Parede pintada. (PR722/724/726/728)</t>
         </is>
       </c>
-      <c r="I26" s="301" t="inlineStr">
+      <c r="I26" s="308" t="inlineStr">
         <is>
           <t>Forro em gesso com sanca: PD 259cm (Garden e Tipo), 267,5cm (Cobertura 1º nível), 272,5cm (Cobertura 2º nível); junta de dilatação em perfil metálico "Z" (DET 09); trechos em laje de concreto aparente. (PR721-728)</t>
         </is>
@@ -15476,14 +15564,14 @@
     </row>
     <row r="27">
       <c r="A27" s="45" t="n"/>
-      <c r="B27" s="269" t="n"/>
+      <c r="B27" s="31" t="n"/>
       <c r="C27" s="32" t="n"/>
       <c r="D27" s="32" t="n"/>
       <c r="E27" s="32" t="n"/>
       <c r="F27" s="32" t="n"/>
       <c r="G27" s="32" t="n"/>
-      <c r="H27" s="271" t="n"/>
-      <c r="I27" s="271" t="n"/>
+      <c r="H27" s="33" t="n"/>
+      <c r="I27" s="33" t="n"/>
       <c r="J27" s="32" t="n"/>
       <c r="K27" s="32" t="n"/>
       <c r="L27" s="32" t="n"/>
@@ -15504,14 +15592,14 @@
     </row>
     <row r="28">
       <c r="A28" s="45" t="n"/>
-      <c r="B28" s="269" t="n"/>
+      <c r="B28" s="31" t="n"/>
       <c r="C28" s="32" t="n"/>
       <c r="D28" s="32" t="n"/>
       <c r="E28" s="32" t="n"/>
       <c r="F28" s="32" t="n"/>
       <c r="G28" s="32" t="n"/>
-      <c r="H28" s="271" t="n"/>
-      <c r="I28" s="271" t="n"/>
+      <c r="H28" s="33" t="n"/>
+      <c r="I28" s="33" t="n"/>
       <c r="J28" s="32" t="n"/>
       <c r="K28" s="32" t="n"/>
       <c r="L28" s="32" t="n"/>
@@ -15532,14 +15620,14 @@
     </row>
     <row r="29">
       <c r="A29" s="45" t="n"/>
-      <c r="B29" s="269" t="n"/>
+      <c r="B29" s="31" t="n"/>
       <c r="C29" s="32" t="n"/>
       <c r="D29" s="32" t="n"/>
       <c r="E29" s="32" t="n"/>
       <c r="F29" s="32" t="n"/>
       <c r="G29" s="32" t="n"/>
-      <c r="H29" s="271" t="n"/>
-      <c r="I29" s="271" t="n"/>
+      <c r="H29" s="33" t="n"/>
+      <c r="I29" s="33" t="n"/>
       <c r="J29" s="32" t="n"/>
       <c r="K29" s="32" t="n"/>
       <c r="L29" s="32" t="n"/>
@@ -15560,14 +15648,14 @@
     </row>
     <row r="30">
       <c r="A30" s="45" t="n"/>
-      <c r="B30" s="269" t="n"/>
+      <c r="B30" s="31" t="n"/>
       <c r="C30" s="32" t="n"/>
       <c r="D30" s="32" t="n"/>
       <c r="E30" s="32" t="n"/>
       <c r="F30" s="32" t="n"/>
       <c r="G30" s="32" t="n"/>
-      <c r="H30" s="271" t="n"/>
-      <c r="I30" s="271" t="n"/>
+      <c r="H30" s="33" t="n"/>
+      <c r="I30" s="33" t="n"/>
       <c r="J30" s="32" t="n"/>
       <c r="K30" s="32" t="n"/>
       <c r="L30" s="32" t="n"/>
@@ -15588,14 +15676,14 @@
     </row>
     <row r="31">
       <c r="A31" s="45" t="n"/>
-      <c r="B31" s="269" t="n"/>
+      <c r="B31" s="31" t="n"/>
       <c r="C31" s="32" t="n"/>
       <c r="D31" s="32" t="n"/>
       <c r="E31" s="32" t="n"/>
       <c r="F31" s="32" t="n"/>
       <c r="G31" s="32" t="n"/>
-      <c r="H31" s="271" t="n"/>
-      <c r="I31" s="271" t="n"/>
+      <c r="H31" s="33" t="n"/>
+      <c r="I31" s="33" t="n"/>
       <c r="J31" s="32" t="n"/>
       <c r="K31" s="32" t="n"/>
       <c r="L31" s="32" t="n"/>
@@ -15679,6 +15767,522 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="328" t="inlineStr">
+        <is>
+          <t>GRADE DE ESPECIFICAÇÕES · EDIFÍCIO JARDIM · ESPECIFICAÇÕES CONFLITANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="329" t="inlineStr">
+        <is>
+          <t>Células em que projetos diferentes trazem especificações diferentes para o mesmo item. As duas versões foram mantidas na grade, em vermelho claro, até a definição da arquitetura. Clique na célula (coluna F) para ir até ela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="330" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B4" s="330" t="inlineStr">
+        <is>
+          <t>ABA</t>
+        </is>
+      </c>
+      <c r="C4" s="330" t="inlineStr">
+        <is>
+          <t>AMBIENTE</t>
+        </is>
+      </c>
+      <c r="D4" s="330" t="inlineStr">
+        <is>
+          <t>GRUPO</t>
+        </is>
+      </c>
+      <c r="E4" s="330" t="inlineStr">
+        <is>
+          <t>ITEM</t>
+        </is>
+      </c>
+      <c r="F4" s="330" t="inlineStr">
+        <is>
+          <t>CÉLULA</t>
+        </is>
+      </c>
+      <c r="G4" s="330" t="inlineStr">
+        <is>
+          <t>ESPECIFICAÇÕES CONFLITANTES (versões e fontes)</t>
+        </is>
+      </c>
+      <c r="H4" s="330" t="inlineStr">
+        <is>
+          <t>DEFINIÇÃO DA ARQUITETURA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="117" customHeight="1">
+      <c r="A5" s="331" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="331" t="inlineStr">
+        <is>
+          <t>TÉRREO</t>
+        </is>
+      </c>
+      <c r="C5" s="332" t="inlineStr">
+        <is>
+          <t>GUARITA</t>
+        </is>
+      </c>
+      <c r="D5" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E5" s="331" t="inlineStr">
+        <is>
+          <t>PISO/REJUNTE</t>
+        </is>
+      </c>
+      <c r="F5" s="333" t="inlineStr">
+        <is>
+          <t>B17</t>
+        </is>
+      </c>
+      <c r="G5" s="334" t="inlineStr">
+        <is>
+          <t>P5 - Piso em porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado. Paginação conforme detalhamento. Ref.: Khali Off White AC; Linha Khali; Eliane. Rejunte Infinity Hard cor Mocha ou cor Branco Pérola Deverá ser testado as duas opções de rejunte para escolher a que mais se aproxima do tom da peça. Amostra a ser aprovada pela GPA&amp;A.
+CONFLITO – Arquitetura: ARQ-P13 - Piso em pedra natural Basaltina. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
+        </is>
+      </c>
+      <c r="H5" s="331" t="inlineStr"/>
+    </row>
+    <row r="6" ht="87" customHeight="1">
+      <c r="A6" s="331" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="331" t="inlineStr">
+        <is>
+          <t>TÉRREO</t>
+        </is>
+      </c>
+      <c r="C6" s="332" t="inlineStr">
+        <is>
+          <t>GUARITA</t>
+        </is>
+      </c>
+      <c r="D6" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E6" s="331" t="inlineStr">
+        <is>
+          <t>PAREDE/REJUNTE</t>
+        </is>
+      </c>
+      <c r="F6" s="333" t="inlineStr">
+        <is>
+          <t>H17</t>
+        </is>
+      </c>
+      <c r="G6" s="334" t="inlineStr">
+        <is>
+          <t>PA1 - Parede em alvenaria com reboco convencional 2,5cm, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.
+CONFLITO – Arquitetura: ARQ-PA02 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor a definir, acabamento acetinado.</t>
+        </is>
+      </c>
+      <c r="H6" s="331" t="inlineStr"/>
+    </row>
+    <row r="7" ht="102" customHeight="1">
+      <c r="A7" s="331" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C7" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO FEMININO</t>
+        </is>
+      </c>
+      <c r="D7" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E7" s="331" t="inlineStr">
+        <is>
+          <t>BANCADA</t>
+        </is>
+      </c>
+      <c r="F7" s="333" t="inlineStr">
+        <is>
+          <t>J35</t>
+        </is>
+      </c>
+      <c r="G7" s="334" t="inlineStr">
+        <is>
+          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
+        </is>
+      </c>
+      <c r="H7" s="331" t="inlineStr"/>
+    </row>
+    <row r="8" ht="87" customHeight="1">
+      <c r="A8" s="331" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C8" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO FEMININO</t>
+        </is>
+      </c>
+      <c r="D8" s="331" t="inlineStr">
+        <is>
+          <t>LOUÇAS E METAIS</t>
+        </is>
+      </c>
+      <c r="E8" s="331" t="inlineStr">
+        <is>
+          <t>TORNEIRAS</t>
+        </is>
+      </c>
+      <c r="F8" s="333" t="inlineStr">
+        <is>
+          <t>O35</t>
+        </is>
+      </c>
+      <c r="G8" s="334" t="inlineStr">
+        <is>
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
+        </is>
+      </c>
+      <c r="H8" s="331" t="inlineStr"/>
+    </row>
+    <row r="9" ht="102" customHeight="1">
+      <c r="A9" s="331" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C9" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO MASCULINO</t>
+        </is>
+      </c>
+      <c r="D9" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E9" s="331" t="inlineStr">
+        <is>
+          <t>BANCADA</t>
+        </is>
+      </c>
+      <c r="F9" s="333" t="inlineStr">
+        <is>
+          <t>J36</t>
+        </is>
+      </c>
+      <c r="G9" s="334" t="inlineStr">
+        <is>
+          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
+        </is>
+      </c>
+      <c r="H9" s="331" t="inlineStr"/>
+    </row>
+    <row r="10" ht="87" customHeight="1">
+      <c r="A10" s="331" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C10" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO MASCULINO</t>
+        </is>
+      </c>
+      <c r="D10" s="331" t="inlineStr">
+        <is>
+          <t>LOUÇAS E METAIS</t>
+        </is>
+      </c>
+      <c r="E10" s="331" t="inlineStr">
+        <is>
+          <t>TORNEIRAS</t>
+        </is>
+      </c>
+      <c r="F10" s="333" t="inlineStr">
+        <is>
+          <t>O36</t>
+        </is>
+      </c>
+      <c r="G10" s="334" t="inlineStr">
+        <is>
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
+        </is>
+      </c>
+      <c r="H10" s="331" t="inlineStr"/>
+    </row>
+    <row r="11" ht="57" customHeight="1">
+      <c r="A11" s="331" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="331" t="inlineStr">
+        <is>
+          <t>APTO TIPO</t>
+        </is>
+      </c>
+      <c r="C11" s="332" t="inlineStr">
+        <is>
+          <t>SALA / VARANDA DA SALA</t>
+        </is>
+      </c>
+      <c r="D11" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E11" s="331" t="inlineStr">
+        <is>
+          <t>RODAPÉ</t>
+        </is>
+      </c>
+      <c r="F11" s="333" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="G11" s="334" t="inlineStr">
+        <is>
+          <t>Rodapé em mármore travertino romano bruto, semi-embutido, h=15cm. (DET PR001/PR002)
+CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+        </is>
+      </c>
+      <c r="H11" s="331" t="inlineStr"/>
+    </row>
+    <row r="12" ht="57" customHeight="1">
+      <c r="A12" s="331" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="331" t="inlineStr">
+        <is>
+          <t>APTO TIPO</t>
+        </is>
+      </c>
+      <c r="C12" s="332" t="inlineStr">
+        <is>
+          <t>LAVABO</t>
+        </is>
+      </c>
+      <c r="D12" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E12" s="331" t="inlineStr">
+        <is>
+          <t>RODAPÉ</t>
+        </is>
+      </c>
+      <c r="F12" s="333" t="inlineStr">
+        <is>
+          <t>F14</t>
+        </is>
+      </c>
+      <c r="G12" s="334" t="inlineStr">
+        <is>
+          <t>Rodapé semi-embutido em mármore travertino romano bruto, h=15cm. (DET PR004)
+CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+        </is>
+      </c>
+      <c r="H12" s="331" t="inlineStr"/>
+    </row>
+    <row r="13" ht="117" customHeight="1">
+      <c r="A13" s="331" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="331" t="inlineStr">
+        <is>
+          <t>APTO TIPO</t>
+        </is>
+      </c>
+      <c r="C13" s="332" t="inlineStr">
+        <is>
+          <t>BANHO SUÍTE MASTER</t>
+        </is>
+      </c>
+      <c r="D13" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E13" s="331" t="inlineStr">
+        <is>
+          <t>PAREDE/REJUNTE</t>
+        </is>
+      </c>
+      <c r="F13" s="333" t="inlineStr">
+        <is>
+          <t>H15</t>
+        </is>
+      </c>
+      <c r="G13" s="334" t="inlineStr">
+        <is>
+          <t>14 - Parede revestida em mármore travertino romano resinado. Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (PR408)
+1 - Parede em alvenaria emassada e regularizada, pintada com tinta acrílica cor branco neve, acabamento acetinado. Ref.: Suvinil. (PR408)
+CONFLITO – Tabela R01: parede em mármore travertino romano BRUTO paginado</t>
+        </is>
+      </c>
+      <c r="H13" s="331" t="inlineStr"/>
+    </row>
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="331" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="331" t="inlineStr">
+        <is>
+          <t>APTO TIPO</t>
+        </is>
+      </c>
+      <c r="C14" s="332" t="inlineStr">
+        <is>
+          <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
+        </is>
+      </c>
+      <c r="D14" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E14" s="331" t="inlineStr">
+        <is>
+          <t>RODAPÉ</t>
+        </is>
+      </c>
+      <c r="F14" s="333" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="G14" s="334" t="inlineStr">
+        <is>
+          <t>Rodapé maciço com o mesmo acabamento do piso, h=10cm. Ref.: Indusparquet. (Tab. R01; quadro do DET PR001)
+CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
+        </is>
+      </c>
+      <c r="H14" s="331" t="inlineStr"/>
+    </row>
+    <row r="15" ht="57" customHeight="1">
+      <c r="A15" s="331" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="331" t="inlineStr">
+        <is>
+          <t>APTO TIPO</t>
+        </is>
+      </c>
+      <c r="C15" s="332" t="inlineStr">
+        <is>
+          <t>COPA NOTURNA</t>
+        </is>
+      </c>
+      <c r="D15" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E15" s="331" t="inlineStr">
+        <is>
+          <t>BANCADA</t>
+        </is>
+      </c>
+      <c r="F15" s="333" t="inlineStr">
+        <is>
+          <t>J18</t>
+        </is>
+      </c>
+      <c r="G15" s="334" t="inlineStr">
+        <is>
+          <t>Bancada esculpida em mármore travertino romano resinado. (DET PR003)
+CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
+        </is>
+      </c>
+      <c r="H15" s="331" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="F5" location="'TÉRREO '!B17" tooltip="Ir para TÉRREO B17"/>
+    <hyperlink ref="F6" location="'TÉRREO '!H17" tooltip="Ir para TÉRREO H17"/>
+    <hyperlink ref="F7" location="'PILOTIS'!J35" tooltip="Ir para PILOTIS J35"/>
+    <hyperlink ref="F8" location="'PILOTIS'!O35" tooltip="Ir para PILOTIS O35"/>
+    <hyperlink ref="F9" location="'PILOTIS'!J36" tooltip="Ir para PILOTIS J36"/>
+    <hyperlink ref="F10" location="'PILOTIS'!O36" tooltip="Ir para PILOTIS O36"/>
+    <hyperlink ref="F11" location="'APTO TIPO'!F13" tooltip="Ir para APTO TIPO F13"/>
+    <hyperlink ref="F12" location="'APTO TIPO'!F14" tooltip="Ir para APTO TIPO F14"/>
+    <hyperlink ref="F13" location="'APTO TIPO'!H15" tooltip="Ir para APTO TIPO H15"/>
+    <hyperlink ref="F14" location="'APTO TIPO'!F17" tooltip="Ir para APTO TIPO F17"/>
+    <hyperlink ref="F15" location="'APTO TIPO'!J18" tooltip="Ir para APTO TIPO J18"/>
+  </hyperlinks>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E544"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Grade R00: conflito só entre arquitetura e detalhamento; detalhamento prevalece sobre a Tabela R01
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -12171,10 +12171,10 @@
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J35" s="321" t="inlineStr">
+      <c r="J35" s="320" t="inlineStr">
         <is>
           <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
+OBS. – As pranchas 37 e 38 do detalhamento R04 indicam bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível (ver PENDÊNCIAS).</t>
         </is>
       </c>
       <c r="K35" s="317" t="inlineStr">
@@ -12185,10 +12185,10 @@
       <c r="L35" s="307" t="n"/>
       <c r="M35" s="308" t="n"/>
       <c r="N35" s="308" t="n"/>
-      <c r="O35" s="321" t="inlineStr">
+      <c r="O35" s="320" t="inlineStr">
         <is>
           <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
+OBS. – As pranchas 37 e 38 do detalhamento R04 indicam torneira de mesa bica baixa Argon, Docol (ver PENDÊNCIAS).</t>
         </is>
       </c>
       <c r="P35" s="320" t="inlineStr">
@@ -12266,10 +12266,10 @@
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J36" s="321" t="inlineStr">
+      <c r="J36" s="320" t="inlineStr">
         <is>
           <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
+OBS. – As pranchas 37 e 38 do detalhamento R04 indicam bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível (ver PENDÊNCIAS).</t>
         </is>
       </c>
       <c r="K36" s="317" t="inlineStr">
@@ -12280,10 +12280,10 @@
       <c r="L36" s="307" t="n"/>
       <c r="M36" s="308" t="n"/>
       <c r="N36" s="308" t="n"/>
-      <c r="O36" s="321" t="inlineStr">
+      <c r="O36" s="320" t="inlineStr">
         <is>
           <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
+OBS. – As pranchas 37 e 38 do detalhamento R04 indicam torneira de mesa bica baixa Argon, Docol (ver PENDÊNCIAS).</t>
         </is>
       </c>
       <c r="P36" s="320" t="inlineStr">
@@ -14693,7 +14693,7 @@
       <c r="Y12" s="241" t="n"/>
       <c r="Z12" s="242" t="n"/>
     </row>
-    <row r="13" ht="89" customHeight="1">
+    <row r="13" ht="74" customHeight="1">
       <c r="A13" s="298" t="inlineStr">
         <is>
           <t>SALA / VARANDA DA SALA</t>
@@ -14707,10 +14707,9 @@
       <c r="C13" s="300" t="n"/>
       <c r="D13" s="300" t="n"/>
       <c r="E13" s="300" t="n"/>
-      <c r="F13" s="304" t="inlineStr">
-        <is>
-          <t>Rodapé em mármore travertino romano bruto, semi-embutido, h=15cm. (DET PR001/PR002)
-CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+      <c r="F13" s="317" t="inlineStr">
+        <is>
+          <t>Rodapé em mármore travertino romano bruto, semi-embutido, h=15cm. (DET PR001/PR002)</t>
         </is>
       </c>
       <c r="G13" s="300" t="n"/>
@@ -14764,10 +14763,9 @@
       </c>
       <c r="D14" s="300" t="n"/>
       <c r="E14" s="300" t="n"/>
-      <c r="F14" s="304" t="inlineStr">
-        <is>
-          <t>Rodapé semi-embutido em mármore travertino romano bruto, h=15cm. (DET PR004)
-CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+      <c r="F14" s="317" t="inlineStr">
+        <is>
+          <t>Rodapé semi-embutido em mármore travertino romano bruto, h=15cm. (DET PR004)</t>
         </is>
       </c>
       <c r="G14" s="300" t="n"/>
@@ -14828,7 +14826,7 @@
       <c r="Y14" s="302" t="n"/>
       <c r="Z14" s="300" t="n"/>
     </row>
-    <row r="15" ht="119" customHeight="1">
+    <row r="15" ht="104" customHeight="1">
       <c r="A15" s="298" t="inlineStr">
         <is>
           <t>BANHO SUÍTE MASTER</t>
@@ -14852,11 +14850,10 @@
         </is>
       </c>
       <c r="G15" s="300" t="n"/>
-      <c r="H15" s="304" t="inlineStr">
+      <c r="H15" s="317" t="inlineStr">
         <is>
           <t>14 - Parede revestida em mármore travertino romano resinado. Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (PR408)
-1 - Parede em alvenaria emassada e regularizada, pintada com tinta acrílica cor branco neve, acabamento acetinado. Ref.: Suvinil. (PR408)
-CONFLITO – Tabela R01: parede em mármore travertino romano BRUTO paginado</t>
+1 - Parede em alvenaria emassada e regularizada, pintada com tinta acrílica cor branco neve, acabamento acetinado. Ref.: Suvinil. (PR408)</t>
         </is>
       </c>
       <c r="I15" s="308" t="inlineStr">
@@ -15026,10 +15023,10 @@
         </is>
       </c>
       <c r="E17" s="300" t="n"/>
-      <c r="F17" s="304" t="inlineStr">
+      <c r="F17" s="317" t="inlineStr">
         <is>
           <t>Rodapé maciço com o mesmo acabamento do piso, h=10cm. Ref.: Indusparquet. (Tab. R01; quadro do DET PR001)
-CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
+OBS. – A legenda de rodapé do DET PR001/PR002 indica h=6,5cm (ver PENDÊNCIAS).</t>
         </is>
       </c>
       <c r="G17" s="300" t="n"/>
@@ -15057,7 +15054,7 @@
       <c r="Y17" s="302" t="n"/>
       <c r="Z17" s="300" t="n"/>
     </row>
-    <row r="18" ht="89" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="298" t="inlineStr">
         <is>
           <t>COPA NOTURNA</t>
@@ -15079,10 +15076,9 @@
       <c r="G18" s="300" t="n"/>
       <c r="H18" s="308" t="n"/>
       <c r="I18" s="308" t="n"/>
-      <c r="J18" s="304" t="inlineStr">
-        <is>
-          <t>Bancada esculpida em mármore travertino romano resinado. (DET PR003)
-CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
+      <c r="J18" s="317" t="inlineStr">
+        <is>
+          <t>Bancada esculpida em mármore travertino romano resinado. (DET PR003)</t>
         </is>
       </c>
       <c r="K18" s="300" t="n"/>
@@ -15767,7 +15763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15911,340 +15907,6 @@
       </c>
       <c r="H6" s="331" t="inlineStr"/>
     </row>
-    <row r="7" ht="102" customHeight="1">
-      <c r="A7" s="331" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="331" t="inlineStr">
-        <is>
-          <t>PILOTIS</t>
-        </is>
-      </c>
-      <c r="C7" s="332" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEMININO</t>
-        </is>
-      </c>
-      <c r="D7" s="331" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="E7" s="331" t="inlineStr">
-        <is>
-          <t>BANCADA</t>
-        </is>
-      </c>
-      <c r="F7" s="333" t="inlineStr">
-        <is>
-          <t>J35</t>
-        </is>
-      </c>
-      <c r="G7" s="334" t="inlineStr">
-        <is>
-          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
-        </is>
-      </c>
-      <c r="H7" s="331" t="inlineStr"/>
-    </row>
-    <row r="8" ht="87" customHeight="1">
-      <c r="A8" s="331" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="331" t="inlineStr">
-        <is>
-          <t>PILOTIS</t>
-        </is>
-      </c>
-      <c r="C8" s="332" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO FEMININO</t>
-        </is>
-      </c>
-      <c r="D8" s="331" t="inlineStr">
-        <is>
-          <t>LOUÇAS E METAIS</t>
-        </is>
-      </c>
-      <c r="E8" s="331" t="inlineStr">
-        <is>
-          <t>TORNEIRAS</t>
-        </is>
-      </c>
-      <c r="F8" s="333" t="inlineStr">
-        <is>
-          <t>O35</t>
-        </is>
-      </c>
-      <c r="G8" s="334" t="inlineStr">
-        <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
-        </is>
-      </c>
-      <c r="H8" s="331" t="inlineStr"/>
-    </row>
-    <row r="9" ht="102" customHeight="1">
-      <c r="A9" s="331" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="331" t="inlineStr">
-        <is>
-          <t>PILOTIS</t>
-        </is>
-      </c>
-      <c r="C9" s="332" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO MASCULINO</t>
-        </is>
-      </c>
-      <c r="D9" s="331" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="E9" s="331" t="inlineStr">
-        <is>
-          <t>BANCADA</t>
-        </is>
-      </c>
-      <c r="F9" s="333" t="inlineStr">
-        <is>
-          <t>J36</t>
-        </is>
-      </c>
-      <c r="G9" s="334" t="inlineStr">
-        <is>
-          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
-        </is>
-      </c>
-      <c r="H9" s="331" t="inlineStr"/>
-    </row>
-    <row r="10" ht="87" customHeight="1">
-      <c r="A10" s="331" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="331" t="inlineStr">
-        <is>
-          <t>PILOTIS</t>
-        </is>
-      </c>
-      <c r="C10" s="332" t="inlineStr">
-        <is>
-          <t>VESTIÁRIO MASCULINO</t>
-        </is>
-      </c>
-      <c r="D10" s="331" t="inlineStr">
-        <is>
-          <t>LOUÇAS E METAIS</t>
-        </is>
-      </c>
-      <c r="E10" s="331" t="inlineStr">
-        <is>
-          <t>TORNEIRAS</t>
-        </is>
-      </c>
-      <c r="F10" s="333" t="inlineStr">
-        <is>
-          <t>O36</t>
-        </is>
-      </c>
-      <c r="G10" s="334" t="inlineStr">
-        <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
-        </is>
-      </c>
-      <c r="H10" s="331" t="inlineStr"/>
-    </row>
-    <row r="11" ht="57" customHeight="1">
-      <c r="A11" s="331" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="331" t="inlineStr">
-        <is>
-          <t>APTO TIPO</t>
-        </is>
-      </c>
-      <c r="C11" s="332" t="inlineStr">
-        <is>
-          <t>SALA / VARANDA DA SALA</t>
-        </is>
-      </c>
-      <c r="D11" s="331" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="E11" s="331" t="inlineStr">
-        <is>
-          <t>RODAPÉ</t>
-        </is>
-      </c>
-      <c r="F11" s="333" t="inlineStr">
-        <is>
-          <t>F13</t>
-        </is>
-      </c>
-      <c r="G11" s="334" t="inlineStr">
-        <is>
-          <t>Rodapé em mármore travertino romano bruto, semi-embutido, h=15cm. (DET PR001/PR002)
-CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
-        </is>
-      </c>
-      <c r="H11" s="331" t="inlineStr"/>
-    </row>
-    <row r="12" ht="57" customHeight="1">
-      <c r="A12" s="331" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="331" t="inlineStr">
-        <is>
-          <t>APTO TIPO</t>
-        </is>
-      </c>
-      <c r="C12" s="332" t="inlineStr">
-        <is>
-          <t>LAVABO</t>
-        </is>
-      </c>
-      <c r="D12" s="331" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="E12" s="331" t="inlineStr">
-        <is>
-          <t>RODAPÉ</t>
-        </is>
-      </c>
-      <c r="F12" s="333" t="inlineStr">
-        <is>
-          <t>F14</t>
-        </is>
-      </c>
-      <c r="G12" s="334" t="inlineStr">
-        <is>
-          <t>Rodapé semi-embutido em mármore travertino romano bruto, h=15cm. (DET PR004)
-CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
-        </is>
-      </c>
-      <c r="H12" s="331" t="inlineStr"/>
-    </row>
-    <row r="13" ht="117" customHeight="1">
-      <c r="A13" s="331" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="331" t="inlineStr">
-        <is>
-          <t>APTO TIPO</t>
-        </is>
-      </c>
-      <c r="C13" s="332" t="inlineStr">
-        <is>
-          <t>BANHO SUÍTE MASTER</t>
-        </is>
-      </c>
-      <c r="D13" s="331" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="E13" s="331" t="inlineStr">
-        <is>
-          <t>PAREDE/REJUNTE</t>
-        </is>
-      </c>
-      <c r="F13" s="333" t="inlineStr">
-        <is>
-          <t>H15</t>
-        </is>
-      </c>
-      <c r="G13" s="334" t="inlineStr">
-        <is>
-          <t>14 - Parede revestida em mármore travertino romano resinado. Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (PR408)
-1 - Parede em alvenaria emassada e regularizada, pintada com tinta acrílica cor branco neve, acabamento acetinado. Ref.: Suvinil. (PR408)
-CONFLITO – Tabela R01: parede em mármore travertino romano BRUTO paginado</t>
-        </is>
-      </c>
-      <c r="H13" s="331" t="inlineStr"/>
-    </row>
-    <row r="14" ht="72" customHeight="1">
-      <c r="A14" s="331" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="331" t="inlineStr">
-        <is>
-          <t>APTO TIPO</t>
-        </is>
-      </c>
-      <c r="C14" s="332" t="inlineStr">
-        <is>
-          <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
-        </is>
-      </c>
-      <c r="D14" s="331" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="E14" s="331" t="inlineStr">
-        <is>
-          <t>RODAPÉ</t>
-        </is>
-      </c>
-      <c r="F14" s="333" t="inlineStr">
-        <is>
-          <t>F17</t>
-        </is>
-      </c>
-      <c r="G14" s="334" t="inlineStr">
-        <is>
-          <t>Rodapé maciço com o mesmo acabamento do piso, h=10cm. Ref.: Indusparquet. (Tab. R01; quadro do DET PR001)
-CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
-        </is>
-      </c>
-      <c r="H14" s="331" t="inlineStr"/>
-    </row>
-    <row r="15" ht="57" customHeight="1">
-      <c r="A15" s="331" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="331" t="inlineStr">
-        <is>
-          <t>APTO TIPO</t>
-        </is>
-      </c>
-      <c r="C15" s="332" t="inlineStr">
-        <is>
-          <t>COPA NOTURNA</t>
-        </is>
-      </c>
-      <c r="D15" s="331" t="inlineStr">
-        <is>
-          <t>REVESTIMENTOS</t>
-        </is>
-      </c>
-      <c r="E15" s="331" t="inlineStr">
-        <is>
-          <t>BANCADA</t>
-        </is>
-      </c>
-      <c r="F15" s="333" t="inlineStr">
-        <is>
-          <t>J18</t>
-        </is>
-      </c>
-      <c r="G15" s="334" t="inlineStr">
-        <is>
-          <t>Bancada esculpida em mármore travertino romano resinado. (DET PR003)
-CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
-        </is>
-      </c>
-      <c r="H15" s="331" t="inlineStr"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -16253,15 +15915,6 @@
   <hyperlinks>
     <hyperlink ref="F5" location="'TÉRREO '!B17" tooltip="Ir para TÉRREO B17"/>
     <hyperlink ref="F6" location="'TÉRREO '!H17" tooltip="Ir para TÉRREO H17"/>
-    <hyperlink ref="F7" location="'PILOTIS'!J35" tooltip="Ir para PILOTIS J35"/>
-    <hyperlink ref="F8" location="'PILOTIS'!O35" tooltip="Ir para PILOTIS O35"/>
-    <hyperlink ref="F9" location="'PILOTIS'!J36" tooltip="Ir para PILOTIS J36"/>
-    <hyperlink ref="F10" location="'PILOTIS'!O36" tooltip="Ir para PILOTIS O36"/>
-    <hyperlink ref="F11" location="'APTO TIPO'!F13" tooltip="Ir para APTO TIPO F13"/>
-    <hyperlink ref="F12" location="'APTO TIPO'!F14" tooltip="Ir para APTO TIPO F14"/>
-    <hyperlink ref="F13" location="'APTO TIPO'!H15" tooltip="Ir para APTO TIPO H15"/>
-    <hyperlink ref="F14" location="'APTO TIPO'!F17" tooltip="Ir para APTO TIPO F17"/>
-    <hyperlink ref="F15" location="'APTO TIPO'!J18" tooltip="Ir para APTO TIPO J18"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
@@ -23398,7 +23051,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Pranchas 37 e 38 citam torneira Argon (Docol) e bancada em granito Branco Siena; a lista R04 traz D29 (Decalux, Deca) e D36 (granito cinza Santa Rosa). Confirmar com a arquitetura.</t>
+          <t>Divergência interna do detalhamento R04: as pranchas 37 e 38 citam torneira Argon (Docol) e bancada em granito Branco Siena com duas cubas esculpidas; a lista R04 traz D29 (Decalux, Deca) e D36 (granito cinza Santa Rosa). Mantida a lista na grade, com OBS. Confirmar.</t>
         </is>
       </c>
     </row>
@@ -28474,7 +28127,7 @@
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>RODAPÉ: CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+          <t>RODAPÉ: Tabela R01 divergente (prevalece o detalhamento): rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
         </is>
       </c>
     </row>
@@ -28486,7 +28139,7 @@
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>RODAPÉ: CONFLITO – Tabela R01: rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
+          <t>RODAPÉ: Tabela R01 divergente (prevalece o detalhamento): rodapé DE SOBREPOR em mármore travertino romano bruto, h=15cm</t>
         </is>
       </c>
     </row>
@@ -28498,7 +28151,7 @@
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>PAREDE/REJUNTE: CONFLITO – Tabela R01: parede em mármore travertino romano BRUTO paginado</t>
+          <t>PAREDE/REJUNTE: Tabela R01 divergente (prevalece o detalhamento): parede em mármore travertino romano BRUTO paginado</t>
         </is>
       </c>
     </row>
@@ -28510,7 +28163,7 @@
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>RODAPÉ: CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm</t>
+          <t>RODAPÉ: divergência interna do detalhamento. O quadro do DET PR001 (e a Tabela R01) indicam h=10cm; a legenda de rodapé do DET PR001/PR002 indica h=6,5cm. Mantido h=10cm na grade. Confirmar.</t>
         </is>
       </c>
     </row>
@@ -28522,7 +28175,7 @@
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>BANCADA: CONFLITO – Tabela R01: bancada "pintura acrílica, cor branco neve"</t>
+          <t>BANCADA: Tabela R01 divergente (prevalece o detalhamento): bancada "pintura acrílica, cor branco neve"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grade R00: divergência entre prancha e tabela da própria prancha também é conflito
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -1492,7 +1492,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="335">
+  <cellXfs count="336">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -2401,6 +2401,9 @@
     </xf>
     <xf numFmtId="0" fontId="73" fillId="14" borderId="73" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="67" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -7566,9 +7569,10 @@
           <t>ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
       </c>
-      <c r="I30" s="307" t="inlineStr">
-        <is>
-          <t>ARQ-T19 - código não existe no quadro de tetos (01 a 06); conferir na planta</t>
+      <c r="I30" s="321" t="inlineStr">
+        <is>
+          <t>ARQ-T19 - código indicado na etiqueta de teto da planta PR003.
+CONFLITO – Quadro de tetos da própria PR003: só traz os códigos 01 a 06; o T19 não existe no quadro.</t>
         </is>
       </c>
       <c r="J30" s="307" t="n"/>
@@ -12171,10 +12175,10 @@
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J35" s="320" t="inlineStr">
+      <c r="J35" s="321" t="inlineStr">
         <is>
           <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-OBS. – As pranchas 37 e 38 do detalhamento R04 indicam bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível (ver PENDÊNCIAS).</t>
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
         </is>
       </c>
       <c r="K35" s="317" t="inlineStr">
@@ -12185,10 +12189,10 @@
       <c r="L35" s="307" t="n"/>
       <c r="M35" s="308" t="n"/>
       <c r="N35" s="308" t="n"/>
-      <c r="O35" s="320" t="inlineStr">
+      <c r="O35" s="321" t="inlineStr">
         <is>
           <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-OBS. – As pranchas 37 e 38 do detalhamento R04 indicam torneira de mesa bica baixa Argon, Docol (ver PENDÊNCIAS).</t>
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
       <c r="P35" s="320" t="inlineStr">
@@ -12266,10 +12270,10 @@
           <t>T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
-      <c r="J36" s="320" t="inlineStr">
+      <c r="J36" s="321" t="inlineStr">
         <is>
           <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-OBS. – As pranchas 37 e 38 do detalhamento R04 indicam bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível (ver PENDÊNCIAS).</t>
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
         </is>
       </c>
       <c r="K36" s="317" t="inlineStr">
@@ -12280,10 +12284,10 @@
       <c r="L36" s="307" t="n"/>
       <c r="M36" s="308" t="n"/>
       <c r="N36" s="308" t="n"/>
-      <c r="O36" s="320" t="inlineStr">
+      <c r="O36" s="321" t="inlineStr">
         <is>
           <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-OBS. – As pranchas 37 e 38 do detalhamento R04 indicam torneira de mesa bica baixa Argon, Docol (ver PENDÊNCIAS).</t>
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
       <c r="P36" s="320" t="inlineStr">
@@ -15023,10 +15027,10 @@
         </is>
       </c>
       <c r="E17" s="300" t="n"/>
-      <c r="F17" s="317" t="inlineStr">
+      <c r="F17" s="335" t="inlineStr">
         <is>
           <t>Rodapé maciço com o mesmo acabamento do piso, h=10cm. Ref.: Indusparquet. (Tab. R01; quadro do DET PR001)
-OBS. – A legenda de rodapé do DET PR001/PR002 indica h=6,5cm (ver PENDÊNCIAS).</t>
+CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm (o quadro da mesma prancha indica h=10cm)</t>
         </is>
       </c>
       <c r="G17" s="300" t="n"/>
@@ -15763,7 +15767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15907,6 +15911,228 @@
       </c>
       <c r="H6" s="331" t="inlineStr"/>
     </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="331" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="331" t="inlineStr">
+        <is>
+          <t>TÉRREO</t>
+        </is>
+      </c>
+      <c r="C7" s="332" t="inlineStr">
+        <is>
+          <t>CONCIERGE</t>
+        </is>
+      </c>
+      <c r="D7" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E7" s="331" t="inlineStr">
+        <is>
+          <t>TETO</t>
+        </is>
+      </c>
+      <c r="F7" s="333" t="inlineStr">
+        <is>
+          <t>I30</t>
+        </is>
+      </c>
+      <c r="G7" s="334" t="inlineStr">
+        <is>
+          <t>ARQ-T19 - código indicado na etiqueta de teto da planta PR003.
+CONFLITO – Quadro de tetos da própria PR003: só traz os códigos 01 a 06; o T19 não existe no quadro.</t>
+        </is>
+      </c>
+      <c r="H7" s="331" t="inlineStr"/>
+    </row>
+    <row r="8" ht="102" customHeight="1">
+      <c r="A8" s="331" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C8" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO FEMININO</t>
+        </is>
+      </c>
+      <c r="D8" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E8" s="331" t="inlineStr">
+        <is>
+          <t>BANCADA</t>
+        </is>
+      </c>
+      <c r="F8" s="333" t="inlineStr">
+        <is>
+          <t>J35</t>
+        </is>
+      </c>
+      <c r="G8" s="334" t="inlineStr">
+        <is>
+          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
+        </is>
+      </c>
+      <c r="H8" s="331" t="inlineStr"/>
+    </row>
+    <row r="9" ht="87" customHeight="1">
+      <c r="A9" s="331" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C9" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO FEMININO</t>
+        </is>
+      </c>
+      <c r="D9" s="331" t="inlineStr">
+        <is>
+          <t>LOUÇAS E METAIS</t>
+        </is>
+      </c>
+      <c r="E9" s="331" t="inlineStr">
+        <is>
+          <t>TORNEIRAS</t>
+        </is>
+      </c>
+      <c r="F9" s="333" t="inlineStr">
+        <is>
+          <t>O35</t>
+        </is>
+      </c>
+      <c r="G9" s="334" t="inlineStr">
+        <is>
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
+        </is>
+      </c>
+      <c r="H9" s="331" t="inlineStr"/>
+    </row>
+    <row r="10" ht="102" customHeight="1">
+      <c r="A10" s="331" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C10" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO MASCULINO</t>
+        </is>
+      </c>
+      <c r="D10" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E10" s="331" t="inlineStr">
+        <is>
+          <t>BANCADA</t>
+        </is>
+      </c>
+      <c r="F10" s="333" t="inlineStr">
+        <is>
+          <t>J36</t>
+        </is>
+      </c>
+      <c r="G10" s="334" t="inlineStr">
+        <is>
+          <t>D36 - Bancada e cubas esculpidas em granito cinza Santa Rosa, acabamento escovado. Desenho e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: bancada em granito Branco Siena com duas cubas esculpidas com bandeja removível</t>
+        </is>
+      </c>
+      <c r="H10" s="331" t="inlineStr"/>
+    </row>
+    <row r="11" ht="87" customHeight="1">
+      <c r="A11" s="331" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="331" t="inlineStr">
+        <is>
+          <t>PILOTIS</t>
+        </is>
+      </c>
+      <c r="C11" s="332" t="inlineStr">
+        <is>
+          <t>VESTIÁRIO MASCULINO</t>
+        </is>
+      </c>
+      <c r="D11" s="331" t="inlineStr">
+        <is>
+          <t>LOUÇAS E METAIS</t>
+        </is>
+      </c>
+      <c r="E11" s="331" t="inlineStr">
+        <is>
+          <t>TORNEIRAS</t>
+        </is>
+      </c>
+      <c r="F11" s="333" t="inlineStr">
+        <is>
+          <t>O36</t>
+        </is>
+      </c>
+      <c r="G11" s="334" t="inlineStr">
+        <is>
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
+        </is>
+      </c>
+      <c r="H11" s="331" t="inlineStr"/>
+    </row>
+    <row r="12" ht="87" customHeight="1">
+      <c r="A12" s="331" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="331" t="inlineStr">
+        <is>
+          <t>APTO TIPO</t>
+        </is>
+      </c>
+      <c r="C12" s="332" t="inlineStr">
+        <is>
+          <t>SUÍTES / QUARTOS / CIRCULAÇÃO / CLOSET / ESTAR ÍNTIMO</t>
+        </is>
+      </c>
+      <c r="D12" s="331" t="inlineStr">
+        <is>
+          <t>REVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="E12" s="331" t="inlineStr">
+        <is>
+          <t>RODAPÉ</t>
+        </is>
+      </c>
+      <c r="F12" s="333" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="G12" s="334" t="inlineStr">
+        <is>
+          <t>Rodapé maciço com o mesmo acabamento do piso, h=10cm. Ref.: Indusparquet. (Tab. R01; quadro do DET PR001)
+CONFLITO – Legenda de rodapé do DET PR001/PR002: h=6,5cm (o quadro da mesma prancha indica h=10cm)</t>
+        </is>
+      </c>
+      <c r="H12" s="331" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -15915,6 +16141,12 @@
   <hyperlinks>
     <hyperlink ref="F5" location="'TÉRREO '!B17" tooltip="Ir para TÉRREO B17"/>
     <hyperlink ref="F6" location="'TÉRREO '!H17" tooltip="Ir para TÉRREO H17"/>
+    <hyperlink ref="F7" location="'TÉRREO '!I30" tooltip="Ir para TÉRREO I30"/>
+    <hyperlink ref="F8" location="'PILOTIS'!J35" tooltip="Ir para PILOTIS J35"/>
+    <hyperlink ref="F9" location="'PILOTIS'!O35" tooltip="Ir para PILOTIS O35"/>
+    <hyperlink ref="F10" location="'PILOTIS'!J36" tooltip="Ir para PILOTIS J36"/>
+    <hyperlink ref="F11" location="'PILOTIS'!O36" tooltip="Ir para PILOTIS O36"/>
+    <hyperlink ref="F12" location="'APTO TIPO'!F17" tooltip="Ir para APTO TIPO F17"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
@@ -23051,7 +23283,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Divergência interna do detalhamento R04: as pranchas 37 e 38 citam torneira Argon (Docol) e bancada em granito Branco Siena com duas cubas esculpidas; a lista R04 traz D29 (Decalux, Deca) e D36 (granito cinza Santa Rosa). Mantida a lista na grade, com OBS. Confirmar.</t>
+          <t>CONFLITO no detalhamento R04 (ver aba CONFLITOS): as pranchas 37 e 38 citam torneira Argon (Docol) e bancada em granito Branco Siena com duas cubas esculpidas; a lista R04 traz D29 (Decalux, Deca) e D36 (granito cinza Santa Rosa).</t>
         </is>
       </c>
     </row>
@@ -28059,7 +28291,7 @@
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>A etiqueta de teto da planta PR003 traz □19, mas o quadro de tetos só vai de 01 a 06. Provável erro de etiqueta; confirmar com a arquitetura.</t>
+          <t>CONFLITO na própria planta (ver aba CONFLITOS): a etiqueta de teto da PR003 traz □19, mas o quadro de tetos da prancha só vai de 01 a 06. Confirmar com a arquitetura.</t>
         </is>
       </c>
     </row>
@@ -28163,7 +28395,7 @@
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>RODAPÉ: divergência interna do detalhamento. O quadro do DET PR001 (e a Tabela R01) indicam h=10cm; a legenda de rodapé do DET PR001/PR002 indica h=6,5cm. Mantido h=10cm na grade. Confirmar.</t>
+          <t>RODAPÉ: CONFLITO na própria prancha (ver aba CONFLITOS). O quadro do DET PR001 indica h=10cm; a legenda de rodapé do DET PR001/PR002 indica h=6,5cm.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grade R00: piso do Terraço do Salão de Festas pela planta PR011 (ARQ-P08)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -11045,13 +11045,17 @@
       <c r="Y14" s="302" t="n"/>
       <c r="Z14" s="300" t="n"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="119" customHeight="1">
       <c r="A15" s="298" t="inlineStr">
         <is>
           <t>TERRAÇO SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="B15" s="302" t="n"/>
+      <c r="B15" s="302" t="inlineStr">
+        <is>
+          <t>ARQ-P08 - Piso elevado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material. (Planta PR011)</t>
+        </is>
+      </c>
       <c r="C15" s="300" t="n"/>
       <c r="D15" s="300" t="n"/>
       <c r="E15" s="300" t="n"/>
@@ -16686,7 +16690,11 @@
         </is>
       </c>
       <c r="C27" s="268" t="inlineStr"/>
-      <c r="D27" s="268" t="inlineStr"/>
+      <c r="D27" s="268" t="inlineStr">
+        <is>
+          <t>Tabela v00 e detalhamento R04 sem especificação de acabamento (a lista R04 só traz códigos sem descrição para "Varanda, terraço, piscina e prainha, braseiro"). A planta de arquitetura PR011 indica piso ○08 (ARQ-P08, lançado na grade) e guarda-corpos GC06/GC07 h=130cm. Sem indicação de rodapé, parede ou teto.</t>
+        </is>
+      </c>
       <c r="E27" s="268" t="inlineStr"/>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Grade R00: conferência visual de todas as etiquetas das plantas de arquitetura
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AF55"/>
+  <dimension ref="A1:AF56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="24"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6761,13 +6761,17 @@
       <c r="Y14" s="295" t="n"/>
       <c r="Z14" s="296" t="n"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="89" customHeight="1">
       <c r="A15" s="294" t="inlineStr">
         <is>
           <t xml:space="preserve">RAMPA ACESSO PEDESTRES </t>
         </is>
       </c>
-      <c r="B15" s="295" t="n"/>
+      <c r="B15" s="295" t="inlineStr">
+        <is>
+          <t>ARQ-P21 - Piso em granito marrom absoluto serrado e envernizado, ou pedra sintética a definir. Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (Planta PR003: plano inclinado - pedestres (social), i=4,99%)</t>
+        </is>
+      </c>
       <c r="C15" s="296" t="n"/>
       <c r="D15" s="296" t="n"/>
       <c r="E15" s="296" t="n"/>
@@ -8669,8 +8673,77 @@
       <c r="Y54" s="307" t="n"/>
       <c r="Z54" s="300" t="n"/>
     </row>
-    <row r="55">
-      <c r="S55" s="3" t="n"/>
+    <row r="55" ht="119" customHeight="1">
+      <c r="A55" s="298" t="inlineStr">
+        <is>
+          <t>PLANO INCLINADO - PEDESTRES (SERVIÇO)</t>
+        </is>
+      </c>
+      <c r="B55" s="307" t="inlineStr">
+        <is>
+          <t>ARQ-P07 - Piso assentado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material. (Planta PR003, i=3,83%)</t>
+        </is>
+      </c>
+      <c r="C55" s="300" t="n"/>
+      <c r="D55" s="307" t="n"/>
+      <c r="E55" s="308" t="n"/>
+      <c r="F55" s="308" t="n"/>
+      <c r="G55" s="300" t="n"/>
+      <c r="H55" s="307" t="n"/>
+      <c r="I55" s="307" t="n"/>
+      <c r="J55" s="307" t="n"/>
+      <c r="K55" s="300" t="n"/>
+      <c r="L55" s="307" t="n"/>
+      <c r="M55" s="308" t="n"/>
+      <c r="N55" s="308" t="n"/>
+      <c r="O55" s="307" t="n"/>
+      <c r="P55" s="302" t="n"/>
+      <c r="Q55" s="300" t="n"/>
+      <c r="R55" s="307" t="n"/>
+      <c r="S55" s="307" t="n"/>
+      <c r="T55" s="307" t="n"/>
+      <c r="U55" s="300" t="n"/>
+      <c r="V55" s="302" t="n"/>
+      <c r="W55" s="307" t="n"/>
+      <c r="X55" s="307" t="n"/>
+      <c r="Y55" s="307" t="n"/>
+      <c r="Z55" s="300" t="n"/>
+    </row>
+    <row r="56" ht="119" customHeight="1">
+      <c r="A56" s="298" t="inlineStr">
+        <is>
+          <t>PLANO INCLINADO - VEÍCULOS</t>
+        </is>
+      </c>
+      <c r="B56" s="307" t="inlineStr">
+        <is>
+          <t>ARQ-P07 - Piso assentado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material. (Planta PR003, dois trechos, i=3,50% e 3,28%)</t>
+        </is>
+      </c>
+      <c r="C56" s="300" t="n"/>
+      <c r="D56" s="307" t="n"/>
+      <c r="E56" s="308" t="n"/>
+      <c r="F56" s="308" t="n"/>
+      <c r="G56" s="300" t="n"/>
+      <c r="H56" s="307" t="n"/>
+      <c r="I56" s="307" t="n"/>
+      <c r="J56" s="307" t="n"/>
+      <c r="K56" s="300" t="n"/>
+      <c r="L56" s="307" t="n"/>
+      <c r="M56" s="308" t="n"/>
+      <c r="N56" s="308" t="n"/>
+      <c r="O56" s="307" t="n"/>
+      <c r="P56" s="302" t="n"/>
+      <c r="Q56" s="300" t="n"/>
+      <c r="R56" s="307" t="n"/>
+      <c r="S56" s="307" t="n"/>
+      <c r="T56" s="307" t="n"/>
+      <c r="U56" s="300" t="n"/>
+      <c r="V56" s="302" t="n"/>
+      <c r="W56" s="307" t="n"/>
+      <c r="X56" s="307" t="n"/>
+      <c r="Y56" s="307" t="n"/>
+      <c r="Z56" s="300" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -11828,13 +11901,17 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1">
+    <row r="28" ht="119" customHeight="1">
       <c r="A28" s="298" t="inlineStr">
         <is>
           <t>VARANDA</t>
         </is>
       </c>
-      <c r="B28" s="307" t="n"/>
+      <c r="B28" s="307" t="inlineStr">
+        <is>
+          <t>ARQ-P08 - Piso elevado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material. (Plantas PR011 e PR012)</t>
+        </is>
+      </c>
       <c r="C28" s="300" t="n"/>
       <c r="D28" s="300" t="n"/>
       <c r="E28" s="308" t="n"/>
@@ -16172,7 +16249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E544"/>
+  <dimension ref="A1:E553"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -28335,7 +28412,7 @@
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>Pranchas de revisão anterior (R11 e R13 de 2025) às demais; não foram usadas.</t>
+          <t>Trecho 2 do 2º pavimento e do Pilotis; conferidas em 02/10/2026 (ver item 7).</t>
         </is>
       </c>
     </row>
@@ -28476,6 +28553,98 @@
       <c r="D544" t="inlineStr">
         <is>
           <t>DET indica "validar com o Setor de Produto"; PR001/PR002 "não liberado para execução, paginação poderá sofrer alterações".</t>
+        </is>
+      </c>
+    </row>
+    <row r="545"/>
+    <row r="546">
+      <c r="A546" s="279" t="inlineStr">
+        <is>
+          <t>7. CONFERÊNCIA VISUAL DAS PLANTAS DE ARQUITETURA (02/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Conferência visual</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Todos os ambientes das plantas PR003, PR004, PR005, PR007, PR008, PR009, PR011, PR012 e PR013 foram conferidos no desenho, etiqueta por etiqueta. Os ambientes já lançados estão de acordo com as plantas. Lista completa: levantamento/arquitetura/conferencia_etiquetas_arquitetura.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>PR008 e PR012</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>São o trecho 2 do 2º pavimento e do Pilotis (não revisões antigas, como estava anotado). PR008 só traz a rampa (○04 △07 □03, igual à PR009). PR012 traz a varanda (○08); piscinas, prainha e deck sem etiqueta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>PILOTIS – VARANDA</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Planta indica só piso ○08 (ARQ-P08), lançado na grade. Detalhamento R04 sem especificação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>PILOTIS – CIRCULAÇÕES EXTERNAS</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>As circulações de 40,36 m² (PR011), 59,22 m² e 83,52 m² (PR013) têm só piso ○08 (ARQ-P08), a mesma especificação já lançada em "CIRCULAÇÃO EXTERNA COBERTA/DESCOBERTA E VARANDA ESPAÇO KIDS". Não foi possível ligar cada uma às linhas "CIRCULAÇÃO JARDINS" e "CIRCULAÇÃO PLAYGROUND" pelo nome; confirmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>TÉRREO – PLANOS INCLINADOS</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Plano inclinado de pedestres (social) com ○21, lançado em RAMPA ACESSO PEDESTRES. Plano inclinado de pedestres (serviço) e de veículos com ○07, em linhas novas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>TÉRREO – MUROS</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Triângulo △04 isolado em três pontos do muro junto ao jardim (PR003): parede em textura acrílica fosca Terra Fértil, Suvinil. Não é um ambiente da grade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Sem etiqueta na planta</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Elevadores, escadas, I.S. P.C.D. e vestíbulo (Térreo), DML e jardinagem (Térreo), jardins sobre laje, piscinas, prainha, deck, playground, lounge quadras, saunas, apoio e DML do salão, lobby pilotis e circulações internas do Pilotis. Hall, lobby, antecâmara (eclusa), espaço kids, gourmet, salão, cozinha, I.S., termas, academia, bar e vestiários do Pilotis têm "ACABAMENTOS VER INTERIORES".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grade R00: piso ○08 nas circulações jardins e playground do Pilotis
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -12144,13 +12144,17 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1">
+    <row r="33" ht="119" customHeight="1">
       <c r="A33" s="298" t="inlineStr">
         <is>
           <t>CIRCULAÇÃO PLAYGROUND</t>
         </is>
       </c>
-      <c r="B33" s="307" t="n"/>
+      <c r="B33" s="307" t="inlineStr">
+        <is>
+          <t>ARQ-P08 - Piso elevado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material. (Planta PR013: circulação junto ao playground)</t>
+        </is>
+      </c>
       <c r="C33" s="300" t="n"/>
       <c r="D33" s="307" t="n"/>
       <c r="E33" s="308" t="n"/>
@@ -12484,13 +12488,17 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="60" customHeight="1">
+    <row r="38" ht="134" customHeight="1">
       <c r="A38" s="298" t="inlineStr">
         <is>
           <t xml:space="preserve">CIRCULAÇÃO JARDINS </t>
         </is>
       </c>
-      <c r="B38" s="307" t="n"/>
+      <c r="B38" s="307" t="inlineStr">
+        <is>
+          <t>ARQ-P08 - Piso elevado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material. (Plantas PR011 e PR013: circulações externas junto aos jardins)</t>
+        </is>
+      </c>
       <c r="C38" s="300" t="n"/>
       <c r="D38" s="307" t="n"/>
       <c r="E38" s="308" t="n"/>
@@ -28608,7 +28616,7 @@
       </c>
       <c r="D550" t="inlineStr">
         <is>
-          <t>As circulações de 40,36 m² (PR011), 59,22 m² e 83,52 m² (PR013) têm só piso ○08 (ARQ-P08), a mesma especificação já lançada em "CIRCULAÇÃO EXTERNA COBERTA/DESCOBERTA E VARANDA ESPAÇO KIDS". Não foi possível ligar cada uma às linhas "CIRCULAÇÃO JARDINS" e "CIRCULAÇÃO PLAYGROUND" pelo nome; confirmar.</t>
+          <t>As circulações de 40,36 m² (PR011), 59,22 m² e 83,52 m² (PR013) têm só piso ○08 (ARQ-P08), a mesma especificação já lançada em "CIRCULAÇÃO EXTERNA COBERTA/DESCOBERTA E VARANDA ESPAÇO KIDS". Lançadas como dois ambientes, "CIRCULAÇÃO JARDINS" e "CIRCULAÇÃO PLAYGROUND", conforme orientação de 02/10/2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grade R00: revisão geral (textos, sumário, controle de revisões e pendências atualizados)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCbvFHcTrLz8qJPTsXqWqD
</commit_message>
<xml_diff>
--- a/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
+++ b/especificacoes/CDJ-GRE-ARQ-AC-R00.xlsx
@@ -5538,7 +5538,7 @@
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="91" t="inlineStr">
         <is>
-          <t xml:space="preserve">PÁGINA </t>
+          <t>ABA</t>
         </is>
       </c>
       <c r="B11" s="217" t="n"/>
@@ -5557,13 +5557,13 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="59" t="inlineStr">
         <is>
-          <t>Página 01 de 11</t>
+          <t>CONTROLE DE REVISÕES</t>
         </is>
       </c>
       <c r="B12" s="217" t="n"/>
       <c r="C12" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUMÁRIO E CONTROLE DE REVISÕES </t>
+          <t>SUMÁRIO E CONTROLE DE REVISÕES</t>
         </is>
       </c>
       <c r="D12" s="230" t="n"/>
@@ -5576,13 +5576,13 @@
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="59" t="inlineStr">
         <is>
-          <t>Página 02 de11</t>
+          <t>TÉRREO</t>
         </is>
       </c>
       <c r="B13" s="217" t="n"/>
       <c r="C13" s="61" t="inlineStr">
         <is>
-          <t>ESPECIFICAÇÃO DE REVESTIMENTOS</t>
+          <t>ESPECIFICAÇÃO DE REVESTIMENTOS, LOUÇAS E METAIS E COMPLEMENTARES</t>
         </is>
       </c>
       <c r="D13" s="230" t="n"/>
@@ -5595,13 +5595,13 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="59" t="inlineStr">
         <is>
-          <t>Página 03 de 11</t>
+          <t>2° PAVTO</t>
         </is>
       </c>
       <c r="B14" s="217" t="n"/>
       <c r="C14" s="61" t="inlineStr">
         <is>
-          <t>ESPECIFICAÇÃO DE REVESTIMENTOS</t>
+          <t>ESPECIFICAÇÃO DE REVESTIMENTOS, LOUÇAS E METAIS E COMPLEMENTARES</t>
         </is>
       </c>
       <c r="D14" s="230" t="n"/>
@@ -5614,13 +5614,13 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="59" t="inlineStr">
         <is>
-          <t>Página 04 de 11</t>
+          <t>PILOTIS</t>
         </is>
       </c>
       <c r="B15" s="217" t="n"/>
       <c r="C15" s="61" t="inlineStr">
         <is>
-          <t>ESPECIFICAÇÃO DE LOUÇAS E METAIS</t>
+          <t>ESPECIFICAÇÃO DE REVESTIMENTOS, LOUÇAS E METAIS E COMPLEMENTARES; IMAGENS AO LADO DA GRADE (LINK "VER IMAGEM")</t>
         </is>
       </c>
       <c r="D15" s="230" t="n"/>
@@ -5633,13 +5633,13 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="59" t="inlineStr">
         <is>
-          <t>Página 05 de 11</t>
+          <t>APTO TIPO</t>
         </is>
       </c>
       <c r="B16" s="217" t="n"/>
       <c r="C16" s="61" t="inlineStr">
         <is>
-          <t>ESPECIFICAÇÃO DE LOUÇAS E METAIS</t>
+          <t>ESPECIFICAÇÃO DO APARTAMENTO TIPO</t>
         </is>
       </c>
       <c r="D16" s="230" t="n"/>
@@ -5652,13 +5652,13 @@
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="59" t="inlineStr">
         <is>
-          <t>Página 06 de 11</t>
+          <t>CONFLITOS</t>
         </is>
       </c>
       <c r="B17" s="217" t="n"/>
       <c r="C17" s="61" t="inlineStr">
         <is>
-          <t>ESPECIFICAÇÃO DE COMPLEMENTARES</t>
+          <t>ESPECIFICAÇÕES CONFLITANTES (ARQUITETURA × DETALHAMENTO; PRANCHA × TABELA DA PRÓPRIA PRANCHA)</t>
         </is>
       </c>
       <c r="D17" s="230" t="n"/>
@@ -5671,13 +5671,13 @@
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="59" t="inlineStr">
         <is>
-          <t>Página 07 de 11</t>
+          <t>PENDÊNCIAS</t>
         </is>
       </c>
       <c r="B18" s="217" t="n"/>
       <c r="C18" s="61" t="inlineStr">
         <is>
-          <t>ESPECIFICAÇÃO DE COMPLEMENTARES</t>
+          <t>PENDÊNCIAS E RASTREABILIDADE DAS FONTES</t>
         </is>
       </c>
       <c r="D18" s="230" t="n"/>
@@ -5688,17 +5688,9 @@
       <c r="I18" s="217" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="59" t="inlineStr">
-        <is>
-          <t>Página 08 de 11</t>
-        </is>
-      </c>
+      <c r="A19" s="59" t="n"/>
       <c r="B19" s="217" t="n"/>
-      <c r="C19" s="61" t="inlineStr">
-        <is>
-          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
-        </is>
-      </c>
+      <c r="C19" s="61" t="n"/>
       <c r="D19" s="230" t="n"/>
       <c r="E19" s="230" t="n"/>
       <c r="F19" s="230" t="n"/>
@@ -5707,17 +5699,9 @@
       <c r="I19" s="217" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="59" t="inlineStr">
-        <is>
-          <t>Página 09 de 11</t>
-        </is>
-      </c>
+      <c r="A20" s="59" t="n"/>
       <c r="B20" s="217" t="n"/>
-      <c r="C20" s="61" t="inlineStr">
-        <is>
-          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
-        </is>
-      </c>
+      <c r="C20" s="61" t="n"/>
       <c r="D20" s="230" t="n"/>
       <c r="E20" s="230" t="n"/>
       <c r="F20" s="230" t="n"/>
@@ -5726,17 +5710,9 @@
       <c r="I20" s="217" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="59" t="inlineStr">
-        <is>
-          <t>Página 10 de 11</t>
-        </is>
-      </c>
+      <c r="A21" s="59" t="n"/>
       <c r="B21" s="217" t="n"/>
-      <c r="C21" s="61" t="inlineStr">
-        <is>
-          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
-        </is>
-      </c>
+      <c r="C21" s="61" t="n"/>
       <c r="D21" s="230" t="n"/>
       <c r="E21" s="230" t="n"/>
       <c r="F21" s="230" t="n"/>
@@ -5745,17 +5721,9 @@
       <c r="I21" s="217" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" thickBot="1">
-      <c r="A22" s="99" t="inlineStr">
-        <is>
-          <t>Página 11 de 11</t>
-        </is>
-      </c>
+      <c r="A22" s="99" t="n"/>
       <c r="B22" s="221" t="n"/>
-      <c r="C22" s="111" t="inlineStr">
-        <is>
-          <t>IMAGENS: AO LADO DA GRADE (LINK "VER IMAGEM")</t>
-        </is>
-      </c>
+      <c r="C22" s="111" t="n"/>
       <c r="D22" s="231" t="n"/>
       <c r="E22" s="231" t="n"/>
       <c r="F22" s="231" t="n"/>
@@ -5821,56 +5789,60 @@
       <c r="I25" s="234" t="n"/>
     </row>
     <row r="26" ht="43.5" customHeight="1">
-      <c r="A26" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>30/09/2026</t>
         </is>
       </c>
-      <c r="C26" s="25" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>R00</t>
         </is>
       </c>
-      <c r="D26" s="235" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>TODAS</t>
+        </is>
+      </c>
+      <c r="E26" s="61" t="inlineStr">
+        <is>
+          <t>Emissão inicial (primeira versão). Prevalece o detalhamento sobre a Tabela 01; divergências entre arquitetura e detalhamento, e entre prancha e tabela da própria prancha, ficam em vermelho e na aba CONFLITOS.</t>
+        </is>
+      </c>
+      <c r="F26" s="230" t="n"/>
+      <c r="G26" s="230" t="n"/>
+      <c r="H26" s="230" t="n"/>
+      <c r="I26" s="217" t="n"/>
+    </row>
+    <row r="27" ht="43.5" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>R00</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
         <is>
           <t>PILOTIS (3º PAVIMENTO)</t>
         </is>
       </c>
-      <c r="E26" s="236" t="inlineStr">
-        <is>
-          <t>Emissão inicial. Especificações levantadas da Tabela de acabamentos Ed. Cidade Jardim v00 (19/06/2026).</t>
-        </is>
-      </c>
-      <c r="F26" s="228" t="n"/>
-      <c r="G26" s="228" t="n"/>
-      <c r="H26" s="228" t="n"/>
-      <c r="I26" s="229" t="n"/>
-    </row>
-    <row r="27" ht="43.5" customHeight="1">
-      <c r="A27" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="B27" s="16" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
-      <c r="C27" s="17" t="inlineStr">
-        <is>
-          <t>R00</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>TÉRREO E 2º PAVIMENTO</t>
-        </is>
-      </c>
-      <c r="E27" s="237" t="inlineStr">
-        <is>
-          <t>Sem especificações na tabela v00 (abrange somente o 3º pavimento - Pilotis). Aguardando informação.</t>
+      <c r="E27" s="61" t="inlineStr">
+        <is>
+          <t>Tabela de acabamentos Ed. Cidade Jardim v00 (19/06/2026), detalhamento de interiores R04 (23/04/2026) e plantas de arquitetura PR011 a PR013.</t>
         </is>
       </c>
       <c r="F27" s="230" t="n"/>
@@ -5879,8 +5851,10 @@
       <c r="I27" s="217" t="n"/>
     </row>
     <row r="28" ht="43.5" customHeight="1">
-      <c r="A28" s="19" t="n">
-        <v>3</v>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
@@ -5892,14 +5866,14 @@
           <t>R00</t>
         </is>
       </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>IMAGENS ESPECIFICAÇÕES</t>
-        </is>
-      </c>
-      <c r="E28" s="237" t="inlineStr">
-        <is>
-          <t>Imagens das fichas TERMAS e VESTIÁRIOS - TERMAS da tabela de acabamentos v00. Em 02/10/2026 passaram para a própria aba PILOTIS, à direita da grade (a partir da coluna AH); o link "► VER IMAGEM (clique)" na célula leva à foto e "◄ VOLTAR" retorna.</t>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>TÉRREO E 2º PAVIMENTO</t>
+        </is>
+      </c>
+      <c r="E28" s="61" t="inlineStr">
+        <is>
+          <t>Detalhamento de interiores R04 (23/04/2026) e plantas de arquitetura CDJ-ARQ-EX PR003 a PR009, conferidas no desenho etiqueta por etiqueta.</t>
         </is>
       </c>
       <c r="F28" s="230" t="n"/>
@@ -5908,8 +5882,10 @@
       <c r="I28" s="217" t="n"/>
     </row>
     <row r="29" ht="43.5" customHeight="1">
-      <c r="A29" s="19" t="n">
-        <v>4</v>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
@@ -5923,12 +5899,12 @@
       </c>
       <c r="D29" s="22" t="inlineStr">
         <is>
-          <t>PENDÊNCIAS</t>
+          <t>APTO TIPO</t>
         </is>
       </c>
       <c r="E29" s="61" t="inlineStr">
         <is>
-          <t>Nova aba com as pendências de especificação e a correspondência ambiente da tabela × linha da grade.</t>
+          <t>Tabela JARDIM-ACABAMENTOS R01 e detalhamento do apartamento (CDJ_DET_EX PR001-PR008, CDJ-ARQ-DT PR406/407/408).</t>
         </is>
       </c>
       <c r="F29" s="230" t="n"/>
@@ -5937,11 +5913,31 @@
       <c r="I29" s="217" t="n"/>
     </row>
     <row r="30" ht="43.5" customHeight="1">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="40" t="n"/>
-      <c r="C30" s="41" t="n"/>
-      <c r="D30" s="39" t="n"/>
-      <c r="E30" s="61" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>R00</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>IMAGENS</t>
+        </is>
+      </c>
+      <c r="E30" s="61" t="inlineStr">
+        <is>
+          <t>Imagens das fichas TERMAS e VESTIÁRIOS - TERMAS na aba PILOTIS, à direita da grade (coluna AH em diante): "► VER IMAGEM (clique)" leva à foto e "◄ VOLTAR" retorna.</t>
+        </is>
+      </c>
       <c r="F30" s="230" t="n"/>
       <c r="G30" s="230" t="n"/>
       <c r="H30" s="230" t="n"/>
@@ -6661,7 +6657,7 @@
       <c r="A12" s="51" t="n"/>
       <c r="B12" s="124" t="inlineStr">
         <is>
-          <t>GERAL — SEM ESPECIFICAÇÕES NA TABELA DE ACABAMENTOS V00 (A TABELA ABRANGE SOMENTE O 3º PAVIMENTO - PILOTIS)</t>
+          <t>GERAL — TÉRREO PELO DETALHAMENTO DE INTERIORES R04 E PELAS PLANTAS DE ARQUITETURA PR003 A PR005</t>
         </is>
       </c>
       <c r="C12" s="241" t="n"/>
@@ -6703,14 +6699,14 @@
           <t>ELEVADORES SOCIAIS</t>
         </is>
       </c>
-      <c r="B13" s="295" t="n"/>
+      <c r="B13" s="327" t="n"/>
       <c r="C13" s="296" t="n"/>
       <c r="D13" s="296" t="n"/>
       <c r="E13" s="296" t="n"/>
       <c r="F13" s="296" t="n"/>
       <c r="G13" s="296" t="n"/>
-      <c r="H13" s="297" t="n"/>
-      <c r="I13" s="297" t="n"/>
+      <c r="H13" s="314" t="n"/>
+      <c r="I13" s="314" t="n"/>
       <c r="J13" s="296" t="n"/>
       <c r="K13" s="296" t="n"/>
       <c r="L13" s="296" t="n"/>
@@ -6725,8 +6721,8 @@
       <c r="U13" s="296" t="n"/>
       <c r="V13" s="296" t="n"/>
       <c r="W13" s="296" t="n"/>
-      <c r="X13" s="295" t="n"/>
-      <c r="Y13" s="295" t="n"/>
+      <c r="X13" s="327" t="n"/>
+      <c r="Y13" s="327" t="n"/>
       <c r="Z13" s="296" t="n"/>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -6735,14 +6731,14 @@
           <t>ELEVADOR SERVIÇO</t>
         </is>
       </c>
-      <c r="B14" s="295" t="n"/>
+      <c r="B14" s="327" t="n"/>
       <c r="C14" s="296" t="n"/>
       <c r="D14" s="296" t="n"/>
       <c r="E14" s="296" t="n"/>
       <c r="F14" s="296" t="n"/>
       <c r="G14" s="296" t="n"/>
-      <c r="H14" s="297" t="n"/>
-      <c r="I14" s="297" t="n"/>
+      <c r="H14" s="314" t="n"/>
+      <c r="I14" s="314" t="n"/>
       <c r="J14" s="296" t="n"/>
       <c r="K14" s="296" t="n"/>
       <c r="L14" s="296" t="n"/>
@@ -6757,17 +6753,17 @@
       <c r="U14" s="296" t="n"/>
       <c r="V14" s="296" t="n"/>
       <c r="W14" s="296" t="n"/>
-      <c r="X14" s="295" t="n"/>
-      <c r="Y14" s="295" t="n"/>
+      <c r="X14" s="327" t="n"/>
+      <c r="Y14" s="327" t="n"/>
       <c r="Z14" s="296" t="n"/>
     </row>
     <row r="15" ht="89" customHeight="1">
       <c r="A15" s="294" t="inlineStr">
         <is>
-          <t xml:space="preserve">RAMPA ACESSO PEDESTRES </t>
-        </is>
-      </c>
-      <c r="B15" s="295" t="inlineStr">
+          <t>RAMPA ACESSO PEDESTRES</t>
+        </is>
+      </c>
+      <c r="B15" s="327" t="inlineStr">
         <is>
           <t>ARQ-P21 - Piso em granito marrom absoluto serrado e envernizado, ou pedra sintética a definir. Paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. (Planta PR003: plano inclinado - pedestres (social), i=4,99%)</t>
         </is>
@@ -6777,8 +6773,8 @@
       <c r="E15" s="296" t="n"/>
       <c r="F15" s="296" t="n"/>
       <c r="G15" s="296" t="n"/>
-      <c r="H15" s="297" t="n"/>
-      <c r="I15" s="297" t="n"/>
+      <c r="H15" s="314" t="n"/>
+      <c r="I15" s="314" t="n"/>
       <c r="J15" s="296" t="n"/>
       <c r="K15" s="296" t="n"/>
       <c r="L15" s="296" t="n"/>
@@ -6793,8 +6789,8 @@
       <c r="U15" s="296" t="n"/>
       <c r="V15" s="296" t="n"/>
       <c r="W15" s="296" t="n"/>
-      <c r="X15" s="295" t="n"/>
-      <c r="Y15" s="295" t="n"/>
+      <c r="X15" s="327" t="n"/>
+      <c r="Y15" s="327" t="n"/>
       <c r="Z15" s="296" t="n"/>
     </row>
     <row r="16" ht="149" customHeight="1">
@@ -6819,7 +6815,7 @@
       <c r="G16" s="300" t="n"/>
       <c r="H16" s="308" t="inlineStr">
         <is>
-          <t>PA56 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica,  revestimento em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>PA56 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica, revestimento em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="I16" s="308" t="inlineStr">
@@ -6848,16 +6844,16 @@
       <c r="X16" s="307" t="inlineStr">
         <is>
           <t>D41 - Porta estruturada em alumínio com fechamento interno e externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A
-D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
-        </is>
-      </c>
-      <c r="Y16" s="302" t="n"/>
+D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+        </is>
+      </c>
+      <c r="Y16" s="320" t="n"/>
       <c r="Z16" s="300" t="n"/>
     </row>
     <row r="17" ht="194" customHeight="1">
       <c r="A17" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">GUARITA </t>
+          <t>GUARITA</t>
         </is>
       </c>
       <c r="B17" s="303" t="inlineStr">
@@ -6906,8 +6902,8 @@
         </is>
       </c>
       <c r="W17" s="300" t="n"/>
-      <c r="X17" s="302" t="n"/>
-      <c r="Y17" s="302" t="n"/>
+      <c r="X17" s="320" t="n"/>
+      <c r="Y17" s="320" t="n"/>
       <c r="Z17" s="300" t="n"/>
     </row>
     <row r="18" ht="89" customHeight="1">
@@ -6954,8 +6950,8 @@
       <c r="U18" s="300" t="n"/>
       <c r="V18" s="300" t="n"/>
       <c r="W18" s="300" t="n"/>
-      <c r="X18" s="302" t="n"/>
-      <c r="Y18" s="302" t="n"/>
+      <c r="X18" s="320" t="n"/>
+      <c r="Y18" s="320" t="n"/>
       <c r="Z18" s="300" t="n"/>
     </row>
     <row r="19" ht="89" customHeight="1">
@@ -7002,8 +6998,8 @@
       <c r="U19" s="300" t="n"/>
       <c r="V19" s="300" t="n"/>
       <c r="W19" s="300" t="n"/>
-      <c r="X19" s="302" t="n"/>
-      <c r="Y19" s="302" t="n"/>
+      <c r="X19" s="320" t="n"/>
+      <c r="Y19" s="320" t="n"/>
       <c r="Z19" s="300" t="n"/>
     </row>
     <row r="20" ht="269" customHeight="1">
@@ -7031,7 +7027,7 @@
           <t>PA1 - Parede em alvenaria com reboco convencional 2,5cm, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.
 PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA54 - Parede em alvenaria regularizada, revestida em pedra natural, Basaltina, acabamento frisado. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
-PA56 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica,  revestimento em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
+PA56 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica, revestimento em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="I20" s="308" t="inlineStr">
@@ -7061,10 +7057,10 @@
       <c r="X20" s="307" t="inlineStr">
         <is>
           <t>D41 - Porta estruturada em alumínio com fechamento interno e externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A
-D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
-        </is>
-      </c>
-      <c r="Y20" s="302" t="n"/>
+D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+        </is>
+      </c>
+      <c r="Y20" s="320" t="n"/>
       <c r="Z20" s="308" t="inlineStr">
         <is>
           <t>D63 - Guarda corpo em chapa metálica dourada colada sobre fechamento em MDF cru 6mm aparafusado em estrutura auxiliar de metalon. Dimensões e detalhes conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A</t>
@@ -7121,8 +7117,8 @@
         </is>
       </c>
       <c r="W21" s="300" t="n"/>
-      <c r="X21" s="302" t="n"/>
-      <c r="Y21" s="302" t="n"/>
+      <c r="X21" s="320" t="n"/>
+      <c r="Y21" s="320" t="n"/>
       <c r="Z21" s="308" t="inlineStr">
         <is>
           <t>D64 - Quadro para elevador em chapa metálica 8mm com acabamento em pintura eletrostática, cor branca. Amostra a ser aprovada pela GPA&amp;A</t>
@@ -7132,7 +7128,7 @@
     <row r="22" ht="74" customHeight="1">
       <c r="A22" s="298" t="inlineStr">
         <is>
-          <t>CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTICÂRA</t>
+          <t>CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTECÂMARA</t>
         </is>
       </c>
       <c r="B22" s="307" t="inlineStr">
@@ -7173,14 +7169,14 @@
       <c r="U22" s="300" t="n"/>
       <c r="V22" s="300" t="n"/>
       <c r="W22" s="300" t="n"/>
-      <c r="X22" s="302" t="n"/>
-      <c r="Y22" s="302" t="n"/>
+      <c r="X22" s="320" t="n"/>
+      <c r="Y22" s="320" t="n"/>
       <c r="Z22" s="300" t="n"/>
     </row>
     <row r="23" ht="134" customHeight="1">
       <c r="A23" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">HALL GARGEM </t>
+          <t>HALL GARAGEM</t>
         </is>
       </c>
       <c r="B23" s="307" t="inlineStr">
@@ -7232,7 +7228,7 @@
 D45 - Porta pivotante em MDF com acabamento em pintura acrílica fosca. Tom a definir. Dimensões conforme Mapa de Esquadrias. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
-      <c r="Y23" s="302" t="n"/>
+      <c r="Y23" s="320" t="n"/>
       <c r="Z23" s="308" t="inlineStr">
         <is>
           <t>D64 - Quadro para elevador em chapa metálica 8mm com acabamento em pintura eletrostática, cor branca. Amostra a ser aprovada pela GPA&amp;A</t>
@@ -7242,7 +7238,7 @@
     <row r="24" ht="74" customHeight="1">
       <c r="A24" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARAGEM </t>
+          <t>GARAGEM</t>
         </is>
       </c>
       <c r="B24" s="307" t="inlineStr">
@@ -7279,8 +7275,8 @@
       <c r="U24" s="300" t="n"/>
       <c r="V24" s="300" t="n"/>
       <c r="W24" s="300" t="n"/>
-      <c r="X24" s="302" t="n"/>
-      <c r="Y24" s="302" t="n"/>
+      <c r="X24" s="320" t="n"/>
+      <c r="Y24" s="320" t="n"/>
       <c r="Z24" s="300" t="n"/>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -7321,10 +7317,10 @@
       <c r="S25" s="300" t="n"/>
       <c r="T25" s="300" t="n"/>
       <c r="U25" s="300" t="n"/>
-      <c r="V25" s="302" t="n"/>
+      <c r="V25" s="320" t="n"/>
       <c r="W25" s="306" t="n"/>
-      <c r="X25" s="302" t="n"/>
-      <c r="Y25" s="302" t="n"/>
+      <c r="X25" s="320" t="n"/>
+      <c r="Y25" s="320" t="n"/>
       <c r="Z25" s="300" t="n"/>
     </row>
     <row r="26" ht="60" customHeight="1">
@@ -7353,16 +7349,16 @@
       <c r="S26" s="300" t="n"/>
       <c r="T26" s="300" t="n"/>
       <c r="U26" s="300" t="n"/>
-      <c r="V26" s="302" t="n"/>
+      <c r="V26" s="320" t="n"/>
       <c r="W26" s="307" t="n"/>
-      <c r="X26" s="302" t="n"/>
-      <c r="Y26" s="302" t="n"/>
+      <c r="X26" s="320" t="n"/>
+      <c r="Y26" s="320" t="n"/>
       <c r="Z26" s="307" t="n"/>
     </row>
     <row r="27" ht="89" customHeight="1">
       <c r="A27" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">CIRCULAÇÃO </t>
+          <t>CIRCULAÇÃO</t>
         </is>
       </c>
       <c r="B27" s="307" t="inlineStr">
@@ -7394,14 +7390,14 @@
       <c r="L27" s="300" t="n"/>
       <c r="M27" s="308" t="n"/>
       <c r="N27" s="308" t="n"/>
-      <c r="O27" s="302" t="n"/>
-      <c r="P27" s="302" t="n"/>
+      <c r="O27" s="320" t="n"/>
+      <c r="P27" s="320" t="n"/>
       <c r="Q27" s="300" t="n"/>
       <c r="R27" s="307" t="n"/>
       <c r="S27" s="300" t="n"/>
       <c r="T27" s="307" t="n"/>
       <c r="U27" s="300" t="n"/>
-      <c r="V27" s="302" t="n"/>
+      <c r="V27" s="320" t="n"/>
       <c r="W27" s="307" t="n"/>
       <c r="X27" s="307" t="n"/>
       <c r="Y27" s="307" t="n"/>
@@ -7478,10 +7474,10 @@
       <c r="W28" s="307" t="n"/>
       <c r="X28" s="307" t="inlineStr">
         <is>
-          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
-        </is>
-      </c>
-      <c r="Y28" s="302" t="n"/>
+          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+        </is>
+      </c>
+      <c r="Y28" s="320" t="n"/>
       <c r="Z28" s="307" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
@@ -7513,7 +7509,7 @@
       <c r="H29" s="307" t="inlineStr">
         <is>
           <t>PA53 - Parede em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
-PA55 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica,  revestimento em vidro 4mm temperado, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
+PA55 - Parede em alvenaria regularizada emassada, pintada com tinta acrílica, revestimento em vidro 4mm temperado, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="I29" s="307" t="inlineStr">
@@ -7541,8 +7537,8 @@
       <c r="W29" s="300" t="n"/>
       <c r="X29" s="308" t="inlineStr">
         <is>
-          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
-D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
+D42 - Porta estruturada em alumínio com fechamento interno ao vestíbulo em vidro 4mm temperado, cor Prada, acabamento acidato; e fechamento externo em vidro extraclean, cor Nebbia, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y29" s="300" t="n"/>
@@ -7591,7 +7587,7 @@
       <c r="S30" s="300" t="n"/>
       <c r="T30" s="307" t="n"/>
       <c r="U30" s="300" t="n"/>
-      <c r="V30" s="302" t="n"/>
+      <c r="V30" s="320" t="n"/>
       <c r="W30" s="300" t="n"/>
       <c r="X30" s="300" t="n"/>
       <c r="Y30" s="300" t="n"/>
@@ -7639,16 +7635,16 @@
       <c r="S31" s="300" t="n"/>
       <c r="T31" s="300" t="n"/>
       <c r="U31" s="300" t="n"/>
-      <c r="V31" s="302" t="n"/>
+      <c r="V31" s="320" t="n"/>
       <c r="W31" s="307" t="n"/>
-      <c r="X31" s="302" t="n"/>
-      <c r="Y31" s="302" t="n"/>
+      <c r="X31" s="320" t="n"/>
+      <c r="Y31" s="320" t="n"/>
       <c r="Z31" s="307" t="n"/>
     </row>
     <row r="32" ht="104" customHeight="1">
       <c r="A32" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">CIRCULAÇÃO SERVIÇO </t>
+          <t>CIRCULAÇÃO SERVIÇO</t>
         </is>
       </c>
       <c r="B32" s="307" t="inlineStr">
@@ -7687,10 +7683,10 @@
       <c r="S32" s="300" t="n"/>
       <c r="T32" s="300" t="n"/>
       <c r="U32" s="300" t="n"/>
-      <c r="V32" s="302" t="n"/>
+      <c r="V32" s="320" t="n"/>
       <c r="W32" s="307" t="n"/>
-      <c r="X32" s="302" t="n"/>
-      <c r="Y32" s="302" t="n"/>
+      <c r="X32" s="320" t="n"/>
+      <c r="Y32" s="320" t="n"/>
       <c r="Z32" s="307" t="n"/>
     </row>
     <row r="33" ht="89" customHeight="1">
@@ -7731,7 +7727,7 @@
       <c r="S33" s="300" t="n"/>
       <c r="T33" s="300" t="n"/>
       <c r="U33" s="300" t="n"/>
-      <c r="V33" s="302" t="n"/>
+      <c r="V33" s="320" t="n"/>
       <c r="W33" s="300" t="n"/>
       <c r="X33" s="300" t="n"/>
       <c r="Y33" s="300" t="n"/>
@@ -7740,7 +7736,7 @@
     <row r="34" ht="89" customHeight="1">
       <c r="A34" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">BICICLETÁRIO </t>
+          <t>BICICLETÁRIO</t>
         </is>
       </c>
       <c r="B34" s="307" t="inlineStr">
@@ -7775,16 +7771,16 @@
       <c r="S34" s="300" t="n"/>
       <c r="T34" s="300" t="n"/>
       <c r="U34" s="300" t="n"/>
-      <c r="V34" s="302" t="n"/>
+      <c r="V34" s="320" t="n"/>
       <c r="W34" s="307" t="n"/>
-      <c r="X34" s="302" t="n"/>
-      <c r="Y34" s="302" t="n"/>
+      <c r="X34" s="320" t="n"/>
+      <c r="Y34" s="320" t="n"/>
       <c r="Z34" s="307" t="n"/>
     </row>
     <row r="35" ht="89" customHeight="1">
       <c r="A35" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZELADORIA </t>
+          <t>ZELADORIA</t>
         </is>
       </c>
       <c r="B35" s="307" t="inlineStr">
@@ -7817,13 +7813,13 @@
       <c r="M35" s="308" t="n"/>
       <c r="N35" s="308" t="n"/>
       <c r="O35" s="307" t="n"/>
-      <c r="P35" s="302" t="n"/>
+      <c r="P35" s="320" t="n"/>
       <c r="Q35" s="300" t="n"/>
       <c r="R35" s="307" t="n"/>
       <c r="S35" s="307" t="n"/>
       <c r="T35" s="307" t="n"/>
       <c r="U35" s="300" t="n"/>
-      <c r="V35" s="302" t="n"/>
+      <c r="V35" s="320" t="n"/>
       <c r="W35" s="307" t="n"/>
       <c r="X35" s="307" t="n"/>
       <c r="Y35" s="307" t="n"/>
@@ -7861,13 +7857,13 @@
       <c r="M36" s="308" t="n"/>
       <c r="N36" s="308" t="n"/>
       <c r="O36" s="307" t="n"/>
-      <c r="P36" s="302" t="n"/>
+      <c r="P36" s="320" t="n"/>
       <c r="Q36" s="300" t="n"/>
       <c r="R36" s="307" t="n"/>
       <c r="S36" s="307" t="n"/>
       <c r="T36" s="307" t="n"/>
       <c r="U36" s="300" t="n"/>
-      <c r="V36" s="302" t="n"/>
+      <c r="V36" s="320" t="n"/>
       <c r="W36" s="307" t="n"/>
       <c r="X36" s="307" t="n"/>
       <c r="Y36" s="307" t="n"/>
@@ -7905,13 +7901,13 @@
       <c r="M37" s="308" t="n"/>
       <c r="N37" s="308" t="n"/>
       <c r="O37" s="307" t="n"/>
-      <c r="P37" s="302" t="n"/>
+      <c r="P37" s="320" t="n"/>
       <c r="Q37" s="300" t="n"/>
       <c r="R37" s="307" t="n"/>
       <c r="S37" s="307" t="n"/>
       <c r="T37" s="307" t="n"/>
       <c r="U37" s="300" t="n"/>
-      <c r="V37" s="302" t="n"/>
+      <c r="V37" s="320" t="n"/>
       <c r="W37" s="307" t="n"/>
       <c r="X37" s="307" t="n"/>
       <c r="Y37" s="307" t="n"/>
@@ -7949,13 +7945,13 @@
       <c r="M38" s="308" t="n"/>
       <c r="N38" s="308" t="n"/>
       <c r="O38" s="307" t="n"/>
-      <c r="P38" s="302" t="n"/>
+      <c r="P38" s="320" t="n"/>
       <c r="Q38" s="300" t="n"/>
       <c r="R38" s="307" t="n"/>
       <c r="S38" s="307" t="n"/>
       <c r="T38" s="307" t="n"/>
       <c r="U38" s="300" t="n"/>
-      <c r="V38" s="302" t="n"/>
+      <c r="V38" s="320" t="n"/>
       <c r="W38" s="307" t="n"/>
       <c r="X38" s="307" t="n"/>
       <c r="Y38" s="307" t="n"/>
@@ -7997,13 +7993,13 @@
       <c r="M39" s="308" t="n"/>
       <c r="N39" s="308" t="n"/>
       <c r="O39" s="307" t="n"/>
-      <c r="P39" s="302" t="n"/>
+      <c r="P39" s="320" t="n"/>
       <c r="Q39" s="300" t="n"/>
       <c r="R39" s="307" t="n"/>
       <c r="S39" s="307" t="n"/>
       <c r="T39" s="307" t="n"/>
       <c r="U39" s="300" t="n"/>
-      <c r="V39" s="302" t="n"/>
+      <c r="V39" s="320" t="n"/>
       <c r="W39" s="307" t="n"/>
       <c r="X39" s="307" t="n"/>
       <c r="Y39" s="307" t="n"/>
@@ -8041,13 +8037,13 @@
       <c r="M40" s="308" t="n"/>
       <c r="N40" s="308" t="n"/>
       <c r="O40" s="307" t="n"/>
-      <c r="P40" s="302" t="n"/>
+      <c r="P40" s="320" t="n"/>
       <c r="Q40" s="300" t="n"/>
       <c r="R40" s="307" t="n"/>
       <c r="S40" s="307" t="n"/>
       <c r="T40" s="307" t="n"/>
       <c r="U40" s="300" t="n"/>
-      <c r="V40" s="302" t="n"/>
+      <c r="V40" s="320" t="n"/>
       <c r="W40" s="307" t="n"/>
       <c r="X40" s="307" t="n"/>
       <c r="Y40" s="307" t="n"/>
@@ -8085,13 +8081,13 @@
       <c r="M41" s="308" t="n"/>
       <c r="N41" s="308" t="n"/>
       <c r="O41" s="307" t="n"/>
-      <c r="P41" s="302" t="n"/>
+      <c r="P41" s="320" t="n"/>
       <c r="Q41" s="300" t="n"/>
       <c r="R41" s="307" t="n"/>
       <c r="S41" s="307" t="n"/>
       <c r="T41" s="307" t="n"/>
       <c r="U41" s="300" t="n"/>
-      <c r="V41" s="302" t="n"/>
+      <c r="V41" s="320" t="n"/>
       <c r="W41" s="307" t="n"/>
       <c r="X41" s="307" t="n"/>
       <c r="Y41" s="307" t="n"/>
@@ -8129,13 +8125,13 @@
       <c r="M42" s="308" t="n"/>
       <c r="N42" s="308" t="n"/>
       <c r="O42" s="307" t="n"/>
-      <c r="P42" s="302" t="n"/>
+      <c r="P42" s="320" t="n"/>
       <c r="Q42" s="300" t="n"/>
       <c r="R42" s="307" t="n"/>
       <c r="S42" s="307" t="n"/>
       <c r="T42" s="307" t="n"/>
       <c r="U42" s="300" t="n"/>
-      <c r="V42" s="302" t="n"/>
+      <c r="V42" s="320" t="n"/>
       <c r="W42" s="307" t="n"/>
       <c r="X42" s="307" t="n"/>
       <c r="Y42" s="307" t="n"/>
@@ -8173,13 +8169,13 @@
       <c r="M43" s="308" t="n"/>
       <c r="N43" s="308" t="n"/>
       <c r="O43" s="307" t="n"/>
-      <c r="P43" s="302" t="n"/>
+      <c r="P43" s="320" t="n"/>
       <c r="Q43" s="300" t="n"/>
       <c r="R43" s="307" t="n"/>
       <c r="S43" s="307" t="n"/>
       <c r="T43" s="307" t="n"/>
       <c r="U43" s="300" t="n"/>
-      <c r="V43" s="302" t="n"/>
+      <c r="V43" s="320" t="n"/>
       <c r="W43" s="307" t="n"/>
       <c r="X43" s="307" t="n"/>
       <c r="Y43" s="307" t="n"/>
@@ -8217,13 +8213,13 @@
       <c r="M44" s="308" t="n"/>
       <c r="N44" s="308" t="n"/>
       <c r="O44" s="307" t="n"/>
-      <c r="P44" s="302" t="n"/>
+      <c r="P44" s="320" t="n"/>
       <c r="Q44" s="300" t="n"/>
       <c r="R44" s="307" t="n"/>
       <c r="S44" s="307" t="n"/>
       <c r="T44" s="307" t="n"/>
       <c r="U44" s="300" t="n"/>
-      <c r="V44" s="302" t="n"/>
+      <c r="V44" s="320" t="n"/>
       <c r="W44" s="307" t="n"/>
       <c r="X44" s="307" t="n"/>
       <c r="Y44" s="307" t="n"/>
@@ -8232,7 +8228,7 @@
     <row r="45" ht="89" customHeight="1">
       <c r="A45" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">CIRCULAÇÃO </t>
+          <t>CIRCULAÇÃO</t>
         </is>
       </c>
       <c r="B45" s="307" t="inlineStr">
@@ -8265,13 +8261,13 @@
       <c r="M45" s="308" t="n"/>
       <c r="N45" s="308" t="n"/>
       <c r="O45" s="307" t="n"/>
-      <c r="P45" s="302" t="n"/>
+      <c r="P45" s="320" t="n"/>
       <c r="Q45" s="300" t="n"/>
       <c r="R45" s="307" t="n"/>
       <c r="S45" s="307" t="n"/>
       <c r="T45" s="307" t="n"/>
       <c r="U45" s="300" t="n"/>
-      <c r="V45" s="302" t="n"/>
+      <c r="V45" s="320" t="n"/>
       <c r="W45" s="307" t="n"/>
       <c r="X45" s="307" t="n"/>
       <c r="Y45" s="307" t="n"/>
@@ -8309,13 +8305,13 @@
       <c r="M46" s="308" t="n"/>
       <c r="N46" s="308" t="n"/>
       <c r="O46" s="307" t="n"/>
-      <c r="P46" s="302" t="n"/>
+      <c r="P46" s="320" t="n"/>
       <c r="Q46" s="300" t="n"/>
       <c r="R46" s="307" t="n"/>
       <c r="S46" s="307" t="n"/>
       <c r="T46" s="307" t="n"/>
       <c r="U46" s="300" t="n"/>
-      <c r="V46" s="302" t="n"/>
+      <c r="V46" s="320" t="n"/>
       <c r="W46" s="307" t="n"/>
       <c r="X46" s="307" t="n"/>
       <c r="Y46" s="307" t="n"/>
@@ -8353,13 +8349,13 @@
       <c r="M47" s="308" t="n"/>
       <c r="N47" s="308" t="n"/>
       <c r="O47" s="307" t="n"/>
-      <c r="P47" s="302" t="n"/>
+      <c r="P47" s="320" t="n"/>
       <c r="Q47" s="300" t="n"/>
       <c r="R47" s="307" t="n"/>
       <c r="S47" s="307" t="n"/>
       <c r="T47" s="307" t="n"/>
       <c r="U47" s="300" t="n"/>
-      <c r="V47" s="302" t="n"/>
+      <c r="V47" s="320" t="n"/>
       <c r="W47" s="307" t="n"/>
       <c r="X47" s="307" t="n"/>
       <c r="Y47" s="307" t="n"/>
@@ -8397,13 +8393,13 @@
       <c r="M48" s="308" t="n"/>
       <c r="N48" s="308" t="n"/>
       <c r="O48" s="307" t="n"/>
-      <c r="P48" s="302" t="n"/>
+      <c r="P48" s="320" t="n"/>
       <c r="Q48" s="300" t="n"/>
       <c r="R48" s="307" t="n"/>
       <c r="S48" s="307" t="n"/>
       <c r="T48" s="307" t="n"/>
       <c r="U48" s="300" t="n"/>
-      <c r="V48" s="302" t="n"/>
+      <c r="V48" s="320" t="n"/>
       <c r="W48" s="307" t="n"/>
       <c r="X48" s="307" t="n"/>
       <c r="Y48" s="307" t="n"/>
@@ -8437,13 +8433,13 @@
       <c r="M49" s="308" t="n"/>
       <c r="N49" s="308" t="n"/>
       <c r="O49" s="307" t="n"/>
-      <c r="P49" s="302" t="n"/>
+      <c r="P49" s="320" t="n"/>
       <c r="Q49" s="300" t="n"/>
       <c r="R49" s="307" t="n"/>
       <c r="S49" s="307" t="n"/>
       <c r="T49" s="307" t="n"/>
       <c r="U49" s="300" t="n"/>
-      <c r="V49" s="302" t="n"/>
+      <c r="V49" s="320" t="n"/>
       <c r="W49" s="307" t="n"/>
       <c r="X49" s="307" t="n"/>
       <c r="Y49" s="307" t="n"/>
@@ -8481,13 +8477,13 @@
       <c r="M50" s="308" t="n"/>
       <c r="N50" s="308" t="n"/>
       <c r="O50" s="307" t="n"/>
-      <c r="P50" s="302" t="n"/>
+      <c r="P50" s="320" t="n"/>
       <c r="Q50" s="300" t="n"/>
       <c r="R50" s="307" t="n"/>
       <c r="S50" s="307" t="n"/>
       <c r="T50" s="307" t="n"/>
       <c r="U50" s="300" t="n"/>
-      <c r="V50" s="302" t="n"/>
+      <c r="V50" s="320" t="n"/>
       <c r="W50" s="307" t="n"/>
       <c r="X50" s="307" t="n"/>
       <c r="Y50" s="307" t="n"/>
@@ -8525,13 +8521,13 @@
       <c r="M51" s="308" t="n"/>
       <c r="N51" s="308" t="n"/>
       <c r="O51" s="307" t="n"/>
-      <c r="P51" s="302" t="n"/>
+      <c r="P51" s="320" t="n"/>
       <c r="Q51" s="300" t="n"/>
       <c r="R51" s="307" t="n"/>
       <c r="S51" s="307" t="n"/>
       <c r="T51" s="307" t="n"/>
       <c r="U51" s="300" t="n"/>
-      <c r="V51" s="302" t="n"/>
+      <c r="V51" s="320" t="n"/>
       <c r="W51" s="307" t="n"/>
       <c r="X51" s="307" t="n"/>
       <c r="Y51" s="307" t="n"/>
@@ -8569,13 +8565,13 @@
       <c r="M52" s="308" t="n"/>
       <c r="N52" s="308" t="n"/>
       <c r="O52" s="307" t="n"/>
-      <c r="P52" s="302" t="n"/>
+      <c r="P52" s="320" t="n"/>
       <c r="Q52" s="300" t="n"/>
       <c r="R52" s="307" t="n"/>
       <c r="S52" s="307" t="n"/>
       <c r="T52" s="307" t="n"/>
       <c r="U52" s="300" t="n"/>
-      <c r="V52" s="302" t="n"/>
+      <c r="V52" s="320" t="n"/>
       <c r="W52" s="307" t="n"/>
       <c r="X52" s="307" t="n"/>
       <c r="Y52" s="307" t="n"/>
@@ -8617,13 +8613,13 @@
       <c r="M53" s="308" t="n"/>
       <c r="N53" s="308" t="n"/>
       <c r="O53" s="307" t="n"/>
-      <c r="P53" s="302" t="n"/>
+      <c r="P53" s="320" t="n"/>
       <c r="Q53" s="300" t="n"/>
       <c r="R53" s="307" t="n"/>
       <c r="S53" s="307" t="n"/>
       <c r="T53" s="307" t="n"/>
       <c r="U53" s="300" t="n"/>
-      <c r="V53" s="302" t="n"/>
+      <c r="V53" s="320" t="n"/>
       <c r="W53" s="307" t="n"/>
       <c r="X53" s="307" t="n"/>
       <c r="Y53" s="307" t="n"/>
@@ -8661,13 +8657,13 @@
       <c r="M54" s="308" t="n"/>
       <c r="N54" s="308" t="n"/>
       <c r="O54" s="307" t="n"/>
-      <c r="P54" s="302" t="n"/>
+      <c r="P54" s="320" t="n"/>
       <c r="Q54" s="300" t="n"/>
       <c r="R54" s="307" t="n"/>
       <c r="S54" s="307" t="n"/>
       <c r="T54" s="307" t="n"/>
       <c r="U54" s="300" t="n"/>
-      <c r="V54" s="302" t="n"/>
+      <c r="V54" s="320" t="n"/>
       <c r="W54" s="307" t="n"/>
       <c r="X54" s="307" t="n"/>
       <c r="Y54" s="307" t="n"/>
@@ -8697,13 +8693,13 @@
       <c r="M55" s="308" t="n"/>
       <c r="N55" s="308" t="n"/>
       <c r="O55" s="307" t="n"/>
-      <c r="P55" s="302" t="n"/>
+      <c r="P55" s="320" t="n"/>
       <c r="Q55" s="300" t="n"/>
       <c r="R55" s="307" t="n"/>
       <c r="S55" s="307" t="n"/>
       <c r="T55" s="307" t="n"/>
       <c r="U55" s="300" t="n"/>
-      <c r="V55" s="302" t="n"/>
+      <c r="V55" s="320" t="n"/>
       <c r="W55" s="307" t="n"/>
       <c r="X55" s="307" t="n"/>
       <c r="Y55" s="307" t="n"/>
@@ -8733,13 +8729,13 @@
       <c r="M56" s="308" t="n"/>
       <c r="N56" s="308" t="n"/>
       <c r="O56" s="307" t="n"/>
-      <c r="P56" s="302" t="n"/>
+      <c r="P56" s="320" t="n"/>
       <c r="Q56" s="300" t="n"/>
       <c r="R56" s="307" t="n"/>
       <c r="S56" s="307" t="n"/>
       <c r="T56" s="307" t="n"/>
       <c r="U56" s="300" t="n"/>
-      <c r="V56" s="302" t="n"/>
+      <c r="V56" s="320" t="n"/>
       <c r="W56" s="307" t="n"/>
       <c r="X56" s="307" t="n"/>
       <c r="Y56" s="307" t="n"/>
@@ -9409,7 +9405,7 @@
       <c r="A12" s="51" t="n"/>
       <c r="B12" s="124" t="inlineStr">
         <is>
-          <t>GERAL — SEM ESPECIFICAÇÕES NA TABELA DE ACABAMENTOS V00 (A TABELA ABRANGE SOMENTE O 3º PAVIMENTO - PILOTIS)</t>
+          <t>GERAL — 2º PAVIMENTO PELAS PLANTAS DE ARQUITETURA PR007 A PR009 (O DETALHAMENTO R04 SÓ TRAZ MOBILIÁRIO)</t>
         </is>
       </c>
       <c r="C12" s="241" t="n"/>
@@ -9485,8 +9481,8 @@
       <c r="U13" s="296" t="n"/>
       <c r="V13" s="296" t="n"/>
       <c r="W13" s="296" t="n"/>
-      <c r="X13" s="295" t="n"/>
-      <c r="Y13" s="295" t="n"/>
+      <c r="X13" s="327" t="n"/>
+      <c r="Y13" s="327" t="n"/>
       <c r="Z13" s="296" t="n"/>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -9529,24 +9525,24 @@
       <c r="U14" s="300" t="n"/>
       <c r="V14" s="300" t="n"/>
       <c r="W14" s="300" t="n"/>
-      <c r="X14" s="302" t="n"/>
-      <c r="Y14" s="302" t="n"/>
+      <c r="X14" s="320" t="n"/>
+      <c r="Y14" s="320" t="n"/>
       <c r="Z14" s="300" t="n"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">HALL GARAGEM </t>
-        </is>
-      </c>
-      <c r="B15" s="302" t="n"/>
+          <t>HALL GARAGEM</t>
+        </is>
+      </c>
+      <c r="B15" s="320" t="n"/>
       <c r="C15" s="300" t="n"/>
       <c r="D15" s="300" t="n"/>
       <c r="E15" s="300" t="n"/>
       <c r="F15" s="300" t="n"/>
       <c r="G15" s="300" t="n"/>
-      <c r="H15" s="311" t="n"/>
-      <c r="I15" s="311" t="n"/>
+      <c r="H15" s="317" t="n"/>
+      <c r="I15" s="317" t="n"/>
       <c r="J15" s="300" t="n"/>
       <c r="K15" s="300" t="n"/>
       <c r="L15" s="300" t="n"/>
@@ -9561,8 +9557,8 @@
       <c r="U15" s="300" t="n"/>
       <c r="V15" s="300" t="n"/>
       <c r="W15" s="300" t="n"/>
-      <c r="X15" s="302" t="n"/>
-      <c r="Y15" s="302" t="n"/>
+      <c r="X15" s="320" t="n"/>
+      <c r="Y15" s="320" t="n"/>
       <c r="Z15" s="300" t="n"/>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -9571,14 +9567,14 @@
           <t>HALL ELEVADOR SOCIAL</t>
         </is>
       </c>
-      <c r="B16" s="302" t="n"/>
+      <c r="B16" s="320" t="n"/>
       <c r="C16" s="300" t="n"/>
       <c r="D16" s="300" t="n"/>
       <c r="E16" s="300" t="n"/>
       <c r="F16" s="300" t="n"/>
       <c r="G16" s="300" t="n"/>
-      <c r="H16" s="311" t="n"/>
-      <c r="I16" s="311" t="n"/>
+      <c r="H16" s="317" t="n"/>
+      <c r="I16" s="317" t="n"/>
       <c r="J16" s="300" t="n"/>
       <c r="K16" s="300" t="n"/>
       <c r="L16" s="300" t="n"/>
@@ -9593,8 +9589,8 @@
       <c r="U16" s="300" t="n"/>
       <c r="V16" s="300" t="n"/>
       <c r="W16" s="300" t="n"/>
-      <c r="X16" s="302" t="n"/>
-      <c r="Y16" s="302" t="n"/>
+      <c r="X16" s="320" t="n"/>
+      <c r="Y16" s="320" t="n"/>
       <c r="Z16" s="300" t="n"/>
     </row>
     <row r="17" ht="119" customHeight="1">
@@ -9642,8 +9638,8 @@
       <c r="U17" s="300" t="n"/>
       <c r="V17" s="300" t="n"/>
       <c r="W17" s="300" t="n"/>
-      <c r="X17" s="302" t="n"/>
-      <c r="Y17" s="302" t="n"/>
+      <c r="X17" s="320" t="n"/>
+      <c r="Y17" s="320" t="n"/>
       <c r="Z17" s="300" t="n"/>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -9686,8 +9682,8 @@
       <c r="U18" s="300" t="n"/>
       <c r="V18" s="300" t="n"/>
       <c r="W18" s="300" t="n"/>
-      <c r="X18" s="302" t="n"/>
-      <c r="Y18" s="302" t="n"/>
+      <c r="X18" s="320" t="n"/>
+      <c r="Y18" s="320" t="n"/>
       <c r="Z18" s="300" t="n"/>
     </row>
     <row r="19" ht="60" customHeight="1">
@@ -9730,8 +9726,8 @@
       <c r="U19" s="300" t="n"/>
       <c r="V19" s="300" t="n"/>
       <c r="W19" s="300" t="n"/>
-      <c r="X19" s="302" t="n"/>
-      <c r="Y19" s="302" t="n"/>
+      <c r="X19" s="320" t="n"/>
+      <c r="Y19" s="320" t="n"/>
       <c r="Z19" s="300" t="n"/>
     </row>
     <row r="20" ht="60" customHeight="1">
@@ -9774,8 +9770,8 @@
       <c r="U20" s="300" t="n"/>
       <c r="V20" s="300" t="n"/>
       <c r="W20" s="300" t="n"/>
-      <c r="X20" s="302" t="n"/>
-      <c r="Y20" s="302" t="n"/>
+      <c r="X20" s="320" t="n"/>
+      <c r="Y20" s="320" t="n"/>
       <c r="Z20" s="300" t="n"/>
     </row>
     <row r="21" ht="74" customHeight="1">
@@ -9816,10 +9812,10 @@
       <c r="S21" s="300" t="n"/>
       <c r="T21" s="300" t="n"/>
       <c r="U21" s="300" t="n"/>
-      <c r="V21" s="302" t="n"/>
+      <c r="V21" s="320" t="n"/>
       <c r="W21" s="306" t="n"/>
-      <c r="X21" s="302" t="n"/>
-      <c r="Y21" s="302" t="n"/>
+      <c r="X21" s="320" t="n"/>
+      <c r="Y21" s="320" t="n"/>
       <c r="Z21" s="300" t="n"/>
     </row>
     <row r="22" ht="74" customHeight="1">
@@ -9860,10 +9856,10 @@
       <c r="S22" s="300" t="n"/>
       <c r="T22" s="300" t="n"/>
       <c r="U22" s="300" t="n"/>
-      <c r="V22" s="302" t="n"/>
+      <c r="V22" s="320" t="n"/>
       <c r="W22" s="307" t="n"/>
-      <c r="X22" s="302" t="n"/>
-      <c r="Y22" s="302" t="n"/>
+      <c r="X22" s="320" t="n"/>
+      <c r="Y22" s="320" t="n"/>
       <c r="Z22" s="307" t="n"/>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -9897,14 +9893,14 @@
       <c r="L23" s="300" t="n"/>
       <c r="M23" s="308" t="n"/>
       <c r="N23" s="308" t="n"/>
-      <c r="O23" s="302" t="n"/>
-      <c r="P23" s="302" t="n"/>
+      <c r="O23" s="320" t="n"/>
+      <c r="P23" s="320" t="n"/>
       <c r="Q23" s="300" t="n"/>
       <c r="R23" s="307" t="n"/>
       <c r="S23" s="300" t="n"/>
       <c r="T23" s="307" t="n"/>
       <c r="U23" s="300" t="n"/>
-      <c r="V23" s="302" t="n"/>
+      <c r="V23" s="320" t="n"/>
       <c r="W23" s="307" t="n"/>
       <c r="X23" s="307" t="n"/>
       <c r="Y23" s="307" t="n"/>
@@ -9948,10 +9944,10 @@
       <c r="S24" s="300" t="n"/>
       <c r="T24" s="307" t="n"/>
       <c r="U24" s="300" t="n"/>
-      <c r="V24" s="302" t="n"/>
+      <c r="V24" s="320" t="n"/>
       <c r="W24" s="307" t="n"/>
-      <c r="X24" s="302" t="n"/>
-      <c r="Y24" s="302" t="n"/>
+      <c r="X24" s="320" t="n"/>
+      <c r="Y24" s="320" t="n"/>
       <c r="Z24" s="307" t="n"/>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -9992,7 +9988,7 @@
       <c r="S25" s="300" t="n"/>
       <c r="T25" s="300" t="n"/>
       <c r="U25" s="300" t="n"/>
-      <c r="V25" s="302" t="n"/>
+      <c r="V25" s="320" t="n"/>
       <c r="W25" s="300" t="n"/>
       <c r="X25" s="300" t="n"/>
       <c r="Y25" s="300" t="n"/>
@@ -10036,7 +10032,7 @@
       <c r="S26" s="300" t="n"/>
       <c r="T26" s="307" t="n"/>
       <c r="U26" s="300" t="n"/>
-      <c r="V26" s="302" t="n"/>
+      <c r="V26" s="320" t="n"/>
       <c r="W26" s="300" t="n"/>
       <c r="X26" s="300" t="n"/>
       <c r="Y26" s="300" t="n"/>
@@ -10080,10 +10076,10 @@
       <c r="S27" s="300" t="n"/>
       <c r="T27" s="300" t="n"/>
       <c r="U27" s="300" t="n"/>
-      <c r="V27" s="302" t="n"/>
+      <c r="V27" s="320" t="n"/>
       <c r="W27" s="307" t="n"/>
-      <c r="X27" s="302" t="n"/>
-      <c r="Y27" s="302" t="n"/>
+      <c r="X27" s="320" t="n"/>
+      <c r="Y27" s="320" t="n"/>
       <c r="Z27" s="307" t="n"/>
     </row>
     <row r="28" ht="60" customHeight="1">
@@ -10124,10 +10120,10 @@
       <c r="S28" s="300" t="n"/>
       <c r="T28" s="300" t="n"/>
       <c r="U28" s="300" t="n"/>
-      <c r="V28" s="302" t="n"/>
+      <c r="V28" s="320" t="n"/>
       <c r="W28" s="307" t="n"/>
-      <c r="X28" s="302" t="n"/>
-      <c r="Y28" s="302" t="n"/>
+      <c r="X28" s="320" t="n"/>
+      <c r="Y28" s="320" t="n"/>
       <c r="Z28" s="307" t="n"/>
     </row>
     <row r="29" ht="74" customHeight="1">
@@ -10168,10 +10164,10 @@
       <c r="S29" s="300" t="n"/>
       <c r="T29" s="300" t="n"/>
       <c r="U29" s="300" t="n"/>
-      <c r="V29" s="302" t="n"/>
+      <c r="V29" s="320" t="n"/>
       <c r="W29" s="307" t="n"/>
-      <c r="X29" s="302" t="n"/>
-      <c r="Y29" s="302" t="n"/>
+      <c r="X29" s="320" t="n"/>
+      <c r="Y29" s="320" t="n"/>
       <c r="Z29" s="307" t="n"/>
     </row>
     <row r="30" ht="60" customHeight="1">
@@ -10212,10 +10208,10 @@
       <c r="S30" s="300" t="n"/>
       <c r="T30" s="300" t="n"/>
       <c r="U30" s="300" t="n"/>
-      <c r="V30" s="302" t="n"/>
+      <c r="V30" s="320" t="n"/>
       <c r="W30" s="307" t="n"/>
-      <c r="X30" s="302" t="n"/>
-      <c r="Y30" s="302" t="n"/>
+      <c r="X30" s="320" t="n"/>
+      <c r="Y30" s="320" t="n"/>
       <c r="Z30" s="307" t="n"/>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -10256,10 +10252,10 @@
       <c r="S31" s="300" t="n"/>
       <c r="T31" s="300" t="n"/>
       <c r="U31" s="300" t="n"/>
-      <c r="V31" s="302" t="n"/>
+      <c r="V31" s="320" t="n"/>
       <c r="W31" s="307" t="n"/>
-      <c r="X31" s="302" t="n"/>
-      <c r="Y31" s="302" t="n"/>
+      <c r="X31" s="320" t="n"/>
+      <c r="Y31" s="320" t="n"/>
       <c r="Z31" s="307" t="n"/>
     </row>
     <row r="32"/>
@@ -10985,7 +10981,7 @@
       <c r="Y12" s="241" t="n"/>
       <c r="Z12" s="242" t="n"/>
     </row>
-    <row r="13" ht="299" customHeight="1">
+    <row r="13" ht="284" customHeight="1">
       <c r="A13" s="294" t="inlineStr">
         <is>
           <t>LOBBY PILOTIS</t>
@@ -11043,13 +11039,13 @@
       <c r="W13" s="296" t="n"/>
       <c r="X13" s="325" t="inlineStr">
         <is>
-          <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
-D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
+          <t>D19 - Porta pivotante estruturada, fechamento em MDF cru, face interna ao I.S. com acabamento em folha madeira natural carvalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
+D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
 D74 - Porta pivotante estruturada, fechamento em MDF cru, acabamento face interna e externa em micropintura cor S168-Sayerlack. Puxador tipo cava, prever tranca. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 D85 - Porta corta fogo em aço inox escovado. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
-      <c r="Y13" s="295" t="n"/>
+      <c r="Y13" s="327" t="n"/>
       <c r="Z13" s="296" t="n"/>
     </row>
     <row r="14" ht="284" customHeight="1">
@@ -11115,7 +11111,7 @@
 D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
-      <c r="Y14" s="302" t="n"/>
+      <c r="Y14" s="320" t="n"/>
       <c r="Z14" s="300" t="n"/>
     </row>
     <row r="15" ht="119" customHeight="1">
@@ -11124,7 +11120,7 @@
           <t>TERRAÇO SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="B15" s="302" t="inlineStr">
+      <c r="B15" s="320" t="inlineStr">
         <is>
           <t>ARQ-P08 - Piso elevado em granito cinza santa rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material. (Planta PR011)</t>
         </is>
@@ -11134,8 +11130,8 @@
       <c r="E15" s="300" t="n"/>
       <c r="F15" s="300" t="n"/>
       <c r="G15" s="300" t="n"/>
-      <c r="H15" s="311" t="n"/>
-      <c r="I15" s="311" t="n"/>
+      <c r="H15" s="317" t="n"/>
+      <c r="I15" s="317" t="n"/>
       <c r="J15" s="300" t="n"/>
       <c r="K15" s="300" t="n"/>
       <c r="L15" s="300" t="n"/>
@@ -11150,8 +11146,8 @@
       <c r="U15" s="300" t="n"/>
       <c r="V15" s="300" t="n"/>
       <c r="W15" s="300" t="n"/>
-      <c r="X15" s="302" t="n"/>
-      <c r="Y15" s="302" t="n"/>
+      <c r="X15" s="320" t="n"/>
+      <c r="Y15" s="320" t="n"/>
       <c r="Z15" s="300" t="n"/>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -11160,14 +11156,14 @@
           <t>CIRCULAÇÃO SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="B16" s="302" t="n"/>
+      <c r="B16" s="320" t="n"/>
       <c r="C16" s="300" t="n"/>
       <c r="D16" s="300" t="n"/>
       <c r="E16" s="300" t="n"/>
       <c r="F16" s="300" t="n"/>
       <c r="G16" s="300" t="n"/>
-      <c r="H16" s="311" t="n"/>
-      <c r="I16" s="311" t="n"/>
+      <c r="H16" s="317" t="n"/>
+      <c r="I16" s="317" t="n"/>
       <c r="J16" s="300" t="n"/>
       <c r="K16" s="300" t="n"/>
       <c r="L16" s="300" t="n"/>
@@ -11182,8 +11178,8 @@
       <c r="U16" s="300" t="n"/>
       <c r="V16" s="300" t="n"/>
       <c r="W16" s="300" t="n"/>
-      <c r="X16" s="302" t="n"/>
-      <c r="Y16" s="302" t="n"/>
+      <c r="X16" s="320" t="n"/>
+      <c r="Y16" s="320" t="n"/>
       <c r="Z16" s="300" t="n"/>
     </row>
     <row r="17" ht="224" customHeight="1">
@@ -11256,7 +11252,7 @@
           <t>D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
-      <c r="Y17" s="302" t="n"/>
+      <c r="Y17" s="320" t="n"/>
       <c r="Z17" s="317" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
@@ -11335,7 +11331,7 @@
           <t>D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
-      <c r="Y18" s="302" t="n"/>
+      <c r="Y18" s="320" t="n"/>
       <c r="Z18" s="317" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
@@ -11350,14 +11346,14 @@
           <t>APOIO COZINHA</t>
         </is>
       </c>
-      <c r="B19" s="302" t="n"/>
+      <c r="B19" s="320" t="n"/>
       <c r="C19" s="300" t="n"/>
       <c r="D19" s="300" t="n"/>
       <c r="E19" s="300" t="n"/>
       <c r="F19" s="300" t="n"/>
       <c r="G19" s="300" t="n"/>
-      <c r="H19" s="311" t="n"/>
-      <c r="I19" s="311" t="n"/>
+      <c r="H19" s="317" t="n"/>
+      <c r="I19" s="317" t="n"/>
       <c r="J19" s="300" t="n"/>
       <c r="K19" s="300" t="n"/>
       <c r="L19" s="300" t="n"/>
@@ -11372,8 +11368,8 @@
       <c r="U19" s="300" t="n"/>
       <c r="V19" s="300" t="n"/>
       <c r="W19" s="300" t="n"/>
-      <c r="X19" s="302" t="n"/>
-      <c r="Y19" s="302" t="n"/>
+      <c r="X19" s="320" t="n"/>
+      <c r="Y19" s="320" t="n"/>
       <c r="Z19" s="300" t="n"/>
     </row>
     <row r="20" ht="224" customHeight="1">
@@ -11423,7 +11419,7 @@
       <c r="N20" s="300" t="n"/>
       <c r="O20" s="317" t="inlineStr">
         <is>
-          <t>D81 - Monocomando de mesa, modelo Angolare, acabamento Scoth Brite, cód.: 94520022. Ref.: Tramontina. ATENÇÃO: vazão máxima de 9 l/min, instalar redutor de vazão se necessário.</t>
+          <t>D81 - Monocomando de mesa, modelo Angolare, acabamento Scotch Brite, cód.: 94520022. Ref.: Tramontina. ATENÇÃO: vazão máxima de 9 l/min, instalar redutor de vazão se necessário.</t>
         </is>
       </c>
       <c r="P20" s="300" t="n"/>
@@ -11444,7 +11440,7 @@
 D74 - Porta pivotante estruturada, fechamento em MDF cru, acabamento face interna e externa em micropintura cor S168-Sayerlack. Puxador tipo cava, prever tranca. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
-      <c r="Y20" s="302" t="n"/>
+      <c r="Y20" s="320" t="n"/>
       <c r="Z20" s="308" t="inlineStr">
         <is>
           <t>D82 - Prateleira em granito cinza Santa Rosa, acabamento escovado, embutido na alvenaria. Amostra a ser aprovada pela GPA&amp;A</t>
@@ -11503,8 +11499,8 @@
       <c r="U21" s="300" t="n"/>
       <c r="V21" s="300" t="n"/>
       <c r="W21" s="300" t="n"/>
-      <c r="X21" s="302" t="n"/>
-      <c r="Y21" s="302" t="n"/>
+      <c r="X21" s="320" t="n"/>
+      <c r="Y21" s="320" t="n"/>
       <c r="Z21" s="300" t="n"/>
     </row>
     <row r="22" ht="104" customHeight="1">
@@ -11549,10 +11545,10 @@
       <c r="S22" s="300" t="n"/>
       <c r="T22" s="300" t="n"/>
       <c r="U22" s="300" t="n"/>
-      <c r="V22" s="302" t="n"/>
+      <c r="V22" s="320" t="n"/>
       <c r="W22" s="306" t="n"/>
-      <c r="X22" s="302" t="n"/>
-      <c r="Y22" s="302" t="n"/>
+      <c r="X22" s="320" t="n"/>
+      <c r="Y22" s="320" t="n"/>
       <c r="Z22" s="300" t="n"/>
     </row>
     <row r="23" ht="269" customHeight="1">
@@ -11578,7 +11574,7 @@
       <c r="H23" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
-PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural caravalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
+PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural carvalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
 PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
@@ -11594,7 +11590,7 @@
       </c>
       <c r="K23" s="317" t="inlineStr">
         <is>
-          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
+          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural carvalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="L23" s="300" t="n"/>
@@ -11623,10 +11619,10 @@
       <c r="W23" s="307" t="n"/>
       <c r="X23" s="307" t="inlineStr">
         <is>
-          <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
-        </is>
-      </c>
-      <c r="Y23" s="302" t="n"/>
+          <t>D19 - Porta pivotante estruturada, fechamento em MDF cru, face interna ao I.S. com acabamento em folha madeira natural carvalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
+        </is>
+      </c>
+      <c r="Y23" s="320" t="n"/>
       <c r="Z23" s="320" t="inlineStr">
         <is>
           <t>D27 - Porta papel higiênico duplo em aço inox, modelo Cai Cai, cód.:70.100. Ref.: Draco
@@ -11638,7 +11634,7 @@
     <row r="24" ht="269" customHeight="1">
       <c r="A24" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">I.S </t>
+          <t>I.S</t>
         </is>
       </c>
       <c r="B24" s="320" t="inlineStr">
@@ -11658,7 +11654,7 @@
       <c r="H24" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
-PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural caravalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
+PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural carvalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
 PA52 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
@@ -11674,7 +11670,7 @@
       </c>
       <c r="K24" s="317" t="inlineStr">
         <is>
-          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
+          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural carvalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="L24" s="300" t="n"/>
@@ -11703,7 +11699,7 @@
       <c r="W24" s="307" t="n"/>
       <c r="X24" s="307" t="inlineStr">
         <is>
-          <t>D19 - Porta pivotante estruturada, fechamento em  MDF cru, face interna ao I.S. com acabamento em folha madeira natural caravalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
+          <t>D19 - Porta pivotante estruturada, fechamento em MDF cru, face interna ao I.S. com acabamento em folha madeira natural carvalho tonalizado e face externa cor S168-Sayerlack. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="Y24" s="307" t="n"/>
@@ -11718,7 +11714,7 @@
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">CIRCULAÇÃO LAVABOS </t>
+          <t>CIRCULAÇÃO LAVABOS</t>
         </is>
       </c>
       <c r="B25" s="307" t="n"/>
@@ -11741,10 +11737,10 @@
       <c r="S25" s="300" t="n"/>
       <c r="T25" s="307" t="n"/>
       <c r="U25" s="300" t="n"/>
-      <c r="V25" s="302" t="n"/>
+      <c r="V25" s="320" t="n"/>
       <c r="W25" s="307" t="n"/>
-      <c r="X25" s="302" t="n"/>
-      <c r="Y25" s="302" t="n"/>
+      <c r="X25" s="320" t="n"/>
+      <c r="Y25" s="320" t="n"/>
       <c r="Z25" s="307" t="n"/>
     </row>
     <row r="26" ht="389" customHeight="1">
@@ -11771,7 +11767,7 @@
       <c r="H26" s="320" t="inlineStr">
         <is>
           <t>PA34 - Parede rebocada regularizada, revestida em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.Obs.: Resina ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.
-PA35 - Parede em alvenaria emassada regularizada, revestida em MDF cru 8mm para regularização da superficie e acabamento em chapa metálica - #16 (aço carbono) colda sobre MDF ou fixada através de fita dupla face 3M -  finalização em micropintura cor S081-Sayerlack. Ver detalhes específicos e amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
+PA35 - Parede em alvenaria emassada regularizada, revestida em MDF cru 8mm para regularização da superficie e acabamento em chapa metálica - #16 (aço carbono) colda sobre MDF ou fixada através de fita dupla face 3M - finalização em micropintura cor S081-Sayerlack. Ver detalhes específicos e amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA36 - Parede em alvenaria emassada regularizada, revestida em painel de MDF cru 8mm + chpa de 4mm com acabamento em mircropintura em cor N081-Sayerlack colada sobre MDF cru. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA37 - Parede emassada regularizada revestida com papel de parede degradê laranja 114-Branco casa. Cód Ref.: BR0114_B10099_PDP_TM. Amostra a ser aprovada pela GPA&amp;A.
 PA38 - Parede em alvenaria emassada regularizada, revestida em painel de marcenaria MDF Nude-linha VEL-Berneck. Amostra a ser aprovada pela GPA&amp;A. Obs.: MDF possui certificação FSC.</t>
@@ -11804,14 +11800,14 @@
       <c r="W26" s="307" t="n"/>
       <c r="X26" s="307" t="inlineStr">
         <is>
-          <t>D11 - Porta pivotante estruturada, fechamento em  MDF cru, acabamento micro pintura face do kids cor S081-Sayerlack e acabamento face do gourmet em folha madeira natural caravalho tonalizado. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
-D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
-        </is>
-      </c>
-      <c r="Y26" s="302" t="n"/>
+          <t>D11 - Porta pivotante estruturada, fechamento em MDF cru, acabamento micro pintura face do kids cor S081-Sayerlack e acabamento face do gourmet em folha madeira natural carvalho tonalizado. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
+D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+        </is>
+      </c>
+      <c r="Y26" s="320" t="n"/>
       <c r="Z26" s="307" t="inlineStr">
         <is>
-          <t>D18 - Módulos compostos por três peças hexagonais com estruturado em peças de madeira maciça,   fechamento em reguas de madeira 25mmx70mm. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
+          <t>D18 - Módulos compostos por três peças hexagonais com estruturado em peças de madeira maciça, fechamento em reguas de madeira 25mmx70mm. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
 D56 - Pendente sob medida em peças de madeira maciça 60x50mm fixados no teto através de cabos de aço e estrutura auxiliar no entreforro, com acabamento no forro em canopla, cor branca. Retroiluminação em fitas de led na parte superior com dimensionamentos conforme projeto luminotécnico. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
@@ -11840,7 +11836,7 @@
       <c r="H27" s="320" t="inlineStr">
         <is>
           <t>PA44 - Parede em alvenaria emassada regularizada, revestida em massa acrílica texturizada cimento queimado, cor 107. Ref.: Terracor CQ. Amostra a ser aprovada pela GPA&amp;A.
-PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural caravalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
+PA32 - Parede em alvenaria emassada regularizada, revestida em mdf cru para regularização da superficie e acabamento em folha madeira natural carvalho tonalizado, acabamento. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural deve possuir certificação FSC ou CERFLOR
 PA33 - Pilar em alvenaria rebocada regularizada, revestida em pedra natural, Basaltina, acabamento frisado. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
@@ -11869,7 +11865,7 @@
       <c r="N27" s="307" t="n"/>
       <c r="O27" s="320" t="inlineStr">
         <is>
-          <t>D9 - Misturador Monocomando Monde Filter Plus em Aço Inox com Saída Adicional para Água Filtrada + Filtro 3M. Cód Ref.:  REF 94520025. Ref.: Tramontina. ATENÇÃO: vazão máxima de 9 l/min, instalar redutor de vazão se necessário</t>
+          <t>D9 - Misturador Monocomando Monde Filter Plus em Aço Inox com Saída Adicional para Água Filtrada + Filtro 3M. Cód Ref.: REF 94520025. Ref.: Tramontina. ATENÇÃO: vazão máxima de 9 l/min, instalar redutor de vazão se necessário</t>
         </is>
       </c>
       <c r="P27" s="300" t="n"/>
@@ -11886,7 +11882,7 @@
       <c r="W27" s="300" t="n"/>
       <c r="X27" s="308" t="inlineStr">
         <is>
-          <t>D11 - Porta pivotante estruturada, fechamento em  MDF cru, acabamento micro pintura face do kids cor S081-Sayerlack e acabamento face do gourmet em folha madeira natural caravalho tonalizado. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
+          <t>D11 - Porta pivotante estruturada, fechamento em MDF cru, acabamento micro pintura face do kids cor S081-Sayerlack e acabamento face do gourmet em folha madeira natural carvalho tonalizado. Batente em cantoneira metálica conforme detalhe. Dimensões e desenho conforme detalhamento. Puxador Round linha Texture, 90cm, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 D83 - Porta pivotante estruturada fechamento em madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador metálico tipo alça padrão Demuner. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
@@ -11894,9 +11890,9 @@
       <c r="Z27" s="307" t="inlineStr">
         <is>
           <t>D13 - Estante suspensa em tubo retangular 25x25mm em aço inox com pintura ouro velho. Fixada no teto através de estrutura auxiliar. Apresentar amostra pintura e solda para aprovação GPA&amp;A.
-D14 - Fechamento cego em mdf cru com acabamento em folha madeira natural caravalho tonalizado. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
+D14 - Fechamento cego em mdf cru com acabamento em folha madeira natural carvalho tonalizado. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
 D15 - Armários em mdf cru com acabamento em folha madeira natural carvalho tonalizado. Puxadore integrado linha Sottile ref. ZEN - acabamento bronze 192mm. Consultar detalhamento.Amostra folha natural madeira com acabamenhto deverá ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
-D16 - Mesa em mdf cru com acabamento em folha madeira natural caravalho tonalizado. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
+D16 - Mesa em mdf cru com acabamento em folha madeira natural carvalho tonalizado. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
 D17 - Armários em ripas de madeira maciça tonalizada seguindo cor folha madeira - ripas de 20x20mm espaçadas 15mm. Portas de giro com puxador no trespasse. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
@@ -11931,7 +11927,7 @@
       <c r="S28" s="300" t="n"/>
       <c r="T28" s="307" t="n"/>
       <c r="U28" s="300" t="n"/>
-      <c r="V28" s="302" t="n"/>
+      <c r="V28" s="320" t="n"/>
       <c r="W28" s="300" t="n"/>
       <c r="X28" s="300" t="n"/>
       <c r="Y28" s="300" t="n"/>
@@ -11940,12 +11936,12 @@
     <row r="29" ht="224" customHeight="1">
       <c r="A29" s="298" t="inlineStr">
         <is>
-          <t>PISCINA DECOBERTA</t>
+          <t>PISCINA DESCOBERTA</t>
         </is>
       </c>
       <c r="B29" s="320" t="inlineStr">
         <is>
-          <t>P18 - Piso revestido em pastilhas de mármore branco selecionado, lote a ser aprovado, acabamento levigado, 3x3cm.  Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Amostra a ser aprovada pela GPA&amp;A
+          <t>P18 - Piso revestido em pastilhas de mármore branco selecionado, lote a ser aprovado, acabamento levigado, 3x3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Amostra a ser aprovada pela GPA&amp;A
 P28 - Piso assentado em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
@@ -11956,7 +11952,7 @@
       <c r="G29" s="300" t="n"/>
       <c r="H29" s="320" t="inlineStr">
         <is>
-          <t>PA59 - Parede revestida em pastilha Jatobá, acabamento cinza cimento brilhante, 5x5cm. Cód.: CJC1614.. Ref.: Ceramicasa. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
+          <t>PA59 - Parede revestida em pastilha Jatobá, acabamento cinza cimento brilhante, 5x5cm. Cód.: CJC1614. Ref.: Ceramicasa. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
       <c r="I29" s="307" t="n"/>
@@ -11984,14 +11980,14 @@
           <t>D79 - Chuveiro de piso para área externa em aço inox 316. cód.: DK5123B. Ref.: Doka</t>
         </is>
       </c>
-      <c r="V29" s="302" t="n"/>
+      <c r="V29" s="320" t="n"/>
       <c r="W29" s="307" t="n"/>
       <c r="X29" s="307" t="inlineStr">
         <is>
           <t>D77 - Porta pivotante para guarda corpo em vidro temperado laminado liso incolor com tubo para pivô em aço inox polido 1 1/4'' fixado no piso com barra lisa soltada com rosca na extremidade para fixação do vidro com botão de acabamento.</t>
         </is>
       </c>
-      <c r="Y29" s="302" t="n"/>
+      <c r="Y29" s="320" t="n"/>
       <c r="Z29" s="307" t="inlineStr">
         <is>
           <t>D76 - Guarda corpo em vidro temperado laminado liso incolor embutido no piso com ancoragem mínima de 70mm através de perfil fixador em aço inox e espaçamento entre vidros de 30mm.</t>
@@ -12006,7 +12002,7 @@
       </c>
       <c r="B30" s="320" t="inlineStr">
         <is>
-          <t>P26 - Piso em deck de madeira Cumaru com tecnica de carbonização Shugi Ban, reguas 20mmx100mmx2000m-acima. Ref.:Madeira Carbonizada.  ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
+          <t>P26 - Piso em deck de madeira Cumaru com tecnica de carbonização Shugi Ban, reguas 20mmx100mmx2000m-acima. Ref.: Madeira Carbonizada. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="C30" s="300" t="n"/>
@@ -12028,10 +12024,10 @@
       <c r="S30" s="300" t="n"/>
       <c r="T30" s="300" t="n"/>
       <c r="U30" s="300" t="n"/>
-      <c r="V30" s="302" t="n"/>
+      <c r="V30" s="320" t="n"/>
       <c r="W30" s="307" t="n"/>
-      <c r="X30" s="302" t="n"/>
-      <c r="Y30" s="302" t="n"/>
+      <c r="X30" s="320" t="n"/>
+      <c r="Y30" s="320" t="n"/>
       <c r="Z30" s="307" t="n"/>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -12060,7 +12056,7 @@
       <c r="S31" s="300" t="n"/>
       <c r="T31" s="300" t="n"/>
       <c r="U31" s="300" t="n"/>
-      <c r="V31" s="302" t="n"/>
+      <c r="V31" s="320" t="n"/>
       <c r="W31" s="300" t="n"/>
       <c r="X31" s="300" t="n"/>
       <c r="Y31" s="300" t="n"/>
@@ -12074,7 +12070,7 @@
       </c>
       <c r="B32" s="307" t="inlineStr">
         <is>
-          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
+          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
       <c r="C32" s="300" t="n"/>
@@ -12094,7 +12090,7 @@
       </c>
       <c r="I32" s="307" t="inlineStr">
         <is>
-          <t>T4 - Forro em madeira pinho autoclavado tonalizado, espessura de 3cm, réguas de 10cm.  ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR
+          <t>T4 - Forro em madeira pinho autoclavado tonalizado, espessura de 3cm, réguas de 10cm. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR
 T1 - Forro em gesso acartonado liso, com acabamento em tinta acrílica, cor branco neve, acabamento fosco, com junta dilatação metálica cor branca. Ref.: Suvinil</t>
         </is>
       </c>
@@ -12113,7 +12109,7 @@
       <c r="N32" s="300" t="n"/>
       <c r="O32" s="308" t="inlineStr">
         <is>
-          <t>D9 - Misturador Monocomando Monde Filter Plus em Aço Inox com Saída Adicional para Água Filtrada + Filtro 3M. Cód Ref.:  REF 94520025. Ref.: Tramontina. ATENÇÃO: vazão máxima de 9 l/min, instalar redutor de vazão se necessário</t>
+          <t>D9 - Misturador Monocomando Monde Filter Plus em Aço Inox com Saída Adicional para Água Filtrada + Filtro 3M. Cód Ref.: REF 94520025. Ref.: Tramontina. ATENÇÃO: vazão máxima de 9 l/min, instalar redutor de vazão se necessário</t>
         </is>
       </c>
       <c r="P32" s="300" t="n"/>
@@ -12133,13 +12129,13 @@
         </is>
       </c>
       <c r="W32" s="307" t="n"/>
-      <c r="X32" s="302" t="n"/>
-      <c r="Y32" s="302" t="n"/>
+      <c r="X32" s="320" t="n"/>
+      <c r="Y32" s="320" t="n"/>
       <c r="Z32" s="307" t="inlineStr">
         <is>
           <t>D47 - Marcenaria sob bancada em MDF Kashimir ref. Arauco - portas e frente gavetas em reguas de madeira maciça engenheirada reflorestada, tonalizada. Acabamento superfície escovada. Painel Bark. Ref.: Demuner. Puxador em cava na marcenaria. Apresentar amostra para aprovação GPA&amp;A Obs.: MDF possui certificação FSC. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR
 D48 - Estante suspensa em tubo retangular 25x25mm em aço inox com pintura ouro velho. Fixada no teto através de estrutura auxiliar. Apresentar amostra pintura e solda para aprovação GPA&amp;A.
-D49 - Armários com interior em MDF madeirado e portas de giro ripadas -  ripas de 20x20mm espaçadas 15mm - puxador executado na marcenaria - prever fechamento face interna porta em vidro liso incolor 4mm. Prateleiras em MDF madeirado com iluminação em LED. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
+D49 - Armários com interior em MDF madeirado e portas de giro ripadas - ripas de 20x20mm espaçadas 15mm - puxador executado na marcenaria - prever fechamento face interna porta em vidro liso incolor 4mm. Prateleiras em MDF madeirado com iluminação em LED. Dimensões e desenho conforme detalhamento.Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
 D50 - Armário sob bancada com portas de giro ripadas para ventilação choppeira. Ripas de 20x20mm espaçadas 15mm - puxador executado na marcenaria. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
@@ -12168,13 +12164,13 @@
       <c r="M33" s="308" t="n"/>
       <c r="N33" s="308" t="n"/>
       <c r="O33" s="307" t="n"/>
-      <c r="P33" s="302" t="n"/>
+      <c r="P33" s="320" t="n"/>
       <c r="Q33" s="300" t="n"/>
       <c r="R33" s="307" t="n"/>
       <c r="S33" s="307" t="n"/>
       <c r="T33" s="307" t="n"/>
       <c r="U33" s="300" t="n"/>
-      <c r="V33" s="302" t="n"/>
+      <c r="V33" s="320" t="n"/>
       <c r="W33" s="307" t="n"/>
       <c r="X33" s="307" t="n"/>
       <c r="Y33" s="307" t="n"/>
@@ -12188,7 +12184,7 @@
       </c>
       <c r="B34" s="307" t="inlineStr">
         <is>
-          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
+          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
       <c r="C34" s="300" t="n"/>
@@ -12212,7 +12208,7 @@
       <c r="M34" s="308" t="n"/>
       <c r="N34" s="308" t="n"/>
       <c r="O34" s="307" t="n"/>
-      <c r="P34" s="302" t="n"/>
+      <c r="P34" s="320" t="n"/>
       <c r="Q34" s="300" t="n"/>
       <c r="R34" s="307" t="n"/>
       <c r="S34" s="307" t="n"/>
@@ -12236,7 +12232,7 @@
       </c>
       <c r="B35" s="320" t="inlineStr">
         <is>
-          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
+          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
       <c r="C35" s="300" t="n"/>
@@ -12276,7 +12272,7 @@
       <c r="N35" s="308" t="n"/>
       <c r="O35" s="321" t="inlineStr">
         <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
 CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
@@ -12300,7 +12296,7 @@
       </c>
       <c r="U35" s="317" t="inlineStr">
         <is>
-          <t>D31 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
+          <t>D31 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
       <c r="V35" s="307" t="inlineStr">
@@ -12326,12 +12322,12 @@
     <row r="36" ht="224" customHeight="1">
       <c r="A36" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">VESTIÁRIO MASCULINO </t>
+          <t>VESTIÁRIO MASCULINO</t>
         </is>
       </c>
       <c r="B36" s="320" t="inlineStr">
         <is>
-          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado.  Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
+          <t>P9 - Piso assentado em granito cinza Santa Rosa, acabamento serrado. Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
       <c r="C36" s="300" t="n"/>
@@ -12371,7 +12367,7 @@
       <c r="N36" s="308" t="n"/>
       <c r="O36" s="321" t="inlineStr">
         <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
 CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
@@ -12395,7 +12391,7 @@
       </c>
       <c r="U36" s="317" t="inlineStr">
         <is>
-          <t>D31 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
+          <t>D31 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
       <c r="V36" s="307" t="inlineStr">
@@ -12442,7 +12438,7 @@
       <c r="H37" s="320" t="inlineStr">
         <is>
           <t>PA26 - Parede em alvenaria rebocada e regularizada revestida em espelho liso incolor 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
-PA27 - Parede em alvenaria rebocada e regularizada revestida em espelho liso fumê 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
+PA27 - Parede em alvenaria rebocada e regularizada revestida em espelho liso fumê 4mm colado sobre MDF cru 6mm aparafusado na alvenaria. Paginação e dimensões conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: o MDF deve possuir certificação FSC ou CERFLOR
 PA28 - Parede em alvenaria rebocada e regularizada revestida em painel de MDF Nero Rust. Paginação conforme detalhamento. Ref.: Berneck. Amostra a ser aprovada pela GPA&amp;A. Obs.: MDF possui certificação FSC.
 PA29 - Fechamento vertical estruturado com acabamento em painel de MDF Nero Rust. Paginação conforme detalhamento. Ref.: Berneck. Amostra a ser aprovada pela GPA&amp;A. Obs.: MDF possui certificação FSC.
 PA30 - Pilar em concreto com acabamento em textura mineral Arch + Concrete ENG, Ref.: Novacolor. Fornecedor: Icolori (31)99952-2442. Amostra a ser aprovada pela GPA&amp;A</t>
@@ -12460,7 +12456,7 @@
       <c r="M37" s="308" t="n"/>
       <c r="N37" s="308" t="n"/>
       <c r="O37" s="307" t="n"/>
-      <c r="P37" s="302" t="n"/>
+      <c r="P37" s="320" t="n"/>
       <c r="Q37" s="300" t="n"/>
       <c r="R37" s="307" t="n"/>
       <c r="S37" s="307" t="n"/>
@@ -12481,7 +12477,7 @@
       <c r="Z37" s="308" t="inlineStr">
         <is>
           <t>D3 - Estante em MDF Nero Rust Ref.: Berneck, desenho conforme detalhamento, Amostra a ser aprovada pela GPA&amp;A. Obs.: MDF possui certificação FSC.
-D4 - Armário em marcenaria, estruturado, com espaço para central de sonorização e automação, quadro de distribuição embutido - verificar dimensões com projetos específico, desenho conforme detalhamento. Porta.  de giro com sistema fecho-toque, acabamento em MDF Nero Rust. Ref.: Berneck. Obs.: MDF possui certificação FSC.
+D4 - Armário em marcenaria, estruturado, com espaço para central de sonorização e automação, quadro de distribuição embutido - verificar dimensões com projetos específico, desenho conforme detalhamento. Porta. de giro com sistema fecho-toque, acabamento em MDF Nero Rust. Ref.: Berneck. Obs.: MDF possui certificação FSC.
 D5 - Painel estruturado com moldura, para encaixe de equipamento, desenho conforme detalhamento, acabamento em MDF Nero Rust. Ref.: Berneck. Obs.: MDF possui certificação FSC.
 D6 - Anéis metálicos acabamento em micropintura perolizada, cor L098, Ref.: Sherwin Williams, fixados em pilar de concreto através de espassadores metálicos. Ver detalhamento. Apresentar protótipo e amostra pintura para aprovação GPA&amp;A.
 D7 - Mesa de apoio metálica em micropintura perolizada, cor L098, Ref.: Sherwin Williams, fixados em pilar de concreto através de estrutura auxiliar. Ver detalhamento. Apresentar protótipo e amostra pintura para aprovação GPA&amp;A.</t>
@@ -12491,7 +12487,7 @@
     <row r="38" ht="134" customHeight="1">
       <c r="A38" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">CIRCULAÇÃO JARDINS </t>
+          <t>CIRCULAÇÃO JARDINS</t>
         </is>
       </c>
       <c r="B38" s="307" t="inlineStr">
@@ -12512,13 +12508,13 @@
       <c r="M38" s="308" t="n"/>
       <c r="N38" s="308" t="n"/>
       <c r="O38" s="307" t="n"/>
-      <c r="P38" s="302" t="n"/>
+      <c r="P38" s="320" t="n"/>
       <c r="Q38" s="300" t="n"/>
       <c r="R38" s="307" t="n"/>
       <c r="S38" s="307" t="n"/>
       <c r="T38" s="307" t="n"/>
       <c r="U38" s="300" t="n"/>
-      <c r="V38" s="302" t="n"/>
+      <c r="V38" s="320" t="n"/>
       <c r="W38" s="307" t="n"/>
       <c r="X38" s="307" t="n"/>
       <c r="Y38" s="307" t="n"/>
@@ -12552,13 +12548,13 @@
       <c r="M39" s="308" t="n"/>
       <c r="N39" s="308" t="n"/>
       <c r="O39" s="307" t="n"/>
-      <c r="P39" s="302" t="n"/>
+      <c r="P39" s="320" t="n"/>
       <c r="Q39" s="300" t="n"/>
       <c r="R39" s="307" t="n"/>
       <c r="S39" s="307" t="n"/>
       <c r="T39" s="307" t="n"/>
       <c r="U39" s="300" t="n"/>
-      <c r="V39" s="302" t="n"/>
+      <c r="V39" s="320" t="n"/>
       <c r="W39" s="307" t="n"/>
       <c r="X39" s="307" t="n"/>
       <c r="Y39" s="307" t="n"/>
@@ -12567,12 +12563,12 @@
     <row r="40" ht="89" customHeight="1">
       <c r="A40" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPA </t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="B40" s="320" t="inlineStr">
         <is>
-          <t>P18 - Piso revestido em pastilhas de mármore branco selecionado, lote a ser aprovado, acabamento levigado, 3x3cm.  Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Amostra a ser aprovada pela GPA&amp;A</t>
+          <t>P18 - Piso revestido em pastilhas de mármore branco selecionado, lote a ser aprovado, acabamento levigado, 3x3cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Amostra a ser aprovada pela GPA&amp;A</t>
         </is>
       </c>
       <c r="C40" s="300" t="n"/>
@@ -12592,13 +12588,13 @@
       <c r="M40" s="308" t="n"/>
       <c r="N40" s="308" t="n"/>
       <c r="O40" s="307" t="n"/>
-      <c r="P40" s="302" t="n"/>
+      <c r="P40" s="320" t="n"/>
       <c r="Q40" s="300" t="n"/>
       <c r="R40" s="307" t="n"/>
       <c r="S40" s="307" t="n"/>
       <c r="T40" s="307" t="n"/>
       <c r="U40" s="300" t="n"/>
-      <c r="V40" s="302" t="n"/>
+      <c r="V40" s="320" t="n"/>
       <c r="W40" s="307" t="n"/>
       <c r="X40" s="307" t="n"/>
       <c r="Y40" s="307" t="n"/>
@@ -12629,7 +12625,7 @@
         <is>
           <t>PA46 - Parede em alvenaria rebocada regularizada revestida em mármore branco selecionado, lote a ser aprovado. Espessura:2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A.
 PA48 - Parede rebocada e regularizada revestida em mármore branco selecionado, lote a ser aprovado, acabamento frisado com ranhuras de 4x4mm espassada a cada 12mm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A
-PA49 - Pilar em concreto rebocados e regularizados revestidos em mosaico de pastilhas, módulos de 32x259cm com pastilhas de 20x20mm, NARCISO Shading BlendDesenho e paginação conforme detalhamento. Argamassa e rejunte recomendados: Filgel plus 1101 bianco alabastro. Ref.:Bisazza. Amostra a ser aprovada pela GPA&amp;A
+PA49 - Pilar em concreto rebocados e regularizados revestidos em mosaico de pastilhas, módulos de 32x259cm com pastilhas de 20x20mm, NARCISO Shading BlendDesenho e paginação conforme detalhamento. Argamassa e rejunte recomendados: Filgel plus 1101 bianco alabastro. Ref.: Bisazza. Amostra a ser aprovada pela GPA&amp;A
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
@@ -12645,7 +12641,7 @@
       <c r="M41" s="308" t="n"/>
       <c r="N41" s="308" t="n"/>
       <c r="O41" s="307" t="n"/>
-      <c r="P41" s="302" t="n"/>
+      <c r="P41" s="320" t="n"/>
       <c r="Q41" s="300" t="n"/>
       <c r="R41" s="307" t="inlineStr">
         <is>
@@ -12672,7 +12668,7 @@
       <c r="W41" s="307" t="n"/>
       <c r="X41" s="307" t="inlineStr">
         <is>
-          <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y41" s="307" t="n"/>
@@ -12699,7 +12695,7 @@
     <row r="42" ht="89" customHeight="1">
       <c r="A42" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAUNA VAPOR </t>
+          <t>SAUNA VAPOR</t>
         </is>
       </c>
       <c r="B42" s="320" t="inlineStr">
@@ -12728,7 +12724,7 @@
       <c r="M42" s="308" t="n"/>
       <c r="N42" s="308" t="n"/>
       <c r="O42" s="307" t="n"/>
-      <c r="P42" s="302" t="n"/>
+      <c r="P42" s="320" t="n"/>
       <c r="Q42" s="300" t="n"/>
       <c r="R42" s="307" t="inlineStr">
         <is>
@@ -12746,7 +12742,7 @@
           <t>D54 - Chuveiro de embutir no teto Raindream, Roca, acabamento cromado, cód.: A5B3250C0C. Ref.: Roca. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
-      <c r="V42" s="302" t="n"/>
+      <c r="V42" s="320" t="n"/>
       <c r="W42" s="307" t="n"/>
       <c r="X42" s="307" t="n"/>
       <c r="Y42" s="307" t="n"/>
@@ -12760,7 +12756,7 @@
       </c>
       <c r="B43" s="320" t="inlineStr">
         <is>
-          <t>P19 - Piso em contrapiso regularizado revestido com porcelanato padrão, coberto com piso tipo deck de madeira Cedro.Reguas 70mmx25mmx comprimento variável e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
+          <t>P19 - Piso em contrapiso regularizado revestido com porcelanato padrão, coberto com piso tipo deck de madeira Cedro.Reguas 70mmx25mmx comprimento variável e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="C43" s="300" t="n"/>
@@ -12775,7 +12771,7 @@
       </c>
       <c r="I43" s="320" t="inlineStr">
         <is>
-          <t>T11 - Laje em concreto revestida em  conjunto com sarrafos de madeira 2,5x5cm a cada 35-40cm, lã de vidro 2,5cm de espessura e fechamento em réguas de madeira Cedro. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A.  ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
+          <t>T11 - Laje em concreto revestida em conjunto com sarrafos de madeira 2,5x5cm a cada 35-40cm, lã de vidro 2,5cm de espessura e fechamento em réguas de madeira Cedro. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="J43" s="307" t="n"/>
@@ -12784,13 +12780,13 @@
       <c r="M43" s="308" t="n"/>
       <c r="N43" s="308" t="n"/>
       <c r="O43" s="307" t="n"/>
-      <c r="P43" s="302" t="n"/>
+      <c r="P43" s="320" t="n"/>
       <c r="Q43" s="300" t="n"/>
       <c r="R43" s="307" t="n"/>
       <c r="S43" s="307" t="n"/>
       <c r="T43" s="307" t="n"/>
       <c r="U43" s="300" t="n"/>
-      <c r="V43" s="302" t="n"/>
+      <c r="V43" s="320" t="n"/>
       <c r="W43" s="307" t="n"/>
       <c r="X43" s="307" t="n"/>
       <c r="Y43" s="307" t="n"/>
@@ -12816,13 +12812,13 @@
       <c r="M44" s="308" t="n"/>
       <c r="N44" s="308" t="n"/>
       <c r="O44" s="307" t="n"/>
-      <c r="P44" s="302" t="n"/>
+      <c r="P44" s="320" t="n"/>
       <c r="Q44" s="300" t="n"/>
       <c r="R44" s="307" t="n"/>
       <c r="S44" s="307" t="n"/>
       <c r="T44" s="307" t="n"/>
       <c r="U44" s="300" t="n"/>
-      <c r="V44" s="302" t="n"/>
+      <c r="V44" s="320" t="n"/>
       <c r="W44" s="307" t="n"/>
       <c r="X44" s="307" t="n"/>
       <c r="Y44" s="307" t="n"/>
@@ -12831,7 +12827,7 @@
     <row r="45" ht="344" customHeight="1">
       <c r="A45" s="298" t="inlineStr">
         <is>
-          <t xml:space="preserve">MASSAGEM </t>
+          <t>MASSAGEM</t>
         </is>
       </c>
       <c r="B45" s="320" t="inlineStr">
@@ -12879,10 +12875,10 @@
       <c r="O45" s="320" t="inlineStr">
         <is>
           <t>D51 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-D53 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
-        </is>
-      </c>
-      <c r="P45" s="302" t="n"/>
+D53 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
+        </is>
+      </c>
+      <c r="P45" s="320" t="n"/>
       <c r="Q45" s="300" t="n"/>
       <c r="R45" s="307" t="n"/>
       <c r="S45" s="307" t="n"/>
@@ -12896,7 +12892,7 @@
       <c r="W45" s="307" t="n"/>
       <c r="X45" s="320" t="inlineStr">
         <is>
-          <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y45" s="307" t="n"/>
@@ -12953,10 +12949,10 @@
       <c r="O46" s="320" t="inlineStr">
         <is>
           <t>D51 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
-D53 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
-        </is>
-      </c>
-      <c r="P46" s="302" t="n"/>
+D53 - Torneira de mesa, linha Mix&amp;Match Presence, com sensor, acabamento grafite escovado. Cód.: 90015460070 Ref.: Docol ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.</t>
+        </is>
+      </c>
+      <c r="P46" s="320" t="n"/>
       <c r="Q46" s="300" t="n"/>
       <c r="R46" s="307" t="n"/>
       <c r="S46" s="307" t="n"/>
@@ -12970,7 +12966,7 @@
       <c r="W46" s="307" t="n"/>
       <c r="X46" s="307" t="inlineStr">
         <is>
-          <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y46" s="307" t="n"/>
@@ -13013,18 +13009,18 @@
       <c r="M47" s="308" t="n"/>
       <c r="N47" s="308" t="n"/>
       <c r="O47" s="307" t="n"/>
-      <c r="P47" s="302" t="n"/>
+      <c r="P47" s="320" t="n"/>
       <c r="Q47" s="300" t="n"/>
       <c r="R47" s="307" t="n"/>
       <c r="S47" s="307" t="n"/>
       <c r="T47" s="307" t="n"/>
       <c r="U47" s="300" t="n"/>
-      <c r="V47" s="302" t="n"/>
+      <c r="V47" s="320" t="n"/>
       <c r="W47" s="307" t="n"/>
       <c r="X47" s="307" t="inlineStr">
         <is>
-          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
-D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
+D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y47" s="307" t="n"/>
@@ -13068,7 +13064,7 @@
       </c>
       <c r="K48" s="308" t="inlineStr">
         <is>
-          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
+          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural carvalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="L48" s="307" t="inlineStr">
@@ -13106,7 +13102,7 @@
       </c>
       <c r="U48" s="308" t="inlineStr">
         <is>
-          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
+          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
       <c r="V48" s="307" t="inlineStr">
@@ -13163,7 +13159,7 @@
       </c>
       <c r="K49" s="308" t="inlineStr">
         <is>
-          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
+          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural carvalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="L49" s="307" t="inlineStr">
@@ -13201,7 +13197,7 @@
       </c>
       <c r="U49" s="308" t="inlineStr">
         <is>
-          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
+          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.</t>
         </is>
       </c>
       <c r="V49" s="307" t="inlineStr">
@@ -13264,13 +13260,13 @@
           <t>D67 - Torneira de parede com arejador, para Jardim e Tanque, linha Izy, acabamento cromado. Cód. 1154.C37; Ref.: Deca.</t>
         </is>
       </c>
-      <c r="P50" s="302" t="n"/>
+      <c r="P50" s="320" t="n"/>
       <c r="Q50" s="300" t="n"/>
       <c r="R50" s="307" t="n"/>
       <c r="S50" s="307" t="n"/>
       <c r="T50" s="307" t="n"/>
       <c r="U50" s="300" t="n"/>
-      <c r="V50" s="302" t="n"/>
+      <c r="V50" s="320" t="n"/>
       <c r="W50" s="307" t="n"/>
       <c r="X50" s="307" t="n"/>
       <c r="Y50" s="307" t="n"/>
@@ -13296,13 +13292,13 @@
       <c r="M51" s="308" t="n"/>
       <c r="N51" s="308" t="n"/>
       <c r="O51" s="307" t="n"/>
-      <c r="P51" s="302" t="n"/>
+      <c r="P51" s="320" t="n"/>
       <c r="Q51" s="300" t="n"/>
       <c r="R51" s="307" t="n"/>
       <c r="S51" s="307" t="n"/>
       <c r="T51" s="307" t="n"/>
       <c r="U51" s="300" t="n"/>
-      <c r="V51" s="302" t="n"/>
+      <c r="V51" s="320" t="n"/>
       <c r="W51" s="307" t="n"/>
       <c r="X51" s="307" t="n"/>
       <c r="Y51" s="307" t="n"/>
@@ -13342,13 +13338,13 @@
       <c r="M52" s="308" t="n"/>
       <c r="N52" s="308" t="n"/>
       <c r="O52" s="307" t="n"/>
-      <c r="P52" s="302" t="n"/>
+      <c r="P52" s="320" t="n"/>
       <c r="Q52" s="300" t="n"/>
       <c r="R52" s="307" t="n"/>
       <c r="S52" s="307" t="n"/>
       <c r="T52" s="307" t="n"/>
       <c r="U52" s="300" t="n"/>
-      <c r="V52" s="302" t="n"/>
+      <c r="V52" s="320" t="n"/>
       <c r="W52" s="307" t="n"/>
       <c r="X52" s="307" t="n"/>
       <c r="Y52" s="307" t="n"/>
@@ -13378,7 +13374,7 @@
       <c r="G53" s="300" t="n"/>
       <c r="H53" s="320" t="inlineStr">
         <is>
-          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali pff white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII
+          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali off white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII
 01| 21 - Pintura acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil, sobre paredes - Reboco (1 demão selador + 3 demãos Latex acrílico)
 ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
@@ -13411,13 +13407,13 @@
           <t>27 - Torneira de parede com arejador, para jardim e tanque, cromado. Ref.: cód.:1154.C37; linha Izy; Deca</t>
         </is>
       </c>
-      <c r="P53" s="302" t="n"/>
+      <c r="P53" s="320" t="n"/>
       <c r="Q53" s="300" t="n"/>
       <c r="R53" s="307" t="n"/>
       <c r="S53" s="307" t="n"/>
       <c r="T53" s="307" t="n"/>
       <c r="U53" s="300" t="n"/>
-      <c r="V53" s="302" t="n"/>
+      <c r="V53" s="320" t="n"/>
       <c r="W53" s="307" t="n"/>
       <c r="X53" s="307" t="n"/>
       <c r="Y53" s="307" t="n"/>
@@ -13447,7 +13443,7 @@
       <c r="G54" s="300" t="n"/>
       <c r="H54" s="320" t="inlineStr">
         <is>
-          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali pff white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII
+          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali off white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII
 01| 21 - Pintura acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil, sobre paredes - Reboco (1 demão selador + 3 demãos Latex acrílico)
 ARQ-PA01 - Parede em alvenaria, emassada e regularizada, pintada com tinta acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil.</t>
         </is>
@@ -13480,13 +13476,13 @@
           <t>27 - Torneira de parede com arejador, para jardim e tanque, cromado. Ref.: cód.:1154.C37; linha Izy; Deca</t>
         </is>
       </c>
-      <c r="P54" s="302" t="n"/>
+      <c r="P54" s="320" t="n"/>
       <c r="Q54" s="300" t="n"/>
       <c r="R54" s="307" t="n"/>
       <c r="S54" s="307" t="n"/>
       <c r="T54" s="307" t="n"/>
       <c r="U54" s="300" t="n"/>
-      <c r="V54" s="302" t="n"/>
+      <c r="V54" s="320" t="n"/>
       <c r="W54" s="307" t="n"/>
       <c r="X54" s="307" t="n"/>
       <c r="Y54" s="307" t="n"/>
@@ -13534,7 +13530,7 @@
       </c>
       <c r="K55" s="317" t="inlineStr">
         <is>
-          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural caravalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
+          <t>D38 - Armário em MDF cru e acabamento em folha madeira natural carvalho tonalizado, com portas em espelho liso incolor, polimento cristal 4mm colado sobre MDF cru 12mm com acabamento das bordas em cantoneiras em aço inox polido. Dimensões e desenho conforme detalhamento. ATENÇÃO: o MDF e a lâmina natural devem possuir certificação FSC ou CERFLOR
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
@@ -13574,7 +13570,7 @@
       </c>
       <c r="U55" s="317" t="inlineStr">
         <is>
-          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol.  ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.
+          <t>D70 - Chuveiro 200 de parede, com tubo reto, linha DocolEden, acabamento cromado, cód.:90008879006. Ref.: Docol. ATENÇÃO: vazão máxima de 8 l/min, instalar restritor de vazão se necessário.
 ► VER IMAGEM (clique)</t>
         </is>
       </c>
@@ -13586,8 +13582,8 @@
       <c r="W55" s="307" t="n"/>
       <c r="X55" s="307" t="inlineStr">
         <is>
-          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture,  com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
-D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura,  acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
+          <t>D39 - Porta estruturada em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.
+D43 - Painel e porta estruturados em alumínio com fechamento interno e externo em vidro, cor Prada, acabamento acidato. Dimensões conforme detalhamento. Ref.: Cinex. Puxador Round linha Texture, 90cm com fechadura, acabamento cromado acetinado. Ref.: La Fonte, Amostra a ser aprovada pela GPA&amp;A.</t>
         </is>
       </c>
       <c r="Y55" s="307" t="n"/>
@@ -13685,13 +13681,13 @@
       <c r="M56" s="308" t="n"/>
       <c r="N56" s="308" t="n"/>
       <c r="O56" s="320" t="n"/>
-      <c r="P56" s="302" t="n"/>
+      <c r="P56" s="320" t="n"/>
       <c r="Q56" s="300" t="n"/>
       <c r="R56" s="307" t="n"/>
       <c r="S56" s="307" t="n"/>
       <c r="T56" s="307" t="n"/>
       <c r="U56" s="300" t="n"/>
-      <c r="V56" s="302" t="n"/>
+      <c r="V56" s="320" t="n"/>
       <c r="W56" s="307" t="n"/>
       <c r="X56" s="307" t="n"/>
       <c r="Y56" s="307" t="n"/>
@@ -13737,13 +13733,13 @@
       <c r="M57" s="308" t="n"/>
       <c r="N57" s="308" t="n"/>
       <c r="O57" s="320" t="n"/>
-      <c r="P57" s="302" t="n"/>
+      <c r="P57" s="320" t="n"/>
       <c r="Q57" s="300" t="n"/>
       <c r="R57" s="307" t="n"/>
       <c r="S57" s="307" t="n"/>
       <c r="T57" s="307" t="n"/>
       <c r="U57" s="300" t="n"/>
-      <c r="V57" s="302" t="n"/>
+      <c r="V57" s="320" t="n"/>
       <c r="W57" s="307" t="n"/>
       <c r="X57" s="307" t="n"/>
       <c r="Y57" s="307" t="n"/>
@@ -13793,7 +13789,7 @@
       <c r="M58" s="308" t="n"/>
       <c r="N58" s="308" t="n"/>
       <c r="O58" s="320" t="n"/>
-      <c r="P58" s="302" t="n"/>
+      <c r="P58" s="320" t="n"/>
       <c r="Q58" s="300" t="n"/>
       <c r="R58" s="307" t="n"/>
       <c r="S58" s="307" t="n"/>
@@ -13818,7 +13814,7 @@
       <c r="B59" s="320" t="inlineStr">
         <is>
           <t>P28 - Piso assentado em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.
-P8 - Piso elevado em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofulgante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
+P8 - Piso elevado em granito cinza Santa Rosa, acabamento serrado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.</t>
         </is>
       </c>
       <c r="C59" s="300" t="n"/>
@@ -13834,7 +13830,7 @@
       <c r="M59" s="308" t="n"/>
       <c r="N59" s="308" t="n"/>
       <c r="O59" s="320" t="n"/>
-      <c r="P59" s="302" t="n"/>
+      <c r="P59" s="320" t="n"/>
       <c r="Q59" s="300" t="n"/>
       <c r="R59" s="307" t="n"/>
       <c r="S59" s="307" t="n"/>
@@ -13844,7 +13840,7 @@
         </is>
       </c>
       <c r="U59" s="300" t="n"/>
-      <c r="V59" s="302" t="n"/>
+      <c r="V59" s="320" t="n"/>
       <c r="W59" s="307" t="n"/>
       <c r="X59" s="307" t="n"/>
       <c r="Y59" s="307" t="n"/>
@@ -13878,13 +13874,13 @@
       <c r="M60" s="308" t="n"/>
       <c r="N60" s="308" t="n"/>
       <c r="O60" s="320" t="n"/>
-      <c r="P60" s="302" t="n"/>
+      <c r="P60" s="320" t="n"/>
       <c r="Q60" s="300" t="n"/>
       <c r="R60" s="307" t="n"/>
       <c r="S60" s="307" t="n"/>
       <c r="T60" s="307" t="n"/>
       <c r="U60" s="300" t="n"/>
-      <c r="V60" s="302" t="n"/>
+      <c r="V60" s="320" t="n"/>
       <c r="W60" s="307" t="n"/>
       <c r="X60" s="307" t="n"/>
       <c r="Y60" s="307" t="n"/>
@@ -13919,13 +13915,13 @@
       <c r="M61" s="308" t="n"/>
       <c r="N61" s="308" t="n"/>
       <c r="O61" s="320" t="n"/>
-      <c r="P61" s="302" t="n"/>
+      <c r="P61" s="320" t="n"/>
       <c r="Q61" s="300" t="n"/>
       <c r="R61" s="307" t="n"/>
       <c r="S61" s="307" t="n"/>
       <c r="T61" s="307" t="n"/>
       <c r="U61" s="300" t="n"/>
-      <c r="V61" s="302" t="n"/>
+      <c r="V61" s="320" t="n"/>
       <c r="W61" s="307" t="n"/>
       <c r="X61" s="307" t="n"/>
       <c r="Y61" s="307" t="n"/>
@@ -13961,13 +13957,13 @@
       <c r="M62" s="308" t="n"/>
       <c r="N62" s="308" t="n"/>
       <c r="O62" s="320" t="n"/>
-      <c r="P62" s="302" t="n"/>
+      <c r="P62" s="320" t="n"/>
       <c r="Q62" s="300" t="n"/>
       <c r="R62" s="307" t="n"/>
       <c r="S62" s="307" t="n"/>
       <c r="T62" s="307" t="n"/>
       <c r="U62" s="300" t="n"/>
-      <c r="V62" s="302" t="n"/>
+      <c r="V62" s="320" t="n"/>
       <c r="W62" s="307" t="n"/>
       <c r="X62" s="307" t="n"/>
       <c r="Y62" s="307" t="n"/>
@@ -13982,7 +13978,7 @@
       <c r="B63" s="320" t="inlineStr">
         <is>
           <t>P7 - Piso assentado em granito cinza Santa Rosa, acabamento escovado, Espessura: 2cm. Dimensões e paginação conforme detalhamento. Rejunte em massa plástica a ser tonalizada de acordo com a cor da pedra. Amostra a ser aprovada pela GPA&amp;A. Obs.: Resina, hidrofugante ou outros acabamentos aplicados no granito devem ser foscos e não podem alterar ou escurecer a cor original do material.
-P27 - Piso em deck de madeira, modelo Tauari Teak encaixe macho e femea, acabamento com cavilha, reguas 20mmx100mmx2000m-acima. Ref.: Indusparquet.  ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
+P27 - Piso em deck de madeira, modelo Tauari Teak encaixe macho e femea, acabamento com cavilha, reguas 20mmx100mmx2000m-acima. Ref.: Indusparquet. ATENÇÃO: a madeira deve possuir certificação FSC ou CERFLOR</t>
         </is>
       </c>
       <c r="C63" s="300" t="n"/>
@@ -14003,13 +13999,13 @@
       <c r="M63" s="308" t="n"/>
       <c r="N63" s="308" t="n"/>
       <c r="O63" s="320" t="n"/>
-      <c r="P63" s="302" t="n"/>
+      <c r="P63" s="320" t="n"/>
       <c r="Q63" s="300" t="n"/>
       <c r="R63" s="307" t="n"/>
       <c r="S63" s="307" t="n"/>
       <c r="T63" s="307" t="n"/>
       <c r="U63" s="300" t="n"/>
-      <c r="V63" s="302" t="n"/>
+      <c r="V63" s="320" t="n"/>
       <c r="W63" s="307" t="n"/>
       <c r="X63" s="307" t="n"/>
       <c r="Y63" s="307" t="n"/>
@@ -14047,13 +14043,13 @@
       <c r="M64" s="308" t="n"/>
       <c r="N64" s="308" t="n"/>
       <c r="O64" s="320" t="n"/>
-      <c r="P64" s="302" t="n"/>
+      <c r="P64" s="320" t="n"/>
       <c r="Q64" s="300" t="n"/>
       <c r="R64" s="307" t="n"/>
       <c r="S64" s="307" t="n"/>
       <c r="T64" s="307" t="n"/>
       <c r="U64" s="300" t="n"/>
-      <c r="V64" s="302" t="n"/>
+      <c r="V64" s="320" t="n"/>
       <c r="W64" s="307" t="n"/>
       <c r="X64" s="307" t="n"/>
       <c r="Y64" s="307" t="n"/>
@@ -14830,8 +14826,8 @@
       <c r="U13" s="300" t="n"/>
       <c r="V13" s="300" t="n"/>
       <c r="W13" s="300" t="n"/>
-      <c r="X13" s="302" t="n"/>
-      <c r="Y13" s="302" t="n"/>
+      <c r="X13" s="320" t="n"/>
+      <c r="Y13" s="320" t="n"/>
       <c r="Z13" s="300" t="inlineStr">
         <is>
           <t>Varanda: mureta h=90cm. (DET PR001)</t>
@@ -14911,12 +14907,12 @@
           <t>Maçaneta Pado Sara, cromo acetinado, interna. (DET PR004)</t>
         </is>
       </c>
-      <c r="X14" s="302" t="inlineStr">
+      <c r="X14" s="320" t="inlineStr">
         <is>
           <t>Porta piso-forro, cor branca, alizar 10cm. (DET PR004)</t>
         </is>
       </c>
-      <c r="Y14" s="302" t="n"/>
+      <c r="Y14" s="320" t="n"/>
       <c r="Z14" s="300" t="n"/>
     </row>
     <row r="15" ht="104" customHeight="1">
@@ -15014,12 +15010,12 @@
           <t>Maçaneta Sara cromo acetinado. Ref.: Pado. (PR408)</t>
         </is>
       </c>
-      <c r="X15" s="302" t="inlineStr">
+      <c r="X15" s="320" t="inlineStr">
         <is>
           <t>38 - Porta em marcenaria piso-forro, cor branca, alizar 10cm. (PR408)</t>
         </is>
       </c>
-      <c r="Y15" s="302" t="n"/>
+      <c r="Y15" s="320" t="n"/>
       <c r="Z15" s="300" t="n"/>
     </row>
     <row r="16" ht="74" customHeight="1">
@@ -15094,8 +15090,8 @@
       <c r="U16" s="300" t="n"/>
       <c r="V16" s="300" t="n"/>
       <c r="W16" s="300" t="n"/>
-      <c r="X16" s="302" t="n"/>
-      <c r="Y16" s="302" t="n"/>
+      <c r="X16" s="320" t="n"/>
+      <c r="Y16" s="320" t="n"/>
       <c r="Z16" s="300" t="n"/>
     </row>
     <row r="17" ht="89" customHeight="1">
@@ -15143,8 +15139,8 @@
       <c r="U17" s="300" t="n"/>
       <c r="V17" s="300" t="n"/>
       <c r="W17" s="300" t="n"/>
-      <c r="X17" s="302" t="n"/>
-      <c r="Y17" s="302" t="n"/>
+      <c r="X17" s="320" t="n"/>
+      <c r="Y17" s="320" t="n"/>
       <c r="Z17" s="300" t="n"/>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -15195,8 +15191,8 @@
       <c r="U18" s="300" t="n"/>
       <c r="V18" s="300" t="n"/>
       <c r="W18" s="300" t="n"/>
-      <c r="X18" s="302" t="n"/>
-      <c r="Y18" s="302" t="n"/>
+      <c r="X18" s="320" t="n"/>
+      <c r="Y18" s="320" t="n"/>
       <c r="Z18" s="300" t="n"/>
     </row>
     <row r="19" ht="74" customHeight="1">
@@ -15256,12 +15252,12 @@
       <c r="U19" s="300" t="n"/>
       <c r="V19" s="300" t="n"/>
       <c r="W19" s="300" t="n"/>
-      <c r="X19" s="302" t="inlineStr">
+      <c r="X19" s="320" t="inlineStr">
         <is>
           <t>Porta em marcenaria. (PR406/407)</t>
         </is>
       </c>
-      <c r="Y19" s="302" t="n"/>
+      <c r="Y19" s="320" t="n"/>
       <c r="Z19" s="300" t="n"/>
     </row>
     <row r="20" ht="74" customHeight="1">
@@ -15336,13 +15332,13 @@
           <t>Maçaneta Pado Sara, cromo acetinado, interna. Porta de segurança: fechadura digital FDE-600W. (DET PR005/PR006)</t>
         </is>
       </c>
-      <c r="X20" s="302" t="inlineStr">
+      <c r="X20" s="320" t="inlineStr">
         <is>
           <t>Porta piso-forro, cor branca, alizar 10cm
 Porta piso-forro especial de segurança, cor branca, alizar 10cm. (DET PR006)</t>
         </is>
       </c>
-      <c r="Y20" s="302" t="n"/>
+      <c r="Y20" s="320" t="n"/>
       <c r="Z20" s="300" t="n"/>
     </row>
     <row r="21" ht="60" customHeight="1">
@@ -15417,8 +15413,8 @@
       <c r="U21" s="300" t="n"/>
       <c r="V21" s="300" t="n"/>
       <c r="W21" s="300" t="n"/>
-      <c r="X21" s="302" t="n"/>
-      <c r="Y21" s="302" t="n"/>
+      <c r="X21" s="320" t="n"/>
+      <c r="Y21" s="320" t="n"/>
       <c r="Z21" s="300" t="n"/>
     </row>
     <row r="22" ht="60" customHeight="1">
@@ -15465,8 +15461,8 @@
       <c r="U22" s="300" t="n"/>
       <c r="V22" s="300" t="n"/>
       <c r="W22" s="300" t="n"/>
-      <c r="X22" s="302" t="n"/>
-      <c r="Y22" s="302" t="n"/>
+      <c r="X22" s="320" t="n"/>
+      <c r="Y22" s="320" t="n"/>
       <c r="Z22" s="300" t="n"/>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -15501,8 +15497,8 @@
       <c r="U23" s="300" t="n"/>
       <c r="V23" s="300" t="n"/>
       <c r="W23" s="300" t="n"/>
-      <c r="X23" s="302" t="n"/>
-      <c r="Y23" s="302" t="n"/>
+      <c r="X23" s="320" t="n"/>
+      <c r="Y23" s="320" t="n"/>
       <c r="Z23" s="300" t="n"/>
     </row>
     <row r="24" ht="60" customHeight="1">
@@ -15546,8 +15542,8 @@
       <c r="U24" s="300" t="n"/>
       <c r="V24" s="300" t="n"/>
       <c r="W24" s="300" t="n"/>
-      <c r="X24" s="302" t="n"/>
-      <c r="Y24" s="302" t="n"/>
+      <c r="X24" s="320" t="n"/>
+      <c r="Y24" s="320" t="n"/>
       <c r="Z24" s="300" t="n"/>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -15591,8 +15587,8 @@
       <c r="U25" s="300" t="n"/>
       <c r="V25" s="300" t="n"/>
       <c r="W25" s="300" t="n"/>
-      <c r="X25" s="302" t="n"/>
-      <c r="Y25" s="302" t="n"/>
+      <c r="X25" s="320" t="n"/>
+      <c r="Y25" s="320" t="n"/>
       <c r="Z25" s="300" t="n"/>
     </row>
     <row r="26" ht="89" customHeight="1">
@@ -15639,12 +15635,12 @@
       <c r="U26" s="300" t="n"/>
       <c r="V26" s="300" t="n"/>
       <c r="W26" s="300" t="n"/>
-      <c r="X26" s="302" t="inlineStr">
+      <c r="X26" s="320" t="inlineStr">
         <is>
           <t>PCF1, PCF2, PE-A, P13, P23, PA05, PCF3, P15A, P15C (vão 90x240cm); material não especificado nas pranchas de circulação. (PR721-728)</t>
         </is>
       </c>
-      <c r="Y26" s="302" t="n"/>
+      <c r="Y26" s="320" t="n"/>
       <c r="Z26" s="300" t="inlineStr">
         <is>
           <t>Sirene de alarme e botoeira; hidrante nos halls conforme projeto PCI. (PR722-728)</t>
@@ -15653,14 +15649,14 @@
     </row>
     <row r="27">
       <c r="A27" s="45" t="n"/>
-      <c r="B27" s="31" t="n"/>
+      <c r="B27" s="245" t="n"/>
       <c r="C27" s="32" t="n"/>
       <c r="D27" s="32" t="n"/>
       <c r="E27" s="32" t="n"/>
       <c r="F27" s="32" t="n"/>
       <c r="G27" s="32" t="n"/>
-      <c r="H27" s="33" t="n"/>
-      <c r="I27" s="33" t="n"/>
+      <c r="H27" s="246" t="n"/>
+      <c r="I27" s="246" t="n"/>
       <c r="J27" s="32" t="n"/>
       <c r="K27" s="32" t="n"/>
       <c r="L27" s="32" t="n"/>
@@ -15675,20 +15671,20 @@
       <c r="U27" s="32" t="n"/>
       <c r="V27" s="32" t="n"/>
       <c r="W27" s="32" t="n"/>
-      <c r="X27" s="31" t="n"/>
-      <c r="Y27" s="31" t="n"/>
+      <c r="X27" s="245" t="n"/>
+      <c r="Y27" s="245" t="n"/>
       <c r="Z27" s="32" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="45" t="n"/>
-      <c r="B28" s="31" t="n"/>
+      <c r="B28" s="245" t="n"/>
       <c r="C28" s="32" t="n"/>
       <c r="D28" s="32" t="n"/>
       <c r="E28" s="32" t="n"/>
       <c r="F28" s="32" t="n"/>
       <c r="G28" s="32" t="n"/>
-      <c r="H28" s="33" t="n"/>
-      <c r="I28" s="33" t="n"/>
+      <c r="H28" s="246" t="n"/>
+      <c r="I28" s="246" t="n"/>
       <c r="J28" s="32" t="n"/>
       <c r="K28" s="32" t="n"/>
       <c r="L28" s="32" t="n"/>
@@ -15703,20 +15699,20 @@
       <c r="U28" s="32" t="n"/>
       <c r="V28" s="32" t="n"/>
       <c r="W28" s="32" t="n"/>
-      <c r="X28" s="31" t="n"/>
-      <c r="Y28" s="31" t="n"/>
+      <c r="X28" s="245" t="n"/>
+      <c r="Y28" s="245" t="n"/>
       <c r="Z28" s="32" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="45" t="n"/>
-      <c r="B29" s="31" t="n"/>
+      <c r="B29" s="245" t="n"/>
       <c r="C29" s="32" t="n"/>
       <c r="D29" s="32" t="n"/>
       <c r="E29" s="32" t="n"/>
       <c r="F29" s="32" t="n"/>
       <c r="G29" s="32" t="n"/>
-      <c r="H29" s="33" t="n"/>
-      <c r="I29" s="33" t="n"/>
+      <c r="H29" s="246" t="n"/>
+      <c r="I29" s="246" t="n"/>
       <c r="J29" s="32" t="n"/>
       <c r="K29" s="32" t="n"/>
       <c r="L29" s="32" t="n"/>
@@ -15731,20 +15727,20 @@
       <c r="U29" s="32" t="n"/>
       <c r="V29" s="32" t="n"/>
       <c r="W29" s="32" t="n"/>
-      <c r="X29" s="31" t="n"/>
-      <c r="Y29" s="31" t="n"/>
+      <c r="X29" s="245" t="n"/>
+      <c r="Y29" s="245" t="n"/>
       <c r="Z29" s="32" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="45" t="n"/>
-      <c r="B30" s="31" t="n"/>
+      <c r="B30" s="245" t="n"/>
       <c r="C30" s="32" t="n"/>
       <c r="D30" s="32" t="n"/>
       <c r="E30" s="32" t="n"/>
       <c r="F30" s="32" t="n"/>
       <c r="G30" s="32" t="n"/>
-      <c r="H30" s="33" t="n"/>
-      <c r="I30" s="33" t="n"/>
+      <c r="H30" s="246" t="n"/>
+      <c r="I30" s="246" t="n"/>
       <c r="J30" s="32" t="n"/>
       <c r="K30" s="32" t="n"/>
       <c r="L30" s="32" t="n"/>
@@ -15759,20 +15755,20 @@
       <c r="U30" s="32" t="n"/>
       <c r="V30" s="32" t="n"/>
       <c r="W30" s="32" t="n"/>
-      <c r="X30" s="31" t="n"/>
-      <c r="Y30" s="31" t="n"/>
+      <c r="X30" s="245" t="n"/>
+      <c r="Y30" s="245" t="n"/>
       <c r="Z30" s="32" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="45" t="n"/>
-      <c r="B31" s="31" t="n"/>
+      <c r="B31" s="245" t="n"/>
       <c r="C31" s="32" t="n"/>
       <c r="D31" s="32" t="n"/>
       <c r="E31" s="32" t="n"/>
       <c r="F31" s="32" t="n"/>
       <c r="G31" s="32" t="n"/>
-      <c r="H31" s="33" t="n"/>
-      <c r="I31" s="33" t="n"/>
+      <c r="H31" s="246" t="n"/>
+      <c r="I31" s="246" t="n"/>
       <c r="J31" s="32" t="n"/>
       <c r="K31" s="32" t="n"/>
       <c r="L31" s="32" t="n"/>
@@ -15787,8 +15783,8 @@
       <c r="U31" s="32" t="n"/>
       <c r="V31" s="32" t="n"/>
       <c r="W31" s="32" t="n"/>
-      <c r="X31" s="31" t="n"/>
-      <c r="Y31" s="31" t="n"/>
+      <c r="X31" s="245" t="n"/>
+      <c r="Y31" s="245" t="n"/>
       <c r="Z31" s="32" t="n"/>
     </row>
     <row r="32"/>
@@ -16074,7 +16070,7 @@
       </c>
       <c r="H8" s="331" t="inlineStr"/>
     </row>
-    <row r="9" ht="87" customHeight="1">
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="331" t="n">
         <v>5</v>
       </c>
@@ -16105,7 +16101,7 @@
       </c>
       <c r="G9" s="334" t="inlineStr">
         <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
 CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
@@ -16148,7 +16144,7 @@
       </c>
       <c r="H10" s="331" t="inlineStr"/>
     </row>
-    <row r="11" ht="87" customHeight="1">
+    <row r="11" ht="72" customHeight="1">
       <c r="A11" s="331" t="n">
         <v>7</v>
       </c>
@@ -16179,7 +16175,7 @@
       </c>
       <c r="G11" s="334" t="inlineStr">
         <is>
-          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca  ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
+          <t>D29 - Torneira de mesa com sensor bivolt e bateria, linha Decalux, acabamento cromado, cód.: 1188.C.N. Ref.: Deca ATENÇÃO: vazão máxima de 6 l/min, instalar restritor de vazão se necessário.
 CONFLITO – Pranchas 37 e 38 do detalhamento R04: torneira de mesa bica baixa Argon, Docol</t>
         </is>
       </c>
@@ -16277,7 +16273,7 @@
     <row r="2">
       <c r="A2" s="264" t="inlineStr">
         <is>
-          <t>Fonte: Tabela de acabamentos Ed. Cidade Jardim v00 (19/06/2026). Emissão 30/09/2026, REV. R00.</t>
+          <t>Fontes: Tabela de acabamentos Ed. Cidade Jardim v00 (19/06/2026); detalhamento de interiores R04 (23/04/2026); plantas de arquitetura CDJ-ARQ-EX PR003–PR013; apartamento tipo: tabela JARDIM-ACABAMENTOS R01 e detalhamento. Emissão 30/09/2026, REV. R00.</t>
         </is>
       </c>
     </row>
@@ -16657,7 +16653,7 @@
       </c>
       <c r="D19" s="268" t="inlineStr">
         <is>
-          <t>Referência grafada "Khali pff white". Considerado Khali off white AC (Eliane).</t>
+          <t>Referência grafada "Khali off white". Considerado Khali off white AC (Eliane).</t>
         </is>
       </c>
       <c r="E19" s="268" t="inlineStr">
@@ -16732,12 +16728,12 @@
       </c>
       <c r="D22" s="268" t="inlineStr">
         <is>
-          <t>A tabela v00 só traz o 3º pavimento - Pilotis. Abas mantidas sem preenchimento.</t>
+          <t>A tabela v00 só traz o 3º pavimento - Pilotis. As abas foram preenchidas pelo detalhamento R04 e pelas plantas de arquitetura (ver itens 5 e 7).</t>
         </is>
       </c>
       <c r="E22" s="268" t="inlineStr">
         <is>
-          <t>Tabela v00</t>
+          <t>Tabela v00 → R04 e arquitetura</t>
         </is>
       </c>
     </row>
@@ -16746,7 +16742,7 @@
     <row r="25">
       <c r="A25" s="265" t="inlineStr">
         <is>
-          <t>2. AMBIENTES DO MODELO (PILOTIS) SEM INFORMAÇÃO NA TABELA</t>
+          <t>2. AMBIENTES DO MODELO (PILOTIS) SEM INFORMAÇÃO NA TABELA V00 — SITUAÇÃO ATUAL</t>
         </is>
       </c>
     </row>
@@ -16761,9 +16757,13 @@
           <t>AMBIENTE NO MODELO</t>
         </is>
       </c>
-      <c r="C26" s="266" t="inlineStr"/>
-      <c r="D26" s="266" t="inlineStr"/>
-      <c r="E26" s="266" t="inlineStr"/>
+      <c r="C26" s="266" t="n"/>
+      <c r="D26" s="266" t="inlineStr">
+        <is>
+          <t>SITUAÇÃO</t>
+        </is>
+      </c>
+      <c r="E26" s="266" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="267" t="n">
@@ -16774,13 +16774,13 @@
           <t>TERRAÇO SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="C27" s="268" t="inlineStr"/>
+      <c r="C27" s="268" t="n"/>
       <c r="D27" s="268" t="inlineStr">
         <is>
           <t>Tabela v00 e detalhamento R04 sem especificação de acabamento (a lista R04 só traz códigos sem descrição para "Varanda, terraço, piscina e prainha, braseiro"). A planta de arquitetura PR011 indica piso ○08 (ARQ-P08, lançado na grade) e guarda-corpos GC06/GC07 h=130cm. Sem indicação de rodapé, parede ou teto.</t>
         </is>
       </c>
-      <c r="E27" s="268" t="inlineStr"/>
+      <c r="E27" s="268" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="267" t="n">
@@ -16791,9 +16791,13 @@
           <t>CIRCULAÇÃO SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="C28" s="268" t="inlineStr"/>
-      <c r="D28" s="268" t="inlineStr"/>
-      <c r="E28" s="268" t="inlineStr"/>
+      <c r="C28" s="268" t="n"/>
+      <c r="D28" s="268" t="inlineStr">
+        <is>
+          <t>Sem especificação em nenhuma fonte recebida (tabela v00, detalhamento R04 e plantas de arquitetura sem etiqueta). Definir.</t>
+        </is>
+      </c>
+      <c r="E28" s="268" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="267" t="n">
@@ -16804,9 +16808,13 @@
           <t>APOIO COZINHA</t>
         </is>
       </c>
-      <c r="C29" s="268" t="inlineStr"/>
-      <c r="D29" s="268" t="inlineStr"/>
-      <c r="E29" s="268" t="inlineStr"/>
+      <c r="C29" s="268" t="n"/>
+      <c r="D29" s="268" t="inlineStr">
+        <is>
+          <t>Sem especificação em nenhuma fonte recebida (tabela v00, detalhamento R04 e plantas de arquitetura sem etiqueta). Definir.</t>
+        </is>
+      </c>
+      <c r="E29" s="268" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="267" t="n">
@@ -16817,9 +16825,13 @@
           <t>CIRCULAÇÃO/ANTECÂMARA ELEVADOR SERVIÇO</t>
         </is>
       </c>
-      <c r="C30" s="268" t="inlineStr"/>
-      <c r="D30" s="268" t="inlineStr"/>
-      <c r="E30" s="268" t="inlineStr"/>
+      <c r="C30" s="268" t="n"/>
+      <c r="D30" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E30" s="268" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="267" t="n">
@@ -16830,9 +16842,13 @@
           <t>CIRCULAÇÃO LAVABOS</t>
         </is>
       </c>
-      <c r="C31" s="268" t="inlineStr"/>
-      <c r="D31" s="268" t="inlineStr"/>
-      <c r="E31" s="268" t="inlineStr"/>
+      <c r="C31" s="268" t="n"/>
+      <c r="D31" s="268" t="inlineStr">
+        <is>
+          <t>Sem especificação em nenhuma fonte recebida (tabela v00, detalhamento R04 e plantas de arquitetura sem etiqueta). Definir.</t>
+        </is>
+      </c>
+      <c r="E31" s="268" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="267" t="n">
@@ -16843,9 +16859,13 @@
           <t>VARANDA</t>
         </is>
       </c>
-      <c r="C32" s="268" t="inlineStr"/>
-      <c r="D32" s="268" t="inlineStr"/>
-      <c r="E32" s="268" t="inlineStr"/>
+      <c r="C32" s="268" t="n"/>
+      <c r="D32" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E32" s="268" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="267" t="n">
@@ -16856,9 +16876,13 @@
           <t>PLAYGROUND</t>
         </is>
       </c>
-      <c r="C33" s="268" t="inlineStr"/>
-      <c r="D33" s="268" t="inlineStr"/>
-      <c r="E33" s="268" t="inlineStr"/>
+      <c r="C33" s="268" t="n"/>
+      <c r="D33" s="268" t="inlineStr">
+        <is>
+          <t>Sem especificação em nenhuma fonte recebida (tabela v00, detalhamento R04 e plantas de arquitetura sem etiqueta). Definir.</t>
+        </is>
+      </c>
+      <c r="E33" s="268" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="267" t="n">
@@ -16869,9 +16893,13 @@
           <t>BAR PISCINA</t>
         </is>
       </c>
-      <c r="C34" s="268" t="inlineStr"/>
-      <c r="D34" s="268" t="inlineStr"/>
-      <c r="E34" s="268" t="inlineStr"/>
+      <c r="C34" s="268" t="n"/>
+      <c r="D34" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E34" s="268" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="267" t="n">
@@ -16882,9 +16910,13 @@
           <t>CIRCULAÇÃO PLAYGROUND</t>
         </is>
       </c>
-      <c r="C35" s="268" t="inlineStr"/>
-      <c r="D35" s="268" t="inlineStr"/>
-      <c r="E35" s="268" t="inlineStr"/>
+      <c r="C35" s="268" t="n"/>
+      <c r="D35" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E35" s="268" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="267" t="n">
@@ -16895,9 +16927,13 @@
           <t>CIRCULAÇÃO VESTIÁRIOS</t>
         </is>
       </c>
-      <c r="C36" s="268" t="inlineStr"/>
-      <c r="D36" s="268" t="inlineStr"/>
-      <c r="E36" s="268" t="inlineStr"/>
+      <c r="C36" s="268" t="n"/>
+      <c r="D36" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E36" s="268" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="267" t="n">
@@ -16908,9 +16944,13 @@
           <t>CIRCULAÇÃO JARDINS</t>
         </is>
       </c>
-      <c r="C37" s="268" t="inlineStr"/>
-      <c r="D37" s="268" t="inlineStr"/>
-      <c r="E37" s="268" t="inlineStr"/>
+      <c r="C37" s="268" t="n"/>
+      <c r="D37" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E37" s="268" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="267" t="n">
@@ -16921,9 +16961,13 @@
           <t>CIRCULAÇÃO MASSAGEM/BELEZA</t>
         </is>
       </c>
-      <c r="C38" s="268" t="inlineStr"/>
-      <c r="D38" s="268" t="inlineStr"/>
-      <c r="E38" s="268" t="inlineStr"/>
+      <c r="C38" s="268" t="n"/>
+      <c r="D38" s="268" t="inlineStr">
+        <is>
+          <t>Sem especificação em nenhuma fonte recebida (tabela v00, detalhamento R04 e plantas de arquitetura sem etiqueta). Definir.</t>
+        </is>
+      </c>
+      <c r="E38" s="268" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="267" t="n">
@@ -16934,9 +16978,13 @@
           <t>HALL VESTIÁRIOS</t>
         </is>
       </c>
-      <c r="C39" s="268" t="inlineStr"/>
-      <c r="D39" s="268" t="inlineStr"/>
-      <c r="E39" s="268" t="inlineStr"/>
+      <c r="C39" s="268" t="n"/>
+      <c r="D39" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E39" s="268" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="267" t="n">
@@ -16947,9 +16995,13 @@
           <t>VEST. P.C.D</t>
         </is>
       </c>
-      <c r="C40" s="268" t="inlineStr"/>
-      <c r="D40" s="268" t="inlineStr"/>
-      <c r="E40" s="268" t="inlineStr"/>
+      <c r="C40" s="268" t="n"/>
+      <c r="D40" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E40" s="268" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="267" t="n">
@@ -16960,9 +17012,13 @@
           <t>VEST. P.C.D</t>
         </is>
       </c>
-      <c r="C41" s="268" t="inlineStr"/>
-      <c r="D41" s="268" t="inlineStr"/>
-      <c r="E41" s="268" t="inlineStr"/>
+      <c r="C41" s="268" t="n"/>
+      <c r="D41" s="268" t="inlineStr">
+        <is>
+          <t>Preenchido pelo detalhamento R04 e/ou pelas plantas de arquitetura.</t>
+        </is>
+      </c>
+      <c r="E41" s="268" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="267" t="n">
@@ -16973,9 +17029,13 @@
           <t>LOUNGE QUADRAS</t>
         </is>
       </c>
-      <c r="C42" s="268" t="inlineStr"/>
-      <c r="D42" s="268" t="inlineStr"/>
-      <c r="E42" s="268" t="inlineStr"/>
+      <c r="C42" s="268" t="n"/>
+      <c r="D42" s="268" t="inlineStr">
+        <is>
+          <t>Sem especificação em nenhuma fonte recebida (tabela v00, detalhamento R04 e plantas de arquitetura sem etiqueta). Definir.</t>
+        </is>
+      </c>
+      <c r="E42" s="268" t="n"/>
     </row>
     <row r="43"/>
     <row r="44"/>
@@ -17002,8 +17062,8 @@
           <t>LINHA(S) NA GRADE</t>
         </is>
       </c>
-      <c r="D46" s="266" t="inlineStr"/>
-      <c r="E46" s="266" t="inlineStr"/>
+      <c r="D46" s="266" t="n"/>
+      <c r="E46" s="266" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="267" t="n">
@@ -17019,8 +17079,8 @@
           <t>LOBBY PILOTIS</t>
         </is>
       </c>
-      <c r="D47" s="268" t="inlineStr"/>
-      <c r="E47" s="268" t="inlineStr"/>
+      <c r="D47" s="268" t="n"/>
+      <c r="E47" s="268" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="267" t="n">
@@ -17036,8 +17096,8 @@
           <t>SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="D48" s="268" t="inlineStr"/>
-      <c r="E48" s="268" t="inlineStr"/>
+      <c r="D48" s="268" t="n"/>
+      <c r="E48" s="268" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="267" t="n">
@@ -17053,8 +17113,8 @@
           <t>I.S FEMININO, I.S MASCULINO</t>
         </is>
       </c>
-      <c r="D49" s="268" t="inlineStr"/>
-      <c r="E49" s="268" t="inlineStr"/>
+      <c r="D49" s="268" t="n"/>
+      <c r="E49" s="268" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="267" t="n">
@@ -17070,8 +17130,8 @@
           <t>COZINHA SALÃO DE FESTAS</t>
         </is>
       </c>
-      <c r="D50" s="268" t="inlineStr"/>
-      <c r="E50" s="268" t="inlineStr"/>
+      <c r="D50" s="268" t="n"/>
+      <c r="E50" s="268" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="267" t="n">
@@ -17087,8 +17147,8 @@
           <t>DML</t>
         </is>
       </c>
-      <c r="D51" s="268" t="inlineStr"/>
-      <c r="E51" s="268" t="inlineStr"/>
+      <c r="D51" s="268" t="n"/>
+      <c r="E51" s="268" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="267" t="n">
@@ -17104,8 +17164,8 @@
           <t>I.S P.C.D, I.S</t>
         </is>
       </c>
-      <c r="D52" s="268" t="inlineStr"/>
-      <c r="E52" s="268" t="inlineStr"/>
+      <c r="D52" s="268" t="n"/>
+      <c r="E52" s="268" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="267" t="n">
@@ -17121,8 +17181,8 @@
           <t>ESPAÇO KIDS</t>
         </is>
       </c>
-      <c r="D53" s="268" t="inlineStr"/>
-      <c r="E53" s="268" t="inlineStr"/>
+      <c r="D53" s="268" t="n"/>
+      <c r="E53" s="268" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="267" t="n">
@@ -17138,8 +17198,8 @@
           <t>ESPAÇO GOURMET</t>
         </is>
       </c>
-      <c r="D54" s="268" t="inlineStr"/>
-      <c r="E54" s="268" t="inlineStr"/>
+      <c r="D54" s="268" t="n"/>
+      <c r="E54" s="268" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="267" t="n">
@@ -17152,11 +17212,11 @@
       </c>
       <c r="C55" s="268" t="inlineStr">
         <is>
-          <t>PISCINA DECOBERTA</t>
-        </is>
-      </c>
-      <c r="D55" s="268" t="inlineStr"/>
-      <c r="E55" s="268" t="inlineStr"/>
+          <t>PISCINA DESCOBERTA</t>
+        </is>
+      </c>
+      <c r="D55" s="268" t="n"/>
+      <c r="E55" s="268" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="267" t="n">
@@ -17172,8 +17232,8 @@
           <t>DECK</t>
         </is>
       </c>
-      <c r="D56" s="268" t="inlineStr"/>
-      <c r="E56" s="268" t="inlineStr"/>
+      <c r="D56" s="268" t="n"/>
+      <c r="E56" s="268" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="267" t="n">
@@ -17189,8 +17249,8 @@
           <t>VESTIÁRIO FEMININO, VESTIÁRIO MASCULINO</t>
         </is>
       </c>
-      <c r="D57" s="268" t="inlineStr"/>
-      <c r="E57" s="268" t="inlineStr"/>
+      <c r="D57" s="268" t="n"/>
+      <c r="E57" s="268" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="267" t="n">
@@ -17206,8 +17266,8 @@
           <t>ACADEMIA</t>
         </is>
       </c>
-      <c r="D58" s="268" t="inlineStr"/>
-      <c r="E58" s="268" t="inlineStr"/>
+      <c r="D58" s="268" t="n"/>
+      <c r="E58" s="268" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="267" t="n">
@@ -17223,8 +17283,8 @@
           <t>PISCINA RAIA, SPA</t>
         </is>
       </c>
-      <c r="D59" s="268" t="inlineStr"/>
-      <c r="E59" s="268" t="inlineStr"/>
+      <c r="D59" s="268" t="n"/>
+      <c r="E59" s="268" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="267" t="n">
@@ -17240,8 +17300,8 @@
           <t>ESPAÇO TERMAS</t>
         </is>
       </c>
-      <c r="D60" s="268" t="inlineStr"/>
-      <c r="E60" s="268" t="inlineStr"/>
+      <c r="D60" s="268" t="n"/>
+      <c r="E60" s="268" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="267" t="n">
@@ -17257,8 +17317,8 @@
           <t>SAUNA VAPOR</t>
         </is>
       </c>
-      <c r="D61" s="268" t="inlineStr"/>
-      <c r="E61" s="268" t="inlineStr"/>
+      <c r="D61" s="268" t="n"/>
+      <c r="E61" s="268" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="267" t="n">
@@ -17274,8 +17334,8 @@
           <t>SAUNA SECA</t>
         </is>
       </c>
-      <c r="D62" s="268" t="inlineStr"/>
-      <c r="E62" s="268" t="inlineStr"/>
+      <c r="D62" s="268" t="n"/>
+      <c r="E62" s="268" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="267" t="n">
@@ -17291,8 +17351,8 @@
           <t>MASSAGEM</t>
         </is>
       </c>
-      <c r="D63" s="268" t="inlineStr"/>
-      <c r="E63" s="268" t="inlineStr"/>
+      <c r="D63" s="268" t="n"/>
+      <c r="E63" s="268" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="267" t="n">
@@ -17308,8 +17368,8 @@
           <t>BELEZA</t>
         </is>
       </c>
-      <c r="D64" s="268" t="inlineStr"/>
-      <c r="E64" s="268" t="inlineStr"/>
+      <c r="D64" s="268" t="n"/>
+      <c r="E64" s="268" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="267" t="n">
@@ -17325,8 +17385,8 @@
           <t>QUADRA TÊNIS</t>
         </is>
       </c>
-      <c r="D65" s="268" t="inlineStr"/>
-      <c r="E65" s="268" t="inlineStr"/>
+      <c r="D65" s="268" t="n"/>
+      <c r="E65" s="268" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="267" t="n">
@@ -17342,8 +17402,8 @@
           <t>DEP JARDIM, DEPÓSITO</t>
         </is>
       </c>
-      <c r="D66" s="268" t="inlineStr"/>
-      <c r="E66" s="268" t="inlineStr"/>
+      <c r="D66" s="268" t="n"/>
+      <c r="E66" s="268" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="267" t="n">
@@ -17359,8 +17419,8 @@
           <t>VESTIÁRIO FEM./MASC. - TERMAS (linha nova)</t>
         </is>
       </c>
-      <c r="D67" s="268" t="inlineStr"/>
-      <c r="E67" s="268" t="inlineStr"/>
+      <c r="D67" s="268" t="n"/>
+      <c r="E67" s="268" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="267" t="n">
@@ -17376,8 +17436,8 @@
           <t>ESCADA DE INCÊNDIO (linha nova)</t>
         </is>
       </c>
-      <c r="D68" s="268" t="inlineStr"/>
-      <c r="E68" s="268" t="inlineStr"/>
+      <c r="D68" s="268" t="n"/>
+      <c r="E68" s="268" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="267" t="n">
@@ -17393,8 +17453,8 @@
           <t>ANTECÂMARA (linha nova)</t>
         </is>
       </c>
-      <c r="D69" s="268" t="inlineStr"/>
-      <c r="E69" s="268" t="inlineStr"/>
+      <c r="D69" s="268" t="n"/>
+      <c r="E69" s="268" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="267" t="n">
@@ -17410,8 +17470,8 @@
           <t>CIRCULAÇÃO (linha nova)</t>
         </is>
       </c>
-      <c r="D70" s="268" t="inlineStr"/>
-      <c r="E70" s="268" t="inlineStr"/>
+      <c r="D70" s="268" t="n"/>
+      <c r="E70" s="268" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="267" t="n">
@@ -17427,8 +17487,8 @@
           <t>ESTAR PISCINA / CIRCULAÇÃO (linha nova)</t>
         </is>
       </c>
-      <c r="D71" s="268" t="inlineStr"/>
-      <c r="E71" s="268" t="inlineStr"/>
+      <c r="D71" s="268" t="n"/>
+      <c r="E71" s="268" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="267" t="n">
@@ -17444,8 +17504,8 @@
           <t>CIRCULAÇÃO EXTERNA COBERTA/DESCOBERTA E VARANDA ESPAÇO KIDS (linha nova)</t>
         </is>
       </c>
-      <c r="D72" s="268" t="inlineStr"/>
-      <c r="E72" s="268" t="inlineStr"/>
+      <c r="D72" s="268" t="n"/>
+      <c r="E72" s="268" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="267" t="n">
@@ -17461,8 +17521,8 @@
           <t>ESCADA EXTERNA (linha nova)</t>
         </is>
       </c>
-      <c r="D73" s="268" t="inlineStr"/>
-      <c r="E73" s="268" t="inlineStr"/>
+      <c r="D73" s="268" t="n"/>
+      <c r="E73" s="268" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="267" t="n">
@@ -17478,8 +17538,8 @@
           <t>QUADRA INFANTIL (linha nova)</t>
         </is>
       </c>
-      <c r="D74" s="268" t="inlineStr"/>
-      <c r="E74" s="268" t="inlineStr"/>
+      <c r="D74" s="268" t="n"/>
+      <c r="E74" s="268" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="267" t="n">
@@ -17495,8 +17555,8 @@
           <t>APOIO QUADRAS (linha nova)</t>
         </is>
       </c>
-      <c r="D75" s="268" t="inlineStr"/>
-      <c r="E75" s="268" t="inlineStr"/>
+      <c r="D75" s="268" t="n"/>
+      <c r="E75" s="268" t="n"/>
     </row>
     <row r="76"/>
     <row r="77"/>
@@ -17528,7 +17588,7 @@
           <t>CRITÉRIO</t>
         </is>
       </c>
-      <c r="E79" s="266" t="inlineStr"/>
+      <c r="E79" s="266" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="267" t="n">
@@ -17549,7 +17609,7 @@
           <t>Transcrição direta.</t>
         </is>
       </c>
-      <c r="E80" s="268" t="inlineStr"/>
+      <c r="E80" s="268" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="267" t="n">
@@ -17570,7 +17630,7 @@
           <t>Revestimentos e pinturas (códigos PA, 01, 06, 09, 12...).</t>
         </is>
       </c>
-      <c r="E81" s="268" t="inlineStr"/>
+      <c r="E81" s="268" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="267" t="n">
@@ -17591,7 +17651,7 @@
           <t>Espelhos sobre armário, fechamentos e painéis decorativos (códigos D), perfis de transição.</t>
         </is>
       </c>
-      <c r="E82" s="268" t="inlineStr"/>
+      <c r="E82" s="268" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="267" t="n">
@@ -17612,7 +17672,7 @@
           <t>P28 (D43) - painel e porta em alumínio e vidro (Massagem).</t>
         </is>
       </c>
-      <c r="E83" s="268" t="inlineStr"/>
+      <c r="E83" s="268" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="267" t="n">
@@ -17633,7 +17693,7 @@
           <t>Bancadas em BANCADA; prateleira e testeira em OUTROS REVESTIMENTOS.</t>
         </is>
       </c>
-      <c r="E84" s="268" t="inlineStr"/>
+      <c r="E84" s="268" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="267" t="n">
@@ -17654,7 +17714,7 @@
           <t>Separado por item; chuveiros em OUTROS LOUÇAS E METAIS.</t>
         </is>
       </c>
-      <c r="E85" s="268" t="inlineStr"/>
+      <c r="E85" s="268" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="267" t="n">
@@ -17675,13 +17735,13 @@
           <t>Ralos em RALOS; saboneteira, porta-papel e papeleira em OUTROS COMPLEMENTARES.</t>
         </is>
       </c>
-      <c r="E86" s="268" t="inlineStr"/>
+      <c r="E86" s="268" t="n"/>
     </row>
     <row r="87"/>
     <row r="88">
       <c r="A88" s="279" t="inlineStr">
         <is>
-          <t>3. LEVANTAMENTO PELOS PROJETOS DE DETALHAMENTO R04 (23/04/2026)</t>
+          <t>5. LEVANTAMENTO PELOS PROJETOS DE DETALHAMENTO R04 (23/04/2026)</t>
         </is>
       </c>
     </row>
@@ -18943,7 +19003,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>PILOTIS – PISCINA DECOBERTA</t>
+          <t>PILOTIS – PISCINA DESCOBERTA</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -18968,7 +19028,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PILOTIS – PISCINA DECOBERTA</t>
+          <t>PILOTIS – PISCINA DESCOBERTA</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -18993,7 +19053,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>PILOTIS – PISCINA DECOBERTA</t>
+          <t>PILOTIS – PISCINA DESCOBERTA</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -19018,12 +19078,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>PILOTIS – PISCINA DECOBERTA</t>
+          <t>PILOTIS – PISCINA DESCOBERTA</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>OUTROS  LOUÇAS E METAIS</t>
+          <t>OUTROS LOUÇAS E METAIS</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -19043,7 +19103,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>PILOTIS – PISCINA DECOBERTA</t>
+          <t>PILOTIS – PISCINA DESCOBERTA</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -19068,7 +19128,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>PILOTIS – PISCINA DECOBERTA</t>
+          <t>PILOTIS – PISCINA DESCOBERTA</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -20323,7 +20383,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>OUTROS  LOUÇAS E METAIS</t>
+          <t>OUTROS LOUÇAS E METAIS</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -21073,7 +21133,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>OUTROS  LOUÇAS E METAIS</t>
+          <t>OUTROS LOUÇAS E METAIS</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -21473,7 +21533,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>OUTROS  LOUÇAS E METAIS</t>
+          <t>OUTROS LOUÇAS E METAIS</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -22693,7 +22753,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>TÉRREO – HALL GARGEM</t>
+          <t>TÉRREO – HALL GARAGEM</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -22718,7 +22778,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>TÉRREO – HALL GARGEM</t>
+          <t>TÉRREO – HALL GARAGEM</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -22743,7 +22803,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>TÉRREO – HALL GARGEM</t>
+          <t>TÉRREO – HALL GARAGEM</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -22768,7 +22828,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>TÉRREO – HALL GARGEM</t>
+          <t>TÉRREO – HALL GARAGEM</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -22793,7 +22853,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>TÉRREO – HALL GARGEM</t>
+          <t>TÉRREO – HALL GARAGEM</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -22818,7 +22878,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>TÉRREO – HALL GARGEM</t>
+          <t>TÉRREO – HALL GARAGEM</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -22843,7 +22903,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>TÉRREO – HALL GARGEM</t>
+          <t>TÉRREO – HALL GARAGEM</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -23316,7 +23376,7 @@
     <row r="315">
       <c r="A315" s="279" t="inlineStr">
         <is>
-          <t>4. OBSERVAÇÕES DO LEVANTAMENTO R04</t>
+          <t>6. OBSERVAÇÕES DO LEVANTAMENTO R04</t>
         </is>
       </c>
     </row>
@@ -23444,7 +23504,7 @@
     <row r="327">
       <c r="A327" s="279" t="inlineStr">
         <is>
-          <t>5. ESPECIFICAÇÕES DAS PLANTAS DE ARQUITETURA (CDJ-ARQ-EX PR003–PR013, Quadro de Especificações - Geral)</t>
+          <t>7. ESPECIFICAÇÕES DAS PLANTAS DE ARQUITETURA (CDJ-ARQ-EX PR003–PR013, Quadro de Especificações - Geral)</t>
         </is>
       </c>
     </row>
@@ -23781,7 +23841,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTICÂRA</t>
+          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTECÂMARA</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -23806,7 +23866,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTICÂRA</t>
+          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTECÂMARA</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -23831,7 +23891,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTICÂRA</t>
+          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTECÂMARA</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -23856,7 +23916,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTICÂRA</t>
+          <t>TÉRREO – CIRCULAÇÃO ELEVADOR DE SERVIÇO/ANTECÂMARA</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -28016,7 +28076,7 @@
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali pff white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII | 01| 21 - Pintura acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil, sobre paredes - Reboco (1 demão selador + 3 demãos Latex acrílico)</t>
+          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali off white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII | 01| 21 - Pintura acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil, sobre paredes - Reboco (1 demão selador + 3 demãos Latex acrílico)</t>
         </is>
       </c>
       <c r="E510" t="inlineStr">
@@ -28116,7 +28176,7 @@
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali pff white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII | 01| 21 - Pintura acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil, sobre paredes - Reboco (1 demão selador + 3 demãos Latex acrílico)</t>
+          <t>12 - Revestimento Porcelanato off white 60x60cm, espessura 1cm, com acabamento acetinado, Ref.: Khali off white AC, linha Khali; Eliane, assentado com argamassa colante em pó ACIII | 01| 21 - Pintura acrílica, cor branco neve, acabamento acetinado. Ref.: Suvinil, sobre paredes - Reboco (1 demão selador + 3 demãos Latex acrílico)</t>
         </is>
       </c>
       <c r="E514" t="inlineStr">
@@ -28440,7 +28500,7 @@
     <row r="534">
       <c r="A534" s="279" t="inlineStr">
         <is>
-          <t>6. APARTAMENTO TIPO (pasta DTL - DETALHAMENTO / APARTAMENTOS)</t>
+          <t>8. APARTAMENTO TIPO (pasta DTL - DETALHAMENTO / APARTAMENTOS)</t>
         </is>
       </c>
     </row>
@@ -28568,7 +28628,7 @@
     <row r="546">
       <c r="A546" s="279" t="inlineStr">
         <is>
-          <t>7. CONFERÊNCIA VISUAL DAS PLANTAS DE ARQUITETURA (02/10/2026)</t>
+          <t>9. CONFERÊNCIA VISUAL DAS PLANTAS DE ARQUITETURA (02/10/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>